<commit_message>
- parsed data from `10.1016/j.actamat.2026.122256`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91878973-5344-0442-AF3D-CD96FEF56F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{422A6709-19E1-FA4D-9CEC-55DCBB9E83FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="85">
   <si>
     <r>
       <rPr>
@@ -318,7 +318,73 @@
     <t>hardness HV</t>
   </si>
   <si>
+    <t>BCC</t>
+  </si>
+  <si>
+    <t>1e-3 strain rate</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>tensile yield stress</t>
+  </si>
+  <si>
+    <t>tensile ductility</t>
+  </si>
+  <si>
+    <t>UTS</t>
+  </si>
+  <si>
+    <t>F5a</t>
+  </si>
+  <si>
     <t>ak@ainm.io</t>
+  </si>
+  <si>
+    <t>Ni43.9 Co17 Fe12 Cr9 Al18 B0.1</t>
+  </si>
+  <si>
+    <t>Eutectic alloy designed with CALPHAD to be FCC+B2</t>
+  </si>
+  <si>
+    <t>RAC</t>
+  </si>
+  <si>
+    <t>Eutectic alloy designed with CALPHAD to be FCC+B2; rolling and annealing cycles (RAC) processing with 5 cycles being cold rolled to 20% reduction and annealed at 1423K for 5min</t>
+  </si>
+  <si>
+    <t>RAC(A)+CR</t>
+  </si>
+  <si>
+    <t>FCC+B2</t>
+  </si>
+  <si>
+    <t>FCC+L10</t>
+  </si>
+  <si>
+    <t>Ni45.5 Co11.2 Cr3.6 Fe7.9 Al31.8</t>
+  </si>
+  <si>
+    <t>stacking fault energy</t>
+  </si>
+  <si>
+    <t>DFT</t>
+  </si>
+  <si>
+    <t>VASP</t>
+  </si>
+  <si>
+    <t>72 atom random supercell; based on 3D-APT composition measurement</t>
+  </si>
+  <si>
+    <t>J/m^2</t>
+  </si>
+  <si>
+    <t>10.1016/j.actamat.2026.122256</t>
   </si>
 </sst>
 </file>
@@ -2909,7 +2975,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="151" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="116"/>
@@ -3183,20 +3249,46 @@
       </c>
     </row>
     <row r="10" spans="1:20" ht="19.5" customHeight="1">
-      <c r="A10" s="29"/>
-      <c r="B10" s="65"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="69"/>
-      <c r="J10" s="34"/>
+      <c r="A10" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="66" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="66" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="67" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="69">
+        <v>298</v>
+      </c>
+      <c r="J10" s="34">
+        <v>630000000</v>
+      </c>
       <c r="K10" s="34"/>
-      <c r="L10" s="67"/>
-      <c r="M10" s="67"/>
-      <c r="N10" s="70"/>
+      <c r="L10" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N10" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O10" s="71"/>
       <c r="P10" s="72"/>
       <c r="Q10" s="72"/>
@@ -3205,20 +3297,46 @@
       <c r="T10" s="71"/>
     </row>
     <row r="11" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A11" s="29"/>
-      <c r="B11" s="65"/>
-      <c r="C11" s="66"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="67"/>
-      <c r="G11" s="67"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="69"/>
-      <c r="J11" s="34"/>
+      <c r="A11" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="66" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="65" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="67" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="69">
+        <v>298</v>
+      </c>
+      <c r="J11" s="34">
+        <v>720000000</v>
+      </c>
       <c r="K11" s="34"/>
-      <c r="L11" s="67"/>
-      <c r="M11" s="67"/>
-      <c r="N11" s="70"/>
+      <c r="L11" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N11" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O11" s="36"/>
       <c r="P11" s="37"/>
       <c r="Q11" s="37"/>
@@ -3227,20 +3345,46 @@
       <c r="T11" s="36"/>
     </row>
     <row r="12" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A12" s="29"/>
-      <c r="B12" s="65"/>
-      <c r="C12" s="66"/>
-      <c r="D12" s="66"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="67"/>
-      <c r="G12" s="67"/>
-      <c r="H12" s="68"/>
-      <c r="I12" s="69"/>
-      <c r="J12" s="34"/>
+      <c r="A12" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="66" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="66" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="69">
+        <v>298</v>
+      </c>
+      <c r="J12" s="34">
+        <v>840000000</v>
+      </c>
       <c r="K12" s="34"/>
-      <c r="L12" s="67"/>
-      <c r="M12" s="67"/>
-      <c r="N12" s="70"/>
+      <c r="L12" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N12" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O12" s="36"/>
       <c r="P12" s="37"/>
       <c r="Q12" s="37"/>
@@ -3249,20 +3393,46 @@
       <c r="T12" s="36"/>
     </row>
     <row r="13" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A13" s="29"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="67"/>
-      <c r="G13" s="67"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="69"/>
-      <c r="J13" s="34"/>
+      <c r="A13" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="66" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="65" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="69">
+        <v>298</v>
+      </c>
+      <c r="J13" s="34">
+        <v>1380000000</v>
+      </c>
       <c r="K13" s="34"/>
-      <c r="L13" s="67"/>
-      <c r="M13" s="67"/>
-      <c r="N13" s="70"/>
+      <c r="L13" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="M13" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N13" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O13" s="36"/>
       <c r="P13" s="37"/>
       <c r="Q13" s="37"/>
@@ -3271,20 +3441,46 @@
       <c r="T13" s="36"/>
     </row>
     <row r="14" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A14" s="29"/>
-      <c r="B14" s="65"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="51"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="69"/>
-      <c r="J14" s="39"/>
+      <c r="A14" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="66" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="66" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="69">
+        <v>298</v>
+      </c>
+      <c r="J14" s="39">
+        <v>7.8</v>
+      </c>
       <c r="K14" s="39"/>
-      <c r="L14" s="67"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="70"/>
+      <c r="L14" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="M14" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N14" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O14" s="36"/>
       <c r="P14" s="36"/>
       <c r="Q14" s="36"/>
@@ -3293,20 +3489,46 @@
       <c r="T14" s="36"/>
     </row>
     <row r="15" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A15" s="29"/>
-      <c r="B15" s="65"/>
-      <c r="C15" s="66"/>
-      <c r="D15" s="66"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="51"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="69"/>
-      <c r="J15" s="39"/>
+      <c r="A15" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="66" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="65" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="68" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="69">
+        <v>298</v>
+      </c>
+      <c r="J15" s="39">
+        <v>24.2</v>
+      </c>
       <c r="K15" s="39"/>
-      <c r="L15" s="67"/>
-      <c r="M15" s="31"/>
-      <c r="N15" s="70"/>
+      <c r="L15" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="M15" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="N15" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O15" s="36"/>
       <c r="P15" s="36"/>
       <c r="Q15" s="36"/>
@@ -3316,19 +3538,37 @@
     </row>
     <row r="16" spans="1:20" ht="18.75" customHeight="1">
       <c r="A16" s="29"/>
-      <c r="B16" s="65"/>
-      <c r="C16" s="66"/>
+      <c r="B16" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="66" t="s">
+        <v>62</v>
+      </c>
       <c r="D16" s="66"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="51"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="54"/>
+      <c r="E16" s="65" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="54" t="s">
+        <v>81</v>
+      </c>
       <c r="I16" s="69"/>
-      <c r="J16" s="39"/>
+      <c r="J16" s="113">
+        <v>0.64600000000000002</v>
+      </c>
       <c r="K16" s="39"/>
-      <c r="L16" s="67"/>
+      <c r="L16" s="67" t="s">
+        <v>83</v>
+      </c>
       <c r="M16" s="31"/>
-      <c r="N16" s="70"/>
+      <c r="N16" s="70" t="s">
+        <v>84</v>
+      </c>
       <c r="O16" s="36"/>
       <c r="P16" s="36"/>
       <c r="Q16" s="36"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.ijrmhm.2026.107677`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C3BD98-0D01-8D42-9CAB-C43AD36D3C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8225294A-F20E-7E49-97F3-7F86E327CD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="118">
   <si>
     <r>
       <rPr>
@@ -424,6 +424,66 @@
   </si>
   <si>
     <t>10.1016/j.ijplas.2026.104622</t>
+  </si>
+  <si>
+    <t>NbMoTa</t>
+  </si>
+  <si>
+    <t>NbMoTaZr0.2</t>
+  </si>
+  <si>
+    <t>NbMoTaZr0.6</t>
+  </si>
+  <si>
+    <t>NbMoTaZr1.0</t>
+  </si>
+  <si>
+    <t>NbMoTaZr1.4</t>
+  </si>
+  <si>
+    <t>Zr0</t>
+  </si>
+  <si>
+    <t>Zr0.2</t>
+  </si>
+  <si>
+    <t>Zr0.6</t>
+  </si>
+  <si>
+    <t>Zr1.0</t>
+  </si>
+  <si>
+    <t>Zr1.4</t>
+  </si>
+  <si>
+    <t>VAM</t>
+  </si>
+  <si>
+    <t>very minor second BCC phase</t>
+  </si>
+  <si>
+    <t>BCC+BCC</t>
+  </si>
+  <si>
+    <t>hardness</t>
+  </si>
+  <si>
+    <t>compressive yield strength</t>
+  </si>
+  <si>
+    <t>compressive plastic strain</t>
+  </si>
+  <si>
+    <t>compressive ductility</t>
+  </si>
+  <si>
+    <t>F7a</t>
+  </si>
+  <si>
+    <t>T3</t>
+  </si>
+  <si>
+    <t>10.1016/j.ijrmhm.2026.107677</t>
   </si>
 </sst>
 </file>
@@ -1458,7 +1518,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="151">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1658,6 +1718,60 @@
     <xf numFmtId="0" fontId="14" fillId="10" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="11" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1718,60 +1832,8 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2988,19 +3050,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="12"/>
-      <c r="D2" s="113" t="s">
+      <c r="D2" s="131" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="114"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="119"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="121"/>
+      <c r="E2" s="132"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="136"/>
+      <c r="H2" s="136"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="138"/>
+      <c r="K2" s="138"/>
+      <c r="L2" s="136"/>
+      <c r="M2" s="136"/>
+      <c r="N2" s="139"/>
       <c r="O2" s="13"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -3012,21 +3074,21 @@
       <c r="A3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="150" t="s">
+      <c r="B3" s="113" t="s">
         <v>72</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="115"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="122"/>
-      <c r="G3" s="122"/>
-      <c r="H3" s="122"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="124"/>
-      <c r="K3" s="124"/>
-      <c r="L3" s="122"/>
-      <c r="M3" s="122"/>
-      <c r="N3" s="125"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="140"/>
+      <c r="H3" s="140"/>
+      <c r="I3" s="141"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="140"/>
+      <c r="M3" s="140"/>
+      <c r="N3" s="143"/>
       <c r="O3" s="13"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -3067,43 +3129,43 @@
       <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="126" t="s">
+      <c r="C5" s="144" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="128" t="s">
+      <c r="D5" s="146" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="128" t="s">
+      <c r="E5" s="146" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="128" t="s">
+      <c r="F5" s="146" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="128" t="s">
+      <c r="G5" s="146" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="129" t="s">
+      <c r="H5" s="147" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="128" t="s">
+      <c r="I5" s="146" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="128" t="s">
+      <c r="J5" s="146" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="128" t="s">
+      <c r="K5" s="146" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="128" t="s">
+      <c r="L5" s="146" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="128" t="s">
+      <c r="M5" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="128" t="s">
+      <c r="N5" s="146" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="133" t="s">
+      <c r="O5" s="114" t="s">
         <v>19</v>
       </c>
       <c r="P5" s="24"/>
@@ -3119,19 +3181,19 @@
       <c r="B6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="127"/>
-      <c r="D6" s="127"/>
-      <c r="E6" s="127"/>
-      <c r="F6" s="127"/>
-      <c r="G6" s="127"/>
-      <c r="H6" s="130"/>
-      <c r="I6" s="131"/>
-      <c r="J6" s="132"/>
-      <c r="K6" s="132"/>
-      <c r="L6" s="127"/>
-      <c r="M6" s="127"/>
-      <c r="N6" s="127"/>
-      <c r="O6" s="134"/>
+      <c r="C6" s="145"/>
+      <c r="D6" s="145"/>
+      <c r="E6" s="145"/>
+      <c r="F6" s="145"/>
+      <c r="G6" s="145"/>
+      <c r="H6" s="148"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="150"/>
+      <c r="K6" s="150"/>
+      <c r="L6" s="145"/>
+      <c r="M6" s="145"/>
+      <c r="N6" s="145"/>
+      <c r="O6" s="115"/>
       <c r="P6" s="24"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="9"/>
@@ -3181,7 +3243,7 @@
       <c r="N7" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="O7" s="135"/>
+      <c r="O7" s="116"/>
       <c r="P7" s="62" t="s">
         <v>61</v>
       </c>
@@ -3196,35 +3258,35 @@
     </row>
     <row r="8" spans="1:20" ht="20.25" customHeight="1" thickBot="1">
       <c r="A8" s="57"/>
-      <c r="B8" s="136" t="s">
+      <c r="B8" s="117" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="137"/>
-      <c r="D8" s="137"/>
-      <c r="E8" s="138"/>
-      <c r="F8" s="139" t="s">
+      <c r="C8" s="118"/>
+      <c r="D8" s="118"/>
+      <c r="E8" s="119"/>
+      <c r="F8" s="120" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="140"/>
-      <c r="H8" s="140"/>
-      <c r="I8" s="141"/>
-      <c r="J8" s="142"/>
-      <c r="K8" s="142"/>
-      <c r="L8" s="143"/>
-      <c r="M8" s="144" t="s">
+      <c r="G8" s="121"/>
+      <c r="H8" s="121"/>
+      <c r="I8" s="122"/>
+      <c r="J8" s="123"/>
+      <c r="K8" s="123"/>
+      <c r="L8" s="124"/>
+      <c r="M8" s="125" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="145"/>
+      <c r="N8" s="126"/>
       <c r="O8" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="P8" s="146" t="s">
+      <c r="P8" s="127" t="s">
         <v>41</v>
       </c>
-      <c r="Q8" s="147"/>
-      <c r="R8" s="148"/>
-      <c r="S8" s="148"/>
-      <c r="T8" s="149"/>
+      <c r="Q8" s="128"/>
+      <c r="R8" s="129"/>
+      <c r="S8" s="129"/>
+      <c r="T8" s="130"/>
     </row>
     <row r="9" spans="1:20" ht="21" customHeight="1" thickBot="1">
       <c r="A9" s="58" t="s">
@@ -4071,20 +4133,42 @@
       <c r="T26" s="36"/>
     </row>
     <row r="27" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A27" s="29"/>
-      <c r="B27" s="40"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="66"/>
+      <c r="A27" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E27" s="65"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="31"/>
+      <c r="F27" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G27" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H27" s="32"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="86"/>
+      <c r="I27" s="69">
+        <v>298</v>
+      </c>
+      <c r="J27" s="86">
+        <v>4550000000</v>
+      </c>
       <c r="K27" s="56"/>
-      <c r="L27" s="31"/>
-      <c r="M27" s="31"/>
-      <c r="N27" s="70"/>
+      <c r="L27" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M27" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N27" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O27" s="36"/>
       <c r="P27" s="36"/>
       <c r="Q27" s="38"/>
@@ -4093,20 +4177,44 @@
       <c r="T27" s="36"/>
     </row>
     <row r="28" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A28" s="29"/>
-      <c r="B28" s="40"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="65"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
+      <c r="A28" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B28" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="66" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="86"/>
+      <c r="I28" s="69">
+        <v>298</v>
+      </c>
+      <c r="J28" s="86">
+        <v>5020000000</v>
+      </c>
       <c r="K28" s="56"/>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="70"/>
+      <c r="L28" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M28" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N28" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O28" s="36"/>
       <c r="P28" s="36"/>
       <c r="Q28" s="38"/>
@@ -4115,20 +4223,42 @@
       <c r="T28" s="36"/>
     </row>
     <row r="29" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A29" s="29"/>
-      <c r="B29" s="40"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="66"/>
+      <c r="A29" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B29" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E29" s="65"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
+      <c r="F29" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H29" s="32"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="86"/>
+      <c r="I29" s="69">
+        <v>298</v>
+      </c>
+      <c r="J29" s="86">
+        <v>5220000000</v>
+      </c>
       <c r="K29" s="56"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="70"/>
+      <c r="L29" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M29" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N29" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O29" s="36"/>
       <c r="P29" s="36"/>
       <c r="Q29" s="38"/>
@@ -4137,20 +4267,42 @@
       <c r="T29" s="36"/>
     </row>
     <row r="30" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A30" s="29"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="66"/>
+      <c r="A30" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="B30" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E30" s="65"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
+      <c r="F30" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="86"/>
+      <c r="I30" s="69">
+        <v>298</v>
+      </c>
+      <c r="J30" s="86">
+        <v>5450000000</v>
+      </c>
       <c r="K30" s="56"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="70"/>
+      <c r="L30" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M30" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N30" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O30" s="36"/>
       <c r="P30" s="36"/>
       <c r="Q30" s="38"/>
@@ -4159,20 +4311,42 @@
       <c r="T30" s="36"/>
     </row>
     <row r="31" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A31" s="29"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="66"/>
+      <c r="A31" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D31" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E31" s="65"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
+      <c r="F31" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G31" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H31" s="32"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="86"/>
+      <c r="I31" s="69">
+        <v>298</v>
+      </c>
+      <c r="J31" s="86">
+        <v>5150000000</v>
+      </c>
       <c r="K31" s="56"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="70"/>
+      <c r="L31" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M31" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N31" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O31" s="36"/>
       <c r="P31" s="36"/>
       <c r="Q31" s="38"/>
@@ -4181,20 +4355,44 @@
       <c r="T31" s="36"/>
     </row>
     <row r="32" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A32" s="29"/>
-      <c r="B32" s="40"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="66"/>
+      <c r="A32" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E32" s="65"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="32"/>
-      <c r="I32" s="33"/>
-      <c r="J32" s="86"/>
+      <c r="F32" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G32" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H32" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I32" s="69">
+        <v>298</v>
+      </c>
+      <c r="J32" s="86">
+        <v>963000000</v>
+      </c>
       <c r="K32" s="56"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="70"/>
+      <c r="L32" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M32" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N32" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O32" s="36"/>
       <c r="P32" s="36"/>
       <c r="Q32" s="38"/>
@@ -4203,20 +4401,46 @@
       <c r="T32" s="36"/>
     </row>
     <row r="33" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A33" s="29"/>
-      <c r="B33" s="40"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="66"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="33"/>
-      <c r="J33" s="86"/>
+      <c r="A33" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D33" s="66" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="F33" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G33" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H33" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I33" s="69">
+        <v>298</v>
+      </c>
+      <c r="J33" s="86">
+        <v>1225000000</v>
+      </c>
       <c r="K33" s="56"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="70"/>
+      <c r="L33" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M33" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N33" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O33" s="36"/>
       <c r="P33" s="36"/>
       <c r="Q33" s="38"/>
@@ -4225,20 +4449,44 @@
       <c r="T33" s="36"/>
     </row>
     <row r="34" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A34" s="29"/>
-      <c r="B34" s="40"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="66"/>
+      <c r="A34" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B34" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D34" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E34" s="65"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="31"/>
-      <c r="H34" s="32"/>
-      <c r="I34" s="33"/>
-      <c r="J34" s="36"/>
+      <c r="F34" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G34" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H34" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I34" s="69">
+        <v>298</v>
+      </c>
+      <c r="J34" s="56">
+        <v>1387000000</v>
+      </c>
       <c r="K34" s="56"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="39"/>
-      <c r="N34" s="70"/>
+      <c r="L34" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M34" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N34" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O34" s="36"/>
       <c r="P34" s="37"/>
       <c r="Q34" s="38"/>
@@ -4247,20 +4495,44 @@
       <c r="T34" s="36"/>
     </row>
     <row r="35" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A35" s="29"/>
-      <c r="B35" s="40"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="66"/>
+      <c r="A35" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="B35" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E35" s="65"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="33"/>
-      <c r="J35" s="36"/>
+      <c r="F35" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G35" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H35" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="69">
+        <v>298</v>
+      </c>
+      <c r="J35" s="56">
+        <v>1457000000</v>
+      </c>
       <c r="K35" s="37"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="39"/>
-      <c r="N35" s="70"/>
+      <c r="L35" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M35" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N35" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O35" s="36"/>
       <c r="P35" s="37"/>
       <c r="Q35" s="38"/>
@@ -4269,20 +4541,44 @@
       <c r="T35" s="36"/>
     </row>
     <row r="36" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A36" s="29"/>
-      <c r="B36" s="40"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="66"/>
+      <c r="A36" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C36" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E36" s="65"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="33"/>
-      <c r="J36" s="36"/>
+      <c r="F36" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G36" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H36" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I36" s="69">
+        <v>298</v>
+      </c>
+      <c r="J36" s="56">
+        <v>1352000000</v>
+      </c>
       <c r="K36" s="37"/>
-      <c r="L36" s="31"/>
-      <c r="M36" s="39"/>
-      <c r="N36" s="70"/>
+      <c r="L36" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M36" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N36" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O36" s="36"/>
       <c r="P36" s="37"/>
       <c r="Q36" s="38"/>
@@ -4291,20 +4587,44 @@
       <c r="T36" s="36"/>
     </row>
     <row r="37" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A37" s="29"/>
-      <c r="B37" s="40"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="66"/>
+      <c r="A37" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D37" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E37" s="65"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="33"/>
-      <c r="J37" s="36"/>
+      <c r="F37" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G37" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H37" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I37" s="69">
+        <v>298</v>
+      </c>
+      <c r="J37" s="36">
+        <v>6.3</v>
+      </c>
       <c r="K37" s="34"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="39"/>
-      <c r="N37" s="70"/>
+      <c r="L37" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M37" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N37" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O37" s="36"/>
       <c r="P37" s="37"/>
       <c r="Q37" s="38"/>
@@ -4313,20 +4633,46 @@
       <c r="T37" s="36"/>
     </row>
     <row r="38" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A38" s="29"/>
-      <c r="B38" s="40"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="66"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="32"/>
-      <c r="I38" s="33"/>
-      <c r="J38" s="43"/>
+      <c r="A38" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="66" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="65" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G38" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H38" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I38" s="69">
+        <v>298</v>
+      </c>
+      <c r="J38" s="43">
+        <v>14.2</v>
+      </c>
       <c r="K38" s="34"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="39"/>
-      <c r="N38" s="70"/>
+      <c r="L38" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M38" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N38" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O38" s="43"/>
       <c r="P38" s="38"/>
       <c r="Q38" s="38"/>
@@ -4335,20 +4681,44 @@
       <c r="T38" s="36"/>
     </row>
     <row r="39" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A39" s="29"/>
-      <c r="B39" s="40"/>
-      <c r="C39" s="29"/>
-      <c r="D39" s="66"/>
+      <c r="A39" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B39" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E39" s="65"/>
-      <c r="F39" s="31"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="33"/>
-      <c r="J39" s="43"/>
+      <c r="F39" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G39" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H39" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I39" s="69">
+        <v>298</v>
+      </c>
+      <c r="J39" s="43">
+        <v>18.100000000000001</v>
+      </c>
       <c r="K39" s="34"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="39"/>
-      <c r="N39" s="70"/>
+      <c r="L39" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M39" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N39" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O39" s="43"/>
       <c r="P39" s="38"/>
       <c r="Q39" s="38"/>
@@ -4357,20 +4727,44 @@
       <c r="T39" s="36"/>
     </row>
     <row r="40" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A40" s="29"/>
-      <c r="B40" s="40"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="66"/>
+      <c r="A40" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D40" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E40" s="65"/>
-      <c r="F40" s="31"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="33"/>
-      <c r="J40" s="43"/>
+      <c r="F40" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H40" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I40" s="69">
+        <v>298</v>
+      </c>
+      <c r="J40" s="43">
+        <v>20.100000000000001</v>
+      </c>
       <c r="K40" s="44"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="39"/>
-      <c r="N40" s="70"/>
+      <c r="L40" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M40" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N40" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O40" s="43"/>
       <c r="P40" s="38"/>
       <c r="Q40" s="43"/>
@@ -4379,20 +4773,44 @@
       <c r="T40" s="36"/>
     </row>
     <row r="41" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A41" s="29"/>
-      <c r="B41" s="40"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="66"/>
+      <c r="A41" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="66" t="s">
+        <v>108</v>
+      </c>
       <c r="E41" s="65"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="32"/>
-      <c r="I41" s="33"/>
-      <c r="J41" s="43"/>
+      <c r="F41" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G41" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H41" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I41" s="69">
+        <v>298</v>
+      </c>
+      <c r="J41" s="43">
+        <v>25.2</v>
+      </c>
       <c r="K41" s="44"/>
-      <c r="L41" s="31"/>
-      <c r="M41" s="39"/>
-      <c r="N41" s="70"/>
+      <c r="L41" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M41" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="N41" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O41" s="43"/>
       <c r="P41" s="38"/>
       <c r="Q41" s="43"/>
@@ -4401,20 +4819,44 @@
       <c r="T41" s="36"/>
     </row>
     <row r="42" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A42" s="29"/>
-      <c r="B42" s="40"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="66"/>
-      <c r="E42" s="65"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="33"/>
-      <c r="J42" s="43"/>
+      <c r="A42" s="151" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="100" t="s">
+        <v>98</v>
+      </c>
+      <c r="C42" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D42" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" s="102"/>
+      <c r="F42" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G42" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H42" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I42" s="69">
+        <v>298</v>
+      </c>
+      <c r="J42" s="43">
+        <v>5.5</v>
+      </c>
       <c r="K42" s="44"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="39"/>
-      <c r="N42" s="70"/>
+      <c r="L42" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M42" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="N42" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O42" s="43"/>
       <c r="P42" s="44"/>
       <c r="Q42" s="43"/>
@@ -4423,20 +4865,46 @@
       <c r="T42" s="36"/>
     </row>
     <row r="43" spans="1:20" ht="18" customHeight="1">
-      <c r="A43" s="29"/>
-      <c r="B43" s="40"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="66"/>
-      <c r="E43" s="65"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="33"/>
-      <c r="J43" s="43"/>
+      <c r="A43" s="152" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="102" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E43" s="102" t="s">
+        <v>109</v>
+      </c>
+      <c r="F43" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G43" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H43" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I43" s="69">
+        <v>298</v>
+      </c>
+      <c r="J43" s="43">
+        <v>13.5</v>
+      </c>
       <c r="K43" s="44"/>
-      <c r="L43" s="31"/>
-      <c r="M43" s="39"/>
-      <c r="N43" s="70"/>
+      <c r="L43" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M43" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="N43" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O43" s="43"/>
       <c r="P43" s="44"/>
       <c r="Q43" s="43"/>
@@ -4445,20 +4913,44 @@
       <c r="T43" s="36"/>
     </row>
     <row r="44" spans="1:20" ht="18" customHeight="1">
-      <c r="A44" s="29"/>
-      <c r="B44" s="40"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="66"/>
-      <c r="E44" s="65"/>
-      <c r="F44" s="31"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="33"/>
-      <c r="J44" s="43"/>
+      <c r="A44" s="152" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" s="102" t="s">
+        <v>100</v>
+      </c>
+      <c r="C44" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="102"/>
+      <c r="F44" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G44" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H44" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I44" s="69">
+        <v>298</v>
+      </c>
+      <c r="J44" s="43">
+        <v>19</v>
+      </c>
       <c r="K44" s="46"/>
-      <c r="L44" s="31"/>
-      <c r="M44" s="39"/>
-      <c r="N44" s="70"/>
+      <c r="L44" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M44" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="N44" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O44" s="43"/>
       <c r="P44" s="43"/>
       <c r="Q44" s="38"/>
@@ -4467,20 +4959,44 @@
       <c r="T44" s="36"/>
     </row>
     <row r="45" spans="1:20" ht="18" customHeight="1">
-      <c r="A45" s="29"/>
-      <c r="B45" s="40"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="66"/>
-      <c r="E45" s="65"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="33"/>
-      <c r="J45" s="43"/>
+      <c r="A45" s="152" t="s">
+        <v>106</v>
+      </c>
+      <c r="B45" s="102" t="s">
+        <v>101</v>
+      </c>
+      <c r="C45" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D45" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E45" s="102"/>
+      <c r="F45" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G45" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H45" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I45" s="69">
+        <v>298</v>
+      </c>
+      <c r="J45" s="43">
+        <v>20</v>
+      </c>
       <c r="K45" s="46"/>
-      <c r="L45" s="31"/>
-      <c r="M45" s="39"/>
-      <c r="N45" s="70"/>
+      <c r="L45" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M45" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="N45" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O45" s="43"/>
       <c r="P45" s="43"/>
       <c r="Q45" s="38"/>
@@ -4489,20 +5005,44 @@
       <c r="T45" s="36"/>
     </row>
     <row r="46" spans="1:20" ht="18" customHeight="1">
-      <c r="A46" s="29"/>
-      <c r="B46" s="40"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="66"/>
-      <c r="E46" s="65"/>
-      <c r="F46" s="31"/>
-      <c r="G46" s="31"/>
-      <c r="H46" s="32"/>
-      <c r="I46" s="33"/>
-      <c r="J46" s="43"/>
+      <c r="A46" s="152" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="102" t="s">
+        <v>102</v>
+      </c>
+      <c r="C46" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E46" s="102"/>
+      <c r="F46" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G46" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H46" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I46" s="69">
+        <v>298</v>
+      </c>
+      <c r="J46" s="43">
+        <v>22</v>
+      </c>
       <c r="K46" s="34"/>
-      <c r="L46" s="31"/>
-      <c r="M46" s="39"/>
-      <c r="N46" s="70"/>
+      <c r="L46" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M46" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="N46" s="70" t="s">
+        <v>117</v>
+      </c>
       <c r="O46" s="43"/>
       <c r="P46" s="43"/>
       <c r="Q46" s="38"/>
@@ -24467,11 +25007,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="P8:T8"/>
     <mergeCell ref="D2:E3"/>
     <mergeCell ref="F2:N3"/>
     <mergeCell ref="C5:C6"/>
@@ -24486,6 +25021,11 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
+    <mergeCell ref="O5:O7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="P8:T8"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.mtadv.2026.100712`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8225294A-F20E-7E49-97F3-7F86E327CD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F81F777-5E3A-2A4F-80BE-60BE54C0C145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="128">
   <si>
     <r>
       <rPr>
@@ -484,6 +484,36 @@
   </si>
   <si>
     <t>10.1016/j.ijrmhm.2026.107677</t>
+  </si>
+  <si>
+    <t>Ti23.5 Zr18.7 Nb35.4 Mo13.8 W8.6</t>
+  </si>
+  <si>
+    <t>Ti11.4 Zr16.3 Nb39.7 Mo11.4 W21.2</t>
+  </si>
+  <si>
+    <t>Ti21.7 Zr24.6 Hf7.1 Ta30.7 W15.9</t>
+  </si>
+  <si>
+    <t>HD1</t>
+  </si>
+  <si>
+    <t>HD2</t>
+  </si>
+  <si>
+    <t>LD</t>
+  </si>
+  <si>
+    <t>F11</t>
+  </si>
+  <si>
+    <t>UCS</t>
+  </si>
+  <si>
+    <t>10.1016/j.mtadv.2026.100712</t>
+  </si>
+  <si>
+    <t>composition was ML-optimized; property value averaged from 3 runs; property uncertainty set as 1/2 of range from 3 runs</t>
   </si>
 </sst>
 </file>
@@ -1518,7 +1548,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1834,6 +1864,8 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="10" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5051,20 +5083,46 @@
       <c r="T46" s="36"/>
     </row>
     <row r="47" spans="1:20" ht="18" customHeight="1">
-      <c r="A47" s="29"/>
-      <c r="B47" s="40"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="66"/>
-      <c r="E47" s="65"/>
-      <c r="F47" s="31"/>
-      <c r="G47" s="31"/>
+      <c r="A47" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D47" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E47" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F47" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G47" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H47" s="32"/>
-      <c r="I47" s="33"/>
-      <c r="J47" s="43"/>
-      <c r="K47" s="44"/>
-      <c r="L47" s="31"/>
-      <c r="M47" s="39"/>
-      <c r="N47" s="70"/>
+      <c r="I47" s="69">
+        <v>298</v>
+      </c>
+      <c r="J47" s="153">
+        <v>1597000000</v>
+      </c>
+      <c r="K47" s="154">
+        <v>18000000</v>
+      </c>
+      <c r="L47" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M47" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N47" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O47" s="43"/>
       <c r="P47" s="43"/>
       <c r="Q47" s="38"/>
@@ -5073,20 +5131,46 @@
       <c r="T47" s="36"/>
     </row>
     <row r="48" spans="1:20" ht="18" customHeight="1">
-      <c r="A48" s="29"/>
-      <c r="B48" s="40"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="66"/>
-      <c r="E48" s="65"/>
-      <c r="F48" s="31"/>
-      <c r="G48" s="31"/>
+      <c r="A48" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="C48" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E48" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F48" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G48" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H48" s="32"/>
-      <c r="I48" s="33"/>
-      <c r="J48" s="43"/>
-      <c r="K48" s="44"/>
-      <c r="L48" s="31"/>
-      <c r="M48" s="39"/>
-      <c r="N48" s="70"/>
+      <c r="I48" s="69">
+        <v>298</v>
+      </c>
+      <c r="J48" s="153">
+        <v>1794000000</v>
+      </c>
+      <c r="K48" s="154">
+        <v>44000000</v>
+      </c>
+      <c r="L48" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M48" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N48" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O48" s="43"/>
       <c r="P48" s="43"/>
       <c r="Q48" s="38"/>
@@ -5095,20 +5179,46 @@
       <c r="T48" s="36"/>
     </row>
     <row r="49" spans="1:20" ht="18" customHeight="1">
-      <c r="A49" s="29"/>
-      <c r="B49" s="40"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="66"/>
-      <c r="E49" s="65"/>
-      <c r="F49" s="31"/>
-      <c r="G49" s="31"/>
+      <c r="A49" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B49" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="C49" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D49" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E49" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F49" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G49" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H49" s="32"/>
-      <c r="I49" s="33"/>
-      <c r="J49" s="43"/>
-      <c r="K49" s="44"/>
-      <c r="L49" s="31"/>
-      <c r="M49" s="39"/>
-      <c r="N49" s="70"/>
+      <c r="I49" s="69">
+        <v>298</v>
+      </c>
+      <c r="J49" s="153">
+        <v>1764000000</v>
+      </c>
+      <c r="K49" s="154">
+        <v>41000000</v>
+      </c>
+      <c r="L49" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M49" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N49" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O49" s="43"/>
       <c r="P49" s="43"/>
       <c r="Q49" s="38"/>
@@ -5117,20 +5227,46 @@
       <c r="T49" s="36"/>
     </row>
     <row r="50" spans="1:20" ht="18" customHeight="1">
-      <c r="A50" s="29"/>
-      <c r="B50" s="40"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="29"/>
-      <c r="E50" s="29"/>
-      <c r="F50" s="31"/>
-      <c r="G50" s="31"/>
+      <c r="A50" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="C50" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D50" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E50" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F50" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G50" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H50" s="32"/>
-      <c r="I50" s="33"/>
-      <c r="J50" s="86"/>
-      <c r="K50" s="44"/>
-      <c r="L50" s="31"/>
-      <c r="M50" s="39"/>
-      <c r="N50" s="35"/>
+      <c r="I50" s="69">
+        <v>298</v>
+      </c>
+      <c r="J50" s="86">
+        <v>2032000000</v>
+      </c>
+      <c r="K50" s="154">
+        <v>17000000</v>
+      </c>
+      <c r="L50" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M50" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N50" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O50" s="43"/>
       <c r="P50" s="43"/>
       <c r="Q50" s="38"/>
@@ -5139,20 +5275,46 @@
       <c r="T50" s="36"/>
     </row>
     <row r="51" spans="1:20" ht="18" customHeight="1">
-      <c r="A51" s="29"/>
-      <c r="B51" s="99"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="29"/>
-      <c r="E51" s="87"/>
-      <c r="F51" s="31"/>
-      <c r="G51" s="31"/>
+      <c r="A51" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B51" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="C51" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D51" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E51" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F51" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G51" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H51" s="32"/>
-      <c r="I51" s="33"/>
-      <c r="J51" s="86"/>
-      <c r="K51" s="46"/>
-      <c r="L51" s="31"/>
-      <c r="M51" s="39"/>
-      <c r="N51" s="35"/>
+      <c r="I51" s="69">
+        <v>298</v>
+      </c>
+      <c r="J51" s="86">
+        <v>2279000000</v>
+      </c>
+      <c r="K51" s="46">
+        <v>61000000</v>
+      </c>
+      <c r="L51" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M51" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N51" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O51" s="43"/>
       <c r="P51" s="43"/>
       <c r="Q51" s="38"/>
@@ -5161,20 +5323,46 @@
       <c r="T51" s="36"/>
     </row>
     <row r="52" spans="1:20" ht="18" customHeight="1">
-      <c r="A52" s="29"/>
-      <c r="B52" s="101"/>
-      <c r="C52" s="29"/>
-      <c r="D52" s="29"/>
-      <c r="E52" s="88"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="31"/>
+      <c r="A52" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B52" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="C52" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D52" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E52" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G52" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H52" s="32"/>
-      <c r="I52" s="33"/>
-      <c r="J52" s="86"/>
-      <c r="K52" s="46"/>
-      <c r="L52" s="31"/>
-      <c r="M52" s="39"/>
-      <c r="N52" s="35"/>
+      <c r="I52" s="69">
+        <v>298</v>
+      </c>
+      <c r="J52" s="86">
+        <v>1914000000</v>
+      </c>
+      <c r="K52" s="46">
+        <v>33000000</v>
+      </c>
+      <c r="L52" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M52" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N52" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O52" s="43"/>
       <c r="P52" s="44"/>
       <c r="Q52" s="38"/>
@@ -5183,20 +5371,46 @@
       <c r="T52" s="36"/>
     </row>
     <row r="53" spans="1:20" ht="18" customHeight="1">
-      <c r="A53" s="29"/>
-      <c r="B53" s="40"/>
-      <c r="C53" s="29"/>
-      <c r="D53" s="29"/>
-      <c r="E53" s="29"/>
-      <c r="F53" s="31"/>
-      <c r="G53" s="31"/>
+      <c r="A53" s="151" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" s="100" t="s">
+        <v>118</v>
+      </c>
+      <c r="C53" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D53" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E53" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F53" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G53" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H53" s="32"/>
-      <c r="I53" s="33"/>
-      <c r="J53" s="86"/>
-      <c r="K53" s="46"/>
-      <c r="L53" s="31"/>
-      <c r="M53" s="39"/>
-      <c r="N53" s="35"/>
+      <c r="I53" s="69">
+        <v>298</v>
+      </c>
+      <c r="J53" s="86">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="K53" s="46">
+        <v>1.8</v>
+      </c>
+      <c r="L53" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M53" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N53" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O53" s="43"/>
       <c r="P53" s="43"/>
       <c r="Q53" s="43"/>
@@ -5205,20 +5419,46 @@
       <c r="T53" s="36"/>
     </row>
     <row r="54" spans="1:20" ht="18" customHeight="1">
-      <c r="A54" s="29"/>
-      <c r="B54" s="40"/>
-      <c r="C54" s="29"/>
-      <c r="D54" s="29"/>
-      <c r="E54" s="29"/>
-      <c r="F54" s="31"/>
-      <c r="G54" s="31"/>
+      <c r="A54" s="152" t="s">
+        <v>122</v>
+      </c>
+      <c r="B54" s="102" t="s">
+        <v>119</v>
+      </c>
+      <c r="C54" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D54" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E54" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F54" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G54" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H54" s="32"/>
-      <c r="I54" s="33"/>
-      <c r="J54" s="86"/>
-      <c r="K54" s="46"/>
-      <c r="L54" s="31"/>
-      <c r="M54" s="39"/>
-      <c r="N54" s="35"/>
+      <c r="I54" s="69">
+        <v>298</v>
+      </c>
+      <c r="J54" s="86">
+        <v>13.9</v>
+      </c>
+      <c r="K54" s="46">
+        <v>3</v>
+      </c>
+      <c r="L54" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M54" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N54" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O54" s="43"/>
       <c r="P54" s="43"/>
       <c r="Q54" s="43"/>
@@ -5227,20 +5467,46 @@
       <c r="T54" s="36"/>
     </row>
     <row r="55" spans="1:20" ht="18" customHeight="1">
-      <c r="A55" s="29"/>
-      <c r="B55" s="99"/>
-      <c r="C55" s="29"/>
-      <c r="D55" s="29"/>
-      <c r="E55" s="87"/>
-      <c r="F55" s="31"/>
-      <c r="G55" s="31"/>
+      <c r="A55" s="152" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" s="102" t="s">
+        <v>120</v>
+      </c>
+      <c r="C55" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="D55" s="88" t="s">
+        <v>108</v>
+      </c>
+      <c r="E55" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F55" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G55" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H55" s="32"/>
-      <c r="I55" s="33"/>
-      <c r="J55" s="86"/>
-      <c r="K55" s="46"/>
-      <c r="L55" s="31"/>
-      <c r="M55" s="39"/>
-      <c r="N55" s="35"/>
+      <c r="I55" s="69">
+        <v>298</v>
+      </c>
+      <c r="J55" s="86">
+        <v>5.2</v>
+      </c>
+      <c r="K55" s="46">
+        <v>1.2</v>
+      </c>
+      <c r="L55" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M55" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="N55" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="O55" s="43"/>
       <c r="P55" s="43"/>
       <c r="Q55" s="43"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jmrt.2025.12.182`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F81F777-5E3A-2A4F-80BE-60BE54C0C145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE686C7-FBB6-5148-BA12-DFF4828F4960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="160">
   <si>
     <r>
       <rPr>
@@ -514,6 +514,102 @@
   </si>
   <si>
     <t>composition was ML-optimized; property value averaged from 3 runs; property uncertainty set as 1/2 of range from 3 runs</t>
+  </si>
+  <si>
+    <t>B1(hs)</t>
+  </si>
+  <si>
+    <t>Ti75 Zr12.5 Hf12.5</t>
+  </si>
+  <si>
+    <t>B1(cs)</t>
+  </si>
+  <si>
+    <t>B2(hs)</t>
+  </si>
+  <si>
+    <t>B2(cs)</t>
+  </si>
+  <si>
+    <t>Ti77.8 Zr11.1 Hf11.1</t>
+  </si>
+  <si>
+    <t>B3(hs)</t>
+  </si>
+  <si>
+    <t>B3(cs)</t>
+  </si>
+  <si>
+    <t>Ti80 Zr10 Hf10</t>
+  </si>
+  <si>
+    <t>Ti60.1 Zr10.1 Hf10.1 Al14 V5</t>
+  </si>
+  <si>
+    <t>B4(hs)</t>
+  </si>
+  <si>
+    <t>B4(cs)</t>
+  </si>
+  <si>
+    <t>Ti63.5 Zr9.1 Hf9.1 Al13.5 V4.8</t>
+  </si>
+  <si>
+    <t>Ti65.7 Zr8.2 Hf8.2 Al13.2 V4.7</t>
+  </si>
+  <si>
+    <t>B5(hs)</t>
+  </si>
+  <si>
+    <t>B5(cs)</t>
+  </si>
+  <si>
+    <t>B6(hs)</t>
+  </si>
+  <si>
+    <t>B6(cs)</t>
+  </si>
+  <si>
+    <t>R1(hs)</t>
+  </si>
+  <si>
+    <t>R1(cs)</t>
+  </si>
+  <si>
+    <t>Ti86.2 Al10.2 V3.6</t>
+  </si>
+  <si>
+    <t>AAM+H+WQ</t>
+  </si>
+  <si>
+    <t>AAM+H+WQ+CT</t>
+  </si>
+  <si>
+    <t>homogenized at 1473K for 2h and water quenched; supposedly BCC+HCP but the XRD appears inconclusive</t>
+  </si>
+  <si>
+    <t>homogenized at 1473K for 2h and water quenched and then cryogenic treated (CT) in liquid nitrogen at 77K for 180s to induce some martensitic transfromation; supposedly BCC+HCP but the XRD appears inconclusive</t>
+  </si>
+  <si>
+    <t>corrosion potential</t>
+  </si>
+  <si>
+    <t>3.5 wt% NaCl</t>
+  </si>
+  <si>
+    <t>corrosion current density</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>A/m^2</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>10.1016/j.jmrt.2025.12.182</t>
   </si>
 </sst>
 </file>
@@ -1548,7 +1644,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1866,6 +1962,12 @@
     <xf numFmtId="0" fontId="13" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="10" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5515,328 +5617,700 @@
       <c r="T55" s="36"/>
     </row>
     <row r="56" spans="1:20" ht="18" customHeight="1">
-      <c r="A56" s="29"/>
-      <c r="B56" s="101"/>
+      <c r="A56" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B56" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C56" s="29"/>
-      <c r="D56" s="29"/>
-      <c r="E56" s="88"/>
-      <c r="F56" s="31"/>
-      <c r="G56" s="31"/>
+      <c r="D56" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E56" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F56" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G56" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H56" s="32"/>
-      <c r="I56" s="33"/>
-      <c r="J56" s="86"/>
+      <c r="I56" s="69">
+        <v>298</v>
+      </c>
+      <c r="J56" s="86">
+        <f>P56*9807000</f>
+        <v>2853837000</v>
+      </c>
       <c r="K56" s="46"/>
-      <c r="L56" s="31"/>
-      <c r="M56" s="39"/>
-      <c r="N56" s="35"/>
+      <c r="L56" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M56" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N56" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O56" s="43"/>
-      <c r="P56" s="43"/>
+      <c r="P56" s="43">
+        <v>291</v>
+      </c>
       <c r="Q56" s="43"/>
       <c r="R56" s="43"/>
       <c r="S56" s="36"/>
       <c r="T56" s="36"/>
     </row>
     <row r="57" spans="1:20" ht="18" customHeight="1">
-      <c r="A57" s="29"/>
-      <c r="B57" s="30"/>
+      <c r="A57" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B57" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C57" s="29"/>
-      <c r="D57" s="29"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="31"/>
-      <c r="G57" s="31"/>
+      <c r="D57" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E57" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F57" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G57" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H57" s="32"/>
-      <c r="I57" s="33"/>
-      <c r="J57" s="34"/>
+      <c r="I57" s="69">
+        <v>298</v>
+      </c>
+      <c r="J57" s="86">
+        <f t="shared" ref="J57:J69" si="0">P57*9807000</f>
+        <v>3667818000</v>
+      </c>
       <c r="K57" s="46"/>
-      <c r="L57" s="31"/>
-      <c r="M57" s="39"/>
-      <c r="N57" s="35"/>
+      <c r="L57" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M57" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N57" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O57" s="43"/>
-      <c r="P57" s="43"/>
+      <c r="P57" s="43">
+        <v>374</v>
+      </c>
       <c r="Q57" s="43"/>
       <c r="R57" s="43"/>
       <c r="S57" s="36"/>
       <c r="T57" s="36"/>
     </row>
     <row r="58" spans="1:20" ht="18" customHeight="1">
-      <c r="A58" s="29"/>
-      <c r="B58" s="30"/>
+      <c r="A58" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B58" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C58" s="29"/>
-      <c r="D58" s="29"/>
-      <c r="E58" s="29"/>
-      <c r="F58" s="31"/>
-      <c r="G58" s="31"/>
+      <c r="D58" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E58" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F58" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G58" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H58" s="32"/>
-      <c r="I58" s="33"/>
-      <c r="J58" s="86"/>
+      <c r="I58" s="69">
+        <v>298</v>
+      </c>
+      <c r="J58" s="86">
+        <f t="shared" si="0"/>
+        <v>2912679000</v>
+      </c>
       <c r="K58" s="46"/>
-      <c r="L58" s="31"/>
-      <c r="M58" s="39"/>
-      <c r="N58" s="35"/>
+      <c r="L58" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M58" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N58" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O58" s="43"/>
-      <c r="P58" s="43"/>
+      <c r="P58" s="43">
+        <v>297</v>
+      </c>
       <c r="Q58" s="43"/>
       <c r="R58" s="43"/>
       <c r="S58" s="36"/>
       <c r="T58" s="36"/>
     </row>
     <row r="59" spans="1:20" ht="18" customHeight="1">
-      <c r="A59" s="29"/>
-      <c r="B59" s="30"/>
+      <c r="A59" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="B59" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C59" s="29"/>
-      <c r="D59" s="29"/>
-      <c r="E59" s="29"/>
-      <c r="F59" s="31"/>
-      <c r="G59" s="31"/>
+      <c r="D59" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E59" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F59" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G59" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H59" s="32"/>
-      <c r="I59" s="33"/>
-      <c r="J59" s="86"/>
+      <c r="I59" s="69">
+        <v>298</v>
+      </c>
+      <c r="J59" s="86">
+        <f t="shared" si="0"/>
+        <v>3932607000</v>
+      </c>
       <c r="K59" s="46"/>
-      <c r="L59" s="31"/>
-      <c r="M59" s="39"/>
-      <c r="N59" s="35"/>
+      <c r="L59" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M59" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N59" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O59" s="43"/>
-      <c r="P59" s="43"/>
+      <c r="P59" s="43">
+        <v>401</v>
+      </c>
       <c r="Q59" s="43"/>
       <c r="R59" s="43"/>
       <c r="S59" s="36"/>
       <c r="T59" s="36"/>
     </row>
     <row r="60" spans="1:20" ht="18" customHeight="1">
-      <c r="A60" s="29"/>
-      <c r="B60" s="30"/>
+      <c r="A60" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B60" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
-      <c r="E60" s="29"/>
-      <c r="F60" s="31"/>
-      <c r="G60" s="31"/>
+      <c r="D60" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E60" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F60" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G60" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H60" s="32"/>
-      <c r="I60" s="33"/>
-      <c r="J60" s="86"/>
+      <c r="I60" s="69">
+        <v>298</v>
+      </c>
+      <c r="J60" s="86">
+        <f t="shared" si="0"/>
+        <v>2804802000</v>
+      </c>
       <c r="K60" s="46"/>
-      <c r="L60" s="31"/>
-      <c r="M60" s="39"/>
-      <c r="N60" s="35"/>
+      <c r="L60" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M60" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N60" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O60" s="43"/>
-      <c r="P60" s="43"/>
+      <c r="P60" s="43">
+        <v>286</v>
+      </c>
       <c r="Q60" s="43"/>
       <c r="R60" s="43"/>
       <c r="S60" s="36"/>
       <c r="T60" s="36"/>
     </row>
     <row r="61" spans="1:20" ht="18" customHeight="1">
-      <c r="A61" s="29"/>
-      <c r="B61" s="30"/>
+      <c r="A61" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="B61" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C61" s="29"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="29"/>
-      <c r="F61" s="31"/>
-      <c r="G61" s="31"/>
+      <c r="D61" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E61" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F61" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G61" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H61" s="32"/>
-      <c r="I61" s="33"/>
-      <c r="J61" s="86"/>
+      <c r="I61" s="69">
+        <v>298</v>
+      </c>
+      <c r="J61" s="86">
+        <f t="shared" si="0"/>
+        <v>3805116000</v>
+      </c>
       <c r="K61" s="46"/>
-      <c r="L61" s="31"/>
-      <c r="M61" s="39"/>
-      <c r="N61" s="35"/>
+      <c r="L61" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M61" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N61" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O61" s="43"/>
-      <c r="P61" s="43"/>
+      <c r="P61" s="43">
+        <v>388</v>
+      </c>
       <c r="Q61" s="43"/>
       <c r="R61" s="43"/>
       <c r="S61" s="36"/>
       <c r="T61" s="36"/>
     </row>
     <row r="62" spans="1:20" ht="18" customHeight="1">
-      <c r="A62" s="29"/>
-      <c r="B62" s="30"/>
+      <c r="A62" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B62" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C62" s="29"/>
-      <c r="D62" s="29"/>
-      <c r="E62" s="29"/>
-      <c r="F62" s="31"/>
-      <c r="G62" s="31"/>
+      <c r="D62" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E62" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F62" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G62" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H62" s="32"/>
-      <c r="I62" s="33"/>
-      <c r="J62" s="86"/>
+      <c r="I62" s="69">
+        <v>298</v>
+      </c>
+      <c r="J62" s="86">
+        <f t="shared" si="0"/>
+        <v>3756081000</v>
+      </c>
       <c r="K62" s="46"/>
-      <c r="L62" s="31"/>
-      <c r="M62" s="39"/>
-      <c r="N62" s="35"/>
+      <c r="L62" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M62" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N62" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O62" s="43"/>
-      <c r="P62" s="43"/>
+      <c r="P62" s="43">
+        <v>383</v>
+      </c>
       <c r="Q62" s="43"/>
       <c r="R62" s="43"/>
       <c r="S62" s="36"/>
       <c r="T62" s="36"/>
     </row>
     <row r="63" spans="1:20" ht="18" customHeight="1">
-      <c r="A63" s="29"/>
-      <c r="B63" s="30"/>
+      <c r="A63" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="B63" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C63" s="29"/>
-      <c r="D63" s="29"/>
-      <c r="E63" s="29"/>
-      <c r="F63" s="31"/>
-      <c r="G63" s="31"/>
+      <c r="D63" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E63" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F63" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G63" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H63" s="32"/>
-      <c r="I63" s="43"/>
-      <c r="J63" s="86"/>
+      <c r="I63" s="69">
+        <v>298</v>
+      </c>
+      <c r="J63" s="86">
+        <f t="shared" si="0"/>
+        <v>4148361000</v>
+      </c>
       <c r="K63" s="46"/>
-      <c r="L63" s="31"/>
-      <c r="M63" s="39"/>
-      <c r="N63" s="35"/>
+      <c r="L63" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M63" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N63" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O63" s="43"/>
-      <c r="P63" s="36"/>
+      <c r="P63" s="36">
+        <v>423</v>
+      </c>
       <c r="Q63" s="43"/>
       <c r="R63" s="43"/>
       <c r="S63" s="36"/>
       <c r="T63" s="36"/>
     </row>
     <row r="64" spans="1:20" ht="18" customHeight="1">
-      <c r="A64" s="29"/>
-      <c r="B64" s="30"/>
+      <c r="A64" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="B64" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C64" s="29"/>
-      <c r="D64" s="29"/>
-      <c r="E64" s="29"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="31"/>
+      <c r="D64" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E64" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F64" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G64" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H64" s="32"/>
-      <c r="I64" s="43"/>
-      <c r="J64" s="86"/>
+      <c r="I64" s="69">
+        <v>298</v>
+      </c>
+      <c r="J64" s="86">
+        <f t="shared" si="0"/>
+        <v>3795309000</v>
+      </c>
       <c r="K64" s="46"/>
-      <c r="L64" s="31"/>
-      <c r="M64" s="39"/>
-      <c r="N64" s="35"/>
+      <c r="L64" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M64" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N64" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O64" s="43"/>
-      <c r="P64" s="36"/>
+      <c r="P64" s="36">
+        <v>387</v>
+      </c>
       <c r="Q64" s="43"/>
       <c r="R64" s="43"/>
       <c r="S64" s="36"/>
       <c r="T64" s="36"/>
     </row>
     <row r="65" spans="1:20" ht="18" customHeight="1">
-      <c r="A65" s="29"/>
-      <c r="B65" s="30"/>
+      <c r="A65" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B65" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C65" s="29"/>
-      <c r="D65" s="29"/>
-      <c r="E65" s="29"/>
-      <c r="F65" s="31"/>
-      <c r="G65" s="31"/>
+      <c r="D65" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E65" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F65" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G65" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H65" s="32"/>
-      <c r="I65" s="43"/>
-      <c r="J65" s="86"/>
+      <c r="I65" s="69">
+        <v>298</v>
+      </c>
+      <c r="J65" s="86">
+        <f t="shared" si="0"/>
+        <v>4217010000</v>
+      </c>
       <c r="K65" s="46"/>
-      <c r="L65" s="31"/>
-      <c r="M65" s="39"/>
-      <c r="N65" s="35"/>
+      <c r="L65" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M65" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N65" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O65" s="43"/>
-      <c r="P65" s="36"/>
+      <c r="P65" s="36">
+        <v>430</v>
+      </c>
       <c r="Q65" s="43"/>
       <c r="R65" s="43"/>
       <c r="S65" s="36"/>
       <c r="T65" s="36"/>
     </row>
     <row r="66" spans="1:20" ht="18" customHeight="1">
-      <c r="A66" s="29"/>
-      <c r="B66" s="30"/>
+      <c r="A66" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B66" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C66" s="29"/>
-      <c r="D66" s="29"/>
-      <c r="E66" s="29"/>
-      <c r="F66" s="31"/>
-      <c r="G66" s="31"/>
+      <c r="D66" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E66" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F66" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G66" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H66" s="32"/>
-      <c r="I66" s="43"/>
-      <c r="J66" s="86"/>
+      <c r="I66" s="69">
+        <v>298</v>
+      </c>
+      <c r="J66" s="86">
+        <f t="shared" si="0"/>
+        <v>3697239000</v>
+      </c>
       <c r="K66" s="44"/>
-      <c r="L66" s="31"/>
-      <c r="M66" s="39"/>
-      <c r="N66" s="35"/>
+      <c r="L66" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M66" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N66" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O66" s="43"/>
-      <c r="P66" s="36"/>
+      <c r="P66" s="36">
+        <v>377</v>
+      </c>
       <c r="Q66" s="43"/>
       <c r="R66" s="43"/>
       <c r="S66" s="36"/>
       <c r="T66" s="36"/>
     </row>
     <row r="67" spans="1:20" ht="18" customHeight="1">
-      <c r="A67" s="29"/>
-      <c r="B67" s="30"/>
+      <c r="A67" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B67" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C67" s="29"/>
-      <c r="D67" s="29"/>
-      <c r="E67" s="29"/>
-      <c r="F67" s="31"/>
-      <c r="G67" s="31"/>
+      <c r="D67" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E67" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F67" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G67" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H67" s="32"/>
-      <c r="I67" s="43"/>
-      <c r="J67" s="86"/>
+      <c r="I67" s="69">
+        <v>298</v>
+      </c>
+      <c r="J67" s="86">
+        <f t="shared" si="0"/>
+        <v>4011063000</v>
+      </c>
       <c r="K67" s="44"/>
-      <c r="L67" s="31"/>
-      <c r="M67" s="39"/>
-      <c r="N67" s="35"/>
+      <c r="L67" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M67" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N67" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O67" s="43"/>
-      <c r="P67" s="36"/>
+      <c r="P67" s="36">
+        <v>409</v>
+      </c>
       <c r="Q67" s="43"/>
       <c r="R67" s="43"/>
       <c r="S67" s="36"/>
       <c r="T67" s="36"/>
     </row>
     <row r="68" spans="1:20" ht="18" customHeight="1">
-      <c r="A68" s="29"/>
-      <c r="B68" s="30"/>
+      <c r="A68" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B68" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C68" s="29"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="29"/>
-      <c r="F68" s="31"/>
-      <c r="G68" s="31"/>
+      <c r="D68" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E68" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F68" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G68" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H68" s="32"/>
-      <c r="I68" s="43"/>
-      <c r="J68" s="86"/>
+      <c r="I68" s="69">
+        <v>298</v>
+      </c>
+      <c r="J68" s="86">
+        <f t="shared" si="0"/>
+        <v>3726660000</v>
+      </c>
       <c r="K68" s="44"/>
-      <c r="L68" s="31"/>
-      <c r="M68" s="39"/>
-      <c r="N68" s="35"/>
+      <c r="L68" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M68" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N68" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O68" s="43"/>
-      <c r="P68" s="36"/>
+      <c r="P68" s="36">
+        <v>380</v>
+      </c>
       <c r="Q68" s="43"/>
       <c r="R68" s="43"/>
       <c r="S68" s="36"/>
       <c r="T68" s="36"/>
     </row>
     <row r="69" spans="1:20" ht="18" customHeight="1">
-      <c r="A69" s="29"/>
-      <c r="B69" s="30"/>
+      <c r="A69" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B69" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C69" s="29"/>
-      <c r="D69" s="29"/>
-      <c r="E69" s="29"/>
-      <c r="F69" s="31"/>
-      <c r="G69" s="31"/>
+      <c r="D69" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E69" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F69" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G69" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H69" s="32"/>
-      <c r="I69" s="43"/>
-      <c r="J69" s="86"/>
+      <c r="I69" s="69">
+        <v>298</v>
+      </c>
+      <c r="J69" s="86">
+        <f t="shared" si="0"/>
+        <v>4079712000</v>
+      </c>
       <c r="K69" s="86"/>
-      <c r="L69" s="31"/>
-      <c r="M69" s="39"/>
-      <c r="N69" s="35"/>
+      <c r="L69" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M69" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="N69" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O69" s="43"/>
-      <c r="P69" s="36"/>
+      <c r="P69" s="36">
+        <v>416</v>
+      </c>
       <c r="Q69" s="46"/>
       <c r="R69" s="43"/>
       <c r="S69" s="36"/>
       <c r="T69" s="36"/>
     </row>
     <row r="70" spans="1:20" ht="18" customHeight="1">
-      <c r="A70" s="29"/>
-      <c r="B70" s="30"/>
+      <c r="A70" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B70" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C70" s="29"/>
-      <c r="D70" s="29"/>
-      <c r="E70" s="29"/>
-      <c r="F70" s="31"/>
-      <c r="G70" s="31"/>
+      <c r="D70" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E70" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F70" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G70" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H70" s="32"/>
-      <c r="I70" s="43"/>
-      <c r="J70" s="86"/>
+      <c r="I70" s="69">
+        <v>298</v>
+      </c>
+      <c r="J70" s="86">
+        <v>750000000</v>
+      </c>
       <c r="K70" s="86"/>
-      <c r="L70" s="31"/>
-      <c r="M70" s="39"/>
-      <c r="N70" s="35"/>
+      <c r="L70" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M70" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N70" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O70" s="43"/>
       <c r="P70" s="36"/>
       <c r="Q70" s="46"/>
@@ -5845,19 +6319,42 @@
       <c r="T70" s="36"/>
     </row>
     <row r="71" spans="1:20" ht="18" customHeight="1">
-      <c r="A71" s="29"/>
-      <c r="B71" s="30"/>
+      <c r="A71" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B71" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C71" s="29"/>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="31"/>
-      <c r="G71" s="31"/>
+      <c r="D71" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E71" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F71" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G71" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H71" s="32"/>
-      <c r="J71" s="86"/>
+      <c r="I71" s="69">
+        <v>298</v>
+      </c>
+      <c r="J71" s="86">
+        <v>763000000</v>
+      </c>
       <c r="K71" s="86"/>
-      <c r="L71" s="31"/>
-      <c r="M71" s="39"/>
-      <c r="N71" s="35"/>
+      <c r="L71" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M71" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N71" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O71" s="43"/>
       <c r="P71" s="36"/>
       <c r="Q71" s="46"/>
@@ -5866,20 +6363,42 @@
       <c r="T71" s="36"/>
     </row>
     <row r="72" spans="1:20" ht="18" customHeight="1">
-      <c r="A72" s="29"/>
-      <c r="B72" s="30"/>
+      <c r="A72" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B72" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C72" s="29"/>
-      <c r="D72" s="29"/>
-      <c r="E72" s="29"/>
-      <c r="F72" s="31"/>
-      <c r="G72" s="31"/>
+      <c r="D72" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E72" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F72" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G72" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H72" s="32"/>
-      <c r="I72" s="44"/>
-      <c r="J72" s="86"/>
+      <c r="I72" s="69">
+        <v>298</v>
+      </c>
+      <c r="J72" s="86">
+        <v>893000000</v>
+      </c>
       <c r="K72" s="86"/>
-      <c r="L72" s="31"/>
-      <c r="M72" s="39"/>
-      <c r="N72" s="35"/>
+      <c r="L72" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M72" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N72" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O72" s="43"/>
       <c r="P72" s="36"/>
       <c r="Q72" s="46"/>
@@ -5888,20 +6407,42 @@
       <c r="T72" s="36"/>
     </row>
     <row r="73" spans="1:20" ht="18" customHeight="1">
-      <c r="A73" s="29"/>
-      <c r="B73" s="30"/>
+      <c r="A73" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B73" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C73" s="29"/>
-      <c r="D73" s="29"/>
-      <c r="E73" s="29"/>
-      <c r="F73" s="31"/>
-      <c r="G73" s="31"/>
+      <c r="D73" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E73" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F73" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G73" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H73" s="32"/>
-      <c r="I73" s="43"/>
-      <c r="J73" s="86"/>
+      <c r="I73" s="69">
+        <v>298</v>
+      </c>
+      <c r="J73" s="86">
+        <v>1078000000</v>
+      </c>
       <c r="K73" s="86"/>
-      <c r="L73" s="31"/>
-      <c r="M73" s="39"/>
-      <c r="N73" s="35"/>
+      <c r="L73" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M73" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N73" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O73" s="43"/>
       <c r="P73" s="36"/>
       <c r="Q73" s="43"/>
@@ -5910,20 +6451,42 @@
       <c r="T73" s="36"/>
     </row>
     <row r="74" spans="1:20" ht="18" customHeight="1">
-      <c r="A74" s="29"/>
-      <c r="B74" s="30"/>
+      <c r="A74" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C74" s="29"/>
-      <c r="D74" s="29"/>
-      <c r="E74" s="29"/>
-      <c r="F74" s="31"/>
-      <c r="G74" s="31"/>
+      <c r="D74" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E74" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F74" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G74" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H74" s="32"/>
-      <c r="I74" s="43"/>
-      <c r="J74" s="86"/>
+      <c r="I74" s="69">
+        <v>298</v>
+      </c>
+      <c r="J74" s="86">
+        <v>1056000000</v>
+      </c>
       <c r="K74" s="86"/>
-      <c r="L74" s="31"/>
-      <c r="M74" s="39"/>
-      <c r="N74" s="35"/>
+      <c r="L74" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M74" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N74" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O74" s="43"/>
       <c r="P74" s="36"/>
       <c r="Q74" s="43"/>
@@ -5932,19 +6495,42 @@
       <c r="T74" s="36"/>
     </row>
     <row r="75" spans="1:20" ht="18" customHeight="1">
-      <c r="A75" s="29"/>
-      <c r="B75" s="30"/>
+      <c r="A75" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B75" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C75" s="29"/>
-      <c r="D75" s="29"/>
-      <c r="E75" s="29"/>
-      <c r="F75" s="31"/>
-      <c r="G75" s="31"/>
+      <c r="D75" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E75" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F75" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G75" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H75" s="32"/>
-      <c r="J75" s="86"/>
+      <c r="I75" s="69">
+        <v>298</v>
+      </c>
+      <c r="J75" s="86">
+        <v>1094000000</v>
+      </c>
       <c r="K75" s="86"/>
-      <c r="L75" s="31"/>
-      <c r="M75" s="39"/>
-      <c r="N75" s="35"/>
+      <c r="L75" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M75" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N75" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O75" s="43"/>
       <c r="P75" s="36"/>
       <c r="Q75" s="38"/>
@@ -5953,20 +6539,42 @@
       <c r="T75" s="36"/>
     </row>
     <row r="76" spans="1:20" ht="18" customHeight="1">
-      <c r="A76" s="29"/>
-      <c r="B76" s="30"/>
+      <c r="A76" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B76" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C76" s="29"/>
-      <c r="D76" s="29"/>
-      <c r="E76" s="29"/>
-      <c r="F76" s="31"/>
-      <c r="G76" s="31"/>
+      <c r="D76" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E76" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F76" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G76" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H76" s="32"/>
-      <c r="I76" s="44"/>
-      <c r="J76" s="86"/>
+      <c r="I76" s="69">
+        <v>298</v>
+      </c>
+      <c r="J76" s="86">
+        <v>879000000</v>
+      </c>
       <c r="K76" s="86"/>
-      <c r="L76" s="31"/>
-      <c r="M76" s="39"/>
-      <c r="N76" s="35"/>
+      <c r="L76" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M76" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N76" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O76" s="43"/>
       <c r="P76" s="36"/>
       <c r="Q76" s="38"/>
@@ -5975,20 +6583,42 @@
       <c r="T76" s="36"/>
     </row>
     <row r="77" spans="1:20" ht="18" customHeight="1">
-      <c r="A77" s="29"/>
-      <c r="B77" s="30"/>
+      <c r="A77" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B77" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C77" s="29"/>
-      <c r="D77" s="29"/>
-      <c r="E77" s="29"/>
-      <c r="F77" s="31"/>
-      <c r="G77" s="31"/>
+      <c r="D77" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E77" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F77" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G77" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H77" s="32"/>
-      <c r="I77" s="43"/>
-      <c r="J77" s="86"/>
+      <c r="I77" s="69">
+        <v>298</v>
+      </c>
+      <c r="J77" s="86">
+        <v>1303000000</v>
+      </c>
       <c r="K77" s="44"/>
-      <c r="L77" s="31"/>
-      <c r="M77" s="39"/>
-      <c r="N77" s="35"/>
+      <c r="L77" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M77" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N77" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O77" s="43"/>
       <c r="P77" s="36"/>
       <c r="Q77" s="38"/>
@@ -5997,20 +6627,42 @@
       <c r="T77" s="36"/>
     </row>
     <row r="78" spans="1:20" ht="18" customHeight="1">
-      <c r="A78" s="29"/>
-      <c r="B78" s="30"/>
+      <c r="A78" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B78" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C78" s="29"/>
-      <c r="D78" s="29"/>
-      <c r="E78" s="29"/>
-      <c r="F78" s="31"/>
-      <c r="G78" s="31"/>
+      <c r="D78" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E78" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F78" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G78" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H78" s="32"/>
-      <c r="I78" s="38"/>
-      <c r="J78" s="86"/>
+      <c r="I78" s="69">
+        <v>298</v>
+      </c>
+      <c r="J78" s="86">
+        <v>1212000000</v>
+      </c>
       <c r="K78" s="44"/>
-      <c r="L78" s="31"/>
-      <c r="M78" s="39"/>
-      <c r="N78" s="35"/>
+      <c r="L78" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M78" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N78" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O78" s="43"/>
       <c r="P78" s="36"/>
       <c r="Q78" s="38"/>
@@ -6019,20 +6671,42 @@
       <c r="T78" s="36"/>
     </row>
     <row r="79" spans="1:20" ht="18" customHeight="1">
-      <c r="A79" s="29"/>
-      <c r="B79" s="30"/>
+      <c r="A79" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B79" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C79" s="29"/>
-      <c r="D79" s="29"/>
-      <c r="E79" s="29"/>
-      <c r="F79" s="31"/>
-      <c r="G79" s="31"/>
+      <c r="D79" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E79" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F79" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G79" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H79" s="32"/>
-      <c r="I79" s="38"/>
-      <c r="J79" s="86"/>
+      <c r="I79" s="69">
+        <v>298</v>
+      </c>
+      <c r="J79" s="86">
+        <v>1183000000</v>
+      </c>
       <c r="K79" s="46"/>
-      <c r="L79" s="31"/>
-      <c r="M79" s="39"/>
-      <c r="N79" s="35"/>
+      <c r="L79" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M79" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N79" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O79" s="43"/>
       <c r="P79" s="36"/>
       <c r="Q79" s="38"/>
@@ -6041,20 +6715,42 @@
       <c r="T79" s="36"/>
     </row>
     <row r="80" spans="1:20" ht="18" customHeight="1">
-      <c r="A80" s="29"/>
-      <c r="B80" s="30"/>
+      <c r="A80" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B80" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C80" s="29"/>
-      <c r="D80" s="29"/>
-      <c r="E80" s="29"/>
-      <c r="F80" s="31"/>
-      <c r="G80" s="31"/>
+      <c r="D80" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E80" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F80" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G80" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H80" s="32"/>
-      <c r="I80" s="38"/>
-      <c r="J80" s="86"/>
+      <c r="I80" s="69">
+        <v>298</v>
+      </c>
+      <c r="J80" s="86">
+        <v>1522000000</v>
+      </c>
       <c r="K80" s="34"/>
-      <c r="L80" s="31"/>
-      <c r="M80" s="39"/>
-      <c r="N80" s="35"/>
+      <c r="L80" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M80" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N80" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O80" s="43"/>
       <c r="P80" s="36"/>
       <c r="Q80" s="38"/>
@@ -6063,20 +6759,42 @@
       <c r="T80" s="36"/>
     </row>
     <row r="81" spans="1:20" ht="18" customHeight="1">
-      <c r="A81" s="29"/>
-      <c r="B81" s="30"/>
+      <c r="A81" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="B81" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C81" s="29"/>
-      <c r="D81" s="29"/>
-      <c r="E81" s="29"/>
-      <c r="F81" s="31"/>
-      <c r="G81" s="31"/>
+      <c r="D81" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E81" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F81" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G81" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H81" s="32"/>
-      <c r="I81" s="38"/>
-      <c r="J81" s="86"/>
+      <c r="I81" s="69">
+        <v>298</v>
+      </c>
+      <c r="J81" s="86">
+        <v>1667000000</v>
+      </c>
       <c r="K81" s="34"/>
-      <c r="L81" s="31"/>
-      <c r="M81" s="39"/>
-      <c r="N81" s="35"/>
+      <c r="L81" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M81" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N81" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O81" s="43"/>
       <c r="P81" s="36"/>
       <c r="Q81" s="38"/>
@@ -6085,20 +6803,42 @@
       <c r="T81" s="36"/>
     </row>
     <row r="82" spans="1:20" ht="18" customHeight="1">
-      <c r="A82" s="29"/>
-      <c r="B82" s="30"/>
+      <c r="A82" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B82" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C82" s="29"/>
-      <c r="D82" s="29"/>
-      <c r="E82" s="29"/>
-      <c r="F82" s="31"/>
-      <c r="G82" s="31"/>
+      <c r="D82" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E82" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F82" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G82" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H82" s="32"/>
-      <c r="I82" s="38"/>
-      <c r="J82" s="86"/>
+      <c r="I82" s="69">
+        <v>298</v>
+      </c>
+      <c r="J82" s="86">
+        <v>1297000000</v>
+      </c>
       <c r="K82" s="34"/>
-      <c r="L82" s="31"/>
-      <c r="M82" s="39"/>
-      <c r="N82" s="35"/>
+      <c r="L82" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M82" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N82" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O82" s="43"/>
       <c r="P82" s="36"/>
       <c r="Q82" s="38"/>
@@ -6107,20 +6847,42 @@
       <c r="T82" s="36"/>
     </row>
     <row r="83" spans="1:20" ht="18" customHeight="1">
-      <c r="A83" s="29"/>
-      <c r="B83" s="30"/>
+      <c r="A83" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B83" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C83" s="29"/>
-      <c r="D83" s="29"/>
-      <c r="E83" s="29"/>
-      <c r="F83" s="31"/>
-      <c r="G83" s="31"/>
+      <c r="D83" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E83" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F83" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="G83" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H83" s="32"/>
-      <c r="I83" s="38"/>
-      <c r="J83" s="86"/>
+      <c r="I83" s="69">
+        <v>298</v>
+      </c>
+      <c r="J83" s="86">
+        <v>1415</v>
+      </c>
       <c r="K83" s="34"/>
-      <c r="L83" s="31"/>
-      <c r="M83" s="39"/>
-      <c r="N83" s="35"/>
+      <c r="L83" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M83" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N83" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O83" s="43"/>
       <c r="P83" s="36"/>
       <c r="Q83" s="38"/>
@@ -6129,20 +6891,42 @@
       <c r="T83" s="36"/>
     </row>
     <row r="84" spans="1:20" ht="18" customHeight="1">
-      <c r="A84" s="29"/>
-      <c r="B84" s="30"/>
-      <c r="C84" s="29"/>
-      <c r="D84" s="29"/>
-      <c r="E84" s="29"/>
-      <c r="F84" s="31"/>
-      <c r="G84" s="31"/>
-      <c r="H84" s="32"/>
-      <c r="I84" s="38"/>
-      <c r="J84" s="86"/>
+      <c r="A84" s="151" t="s">
+        <v>128</v>
+      </c>
+      <c r="B84" s="102" t="s">
+        <v>129</v>
+      </c>
+      <c r="C84" s="87"/>
+      <c r="D84" s="87" t="s">
+        <v>149</v>
+      </c>
+      <c r="E84" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F84" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G84" s="94" t="s">
+        <v>28</v>
+      </c>
+      <c r="H84" s="155"/>
+      <c r="I84" s="108">
+        <v>298</v>
+      </c>
+      <c r="J84" s="86">
+        <v>23.1</v>
+      </c>
       <c r="K84" s="34"/>
-      <c r="L84" s="31"/>
-      <c r="M84" s="39"/>
-      <c r="N84" s="35"/>
+      <c r="L84" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M84" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N84" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O84" s="43"/>
       <c r="P84" s="36"/>
       <c r="Q84" s="38"/>
@@ -6151,20 +6935,42 @@
       <c r="T84" s="36"/>
     </row>
     <row r="85" spans="1:20" ht="18" customHeight="1">
-      <c r="A85" s="29"/>
-      <c r="B85" s="30"/>
-      <c r="C85" s="29"/>
-      <c r="D85" s="29"/>
-      <c r="E85" s="29"/>
-      <c r="F85" s="31"/>
-      <c r="G85" s="31"/>
-      <c r="H85" s="32"/>
-      <c r="I85" s="38"/>
-      <c r="J85" s="86"/>
+      <c r="A85" s="152" t="s">
+        <v>131</v>
+      </c>
+      <c r="B85" s="102" t="s">
+        <v>133</v>
+      </c>
+      <c r="C85" s="88"/>
+      <c r="D85" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E85" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F85" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G85" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H85" s="156"/>
+      <c r="I85" s="108">
+        <v>298</v>
+      </c>
+      <c r="J85" s="86">
+        <v>26.9</v>
+      </c>
       <c r="K85" s="34"/>
-      <c r="L85" s="31"/>
-      <c r="M85" s="39"/>
-      <c r="N85" s="35"/>
+      <c r="L85" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M85" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N85" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O85" s="43"/>
       <c r="P85" s="36"/>
       <c r="Q85" s="38"/>
@@ -6173,20 +6979,42 @@
       <c r="T85" s="36"/>
     </row>
     <row r="86" spans="1:20" ht="18" customHeight="1">
-      <c r="A86" s="29"/>
-      <c r="B86" s="30"/>
-      <c r="C86" s="29"/>
-      <c r="D86" s="29"/>
-      <c r="E86" s="29"/>
-      <c r="F86" s="31"/>
-      <c r="G86" s="31"/>
-      <c r="H86" s="32"/>
-      <c r="I86" s="44"/>
-      <c r="J86" s="86"/>
+      <c r="A86" s="152" t="s">
+        <v>134</v>
+      </c>
+      <c r="B86" s="102" t="s">
+        <v>136</v>
+      </c>
+      <c r="C86" s="88"/>
+      <c r="D86" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E86" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F86" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G86" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H86" s="156"/>
+      <c r="I86" s="108">
+        <v>298</v>
+      </c>
+      <c r="J86" s="86">
+        <v>7.7</v>
+      </c>
       <c r="K86" s="46"/>
-      <c r="L86" s="31"/>
-      <c r="M86" s="39"/>
-      <c r="N86" s="35"/>
+      <c r="L86" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M86" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N86" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O86" s="43"/>
       <c r="P86" s="36"/>
       <c r="Q86" s="38"/>
@@ -6195,20 +7023,42 @@
       <c r="T86" s="36"/>
     </row>
     <row r="87" spans="1:20" ht="18" customHeight="1">
-      <c r="A87" s="29"/>
-      <c r="B87" s="30"/>
-      <c r="C87" s="29"/>
-      <c r="D87" s="29"/>
-      <c r="E87" s="29"/>
-      <c r="F87" s="31"/>
-      <c r="G87" s="31"/>
-      <c r="H87" s="32"/>
-      <c r="I87" s="44"/>
-      <c r="J87" s="86"/>
+      <c r="A87" s="152" t="s">
+        <v>138</v>
+      </c>
+      <c r="B87" s="102" t="s">
+        <v>137</v>
+      </c>
+      <c r="C87" s="88"/>
+      <c r="D87" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E87" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F87" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G87" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H87" s="156"/>
+      <c r="I87" s="108">
+        <v>298</v>
+      </c>
+      <c r="J87" s="86">
+        <v>31.1</v>
+      </c>
       <c r="K87" s="46"/>
-      <c r="L87" s="31"/>
-      <c r="M87" s="39"/>
-      <c r="N87" s="35"/>
+      <c r="L87" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M87" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N87" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O87" s="43"/>
       <c r="P87" s="36"/>
       <c r="Q87" s="38"/>
@@ -6217,20 +7067,42 @@
       <c r="T87" s="36"/>
     </row>
     <row r="88" spans="1:20" ht="18" customHeight="1">
-      <c r="A88" s="29"/>
-      <c r="B88" s="30"/>
-      <c r="C88" s="29"/>
-      <c r="D88" s="29"/>
-      <c r="E88" s="29"/>
-      <c r="F88" s="31"/>
-      <c r="G88" s="31"/>
-      <c r="H88" s="32"/>
-      <c r="I88" s="44"/>
-      <c r="J88" s="86"/>
+      <c r="A88" s="152" t="s">
+        <v>142</v>
+      </c>
+      <c r="B88" s="102" t="s">
+        <v>140</v>
+      </c>
+      <c r="C88" s="88"/>
+      <c r="D88" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E88" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F88" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G88" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H88" s="156"/>
+      <c r="I88" s="108">
+        <v>298</v>
+      </c>
+      <c r="J88" s="86">
+        <v>32.5</v>
+      </c>
       <c r="K88" s="46"/>
-      <c r="L88" s="31"/>
-      <c r="M88" s="39"/>
-      <c r="N88" s="35"/>
+      <c r="L88" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M88" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N88" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O88" s="43"/>
       <c r="P88" s="36"/>
       <c r="Q88" s="38"/>
@@ -6239,20 +7111,42 @@
       <c r="T88" s="36"/>
     </row>
     <row r="89" spans="1:20" ht="18" customHeight="1">
-      <c r="A89" s="29"/>
-      <c r="B89" s="30"/>
-      <c r="C89" s="29"/>
-      <c r="D89" s="29"/>
-      <c r="E89" s="29"/>
-      <c r="F89" s="31"/>
-      <c r="G89" s="31"/>
-      <c r="H89" s="32"/>
-      <c r="I89" s="44"/>
-      <c r="J89" s="86"/>
+      <c r="A89" s="152" t="s">
+        <v>144</v>
+      </c>
+      <c r="B89" s="102" t="s">
+        <v>141</v>
+      </c>
+      <c r="C89" s="88"/>
+      <c r="D89" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E89" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F89" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G89" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H89" s="156"/>
+      <c r="I89" s="108">
+        <v>298</v>
+      </c>
+      <c r="J89" s="86">
+        <v>13.8</v>
+      </c>
       <c r="K89" s="46"/>
-      <c r="L89" s="31"/>
-      <c r="M89" s="39"/>
-      <c r="N89" s="35"/>
+      <c r="L89" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M89" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N89" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O89" s="43"/>
       <c r="P89" s="36"/>
       <c r="Q89" s="38"/>
@@ -6261,20 +7155,42 @@
       <c r="T89" s="36"/>
     </row>
     <row r="90" spans="1:20" ht="18" customHeight="1">
-      <c r="A90" s="29"/>
-      <c r="B90" s="30"/>
-      <c r="C90" s="29"/>
-      <c r="D90" s="29"/>
-      <c r="E90" s="29"/>
-      <c r="F90" s="31"/>
-      <c r="G90" s="31"/>
-      <c r="H90" s="32"/>
-      <c r="I90" s="44"/>
-      <c r="J90" s="86"/>
+      <c r="A90" s="152" t="s">
+        <v>146</v>
+      </c>
+      <c r="B90" s="102" t="s">
+        <v>148</v>
+      </c>
+      <c r="C90" s="88"/>
+      <c r="D90" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="E90" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F90" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G90" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H90" s="156"/>
+      <c r="I90" s="108">
+        <v>298</v>
+      </c>
+      <c r="J90" s="86">
+        <v>26.3</v>
+      </c>
       <c r="K90" s="46"/>
-      <c r="L90" s="31"/>
-      <c r="M90" s="39"/>
-      <c r="N90" s="35"/>
+      <c r="L90" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M90" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N90" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O90" s="43"/>
       <c r="P90" s="36"/>
       <c r="Q90" s="38"/>
@@ -6283,616 +7199,1372 @@
       <c r="T90" s="36"/>
     </row>
     <row r="91" spans="1:20" ht="18" customHeight="1">
-      <c r="A91" s="29"/>
-      <c r="B91" s="30"/>
+      <c r="A91" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B91" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C91" s="29"/>
-      <c r="D91" s="29"/>
-      <c r="E91" s="29"/>
-      <c r="F91" s="31"/>
-      <c r="G91" s="31"/>
-      <c r="H91" s="32"/>
-      <c r="I91" s="43"/>
-      <c r="J91" s="86"/>
+      <c r="D91" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E91" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F91" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G91" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H91" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I91" s="108">
+        <v>298</v>
+      </c>
+      <c r="J91" s="86">
+        <f>-1-P91/100</f>
+        <v>-1.51</v>
+      </c>
       <c r="K91" s="46"/>
-      <c r="L91" s="31"/>
-      <c r="M91" s="39"/>
-      <c r="N91" s="35"/>
+      <c r="L91" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M91" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N91" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O91" s="43"/>
-      <c r="P91" s="36"/>
+      <c r="P91" s="36">
+        <v>51</v>
+      </c>
       <c r="Q91" s="38"/>
       <c r="R91" s="43"/>
       <c r="S91" s="36"/>
       <c r="T91" s="36"/>
     </row>
     <row r="92" spans="1:20" ht="18" customHeight="1">
-      <c r="A92" s="29"/>
-      <c r="B92" s="30"/>
+      <c r="A92" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B92" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C92" s="29"/>
-      <c r="D92" s="29"/>
-      <c r="E92" s="29"/>
-      <c r="F92" s="31"/>
-      <c r="G92" s="31"/>
-      <c r="H92" s="32"/>
-      <c r="I92" s="43"/>
-      <c r="J92" s="86"/>
+      <c r="D92" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E92" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F92" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G92" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H92" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I92" s="108">
+        <v>298</v>
+      </c>
+      <c r="J92" s="86">
+        <f t="shared" ref="J92:J104" si="1">-1-P92/100</f>
+        <v>-1.54</v>
+      </c>
       <c r="K92" s="46"/>
-      <c r="L92" s="31"/>
-      <c r="M92" s="39"/>
-      <c r="N92" s="35"/>
+      <c r="L92" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M92" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N92" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O92" s="43"/>
-      <c r="P92" s="36"/>
+      <c r="P92" s="36">
+        <v>54</v>
+      </c>
       <c r="Q92" s="43"/>
       <c r="R92" s="43"/>
       <c r="S92" s="36"/>
       <c r="T92" s="36"/>
     </row>
     <row r="93" spans="1:20" ht="18" customHeight="1">
-      <c r="A93" s="29"/>
-      <c r="B93" s="30"/>
+      <c r="A93" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B93" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C93" s="29"/>
-      <c r="D93" s="29"/>
-      <c r="E93" s="29"/>
-      <c r="F93" s="31"/>
-      <c r="G93" s="31"/>
-      <c r="H93" s="32"/>
-      <c r="I93" s="43"/>
-      <c r="J93" s="86"/>
+      <c r="D93" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E93" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F93" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G93" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H93" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I93" s="108">
+        <v>298</v>
+      </c>
+      <c r="J93" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.48</v>
+      </c>
       <c r="K93" s="46"/>
-      <c r="L93" s="31"/>
-      <c r="M93" s="39"/>
-      <c r="N93" s="35"/>
+      <c r="L93" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M93" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N93" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O93" s="43"/>
-      <c r="P93" s="36"/>
+      <c r="P93" s="36">
+        <v>48</v>
+      </c>
       <c r="Q93" s="43"/>
       <c r="R93" s="43"/>
       <c r="S93" s="36"/>
       <c r="T93" s="36"/>
     </row>
     <row r="94" spans="1:20" ht="18" customHeight="1">
-      <c r="A94" s="29"/>
-      <c r="B94" s="30"/>
+      <c r="A94" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="B94" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C94" s="29"/>
-      <c r="D94" s="29"/>
-      <c r="E94" s="29"/>
-      <c r="F94" s="31"/>
-      <c r="G94" s="31"/>
-      <c r="H94" s="32"/>
-      <c r="I94" s="43"/>
-      <c r="J94" s="86"/>
+      <c r="D94" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E94" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F94" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G94" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H94" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I94" s="108">
+        <v>298</v>
+      </c>
+      <c r="J94" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.55</v>
+      </c>
       <c r="K94" s="46"/>
-      <c r="L94" s="31"/>
-      <c r="M94" s="39"/>
-      <c r="N94" s="35"/>
+      <c r="L94" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M94" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N94" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O94" s="43"/>
-      <c r="P94" s="36"/>
+      <c r="P94" s="36">
+        <v>55</v>
+      </c>
       <c r="Q94" s="43"/>
       <c r="R94" s="43"/>
       <c r="S94" s="36"/>
       <c r="T94" s="36"/>
     </row>
     <row r="95" spans="1:20" ht="18" customHeight="1">
-      <c r="A95" s="29"/>
-      <c r="B95" s="30"/>
+      <c r="A95" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B95" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C95" s="29"/>
-      <c r="D95" s="29"/>
-      <c r="E95" s="29"/>
-      <c r="F95" s="31"/>
-      <c r="G95" s="31"/>
-      <c r="H95" s="32"/>
-      <c r="I95" s="43"/>
-      <c r="J95" s="86"/>
+      <c r="D95" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E95" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F95" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G95" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H95" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I95" s="108">
+        <v>298</v>
+      </c>
+      <c r="J95" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.42</v>
+      </c>
       <c r="K95" s="46"/>
-      <c r="L95" s="31"/>
-      <c r="M95" s="39"/>
-      <c r="N95" s="35"/>
+      <c r="L95" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M95" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N95" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O95" s="43"/>
-      <c r="P95" s="36"/>
+      <c r="P95" s="36">
+        <v>42</v>
+      </c>
       <c r="Q95" s="43"/>
       <c r="R95" s="43"/>
       <c r="S95" s="36"/>
       <c r="T95" s="36"/>
     </row>
     <row r="96" spans="1:20" ht="18" customHeight="1">
-      <c r="A96" s="29"/>
-      <c r="B96" s="30"/>
+      <c r="A96" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="B96" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C96" s="29"/>
-      <c r="D96" s="29"/>
-      <c r="E96" s="29"/>
-      <c r="F96" s="31"/>
-      <c r="G96" s="31"/>
-      <c r="H96" s="32"/>
-      <c r="I96" s="43"/>
-      <c r="J96" s="86"/>
+      <c r="D96" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E96" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F96" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G96" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H96" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I96" s="108">
+        <v>298</v>
+      </c>
+      <c r="J96" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.45</v>
+      </c>
       <c r="K96" s="46"/>
-      <c r="L96" s="31"/>
-      <c r="M96" s="39"/>
-      <c r="N96" s="35"/>
+      <c r="L96" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M96" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N96" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O96" s="43"/>
-      <c r="P96" s="36"/>
+      <c r="P96" s="36">
+        <v>45</v>
+      </c>
       <c r="Q96" s="43"/>
       <c r="R96" s="43"/>
       <c r="S96" s="36"/>
       <c r="T96" s="36"/>
     </row>
     <row r="97" spans="1:20" ht="18" customHeight="1">
-      <c r="A97" s="29"/>
-      <c r="B97" s="30"/>
+      <c r="A97" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B97" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C97" s="29"/>
-      <c r="D97" s="29"/>
-      <c r="E97" s="29"/>
-      <c r="F97" s="31"/>
-      <c r="G97" s="31"/>
-      <c r="H97" s="32"/>
-      <c r="I97" s="43"/>
-      <c r="J97" s="86"/>
+      <c r="D97" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E97" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F97" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G97" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H97" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I97" s="108">
+        <v>298</v>
+      </c>
+      <c r="J97" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.45</v>
+      </c>
       <c r="K97" s="46"/>
-      <c r="L97" s="31"/>
-      <c r="M97" s="39"/>
-      <c r="N97" s="35"/>
+      <c r="L97" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M97" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N97" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O97" s="43"/>
-      <c r="P97" s="36"/>
+      <c r="P97" s="36">
+        <v>45</v>
+      </c>
       <c r="Q97" s="43"/>
       <c r="R97" s="43"/>
       <c r="S97" s="36"/>
       <c r="T97" s="36"/>
     </row>
     <row r="98" spans="1:20" ht="18" customHeight="1">
-      <c r="A98" s="29"/>
-      <c r="B98" s="30"/>
+      <c r="A98" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="B98" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C98" s="29"/>
-      <c r="D98" s="29"/>
-      <c r="E98" s="29"/>
-      <c r="F98" s="31"/>
-      <c r="G98" s="31"/>
-      <c r="H98" s="32"/>
-      <c r="I98" s="38"/>
-      <c r="J98" s="86"/>
+      <c r="D98" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E98" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F98" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G98" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H98" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I98" s="108">
+        <v>298</v>
+      </c>
+      <c r="J98" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.46</v>
+      </c>
       <c r="K98" s="46"/>
-      <c r="L98" s="31"/>
-      <c r="M98" s="39"/>
-      <c r="N98" s="35"/>
+      <c r="L98" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M98" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N98" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O98" s="43"/>
-      <c r="P98" s="36"/>
+      <c r="P98" s="36">
+        <v>46</v>
+      </c>
       <c r="Q98" s="36"/>
       <c r="R98" s="43"/>
       <c r="S98" s="36"/>
       <c r="T98" s="36"/>
     </row>
     <row r="99" spans="1:20" ht="18" customHeight="1">
-      <c r="A99" s="29"/>
-      <c r="B99" s="30"/>
+      <c r="A99" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="B99" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C99" s="29"/>
-      <c r="D99" s="29"/>
-      <c r="E99" s="29"/>
-      <c r="F99" s="31"/>
-      <c r="G99" s="31"/>
-      <c r="H99" s="32"/>
-      <c r="I99" s="38"/>
-      <c r="J99" s="86"/>
+      <c r="D99" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E99" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F99" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G99" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H99" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I99" s="108">
+        <v>298</v>
+      </c>
+      <c r="J99" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.54</v>
+      </c>
       <c r="K99" s="46"/>
-      <c r="L99" s="31"/>
-      <c r="M99" s="39"/>
-      <c r="N99" s="35"/>
+      <c r="L99" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M99" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N99" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O99" s="43"/>
-      <c r="P99" s="36"/>
+      <c r="P99" s="36">
+        <v>54</v>
+      </c>
       <c r="Q99" s="38"/>
       <c r="R99" s="43"/>
       <c r="S99" s="36"/>
       <c r="T99" s="36"/>
     </row>
     <row r="100" spans="1:20" ht="18" customHeight="1">
-      <c r="A100" s="29"/>
-      <c r="B100" s="30"/>
+      <c r="A100" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B100" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C100" s="29"/>
-      <c r="D100" s="29"/>
-      <c r="E100" s="29"/>
-      <c r="F100" s="31"/>
-      <c r="G100" s="31"/>
-      <c r="H100" s="32"/>
-      <c r="I100" s="38"/>
-      <c r="J100" s="86"/>
+      <c r="D100" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E100" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F100" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G100" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H100" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I100" s="108">
+        <v>298</v>
+      </c>
+      <c r="J100" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.44</v>
+      </c>
       <c r="K100" s="46"/>
-      <c r="L100" s="31"/>
-      <c r="M100" s="39"/>
-      <c r="N100" s="35"/>
+      <c r="L100" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M100" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N100" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O100" s="43"/>
-      <c r="P100" s="36"/>
+      <c r="P100" s="36">
+        <v>44</v>
+      </c>
       <c r="Q100" s="38"/>
       <c r="R100" s="43"/>
       <c r="S100" s="36"/>
       <c r="T100" s="36"/>
     </row>
     <row r="101" spans="1:20" ht="18" customHeight="1">
-      <c r="A101" s="29"/>
-      <c r="B101" s="30"/>
+      <c r="A101" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B101" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C101" s="29"/>
-      <c r="D101" s="29"/>
-      <c r="E101" s="29"/>
-      <c r="F101" s="31"/>
-      <c r="G101" s="31"/>
-      <c r="H101" s="32"/>
-      <c r="I101" s="38"/>
-      <c r="J101" s="86"/>
+      <c r="D101" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E101" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F101" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G101" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H101" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I101" s="108">
+        <v>298</v>
+      </c>
+      <c r="J101" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.42</v>
+      </c>
       <c r="K101" s="46"/>
-      <c r="L101" s="31"/>
-      <c r="M101" s="39"/>
-      <c r="N101" s="35"/>
+      <c r="L101" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M101" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N101" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O101" s="43"/>
-      <c r="P101" s="36"/>
+      <c r="P101" s="36">
+        <v>42</v>
+      </c>
       <c r="Q101" s="38"/>
       <c r="R101" s="43"/>
       <c r="S101" s="36"/>
       <c r="T101" s="36"/>
     </row>
     <row r="102" spans="1:20" ht="18" customHeight="1">
-      <c r="A102" s="29"/>
-      <c r="B102" s="30"/>
+      <c r="A102" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B102" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C102" s="29"/>
-      <c r="D102" s="29"/>
-      <c r="E102" s="29"/>
-      <c r="F102" s="31"/>
-      <c r="G102" s="31"/>
-      <c r="H102" s="32"/>
-      <c r="I102" s="38"/>
-      <c r="J102" s="86"/>
+      <c r="D102" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E102" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F102" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G102" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H102" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I102" s="108">
+        <v>298</v>
+      </c>
+      <c r="J102" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.49</v>
+      </c>
       <c r="K102" s="46"/>
-      <c r="L102" s="31"/>
-      <c r="M102" s="39"/>
-      <c r="N102" s="35"/>
+      <c r="L102" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M102" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N102" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O102" s="43"/>
-      <c r="P102" s="36"/>
+      <c r="P102" s="36">
+        <v>49</v>
+      </c>
       <c r="Q102" s="38"/>
       <c r="R102" s="43"/>
       <c r="S102" s="36"/>
       <c r="T102" s="36"/>
     </row>
     <row r="103" spans="1:20" ht="18" customHeight="1">
-      <c r="A103" s="29"/>
-      <c r="B103" s="30"/>
+      <c r="A103" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B103" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C103" s="29"/>
-      <c r="D103" s="29"/>
-      <c r="E103" s="29"/>
-      <c r="F103" s="31"/>
-      <c r="G103" s="31"/>
-      <c r="H103" s="32"/>
-      <c r="I103" s="38"/>
-      <c r="J103" s="86"/>
+      <c r="D103" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E103" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F103" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G103" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H103" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I103" s="108">
+        <v>298</v>
+      </c>
+      <c r="J103" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.46</v>
+      </c>
       <c r="K103" s="46"/>
-      <c r="L103" s="31"/>
-      <c r="M103" s="39"/>
-      <c r="N103" s="35"/>
+      <c r="L103" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M103" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N103" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O103" s="43"/>
-      <c r="P103" s="36"/>
+      <c r="P103" s="36">
+        <v>46</v>
+      </c>
       <c r="Q103" s="38"/>
       <c r="R103" s="43"/>
       <c r="S103" s="36"/>
       <c r="T103" s="36"/>
     </row>
     <row r="104" spans="1:20" ht="18" customHeight="1">
-      <c r="A104" s="29"/>
-      <c r="B104" s="30"/>
+      <c r="A104" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B104" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C104" s="29"/>
-      <c r="D104" s="29"/>
-      <c r="E104" s="29"/>
-      <c r="F104" s="31"/>
-      <c r="G104" s="31"/>
-      <c r="H104" s="32"/>
-      <c r="I104" s="38"/>
-      <c r="J104" s="86"/>
+      <c r="D104" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E104" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F104" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G104" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H104" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I104" s="108">
+        <v>298</v>
+      </c>
+      <c r="J104" s="86">
+        <f t="shared" si="1"/>
+        <v>-1.52</v>
+      </c>
       <c r="K104" s="46"/>
-      <c r="L104" s="31"/>
-      <c r="M104" s="39"/>
-      <c r="N104" s="35"/>
+      <c r="L104" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M104" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N104" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O104" s="43"/>
-      <c r="P104" s="36"/>
+      <c r="P104" s="36">
+        <v>52</v>
+      </c>
       <c r="Q104" s="38"/>
       <c r="R104" s="43"/>
       <c r="S104" s="36"/>
       <c r="T104" s="36"/>
     </row>
     <row r="105" spans="1:20" ht="18" customHeight="1">
-      <c r="A105" s="29"/>
-      <c r="B105" s="30"/>
+      <c r="A105" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B105" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C105" s="29"/>
-      <c r="D105" s="29"/>
-      <c r="E105" s="29"/>
-      <c r="F105" s="95"/>
-      <c r="G105" s="31"/>
-      <c r="H105" s="32"/>
-      <c r="I105" s="38"/>
-      <c r="J105" s="43"/>
+      <c r="D105" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E105" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F105" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G105" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H105" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I105" s="108">
+        <v>298</v>
+      </c>
+      <c r="J105" s="86">
+        <f>P105*10000/1000000</f>
+        <v>0.51800000000000002</v>
+      </c>
       <c r="K105" s="46"/>
-      <c r="L105" s="31"/>
-      <c r="M105" s="39"/>
-      <c r="N105" s="35"/>
+      <c r="L105" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M105" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N105" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O105" s="43"/>
-      <c r="P105" s="43"/>
+      <c r="P105" s="43">
+        <v>51.8</v>
+      </c>
       <c r="Q105" s="43"/>
       <c r="R105" s="43"/>
       <c r="S105" s="36"/>
       <c r="T105" s="36"/>
     </row>
     <row r="106" spans="1:20" ht="18" customHeight="1">
-      <c r="A106" s="29"/>
-      <c r="B106" s="30"/>
+      <c r="A106" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B106" s="101" t="s">
+        <v>129</v>
+      </c>
       <c r="C106" s="29"/>
-      <c r="D106" s="29"/>
-      <c r="E106" s="29"/>
-      <c r="F106" s="95"/>
-      <c r="G106" s="31"/>
-      <c r="H106" s="32"/>
-      <c r="I106" s="38"/>
-      <c r="J106" s="43"/>
+      <c r="D106" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E106" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F106" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G106" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H106" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I106" s="108">
+        <v>298</v>
+      </c>
+      <c r="J106" s="86">
+        <f t="shared" ref="J106:J118" si="2">P106*10000/1000000</f>
+        <v>0.57199999999999995</v>
+      </c>
       <c r="K106" s="49"/>
-      <c r="L106" s="31"/>
-      <c r="M106" s="39"/>
-      <c r="N106" s="35"/>
+      <c r="L106" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M106" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N106" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O106" s="43"/>
-      <c r="P106" s="43"/>
+      <c r="P106" s="43">
+        <v>57.2</v>
+      </c>
       <c r="Q106" s="43"/>
       <c r="R106" s="43"/>
       <c r="S106" s="36"/>
       <c r="T106" s="36"/>
     </row>
     <row r="107" spans="1:20" ht="18" customHeight="1">
-      <c r="A107" s="29"/>
-      <c r="B107" s="30"/>
+      <c r="A107" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B107" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C107" s="29"/>
-      <c r="D107" s="29"/>
-      <c r="E107" s="29"/>
-      <c r="F107" s="95"/>
-      <c r="G107" s="31"/>
-      <c r="H107" s="32"/>
-      <c r="I107" s="38"/>
-      <c r="J107" s="43"/>
+      <c r="D107" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E107" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F107" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G107" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H107" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I107" s="108">
+        <v>298</v>
+      </c>
+      <c r="J107" s="86">
+        <f t="shared" si="2"/>
+        <v>0.52600000000000002</v>
+      </c>
       <c r="K107" s="49"/>
-      <c r="L107" s="31"/>
-      <c r="M107" s="39"/>
-      <c r="N107" s="35"/>
+      <c r="L107" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M107" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N107" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O107" s="43"/>
-      <c r="P107" s="43"/>
+      <c r="P107" s="43">
+        <v>52.6</v>
+      </c>
       <c r="Q107" s="43"/>
       <c r="R107" s="43"/>
       <c r="S107" s="36"/>
       <c r="T107" s="36"/>
     </row>
     <row r="108" spans="1:20" ht="18" customHeight="1">
-      <c r="A108" s="29"/>
-      <c r="B108" s="30"/>
+      <c r="A108" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="B108" s="30" t="s">
+        <v>133</v>
+      </c>
       <c r="C108" s="29"/>
-      <c r="D108" s="29"/>
-      <c r="E108" s="29"/>
-      <c r="F108" s="95"/>
-      <c r="G108" s="31"/>
-      <c r="H108" s="32"/>
-      <c r="I108" s="38"/>
-      <c r="J108" s="43"/>
+      <c r="D108" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E108" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F108" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G108" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H108" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I108" s="108">
+        <v>298</v>
+      </c>
+      <c r="J108" s="86">
+        <f t="shared" si="2"/>
+        <v>0.60699999999999998</v>
+      </c>
       <c r="K108" s="46"/>
-      <c r="L108" s="31"/>
-      <c r="M108" s="39"/>
-      <c r="N108" s="35"/>
+      <c r="L108" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M108" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N108" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O108" s="43"/>
-      <c r="P108" s="43"/>
+      <c r="P108" s="43">
+        <v>60.7</v>
+      </c>
       <c r="Q108" s="43"/>
       <c r="R108" s="43"/>
       <c r="S108" s="36"/>
       <c r="T108" s="36"/>
     </row>
     <row r="109" spans="1:20" ht="18" customHeight="1">
-      <c r="A109" s="29"/>
-      <c r="B109" s="30"/>
+      <c r="A109" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B109" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C109" s="29"/>
-      <c r="D109" s="29"/>
-      <c r="E109" s="29"/>
-      <c r="F109" s="95"/>
-      <c r="G109" s="31"/>
-      <c r="H109" s="32"/>
-      <c r="I109" s="38"/>
-      <c r="J109" s="43"/>
+      <c r="D109" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E109" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F109" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G109" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H109" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I109" s="108">
+        <v>298</v>
+      </c>
+      <c r="J109" s="86">
+        <f t="shared" si="2"/>
+        <v>0.58099999999999996</v>
+      </c>
       <c r="K109" s="46"/>
-      <c r="L109" s="31"/>
-      <c r="M109" s="39"/>
-      <c r="N109" s="35"/>
-      <c r="O109" s="36"/>
-      <c r="P109" s="36"/>
+      <c r="L109" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M109" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N109" s="35" t="s">
+        <v>159</v>
+      </c>
+      <c r="O109" s="43"/>
+      <c r="P109" s="36">
+        <v>58.1</v>
+      </c>
       <c r="Q109" s="36"/>
       <c r="R109" s="43"/>
       <c r="S109" s="36"/>
       <c r="T109" s="36"/>
     </row>
     <row r="110" spans="1:20" ht="18" customHeight="1">
-      <c r="A110" s="29"/>
-      <c r="B110" s="30"/>
+      <c r="A110" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="B110" s="30" t="s">
+        <v>136</v>
+      </c>
       <c r="C110" s="29"/>
-      <c r="D110" s="29"/>
-      <c r="E110" s="29"/>
-      <c r="F110" s="95"/>
-      <c r="G110" s="31"/>
-      <c r="H110" s="32"/>
-      <c r="I110" s="38"/>
-      <c r="J110" s="43"/>
+      <c r="D110" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E110" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F110" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G110" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H110" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I110" s="108">
+        <v>298</v>
+      </c>
+      <c r="J110" s="86">
+        <f t="shared" si="2"/>
+        <v>0.61799999999999999</v>
+      </c>
       <c r="K110" s="46"/>
-      <c r="L110" s="31"/>
-      <c r="M110" s="39"/>
-      <c r="N110" s="35"/>
+      <c r="L110" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M110" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N110" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O110" s="36"/>
-      <c r="P110" s="36"/>
+      <c r="P110" s="36">
+        <v>61.8</v>
+      </c>
       <c r="Q110" s="36"/>
       <c r="R110" s="43"/>
       <c r="S110" s="36"/>
       <c r="T110" s="36"/>
     </row>
     <row r="111" spans="1:20" ht="18" customHeight="1">
-      <c r="A111" s="29"/>
-      <c r="B111" s="30"/>
+      <c r="A111" s="29" t="s">
+        <v>138</v>
+      </c>
+      <c r="B111" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C111" s="29"/>
-      <c r="D111" s="29"/>
-      <c r="E111" s="29"/>
-      <c r="F111" s="95"/>
-      <c r="G111" s="31"/>
-      <c r="H111" s="32"/>
-      <c r="I111" s="38"/>
-      <c r="J111" s="43"/>
+      <c r="D111" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E111" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F111" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G111" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H111" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I111" s="108">
+        <v>298</v>
+      </c>
+      <c r="J111" s="86">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
       <c r="K111" s="34"/>
-      <c r="L111" s="31"/>
-      <c r="M111" s="39"/>
-      <c r="N111" s="35"/>
-      <c r="O111" s="43"/>
-      <c r="P111" s="43"/>
+      <c r="L111" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M111" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N111" s="35" t="s">
+        <v>159</v>
+      </c>
+      <c r="O111" s="36"/>
+      <c r="P111" s="43">
+        <v>50</v>
+      </c>
       <c r="Q111" s="43"/>
       <c r="R111" s="43"/>
       <c r="S111" s="36"/>
       <c r="T111" s="36"/>
     </row>
     <row r="112" spans="1:20" ht="18" customHeight="1">
-      <c r="A112" s="29"/>
-      <c r="B112" s="30"/>
+      <c r="A112" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="B112" s="30" t="s">
+        <v>137</v>
+      </c>
       <c r="C112" s="29"/>
-      <c r="D112" s="29"/>
-      <c r="E112" s="29"/>
-      <c r="F112" s="95"/>
-      <c r="G112" s="31"/>
-      <c r="H112" s="32"/>
-      <c r="I112" s="38"/>
-      <c r="J112" s="43"/>
+      <c r="D112" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E112" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F112" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G112" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H112" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I112" s="108">
+        <v>298</v>
+      </c>
+      <c r="J112" s="86">
+        <f t="shared" si="2"/>
+        <v>0.60699999999999998</v>
+      </c>
       <c r="K112" s="34"/>
-      <c r="L112" s="31"/>
-      <c r="M112" s="39"/>
-      <c r="N112" s="35"/>
+      <c r="L112" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M112" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N112" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O112" s="43"/>
-      <c r="P112" s="43"/>
+      <c r="P112" s="43">
+        <v>60.7</v>
+      </c>
       <c r="Q112" s="43"/>
       <c r="R112" s="43"/>
       <c r="S112" s="36"/>
       <c r="T112" s="36"/>
     </row>
     <row r="113" spans="1:20" ht="18" customHeight="1">
-      <c r="A113" s="29"/>
-      <c r="B113" s="30"/>
+      <c r="A113" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="B113" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C113" s="29"/>
-      <c r="D113" s="29"/>
-      <c r="E113" s="29"/>
-      <c r="F113" s="95"/>
-      <c r="G113" s="31"/>
-      <c r="H113" s="32"/>
-      <c r="I113" s="38"/>
-      <c r="J113" s="43"/>
+      <c r="D113" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E113" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F113" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G113" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H113" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I113" s="108">
+        <v>298</v>
+      </c>
+      <c r="J113" s="86">
+        <f t="shared" si="2"/>
+        <v>0.63100000000000001</v>
+      </c>
       <c r="K113" s="34"/>
-      <c r="L113" s="31"/>
-      <c r="M113" s="39"/>
-      <c r="N113" s="35"/>
+      <c r="L113" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M113" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N113" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O113" s="43"/>
-      <c r="P113" s="43"/>
+      <c r="P113" s="43">
+        <v>63.1</v>
+      </c>
       <c r="Q113" s="43"/>
       <c r="R113" s="43"/>
       <c r="S113" s="36"/>
       <c r="T113" s="36"/>
     </row>
     <row r="114" spans="1:20" ht="18" customHeight="1">
-      <c r="A114" s="29"/>
-      <c r="B114" s="30"/>
+      <c r="A114" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B114" s="30" t="s">
+        <v>140</v>
+      </c>
       <c r="C114" s="29"/>
-      <c r="D114" s="29"/>
-      <c r="E114" s="29"/>
-      <c r="F114" s="95"/>
-      <c r="G114" s="31"/>
-      <c r="H114" s="32"/>
-      <c r="I114" s="38"/>
-      <c r="J114" s="43"/>
+      <c r="D114" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E114" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F114" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G114" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H114" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I114" s="108">
+        <v>298</v>
+      </c>
+      <c r="J114" s="86">
+        <f t="shared" si="2"/>
+        <v>0.51800000000000002</v>
+      </c>
       <c r="K114" s="34"/>
-      <c r="L114" s="31"/>
-      <c r="M114" s="39"/>
-      <c r="N114" s="35"/>
+      <c r="L114" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M114" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N114" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O114" s="43"/>
-      <c r="P114" s="43"/>
+      <c r="P114" s="43">
+        <v>51.8</v>
+      </c>
       <c r="Q114" s="43"/>
       <c r="R114" s="43"/>
       <c r="S114" s="36"/>
       <c r="T114" s="36"/>
     </row>
     <row r="115" spans="1:20" ht="18" customHeight="1">
-      <c r="A115" s="29"/>
-      <c r="B115" s="30"/>
+      <c r="A115" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B115" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C115" s="29"/>
-      <c r="D115" s="29"/>
-      <c r="E115" s="29"/>
-      <c r="F115" s="95"/>
-      <c r="G115" s="31"/>
-      <c r="H115" s="32"/>
-      <c r="I115" s="38"/>
-      <c r="J115" s="43"/>
+      <c r="D115" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E115" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F115" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G115" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H115" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I115" s="108">
+        <v>298</v>
+      </c>
+      <c r="J115" s="86">
+        <f t="shared" si="2"/>
+        <v>0.43</v>
+      </c>
       <c r="K115" s="34"/>
-      <c r="L115" s="31"/>
-      <c r="M115" s="39"/>
-      <c r="N115" s="35"/>
+      <c r="L115" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M115" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N115" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O115" s="43"/>
-      <c r="P115" s="43"/>
+      <c r="P115" s="43">
+        <v>43</v>
+      </c>
       <c r="Q115" s="43"/>
       <c r="R115" s="43"/>
       <c r="S115" s="36"/>
       <c r="T115" s="36"/>
     </row>
     <row r="116" spans="1:20" ht="18" customHeight="1">
-      <c r="A116" s="29"/>
-      <c r="B116" s="30"/>
+      <c r="A116" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B116" s="30" t="s">
+        <v>141</v>
+      </c>
       <c r="C116" s="29"/>
-      <c r="D116" s="29"/>
-      <c r="E116" s="29"/>
-      <c r="F116" s="95"/>
-      <c r="G116" s="31"/>
-      <c r="H116" s="32"/>
-      <c r="I116" s="38"/>
-      <c r="J116" s="43"/>
+      <c r="D116" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E116" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F116" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G116" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H116" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I116" s="108">
+        <v>298</v>
+      </c>
+      <c r="J116" s="86">
+        <f t="shared" si="2"/>
+        <v>0.56699999999999995</v>
+      </c>
       <c r="K116" s="34"/>
-      <c r="L116" s="31"/>
-      <c r="M116" s="39"/>
-      <c r="N116" s="35"/>
+      <c r="L116" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M116" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N116" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O116" s="43"/>
-      <c r="P116" s="43"/>
+      <c r="P116" s="43">
+        <v>56.7</v>
+      </c>
       <c r="Q116" s="43"/>
       <c r="R116" s="43"/>
       <c r="S116" s="36"/>
       <c r="T116" s="36"/>
     </row>
     <row r="117" spans="1:20" ht="18" customHeight="1">
-      <c r="A117" s="29"/>
-      <c r="B117" s="30"/>
+      <c r="A117" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B117" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C117" s="29"/>
-      <c r="D117" s="29"/>
-      <c r="E117" s="29"/>
-      <c r="F117" s="31"/>
-      <c r="G117" s="31"/>
-      <c r="H117" s="32"/>
-      <c r="I117" s="38"/>
-      <c r="J117" s="86"/>
+      <c r="D117" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="E117" s="88" t="s">
+        <v>151</v>
+      </c>
+      <c r="F117" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G117" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H117" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I117" s="108">
+        <v>298</v>
+      </c>
+      <c r="J117" s="86">
+        <f t="shared" si="2"/>
+        <v>0.51800000000000002</v>
+      </c>
       <c r="K117" s="34"/>
-      <c r="L117" s="31"/>
-      <c r="M117" s="39"/>
-      <c r="N117" s="35"/>
+      <c r="L117" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M117" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N117" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O117" s="43"/>
-      <c r="P117" s="43"/>
+      <c r="P117" s="43">
+        <v>51.8</v>
+      </c>
       <c r="Q117" s="37"/>
       <c r="R117" s="43"/>
       <c r="S117" s="36"/>
       <c r="T117" s="36"/>
     </row>
     <row r="118" spans="1:20" ht="18" customHeight="1">
-      <c r="A118" s="29"/>
-      <c r="B118" s="30"/>
+      <c r="A118" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B118" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="C118" s="29"/>
-      <c r="D118" s="29"/>
-      <c r="E118" s="29"/>
-      <c r="F118" s="31"/>
-      <c r="G118" s="31"/>
-      <c r="H118" s="32"/>
-      <c r="I118" s="38"/>
-      <c r="J118" s="86"/>
+      <c r="D118" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="E118" s="88" t="s">
+        <v>152</v>
+      </c>
+      <c r="F118" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="G118" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H118" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I118" s="108">
+        <v>298</v>
+      </c>
+      <c r="J118" s="86">
+        <f t="shared" si="2"/>
+        <v>0.49399999999999999</v>
+      </c>
       <c r="K118" s="34"/>
-      <c r="L118" s="31"/>
-      <c r="M118" s="39"/>
-      <c r="N118" s="35"/>
+      <c r="L118" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="M118" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="N118" s="35" t="s">
+        <v>159</v>
+      </c>
       <c r="O118" s="43"/>
-      <c r="P118" s="43"/>
+      <c r="P118" s="43">
+        <v>49.4</v>
+      </c>
       <c r="Q118" s="37"/>
       <c r="R118" s="43"/>
       <c r="S118" s="36"/>
@@ -7023,7 +8695,7 @@
       <c r="L124" s="31"/>
       <c r="M124" s="39"/>
       <c r="N124" s="35"/>
-      <c r="O124" s="36"/>
+      <c r="O124" s="43"/>
       <c r="P124" s="36"/>
       <c r="Q124" s="37"/>
       <c r="R124" s="43"/>
@@ -9047,7 +10719,7 @@
       <c r="L216" s="39"/>
       <c r="M216" s="39"/>
       <c r="N216" s="29"/>
-      <c r="O216" s="42"/>
+      <c r="O216" s="36"/>
       <c r="P216" s="42"/>
       <c r="Q216" s="42"/>
       <c r="R216" s="36"/>
@@ -10367,7 +12039,7 @@
       <c r="L276" s="39"/>
       <c r="M276" s="39"/>
       <c r="N276" s="39"/>
-      <c r="O276" s="89"/>
+      <c r="O276" s="42"/>
       <c r="P276" s="42"/>
       <c r="Q276" s="42"/>
       <c r="R276" s="42"/>
@@ -10389,7 +12061,7 @@
       <c r="L277" s="55"/>
       <c r="M277" s="55"/>
       <c r="N277" s="39"/>
-      <c r="O277" s="42"/>
+      <c r="O277" s="89"/>
       <c r="P277" s="42"/>
       <c r="Q277" s="42"/>
       <c r="R277" s="42"/>
@@ -25252,6 +26924,7 @@
       <c r="T956" s="42"/>
     </row>
     <row r="957" spans="1:20" ht="15" customHeight="1">
+      <c r="O957" s="42"/>
       <c r="R957" s="42"/>
       <c r="S957" s="42"/>
       <c r="T957" s="42"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jmrt.2026.05.105`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE686C7-FBB6-5148-BA12-DFF4828F4960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010B7EF2-4B12-8945-802B-53C9FE7C4A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="162">
   <si>
     <r>
       <rPr>
@@ -610,6 +610,12 @@
   </si>
   <si>
     <t>10.1016/j.jmrt.2025.12.182</t>
+  </si>
+  <si>
+    <t>Mo7 Nb15 Ta26 V45 W7</t>
+  </si>
+  <si>
+    <t>10.1016/j.jmrt.2026.05.105</t>
   </si>
 </sst>
 </file>
@@ -1847,56 +1853,15 @@
     <xf numFmtId="49" fontId="17" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="10" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1958,15 +1923,56 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="10" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="10" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3184,19 +3190,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="12"/>
-      <c r="D2" s="131" t="s">
+      <c r="D2" s="120" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="132"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="136"/>
-      <c r="H2" s="136"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="138"/>
-      <c r="K2" s="138"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="139"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="124"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="127"/>
+      <c r="K2" s="127"/>
+      <c r="L2" s="125"/>
+      <c r="M2" s="125"/>
+      <c r="N2" s="128"/>
       <c r="O2" s="13"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -3212,17 +3218,17 @@
         <v>72</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="133"/>
-      <c r="E3" s="134"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="140"/>
-      <c r="H3" s="140"/>
-      <c r="I3" s="141"/>
-      <c r="J3" s="142"/>
-      <c r="K3" s="142"/>
-      <c r="L3" s="140"/>
-      <c r="M3" s="140"/>
-      <c r="N3" s="143"/>
+      <c r="D3" s="122"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="129"/>
+      <c r="G3" s="129"/>
+      <c r="H3" s="129"/>
+      <c r="I3" s="130"/>
+      <c r="J3" s="131"/>
+      <c r="K3" s="131"/>
+      <c r="L3" s="129"/>
+      <c r="M3" s="129"/>
+      <c r="N3" s="132"/>
       <c r="O3" s="13"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -3263,43 +3269,43 @@
       <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="144" t="s">
+      <c r="C5" s="133" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="146" t="s">
+      <c r="D5" s="135" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="146" t="s">
+      <c r="E5" s="135" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="146" t="s">
+      <c r="F5" s="135" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="146" t="s">
+      <c r="G5" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="147" t="s">
+      <c r="H5" s="136" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="146" t="s">
+      <c r="I5" s="135" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="146" t="s">
+      <c r="J5" s="135" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="146" t="s">
+      <c r="K5" s="135" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="146" t="s">
+      <c r="L5" s="135" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="146" t="s">
+      <c r="M5" s="135" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="146" t="s">
+      <c r="N5" s="135" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="114" t="s">
+      <c r="O5" s="140" t="s">
         <v>19</v>
       </c>
       <c r="P5" s="24"/>
@@ -3315,19 +3321,19 @@
       <c r="B6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="145"/>
-      <c r="D6" s="145"/>
-      <c r="E6" s="145"/>
-      <c r="F6" s="145"/>
-      <c r="G6" s="145"/>
-      <c r="H6" s="148"/>
-      <c r="I6" s="149"/>
-      <c r="J6" s="150"/>
-      <c r="K6" s="150"/>
-      <c r="L6" s="145"/>
-      <c r="M6" s="145"/>
-      <c r="N6" s="145"/>
-      <c r="O6" s="115"/>
+      <c r="C6" s="134"/>
+      <c r="D6" s="134"/>
+      <c r="E6" s="134"/>
+      <c r="F6" s="134"/>
+      <c r="G6" s="134"/>
+      <c r="H6" s="137"/>
+      <c r="I6" s="138"/>
+      <c r="J6" s="139"/>
+      <c r="K6" s="139"/>
+      <c r="L6" s="134"/>
+      <c r="M6" s="134"/>
+      <c r="N6" s="134"/>
+      <c r="O6" s="141"/>
       <c r="P6" s="24"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="9"/>
@@ -3377,7 +3383,7 @@
       <c r="N7" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="O7" s="116"/>
+      <c r="O7" s="142"/>
       <c r="P7" s="62" t="s">
         <v>61</v>
       </c>
@@ -3392,35 +3398,35 @@
     </row>
     <row r="8" spans="1:20" ht="20.25" customHeight="1" thickBot="1">
       <c r="A8" s="57"/>
-      <c r="B8" s="117" t="s">
+      <c r="B8" s="143" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="118"/>
-      <c r="D8" s="118"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="120" t="s">
+      <c r="C8" s="144"/>
+      <c r="D8" s="144"/>
+      <c r="E8" s="145"/>
+      <c r="F8" s="146" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="121"/>
-      <c r="H8" s="121"/>
-      <c r="I8" s="122"/>
-      <c r="J8" s="123"/>
-      <c r="K8" s="123"/>
-      <c r="L8" s="124"/>
-      <c r="M8" s="125" t="s">
+      <c r="G8" s="147"/>
+      <c r="H8" s="147"/>
+      <c r="I8" s="148"/>
+      <c r="J8" s="149"/>
+      <c r="K8" s="149"/>
+      <c r="L8" s="150"/>
+      <c r="M8" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="126"/>
+      <c r="N8" s="152"/>
       <c r="O8" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="P8" s="127" t="s">
+      <c r="P8" s="153" t="s">
         <v>41</v>
       </c>
-      <c r="Q8" s="128"/>
-      <c r="R8" s="129"/>
-      <c r="S8" s="129"/>
-      <c r="T8" s="130"/>
+      <c r="Q8" s="154"/>
+      <c r="R8" s="155"/>
+      <c r="S8" s="155"/>
+      <c r="T8" s="156"/>
     </row>
     <row r="9" spans="1:20" ht="21" customHeight="1" thickBot="1">
       <c r="A9" s="58" t="s">
@@ -4953,7 +4959,7 @@
       <c r="T41" s="36"/>
     </row>
     <row r="42" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A42" s="151" t="s">
+      <c r="A42" s="114" t="s">
         <v>103</v>
       </c>
       <c r="B42" s="100" t="s">
@@ -4999,7 +5005,7 @@
       <c r="T42" s="36"/>
     </row>
     <row r="43" spans="1:20" ht="18" customHeight="1">
-      <c r="A43" s="152" t="s">
+      <c r="A43" s="115" t="s">
         <v>104</v>
       </c>
       <c r="B43" s="102" t="s">
@@ -5047,7 +5053,7 @@
       <c r="T43" s="36"/>
     </row>
     <row r="44" spans="1:20" ht="18" customHeight="1">
-      <c r="A44" s="152" t="s">
+      <c r="A44" s="115" t="s">
         <v>105</v>
       </c>
       <c r="B44" s="102" t="s">
@@ -5093,7 +5099,7 @@
       <c r="T44" s="36"/>
     </row>
     <row r="45" spans="1:20" ht="18" customHeight="1">
-      <c r="A45" s="152" t="s">
+      <c r="A45" s="115" t="s">
         <v>106</v>
       </c>
       <c r="B45" s="102" t="s">
@@ -5139,7 +5145,7 @@
       <c r="T45" s="36"/>
     </row>
     <row r="46" spans="1:20" ht="18" customHeight="1">
-      <c r="A46" s="152" t="s">
+      <c r="A46" s="115" t="s">
         <v>107</v>
       </c>
       <c r="B46" s="102" t="s">
@@ -5210,10 +5216,10 @@
       <c r="I47" s="69">
         <v>298</v>
       </c>
-      <c r="J47" s="153">
+      <c r="J47" s="116">
         <v>1597000000</v>
       </c>
-      <c r="K47" s="154">
+      <c r="K47" s="117">
         <v>18000000</v>
       </c>
       <c r="L47" s="31" t="s">
@@ -5258,10 +5264,10 @@
       <c r="I48" s="69">
         <v>298</v>
       </c>
-      <c r="J48" s="153">
+      <c r="J48" s="116">
         <v>1794000000</v>
       </c>
-      <c r="K48" s="154">
+      <c r="K48" s="117">
         <v>44000000</v>
       </c>
       <c r="L48" s="31" t="s">
@@ -5306,10 +5312,10 @@
       <c r="I49" s="69">
         <v>298</v>
       </c>
-      <c r="J49" s="153">
+      <c r="J49" s="116">
         <v>1764000000</v>
       </c>
-      <c r="K49" s="154">
+      <c r="K49" s="117">
         <v>41000000</v>
       </c>
       <c r="L49" s="31" t="s">
@@ -5357,7 +5363,7 @@
       <c r="J50" s="86">
         <v>2032000000</v>
       </c>
-      <c r="K50" s="154">
+      <c r="K50" s="117">
         <v>17000000</v>
       </c>
       <c r="L50" s="31" t="s">
@@ -5473,7 +5479,7 @@
       <c r="T52" s="36"/>
     </row>
     <row r="53" spans="1:20" ht="18" customHeight="1">
-      <c r="A53" s="151" t="s">
+      <c r="A53" s="114" t="s">
         <v>121</v>
       </c>
       <c r="B53" s="100" t="s">
@@ -5521,7 +5527,7 @@
       <c r="T53" s="36"/>
     </row>
     <row r="54" spans="1:20" ht="18" customHeight="1">
-      <c r="A54" s="152" t="s">
+      <c r="A54" s="115" t="s">
         <v>122</v>
       </c>
       <c r="B54" s="102" t="s">
@@ -5569,7 +5575,7 @@
       <c r="T54" s="36"/>
     </row>
     <row r="55" spans="1:20" ht="18" customHeight="1">
-      <c r="A55" s="152" t="s">
+      <c r="A55" s="115" t="s">
         <v>123</v>
       </c>
       <c r="B55" s="102" t="s">
@@ -6891,7 +6897,7 @@
       <c r="T83" s="36"/>
     </row>
     <row r="84" spans="1:20" ht="18" customHeight="1">
-      <c r="A84" s="151" t="s">
+      <c r="A84" s="114" t="s">
         <v>128</v>
       </c>
       <c r="B84" s="102" t="s">
@@ -6910,7 +6916,7 @@
       <c r="G84" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H84" s="155"/>
+      <c r="H84" s="118"/>
       <c r="I84" s="108">
         <v>298</v>
       </c>
@@ -6935,7 +6941,7 @@
       <c r="T84" s="36"/>
     </row>
     <row r="85" spans="1:20" ht="18" customHeight="1">
-      <c r="A85" s="152" t="s">
+      <c r="A85" s="115" t="s">
         <v>131</v>
       </c>
       <c r="B85" s="102" t="s">
@@ -6954,7 +6960,7 @@
       <c r="G85" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H85" s="156"/>
+      <c r="H85" s="119"/>
       <c r="I85" s="108">
         <v>298</v>
       </c>
@@ -6979,7 +6985,7 @@
       <c r="T85" s="36"/>
     </row>
     <row r="86" spans="1:20" ht="18" customHeight="1">
-      <c r="A86" s="152" t="s">
+      <c r="A86" s="115" t="s">
         <v>134</v>
       </c>
       <c r="B86" s="102" t="s">
@@ -6998,7 +7004,7 @@
       <c r="G86" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H86" s="156"/>
+      <c r="H86" s="119"/>
       <c r="I86" s="108">
         <v>298</v>
       </c>
@@ -7023,7 +7029,7 @@
       <c r="T86" s="36"/>
     </row>
     <row r="87" spans="1:20" ht="18" customHeight="1">
-      <c r="A87" s="152" t="s">
+      <c r="A87" s="115" t="s">
         <v>138</v>
       </c>
       <c r="B87" s="102" t="s">
@@ -7042,7 +7048,7 @@
       <c r="G87" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H87" s="156"/>
+      <c r="H87" s="119"/>
       <c r="I87" s="108">
         <v>298</v>
       </c>
@@ -7067,7 +7073,7 @@
       <c r="T87" s="36"/>
     </row>
     <row r="88" spans="1:20" ht="18" customHeight="1">
-      <c r="A88" s="152" t="s">
+      <c r="A88" s="115" t="s">
         <v>142</v>
       </c>
       <c r="B88" s="102" t="s">
@@ -7086,7 +7092,7 @@
       <c r="G88" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H88" s="156"/>
+      <c r="H88" s="119"/>
       <c r="I88" s="108">
         <v>298</v>
       </c>
@@ -7111,7 +7117,7 @@
       <c r="T88" s="36"/>
     </row>
     <row r="89" spans="1:20" ht="18" customHeight="1">
-      <c r="A89" s="152" t="s">
+      <c r="A89" s="115" t="s">
         <v>144</v>
       </c>
       <c r="B89" s="102" t="s">
@@ -7130,7 +7136,7 @@
       <c r="G89" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H89" s="156"/>
+      <c r="H89" s="119"/>
       <c r="I89" s="108">
         <v>298</v>
       </c>
@@ -7155,7 +7161,7 @@
       <c r="T89" s="36"/>
     </row>
     <row r="90" spans="1:20" ht="18" customHeight="1">
-      <c r="A90" s="152" t="s">
+      <c r="A90" s="115" t="s">
         <v>146</v>
       </c>
       <c r="B90" s="102" t="s">
@@ -7174,7 +7180,7 @@
       <c r="G90" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="H90" s="156"/>
+      <c r="H90" s="119"/>
       <c r="I90" s="108">
         <v>298</v>
       </c>
@@ -8572,19 +8578,41 @@
     </row>
     <row r="119" spans="1:20" ht="18" customHeight="1">
       <c r="A119" s="29"/>
-      <c r="B119" s="30"/>
-      <c r="C119" s="29"/>
-      <c r="D119" s="29"/>
+      <c r="B119" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C119" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D119" s="29" t="s">
+        <v>65</v>
+      </c>
       <c r="E119" s="29"/>
-      <c r="F119" s="31"/>
-      <c r="G119" s="31"/>
+      <c r="F119" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G119" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H119" s="32"/>
-      <c r="I119" s="38"/>
-      <c r="J119" s="86"/>
-      <c r="K119" s="34"/>
-      <c r="L119" s="31"/>
-      <c r="M119" s="39"/>
-      <c r="N119" s="35"/>
+      <c r="I119" s="108">
+        <v>298</v>
+      </c>
+      <c r="J119" s="86">
+        <v>1720000000</v>
+      </c>
+      <c r="K119" s="34">
+        <v>30000000</v>
+      </c>
+      <c r="L119" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M119" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N119" s="35" t="s">
+        <v>161</v>
+      </c>
       <c r="O119" s="43"/>
       <c r="P119" s="43"/>
       <c r="Q119" s="37"/>
@@ -8594,19 +8622,41 @@
     </row>
     <row r="120" spans="1:20" ht="18" customHeight="1">
       <c r="A120" s="29"/>
-      <c r="B120" s="30"/>
-      <c r="C120" s="29"/>
-      <c r="D120" s="29"/>
+      <c r="B120" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C120" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D120" s="29" t="s">
+        <v>65</v>
+      </c>
       <c r="E120" s="29"/>
-      <c r="F120" s="31"/>
-      <c r="G120" s="31"/>
+      <c r="F120" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G120" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H120" s="32"/>
-      <c r="I120" s="38"/>
-      <c r="J120" s="86"/>
-      <c r="K120" s="34"/>
-      <c r="L120" s="31"/>
-      <c r="M120" s="39"/>
-      <c r="N120" s="35"/>
+      <c r="I120" s="108">
+        <v>298</v>
+      </c>
+      <c r="J120" s="86">
+        <v>41.7</v>
+      </c>
+      <c r="K120" s="34">
+        <v>2.1</v>
+      </c>
+      <c r="L120" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M120" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N120" s="35" t="s">
+        <v>161</v>
+      </c>
       <c r="O120" s="43"/>
       <c r="P120" s="43"/>
       <c r="Q120" s="37"/>
@@ -8616,22 +8666,50 @@
     </row>
     <row r="121" spans="1:20" ht="18" customHeight="1">
       <c r="A121" s="29"/>
-      <c r="B121" s="30"/>
-      <c r="C121" s="29"/>
-      <c r="D121" s="29"/>
+      <c r="B121" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C121" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D121" s="29" t="s">
+        <v>65</v>
+      </c>
       <c r="E121" s="29"/>
-      <c r="F121" s="31"/>
-      <c r="G121" s="31"/>
+      <c r="F121" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G121" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H121" s="32"/>
-      <c r="I121" s="38"/>
-      <c r="J121" s="86"/>
-      <c r="K121" s="34"/>
-      <c r="L121" s="31"/>
-      <c r="M121" s="39"/>
-      <c r="N121" s="35"/>
+      <c r="I121" s="108">
+        <v>298</v>
+      </c>
+      <c r="J121" s="86">
+        <f t="shared" ref="J121:K121" si="3">P121*9807000</f>
+        <v>5285973000</v>
+      </c>
+      <c r="K121" s="86">
+        <f t="shared" si="3"/>
+        <v>117684000</v>
+      </c>
+      <c r="L121" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M121" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="N121" s="35" t="s">
+        <v>161</v>
+      </c>
       <c r="O121" s="43"/>
-      <c r="P121" s="43"/>
-      <c r="Q121" s="37"/>
+      <c r="P121" s="43">
+        <v>539</v>
+      </c>
+      <c r="Q121" s="37">
+        <v>12</v>
+      </c>
       <c r="R121" s="43"/>
       <c r="S121" s="36"/>
       <c r="T121" s="36"/>
@@ -8777,7 +8855,7 @@
       <c r="F128" s="31"/>
       <c r="G128" s="31"/>
       <c r="H128" s="32"/>
-      <c r="I128" s="38"/>
+      <c r="I128" s="33"/>
       <c r="J128" s="86"/>
       <c r="K128" s="34"/>
       <c r="L128" s="31"/>
@@ -8866,7 +8944,7 @@
       <c r="G132" s="31"/>
       <c r="H132" s="32"/>
       <c r="I132" s="33"/>
-      <c r="J132" s="86"/>
+      <c r="J132" s="43"/>
       <c r="K132" s="34"/>
       <c r="L132" s="31"/>
       <c r="M132" s="31"/>
@@ -8998,7 +9076,7 @@
       <c r="G138" s="31"/>
       <c r="H138" s="32"/>
       <c r="I138" s="33"/>
-      <c r="J138" s="43"/>
+      <c r="J138" s="34"/>
       <c r="K138" s="34"/>
       <c r="L138" s="31"/>
       <c r="M138" s="31"/>
@@ -9033,11 +9111,11 @@
       <c r="T139" s="36"/>
     </row>
     <row r="140" spans="1:20" ht="18" customHeight="1">
-      <c r="A140" s="29"/>
+      <c r="A140" s="48"/>
       <c r="B140" s="30"/>
-      <c r="C140" s="29"/>
+      <c r="C140" s="88"/>
       <c r="D140" s="29"/>
-      <c r="E140" s="29"/>
+      <c r="E140" s="30"/>
       <c r="F140" s="31"/>
       <c r="G140" s="31"/>
       <c r="H140" s="32"/>
@@ -9079,7 +9157,7 @@
     <row r="142" spans="1:20" ht="18" customHeight="1">
       <c r="A142" s="48"/>
       <c r="B142" s="30"/>
-      <c r="C142" s="88"/>
+      <c r="C142" s="29"/>
       <c r="D142" s="29"/>
       <c r="E142" s="30"/>
       <c r="F142" s="31"/>
@@ -9101,7 +9179,7 @@
     <row r="143" spans="1:20" ht="18" customHeight="1">
       <c r="A143" s="48"/>
       <c r="B143" s="30"/>
-      <c r="C143" s="29"/>
+      <c r="C143" s="88"/>
       <c r="D143" s="29"/>
       <c r="E143" s="30"/>
       <c r="F143" s="31"/>
@@ -9167,7 +9245,7 @@
     <row r="146" spans="1:20" ht="18" customHeight="1">
       <c r="A146" s="48"/>
       <c r="B146" s="30"/>
-      <c r="C146" s="88"/>
+      <c r="C146" s="29"/>
       <c r="D146" s="29"/>
       <c r="E146" s="30"/>
       <c r="F146" s="31"/>
@@ -9189,15 +9267,15 @@
     <row r="147" spans="1:20" ht="18" customHeight="1">
       <c r="A147" s="48"/>
       <c r="B147" s="30"/>
-      <c r="C147" s="29"/>
+      <c r="C147" s="88"/>
       <c r="D147" s="29"/>
       <c r="E147" s="30"/>
-      <c r="F147" s="31"/>
+      <c r="F147" s="50"/>
       <c r="G147" s="31"/>
       <c r="H147" s="32"/>
       <c r="I147" s="33"/>
-      <c r="J147" s="34"/>
-      <c r="K147" s="34"/>
+      <c r="J147" s="56"/>
+      <c r="K147" s="49"/>
       <c r="L147" s="31"/>
       <c r="M147" s="31"/>
       <c r="N147" s="29"/>
@@ -9211,7 +9289,7 @@
     <row r="148" spans="1:20" ht="18" customHeight="1">
       <c r="A148" s="48"/>
       <c r="B148" s="30"/>
-      <c r="C148" s="88"/>
+      <c r="C148" s="29"/>
       <c r="D148" s="29"/>
       <c r="E148" s="30"/>
       <c r="F148" s="50"/>
@@ -9241,7 +9319,7 @@
       <c r="H149" s="32"/>
       <c r="I149" s="33"/>
       <c r="J149" s="56"/>
-      <c r="K149" s="49"/>
+      <c r="K149" s="46"/>
       <c r="L149" s="31"/>
       <c r="M149" s="47"/>
       <c r="N149" s="29"/>
@@ -9284,7 +9362,7 @@
       <c r="G151" s="31"/>
       <c r="H151" s="32"/>
       <c r="I151" s="33"/>
-      <c r="J151" s="56"/>
+      <c r="J151" s="46"/>
       <c r="K151" s="46"/>
       <c r="L151" s="31"/>
       <c r="M151" s="47"/>
@@ -9373,7 +9451,7 @@
       <c r="H155" s="32"/>
       <c r="I155" s="33"/>
       <c r="J155" s="46"/>
-      <c r="K155" s="46"/>
+      <c r="K155" s="37"/>
       <c r="L155" s="31"/>
       <c r="M155" s="47"/>
       <c r="N155" s="29"/>
@@ -9452,10 +9530,10 @@
     </row>
     <row r="159" spans="1:20" ht="18" customHeight="1">
       <c r="A159" s="48"/>
-      <c r="B159" s="30"/>
-      <c r="C159" s="29"/>
-      <c r="D159" s="29"/>
-      <c r="E159" s="30"/>
+      <c r="B159" s="99"/>
+      <c r="C159" s="87"/>
+      <c r="D159" s="87"/>
+      <c r="E159" s="100"/>
       <c r="F159" s="50"/>
       <c r="G159" s="31"/>
       <c r="H159" s="32"/>
@@ -9474,16 +9552,16 @@
     </row>
     <row r="160" spans="1:20" ht="18" customHeight="1">
       <c r="A160" s="48"/>
-      <c r="B160" s="99"/>
-      <c r="C160" s="87"/>
-      <c r="D160" s="87"/>
-      <c r="E160" s="100"/>
+      <c r="B160" s="101"/>
+      <c r="C160" s="88"/>
+      <c r="D160" s="88"/>
+      <c r="E160" s="102"/>
       <c r="F160" s="50"/>
       <c r="G160" s="31"/>
       <c r="H160" s="32"/>
       <c r="I160" s="33"/>
       <c r="J160" s="46"/>
-      <c r="K160" s="37"/>
+      <c r="K160" s="49"/>
       <c r="L160" s="31"/>
       <c r="M160" s="47"/>
       <c r="N160" s="29"/>
@@ -9518,10 +9596,10 @@
     </row>
     <row r="162" spans="1:20" ht="18" customHeight="1">
       <c r="A162" s="48"/>
-      <c r="B162" s="101"/>
-      <c r="C162" s="88"/>
-      <c r="D162" s="88"/>
-      <c r="E162" s="102"/>
+      <c r="B162" s="99"/>
+      <c r="C162" s="87"/>
+      <c r="D162" s="87"/>
+      <c r="E162" s="100"/>
       <c r="F162" s="50"/>
       <c r="G162" s="31"/>
       <c r="H162" s="32"/>
@@ -9540,10 +9618,10 @@
     </row>
     <row r="163" spans="1:20" ht="18" customHeight="1">
       <c r="A163" s="48"/>
-      <c r="B163" s="99"/>
-      <c r="C163" s="87"/>
-      <c r="D163" s="87"/>
-      <c r="E163" s="100"/>
+      <c r="B163" s="101"/>
+      <c r="C163" s="88"/>
+      <c r="D163" s="88"/>
+      <c r="E163" s="102"/>
       <c r="F163" s="50"/>
       <c r="G163" s="31"/>
       <c r="H163" s="32"/>
@@ -9571,7 +9649,7 @@
       <c r="H164" s="32"/>
       <c r="I164" s="33"/>
       <c r="J164" s="46"/>
-      <c r="K164" s="49"/>
+      <c r="K164" s="37"/>
       <c r="L164" s="31"/>
       <c r="M164" s="47"/>
       <c r="N164" s="29"/>
@@ -9584,15 +9662,15 @@
     </row>
     <row r="165" spans="1:20" ht="18" customHeight="1">
       <c r="A165" s="48"/>
-      <c r="B165" s="101"/>
-      <c r="C165" s="88"/>
-      <c r="D165" s="88"/>
-      <c r="E165" s="102"/>
+      <c r="B165" s="30"/>
+      <c r="C165" s="29"/>
+      <c r="D165" s="29"/>
+      <c r="E165" s="30"/>
       <c r="F165" s="50"/>
       <c r="G165" s="31"/>
       <c r="H165" s="32"/>
       <c r="I165" s="33"/>
-      <c r="J165" s="46"/>
+      <c r="J165" s="34"/>
       <c r="K165" s="37"/>
       <c r="L165" s="31"/>
       <c r="M165" s="47"/>
@@ -9680,7 +9758,7 @@
       <c r="G169" s="31"/>
       <c r="H169" s="32"/>
       <c r="I169" s="33"/>
-      <c r="J169" s="34"/>
+      <c r="J169" s="46"/>
       <c r="K169" s="37"/>
       <c r="L169" s="31"/>
       <c r="M169" s="47"/>
@@ -9759,15 +9837,15 @@
       <c r="T172" s="36"/>
     </row>
     <row r="173" spans="1:20" ht="18" customHeight="1">
-      <c r="A173" s="48"/>
-      <c r="B173" s="30"/>
-      <c r="C173" s="29"/>
-      <c r="D173" s="29"/>
-      <c r="E173" s="30"/>
-      <c r="F173" s="50"/>
-      <c r="G173" s="31"/>
+      <c r="A173" s="105"/>
+      <c r="B173" s="100"/>
+      <c r="C173" s="87"/>
+      <c r="D173" s="87"/>
+      <c r="E173" s="100"/>
+      <c r="F173" s="94"/>
+      <c r="G173" s="94"/>
       <c r="H173" s="32"/>
-      <c r="I173" s="33"/>
+      <c r="I173" s="106"/>
       <c r="J173" s="46"/>
       <c r="K173" s="37"/>
       <c r="L173" s="31"/>
@@ -9781,15 +9859,15 @@
       <c r="T173" s="36"/>
     </row>
     <row r="174" spans="1:20" ht="18" customHeight="1">
-      <c r="A174" s="105"/>
-      <c r="B174" s="100"/>
-      <c r="C174" s="87"/>
-      <c r="D174" s="87"/>
-      <c r="E174" s="100"/>
+      <c r="A174" s="107"/>
+      <c r="B174" s="102"/>
+      <c r="C174" s="88"/>
+      <c r="D174" s="88"/>
+      <c r="E174" s="102"/>
       <c r="F174" s="94"/>
-      <c r="G174" s="94"/>
+      <c r="G174" s="95"/>
       <c r="H174" s="32"/>
-      <c r="I174" s="106"/>
+      <c r="I174" s="108"/>
       <c r="J174" s="46"/>
       <c r="K174" s="37"/>
       <c r="L174" s="31"/>
@@ -9834,7 +9912,7 @@
       <c r="G176" s="95"/>
       <c r="H176" s="32"/>
       <c r="I176" s="108"/>
-      <c r="J176" s="46"/>
+      <c r="J176" s="34"/>
       <c r="K176" s="37"/>
       <c r="L176" s="31"/>
       <c r="M176" s="47"/>
@@ -9847,15 +9925,15 @@
       <c r="T176" s="36"/>
     </row>
     <row r="177" spans="1:20" ht="18" customHeight="1">
-      <c r="A177" s="107"/>
-      <c r="B177" s="102"/>
-      <c r="C177" s="88"/>
-      <c r="D177" s="88"/>
-      <c r="E177" s="102"/>
+      <c r="A177" s="105"/>
+      <c r="B177" s="100"/>
+      <c r="C177" s="87"/>
+      <c r="D177" s="87"/>
+      <c r="E177" s="100"/>
       <c r="F177" s="94"/>
-      <c r="G177" s="95"/>
+      <c r="G177" s="94"/>
       <c r="H177" s="32"/>
-      <c r="I177" s="108"/>
+      <c r="I177" s="106"/>
       <c r="J177" s="34"/>
       <c r="K177" s="37"/>
       <c r="L177" s="31"/>
@@ -9869,15 +9947,15 @@
       <c r="T177" s="36"/>
     </row>
     <row r="178" spans="1:20" ht="18" customHeight="1">
-      <c r="A178" s="105"/>
-      <c r="B178" s="100"/>
-      <c r="C178" s="87"/>
-      <c r="D178" s="87"/>
-      <c r="E178" s="100"/>
+      <c r="A178" s="107"/>
+      <c r="B178" s="102"/>
+      <c r="C178" s="88"/>
+      <c r="D178" s="88"/>
+      <c r="E178" s="102"/>
       <c r="F178" s="94"/>
-      <c r="G178" s="94"/>
+      <c r="G178" s="95"/>
       <c r="H178" s="32"/>
-      <c r="I178" s="106"/>
+      <c r="I178" s="108"/>
       <c r="J178" s="34"/>
       <c r="K178" s="37"/>
       <c r="L178" s="31"/>
@@ -9935,16 +10013,16 @@
       <c r="T180" s="36"/>
     </row>
     <row r="181" spans="1:20" ht="18" customHeight="1">
-      <c r="A181" s="107"/>
-      <c r="B181" s="102"/>
-      <c r="C181" s="88"/>
-      <c r="D181" s="88"/>
-      <c r="E181" s="102"/>
-      <c r="F181" s="94"/>
-      <c r="G181" s="95"/>
-      <c r="H181" s="32"/>
-      <c r="I181" s="108"/>
-      <c r="J181" s="34"/>
+      <c r="A181" s="48"/>
+      <c r="B181" s="30"/>
+      <c r="C181" s="29"/>
+      <c r="D181" s="29"/>
+      <c r="E181" s="30"/>
+      <c r="F181" s="50"/>
+      <c r="G181" s="31"/>
+      <c r="H181" s="54"/>
+      <c r="I181" s="52"/>
+      <c r="J181" s="49"/>
       <c r="K181" s="37"/>
       <c r="L181" s="31"/>
       <c r="M181" s="47"/>
@@ -10023,13 +10101,13 @@
       <c r="T184" s="36"/>
     </row>
     <row r="185" spans="1:20" ht="18" customHeight="1">
-      <c r="A185" s="48"/>
-      <c r="B185" s="30"/>
-      <c r="C185" s="29"/>
-      <c r="D185" s="29"/>
-      <c r="E185" s="30"/>
-      <c r="F185" s="50"/>
-      <c r="G185" s="31"/>
+      <c r="A185" s="105"/>
+      <c r="B185" s="100"/>
+      <c r="C185" s="87"/>
+      <c r="D185" s="87"/>
+      <c r="E185" s="100"/>
+      <c r="F185" s="94"/>
+      <c r="G185" s="94"/>
       <c r="H185" s="54"/>
       <c r="I185" s="52"/>
       <c r="J185" s="49"/>
@@ -10045,13 +10123,13 @@
       <c r="T185" s="36"/>
     </row>
     <row r="186" spans="1:20" ht="18" customHeight="1">
-      <c r="A186" s="105"/>
-      <c r="B186" s="100"/>
-      <c r="C186" s="87"/>
-      <c r="D186" s="87"/>
-      <c r="E186" s="100"/>
+      <c r="A186" s="107"/>
+      <c r="B186" s="102"/>
+      <c r="C186" s="88"/>
+      <c r="D186" s="88"/>
+      <c r="E186" s="102"/>
       <c r="F186" s="94"/>
-      <c r="G186" s="94"/>
+      <c r="G186" s="95"/>
       <c r="H186" s="54"/>
       <c r="I186" s="52"/>
       <c r="J186" s="49"/>
@@ -10111,13 +10189,13 @@
       <c r="T188" s="36"/>
     </row>
     <row r="189" spans="1:20" ht="18" customHeight="1">
-      <c r="A189" s="107"/>
-      <c r="B189" s="102"/>
-      <c r="C189" s="88"/>
-      <c r="D189" s="88"/>
-      <c r="E189" s="102"/>
+      <c r="A189" s="105"/>
+      <c r="B189" s="100"/>
+      <c r="C189" s="87"/>
+      <c r="D189" s="87"/>
+      <c r="E189" s="100"/>
       <c r="F189" s="94"/>
-      <c r="G189" s="95"/>
+      <c r="G189" s="94"/>
       <c r="H189" s="54"/>
       <c r="I189" s="52"/>
       <c r="J189" s="49"/>
@@ -10133,13 +10211,13 @@
       <c r="T189" s="36"/>
     </row>
     <row r="190" spans="1:20" ht="18" customHeight="1">
-      <c r="A190" s="105"/>
-      <c r="B190" s="100"/>
-      <c r="C190" s="87"/>
-      <c r="D190" s="87"/>
-      <c r="E190" s="100"/>
+      <c r="A190" s="107"/>
+      <c r="B190" s="102"/>
+      <c r="C190" s="88"/>
+      <c r="D190" s="88"/>
+      <c r="E190" s="102"/>
       <c r="F190" s="94"/>
-      <c r="G190" s="94"/>
+      <c r="G190" s="95"/>
       <c r="H190" s="54"/>
       <c r="I190" s="52"/>
       <c r="J190" s="49"/>
@@ -10199,16 +10277,16 @@
       <c r="T192" s="36"/>
     </row>
     <row r="193" spans="1:20" ht="18" customHeight="1">
-      <c r="A193" s="107"/>
-      <c r="B193" s="102"/>
-      <c r="C193" s="88"/>
-      <c r="D193" s="88"/>
-      <c r="E193" s="102"/>
-      <c r="F193" s="94"/>
+      <c r="A193" s="39"/>
+      <c r="B193" s="30"/>
+      <c r="C193" s="29"/>
+      <c r="D193" s="29"/>
+      <c r="E193" s="30"/>
+      <c r="F193" s="50"/>
       <c r="G193" s="95"/>
       <c r="H193" s="54"/>
       <c r="I193" s="52"/>
-      <c r="J193" s="49"/>
+      <c r="J193" s="37"/>
       <c r="K193" s="37"/>
       <c r="L193" s="47"/>
       <c r="M193" s="47"/>
@@ -10272,7 +10350,7 @@
       <c r="E196" s="30"/>
       <c r="F196" s="50"/>
       <c r="G196" s="95"/>
-      <c r="H196" s="54"/>
+      <c r="H196" s="45"/>
       <c r="I196" s="52"/>
       <c r="J196" s="37"/>
       <c r="K196" s="37"/>
@@ -10310,7 +10388,7 @@
     </row>
     <row r="198" spans="1:20" ht="18" customHeight="1">
       <c r="A198" s="39"/>
-      <c r="B198" s="30"/>
+      <c r="B198" s="40"/>
       <c r="C198" s="29"/>
       <c r="D198" s="29"/>
       <c r="E198" s="30"/>
@@ -10332,16 +10410,16 @@
     </row>
     <row r="199" spans="1:20" ht="18" customHeight="1">
       <c r="A199" s="39"/>
-      <c r="B199" s="40"/>
+      <c r="B199" s="30"/>
       <c r="C199" s="29"/>
       <c r="D199" s="29"/>
       <c r="E199" s="30"/>
-      <c r="F199" s="50"/>
-      <c r="G199" s="95"/>
-      <c r="H199" s="45"/>
+      <c r="F199" s="109"/>
+      <c r="G199" s="31"/>
+      <c r="H199" s="54"/>
       <c r="I199" s="52"/>
-      <c r="J199" s="37"/>
-      <c r="K199" s="37"/>
+      <c r="J199" s="34"/>
+      <c r="K199" s="34"/>
       <c r="L199" s="47"/>
       <c r="M199" s="39"/>
       <c r="N199" s="29"/>
@@ -10358,7 +10436,7 @@
       <c r="C200" s="29"/>
       <c r="D200" s="29"/>
       <c r="E200" s="30"/>
-      <c r="F200" s="109"/>
+      <c r="F200" s="50"/>
       <c r="G200" s="31"/>
       <c r="H200" s="54"/>
       <c r="I200" s="52"/>
@@ -10406,8 +10484,8 @@
       <c r="G202" s="31"/>
       <c r="H202" s="54"/>
       <c r="I202" s="52"/>
-      <c r="J202" s="34"/>
-      <c r="K202" s="34"/>
+      <c r="J202" s="56"/>
+      <c r="K202" s="49"/>
       <c r="L202" s="39"/>
       <c r="M202" s="39"/>
       <c r="N202" s="29"/>
@@ -10495,7 +10573,7 @@
       <c r="H206" s="54"/>
       <c r="I206" s="52"/>
       <c r="J206" s="56"/>
-      <c r="K206" s="49"/>
+      <c r="K206" s="37"/>
       <c r="L206" s="39"/>
       <c r="M206" s="39"/>
       <c r="N206" s="29"/>
@@ -10534,7 +10612,7 @@
       <c r="C208" s="29"/>
       <c r="D208" s="29"/>
       <c r="E208" s="30"/>
-      <c r="F208" s="50"/>
+      <c r="F208" s="94"/>
       <c r="G208" s="31"/>
       <c r="H208" s="54"/>
       <c r="I208" s="52"/>
@@ -10670,8 +10748,8 @@
       <c r="G214" s="31"/>
       <c r="H214" s="54"/>
       <c r="I214" s="52"/>
-      <c r="J214" s="56"/>
-      <c r="K214" s="37"/>
+      <c r="J214" s="86"/>
+      <c r="K214" s="49"/>
       <c r="L214" s="39"/>
       <c r="M214" s="39"/>
       <c r="N214" s="29"/>
@@ -10705,12 +10783,12 @@
       <c r="T215" s="36"/>
     </row>
     <row r="216" spans="1:20" ht="18" customHeight="1">
-      <c r="A216" s="39"/>
-      <c r="B216" s="30"/>
-      <c r="C216" s="29"/>
-      <c r="D216" s="29"/>
-      <c r="E216" s="30"/>
-      <c r="F216" s="94"/>
+      <c r="A216" s="110"/>
+      <c r="B216" s="100"/>
+      <c r="C216" s="87"/>
+      <c r="D216" s="87"/>
+      <c r="E216" s="100"/>
+      <c r="F216" s="51"/>
       <c r="G216" s="31"/>
       <c r="H216" s="54"/>
       <c r="I216" s="52"/>
@@ -10727,11 +10805,11 @@
       <c r="T216" s="36"/>
     </row>
     <row r="217" spans="1:20" ht="18" customHeight="1">
-      <c r="A217" s="110"/>
-      <c r="B217" s="100"/>
-      <c r="C217" s="87"/>
-      <c r="D217" s="87"/>
-      <c r="E217" s="100"/>
+      <c r="A217" s="111"/>
+      <c r="B217" s="102"/>
+      <c r="C217" s="88"/>
+      <c r="D217" s="88"/>
+      <c r="E217" s="102"/>
       <c r="F217" s="51"/>
       <c r="G217" s="31"/>
       <c r="H217" s="54"/>
@@ -10759,7 +10837,7 @@
       <c r="H218" s="54"/>
       <c r="I218" s="52"/>
       <c r="J218" s="86"/>
-      <c r="K218" s="49"/>
+      <c r="K218" s="37"/>
       <c r="L218" s="39"/>
       <c r="M218" s="39"/>
       <c r="N218" s="29"/>
@@ -10802,7 +10880,7 @@
       <c r="G220" s="31"/>
       <c r="H220" s="54"/>
       <c r="I220" s="52"/>
-      <c r="J220" s="86"/>
+      <c r="J220" s="42"/>
       <c r="K220" s="37"/>
       <c r="L220" s="39"/>
       <c r="M220" s="39"/>
@@ -10881,11 +10959,11 @@
       <c r="T223" s="36"/>
     </row>
     <row r="224" spans="1:20" ht="18" customHeight="1">
-      <c r="A224" s="111"/>
-      <c r="B224" s="102"/>
-      <c r="C224" s="88"/>
-      <c r="D224" s="88"/>
-      <c r="E224" s="102"/>
+      <c r="A224" s="110"/>
+      <c r="B224" s="100"/>
+      <c r="C224" s="87"/>
+      <c r="D224" s="87"/>
+      <c r="E224" s="100"/>
       <c r="F224" s="51"/>
       <c r="G224" s="31"/>
       <c r="H224" s="54"/>
@@ -10903,11 +10981,11 @@
       <c r="T224" s="36"/>
     </row>
     <row r="225" spans="1:20" ht="18" customHeight="1">
-      <c r="A225" s="110"/>
-      <c r="B225" s="100"/>
-      <c r="C225" s="87"/>
-      <c r="D225" s="87"/>
-      <c r="E225" s="100"/>
+      <c r="A225" s="111"/>
+      <c r="B225" s="102"/>
+      <c r="C225" s="88"/>
+      <c r="D225" s="88"/>
+      <c r="E225" s="102"/>
       <c r="F225" s="51"/>
       <c r="G225" s="31"/>
       <c r="H225" s="54"/>
@@ -11057,16 +11135,16 @@
       <c r="T231" s="36"/>
     </row>
     <row r="232" spans="1:20" ht="18" customHeight="1">
-      <c r="A232" s="111"/>
-      <c r="B232" s="102"/>
-      <c r="C232" s="88"/>
-      <c r="D232" s="88"/>
-      <c r="E232" s="102"/>
+      <c r="A232" s="110"/>
+      <c r="B232" s="100"/>
+      <c r="C232" s="87"/>
+      <c r="D232" s="87"/>
+      <c r="E232" s="100"/>
       <c r="F232" s="51"/>
       <c r="G232" s="31"/>
       <c r="H232" s="54"/>
       <c r="I232" s="52"/>
-      <c r="J232" s="42"/>
+      <c r="J232" s="34"/>
       <c r="K232" s="37"/>
       <c r="L232" s="39"/>
       <c r="M232" s="39"/>
@@ -11079,11 +11157,11 @@
       <c r="T232" s="36"/>
     </row>
     <row r="233" spans="1:20" ht="18" customHeight="1">
-      <c r="A233" s="110"/>
-      <c r="B233" s="100"/>
-      <c r="C233" s="87"/>
-      <c r="D233" s="87"/>
-      <c r="E233" s="100"/>
+      <c r="A233" s="111"/>
+      <c r="B233" s="102"/>
+      <c r="C233" s="88"/>
+      <c r="D233" s="88"/>
+      <c r="E233" s="102"/>
       <c r="F233" s="51"/>
       <c r="G233" s="31"/>
       <c r="H233" s="54"/>
@@ -11233,16 +11311,16 @@
       <c r="T239" s="36"/>
     </row>
     <row r="240" spans="1:20" ht="18" customHeight="1">
-      <c r="A240" s="111"/>
-      <c r="B240" s="102"/>
-      <c r="C240" s="88"/>
-      <c r="D240" s="88"/>
-      <c r="E240" s="102"/>
+      <c r="A240" s="110"/>
+      <c r="B240" s="100"/>
+      <c r="C240" s="87"/>
+      <c r="D240" s="87"/>
+      <c r="E240" s="100"/>
       <c r="F240" s="51"/>
       <c r="G240" s="31"/>
       <c r="H240" s="54"/>
       <c r="I240" s="52"/>
-      <c r="J240" s="34"/>
+      <c r="J240" s="39"/>
       <c r="K240" s="37"/>
       <c r="L240" s="39"/>
       <c r="M240" s="39"/>
@@ -11255,11 +11333,11 @@
       <c r="T240" s="36"/>
     </row>
     <row r="241" spans="1:20" ht="18" customHeight="1">
-      <c r="A241" s="110"/>
-      <c r="B241" s="100"/>
-      <c r="C241" s="87"/>
-      <c r="D241" s="87"/>
-      <c r="E241" s="100"/>
+      <c r="A241" s="111"/>
+      <c r="B241" s="102"/>
+      <c r="C241" s="88"/>
+      <c r="D241" s="88"/>
+      <c r="E241" s="102"/>
       <c r="F241" s="51"/>
       <c r="G241" s="31"/>
       <c r="H241" s="54"/>
@@ -11409,11 +11487,11 @@
       <c r="T247" s="42"/>
     </row>
     <row r="248" spans="1:20" ht="18" customHeight="1">
-      <c r="A248" s="111"/>
-      <c r="B248" s="102"/>
-      <c r="C248" s="88"/>
-      <c r="D248" s="88"/>
-      <c r="E248" s="102"/>
+      <c r="A248" s="110"/>
+      <c r="B248" s="100"/>
+      <c r="C248" s="87"/>
+      <c r="D248" s="87"/>
+      <c r="E248" s="100"/>
       <c r="F248" s="51"/>
       <c r="G248" s="31"/>
       <c r="H248" s="54"/>
@@ -11431,11 +11509,11 @@
       <c r="T248" s="42"/>
     </row>
     <row r="249" spans="1:20" ht="18" customHeight="1">
-      <c r="A249" s="110"/>
-      <c r="B249" s="100"/>
-      <c r="C249" s="87"/>
-      <c r="D249" s="87"/>
-      <c r="E249" s="100"/>
+      <c r="A249" s="111"/>
+      <c r="B249" s="102"/>
+      <c r="C249" s="88"/>
+      <c r="D249" s="88"/>
+      <c r="E249" s="102"/>
       <c r="F249" s="51"/>
       <c r="G249" s="31"/>
       <c r="H249" s="54"/>
@@ -11585,11 +11663,11 @@
       <c r="T255" s="36"/>
     </row>
     <row r="256" spans="1:20" ht="18" customHeight="1">
-      <c r="A256" s="111"/>
-      <c r="B256" s="102"/>
-      <c r="C256" s="88"/>
-      <c r="D256" s="88"/>
-      <c r="E256" s="102"/>
+      <c r="A256" s="110"/>
+      <c r="B256" s="100"/>
+      <c r="C256" s="87"/>
+      <c r="D256" s="87"/>
+      <c r="E256" s="100"/>
       <c r="F256" s="51"/>
       <c r="G256" s="31"/>
       <c r="H256" s="54"/>
@@ -11607,11 +11685,11 @@
       <c r="T256" s="36"/>
     </row>
     <row r="257" spans="1:20" ht="18" customHeight="1">
-      <c r="A257" s="110"/>
-      <c r="B257" s="100"/>
-      <c r="C257" s="87"/>
-      <c r="D257" s="87"/>
-      <c r="E257" s="100"/>
+      <c r="A257" s="111"/>
+      <c r="B257" s="102"/>
+      <c r="C257" s="88"/>
+      <c r="D257" s="88"/>
+      <c r="E257" s="102"/>
       <c r="F257" s="51"/>
       <c r="G257" s="31"/>
       <c r="H257" s="54"/>
@@ -11761,16 +11839,16 @@
       <c r="T263" s="36"/>
     </row>
     <row r="264" spans="1:20" ht="18" customHeight="1">
-      <c r="A264" s="111"/>
-      <c r="B264" s="102"/>
-      <c r="C264" s="88"/>
-      <c r="D264" s="88"/>
-      <c r="E264" s="102"/>
+      <c r="A264" s="55"/>
+      <c r="B264" s="40"/>
+      <c r="C264" s="29"/>
+      <c r="D264" s="29"/>
+      <c r="E264" s="30"/>
       <c r="F264" s="51"/>
       <c r="G264" s="31"/>
       <c r="H264" s="54"/>
       <c r="I264" s="52"/>
-      <c r="J264" s="39"/>
+      <c r="J264" s="112"/>
       <c r="K264" s="37"/>
       <c r="L264" s="39"/>
       <c r="M264" s="39"/>
@@ -11853,12 +11931,12 @@
       <c r="B268" s="40"/>
       <c r="C268" s="29"/>
       <c r="D268" s="29"/>
-      <c r="E268" s="30"/>
+      <c r="E268" s="53"/>
       <c r="F268" s="51"/>
       <c r="G268" s="31"/>
       <c r="H268" s="54"/>
       <c r="I268" s="52"/>
-      <c r="J268" s="112"/>
+      <c r="J268" s="34"/>
       <c r="K268" s="37"/>
       <c r="L268" s="39"/>
       <c r="M268" s="39"/>
@@ -11898,11 +11976,11 @@
       <c r="C270" s="29"/>
       <c r="D270" s="29"/>
       <c r="E270" s="53"/>
-      <c r="F270" s="51"/>
+      <c r="F270" s="55"/>
       <c r="G270" s="31"/>
       <c r="H270" s="54"/>
       <c r="I270" s="52"/>
-      <c r="J270" s="34"/>
+      <c r="J270" s="49"/>
       <c r="K270" s="37"/>
       <c r="L270" s="39"/>
       <c r="M270" s="39"/>
@@ -11925,7 +12003,7 @@
       <c r="H271" s="54"/>
       <c r="I271" s="52"/>
       <c r="J271" s="49"/>
-      <c r="K271" s="37"/>
+      <c r="K271" s="49"/>
       <c r="L271" s="39"/>
       <c r="M271" s="39"/>
       <c r="N271" s="39"/>
@@ -11969,7 +12047,7 @@
       <c r="H273" s="54"/>
       <c r="I273" s="52"/>
       <c r="J273" s="49"/>
-      <c r="K273" s="49"/>
+      <c r="K273" s="37"/>
       <c r="L273" s="39"/>
       <c r="M273" s="39"/>
       <c r="N273" s="39"/>
@@ -12013,7 +12091,7 @@
       <c r="H275" s="54"/>
       <c r="I275" s="52"/>
       <c r="J275" s="49"/>
-      <c r="K275" s="37"/>
+      <c r="K275" s="42"/>
       <c r="L275" s="39"/>
       <c r="M275" s="39"/>
       <c r="N275" s="39"/>
@@ -12025,10 +12103,10 @@
       <c r="T275" s="36"/>
     </row>
     <row r="276" spans="1:20" ht="18" customHeight="1">
-      <c r="A276" s="55"/>
-      <c r="B276" s="40"/>
-      <c r="C276" s="29"/>
-      <c r="D276" s="29"/>
+      <c r="A276" s="90"/>
+      <c r="B276" s="100"/>
+      <c r="C276" s="87"/>
+      <c r="D276" s="87"/>
       <c r="E276" s="53"/>
       <c r="F276" s="55"/>
       <c r="G276" s="31"/>
@@ -12047,10 +12125,10 @@
       <c r="T276" s="36"/>
     </row>
     <row r="277" spans="1:20" ht="18" customHeight="1">
-      <c r="A277" s="90"/>
-      <c r="B277" s="100"/>
-      <c r="C277" s="87"/>
-      <c r="D277" s="87"/>
+      <c r="A277" s="92"/>
+      <c r="B277" s="102"/>
+      <c r="C277" s="88"/>
+      <c r="D277" s="88"/>
       <c r="E277" s="53"/>
       <c r="F277" s="55"/>
       <c r="G277" s="31"/>
@@ -12078,7 +12156,7 @@
       <c r="G278" s="31"/>
       <c r="H278" s="54"/>
       <c r="I278" s="52"/>
-      <c r="J278" s="49"/>
+      <c r="J278" s="42"/>
       <c r="K278" s="42"/>
       <c r="L278" s="55"/>
       <c r="M278" s="55"/>
@@ -12157,17 +12235,17 @@
       <c r="T281" s="36"/>
     </row>
     <row r="282" spans="1:20" ht="18" customHeight="1">
-      <c r="A282" s="92"/>
-      <c r="B282" s="102"/>
-      <c r="C282" s="88"/>
-      <c r="D282" s="88"/>
-      <c r="E282" s="53"/>
+      <c r="A282" s="55"/>
+      <c r="B282" s="55"/>
+      <c r="C282" s="55"/>
+      <c r="D282" s="55"/>
+      <c r="E282" s="55"/>
       <c r="F282" s="55"/>
       <c r="G282" s="31"/>
-      <c r="H282" s="54"/>
+      <c r="H282" s="55"/>
       <c r="I282" s="52"/>
-      <c r="J282" s="42"/>
-      <c r="K282" s="42"/>
+      <c r="J282" s="56"/>
+      <c r="K282" s="46"/>
       <c r="L282" s="55"/>
       <c r="M282" s="55"/>
       <c r="N282" s="39"/>
@@ -12189,7 +12267,7 @@
       <c r="H283" s="55"/>
       <c r="I283" s="52"/>
       <c r="J283" s="56"/>
-      <c r="K283" s="46"/>
+      <c r="K283" s="56"/>
       <c r="L283" s="55"/>
       <c r="M283" s="55"/>
       <c r="N283" s="39"/>
@@ -12233,7 +12311,7 @@
       <c r="H285" s="55"/>
       <c r="I285" s="52"/>
       <c r="J285" s="56"/>
-      <c r="K285" s="56"/>
+      <c r="K285" s="42"/>
       <c r="L285" s="55"/>
       <c r="M285" s="55"/>
       <c r="N285" s="39"/>
@@ -12277,7 +12355,7 @@
       <c r="H287" s="55"/>
       <c r="I287" s="52"/>
       <c r="J287" s="56"/>
-      <c r="K287" s="42"/>
+      <c r="K287" s="56"/>
       <c r="L287" s="55"/>
       <c r="M287" s="55"/>
       <c r="N287" s="39"/>
@@ -12299,7 +12377,7 @@
       <c r="H288" s="55"/>
       <c r="I288" s="52"/>
       <c r="J288" s="56"/>
-      <c r="K288" s="56"/>
+      <c r="K288" s="42"/>
       <c r="L288" s="55"/>
       <c r="M288" s="55"/>
       <c r="N288" s="39"/>
@@ -12320,7 +12398,7 @@
       <c r="G289" s="31"/>
       <c r="H289" s="55"/>
       <c r="I289" s="52"/>
-      <c r="J289" s="56"/>
+      <c r="J289" s="49"/>
       <c r="K289" s="42"/>
       <c r="L289" s="55"/>
       <c r="M289" s="55"/>
@@ -12342,7 +12420,7 @@
       <c r="G290" s="31"/>
       <c r="H290" s="55"/>
       <c r="I290" s="52"/>
-      <c r="J290" s="49"/>
+      <c r="J290" s="42"/>
       <c r="K290" s="42"/>
       <c r="L290" s="55"/>
       <c r="M290" s="55"/>
@@ -12425,11 +12503,11 @@
       <c r="B294" s="55"/>
       <c r="C294" s="55"/>
       <c r="D294" s="55"/>
-      <c r="E294" s="55"/>
+      <c r="E294" s="53"/>
       <c r="F294" s="55"/>
       <c r="G294" s="31"/>
       <c r="H294" s="55"/>
-      <c r="I294" s="52"/>
+      <c r="I294" s="37"/>
       <c r="J294" s="42"/>
       <c r="K294" s="42"/>
       <c r="L294" s="55"/>
@@ -12540,7 +12618,7 @@
       <c r="G299" s="31"/>
       <c r="H299" s="55"/>
       <c r="I299" s="37"/>
-      <c r="J299" s="42"/>
+      <c r="J299" s="56"/>
       <c r="K299" s="42"/>
       <c r="L299" s="55"/>
       <c r="M299" s="55"/>
@@ -12597,7 +12675,7 @@
       <c r="T301" s="36"/>
     </row>
     <row r="302" spans="1:20" ht="18" customHeight="1">
-      <c r="A302" s="55"/>
+      <c r="A302" s="90"/>
       <c r="B302" s="55"/>
       <c r="C302" s="55"/>
       <c r="D302" s="55"/>
@@ -12619,7 +12697,7 @@
       <c r="T302" s="36"/>
     </row>
     <row r="303" spans="1:20" ht="18" customHeight="1">
-      <c r="A303" s="90"/>
+      <c r="A303" s="92"/>
       <c r="B303" s="55"/>
       <c r="C303" s="55"/>
       <c r="D303" s="55"/>
@@ -12646,7 +12724,7 @@
       <c r="C304" s="55"/>
       <c r="D304" s="55"/>
       <c r="E304" s="53"/>
-      <c r="F304" s="55"/>
+      <c r="F304" s="91"/>
       <c r="G304" s="31"/>
       <c r="H304" s="55"/>
       <c r="I304" s="37"/>
@@ -12663,7 +12741,7 @@
       <c r="T304" s="36"/>
     </row>
     <row r="305" spans="1:20" ht="18" customHeight="1">
-      <c r="A305" s="92"/>
+      <c r="A305" s="90"/>
       <c r="B305" s="55"/>
       <c r="C305" s="55"/>
       <c r="D305" s="55"/>
@@ -12685,7 +12763,7 @@
       <c r="T305" s="36"/>
     </row>
     <row r="306" spans="1:20" ht="18" customHeight="1">
-      <c r="A306" s="90"/>
+      <c r="A306" s="92"/>
       <c r="B306" s="55"/>
       <c r="C306" s="55"/>
       <c r="D306" s="55"/>
@@ -12729,7 +12807,7 @@
       <c r="T307" s="36"/>
     </row>
     <row r="308" spans="1:20" ht="18" customHeight="1">
-      <c r="A308" s="92"/>
+      <c r="A308" s="55"/>
       <c r="B308" s="55"/>
       <c r="C308" s="55"/>
       <c r="D308" s="55"/>
@@ -12752,15 +12830,15 @@
     </row>
     <row r="309" spans="1:20" ht="18" customHeight="1">
       <c r="A309" s="55"/>
-      <c r="B309" s="55"/>
-      <c r="C309" s="55"/>
-      <c r="D309" s="55"/>
-      <c r="E309" s="53"/>
-      <c r="F309" s="91"/>
+      <c r="B309" s="90"/>
+      <c r="C309" s="91"/>
+      <c r="D309" s="91"/>
+      <c r="E309" s="103"/>
+      <c r="F309" s="55"/>
       <c r="G309" s="31"/>
       <c r="H309" s="55"/>
       <c r="I309" s="37"/>
-      <c r="J309" s="56"/>
+      <c r="J309" s="42"/>
       <c r="K309" s="42"/>
       <c r="L309" s="55"/>
       <c r="M309" s="55"/>
@@ -12774,10 +12852,10 @@
     </row>
     <row r="310" spans="1:20" ht="18" customHeight="1">
       <c r="A310" s="55"/>
-      <c r="B310" s="90"/>
-      <c r="C310" s="91"/>
-      <c r="D310" s="91"/>
-      <c r="E310" s="103"/>
+      <c r="B310" s="92"/>
+      <c r="C310" s="93"/>
+      <c r="D310" s="93"/>
+      <c r="E310" s="104"/>
       <c r="F310" s="55"/>
       <c r="G310" s="31"/>
       <c r="H310" s="55"/>
@@ -12862,16 +12940,16 @@
     </row>
     <row r="314" spans="1:20" ht="18" customHeight="1">
       <c r="A314" s="55"/>
-      <c r="B314" s="92"/>
-      <c r="C314" s="93"/>
-      <c r="D314" s="93"/>
-      <c r="E314" s="104"/>
+      <c r="B314" s="90"/>
+      <c r="C314" s="91"/>
+      <c r="D314" s="91"/>
+      <c r="E314" s="103"/>
       <c r="F314" s="55"/>
       <c r="G314" s="31"/>
       <c r="H314" s="55"/>
       <c r="I314" s="37"/>
-      <c r="J314" s="42"/>
-      <c r="K314" s="42"/>
+      <c r="J314" s="34"/>
+      <c r="K314" s="34"/>
       <c r="L314" s="55"/>
       <c r="M314" s="55"/>
       <c r="N314" s="39"/>
@@ -12884,10 +12962,10 @@
     </row>
     <row r="315" spans="1:20" ht="18" customHeight="1">
       <c r="A315" s="55"/>
-      <c r="B315" s="90"/>
-      <c r="C315" s="91"/>
-      <c r="D315" s="91"/>
-      <c r="E315" s="103"/>
+      <c r="B315" s="92"/>
+      <c r="C315" s="93"/>
+      <c r="D315" s="93"/>
+      <c r="E315" s="104"/>
       <c r="F315" s="55"/>
       <c r="G315" s="31"/>
       <c r="H315" s="55"/>
@@ -12972,16 +13050,16 @@
     </row>
     <row r="319" spans="1:20" ht="18" customHeight="1">
       <c r="A319" s="55"/>
-      <c r="B319" s="92"/>
-      <c r="C319" s="93"/>
-      <c r="D319" s="93"/>
-      <c r="E319" s="104"/>
+      <c r="B319" s="90"/>
+      <c r="C319" s="91"/>
+      <c r="D319" s="55"/>
+      <c r="E319" s="55"/>
       <c r="F319" s="55"/>
       <c r="G319" s="31"/>
       <c r="H319" s="55"/>
-      <c r="I319" s="37"/>
-      <c r="J319" s="34"/>
-      <c r="K319" s="34"/>
+      <c r="I319" s="42"/>
+      <c r="J319" s="42"/>
+      <c r="K319" s="42"/>
       <c r="L319" s="55"/>
       <c r="M319" s="55"/>
       <c r="N319" s="39"/>
@@ -12994,8 +13072,8 @@
     </row>
     <row r="320" spans="1:20" ht="18" customHeight="1">
       <c r="A320" s="55"/>
-      <c r="B320" s="90"/>
-      <c r="C320" s="91"/>
+      <c r="B320" s="92"/>
+      <c r="C320" s="93"/>
       <c r="D320" s="55"/>
       <c r="E320" s="55"/>
       <c r="F320" s="55"/>
@@ -13003,7 +13081,7 @@
       <c r="H320" s="55"/>
       <c r="I320" s="42"/>
       <c r="J320" s="42"/>
-      <c r="K320" s="42"/>
+      <c r="K320" s="46"/>
       <c r="L320" s="55"/>
       <c r="M320" s="55"/>
       <c r="N320" s="39"/>
@@ -13044,7 +13122,7 @@
       <c r="E322" s="55"/>
       <c r="F322" s="55"/>
       <c r="G322" s="31"/>
-      <c r="H322" s="55"/>
+      <c r="H322" s="42"/>
       <c r="I322" s="42"/>
       <c r="J322" s="42"/>
       <c r="K322" s="46"/>
@@ -13082,15 +13160,15 @@
     </row>
     <row r="324" spans="1:20" ht="18" customHeight="1">
       <c r="A324" s="55"/>
-      <c r="B324" s="92"/>
-      <c r="C324" s="93"/>
+      <c r="B324" s="90"/>
+      <c r="C324" s="91"/>
       <c r="D324" s="55"/>
       <c r="E324" s="55"/>
       <c r="F324" s="55"/>
       <c r="G324" s="31"/>
       <c r="H324" s="42"/>
       <c r="I324" s="42"/>
-      <c r="J324" s="42"/>
+      <c r="J324" s="56"/>
       <c r="K324" s="46"/>
       <c r="L324" s="55"/>
       <c r="M324" s="55"/>
@@ -13104,8 +13182,8 @@
     </row>
     <row r="325" spans="1:20" ht="18" customHeight="1">
       <c r="A325" s="55"/>
-      <c r="B325" s="90"/>
-      <c r="C325" s="91"/>
+      <c r="B325" s="92"/>
+      <c r="C325" s="93"/>
       <c r="D325" s="55"/>
       <c r="E325" s="55"/>
       <c r="F325" s="55"/>
@@ -13192,15 +13270,15 @@
     </row>
     <row r="329" spans="1:20" ht="18" customHeight="1">
       <c r="A329" s="55"/>
-      <c r="B329" s="92"/>
-      <c r="C329" s="93"/>
-      <c r="D329" s="55"/>
-      <c r="E329" s="55"/>
-      <c r="F329" s="55"/>
-      <c r="G329" s="31"/>
+      <c r="B329" s="90"/>
+      <c r="C329" s="91"/>
+      <c r="D329" s="91"/>
+      <c r="E329" s="91"/>
+      <c r="F329" s="91"/>
+      <c r="G329" s="94"/>
       <c r="H329" s="42"/>
       <c r="I329" s="42"/>
-      <c r="J329" s="56"/>
+      <c r="J329" s="42"/>
       <c r="K329" s="46"/>
       <c r="L329" s="55"/>
       <c r="M329" s="55"/>
@@ -13214,12 +13292,12 @@
     </row>
     <row r="330" spans="1:20" ht="18" customHeight="1">
       <c r="A330" s="55"/>
-      <c r="B330" s="90"/>
-      <c r="C330" s="91"/>
-      <c r="D330" s="91"/>
-      <c r="E330" s="91"/>
+      <c r="B330" s="92"/>
+      <c r="C330" s="93"/>
+      <c r="D330" s="93"/>
+      <c r="E330" s="93"/>
       <c r="F330" s="91"/>
-      <c r="G330" s="94"/>
+      <c r="G330" s="95"/>
       <c r="H330" s="42"/>
       <c r="I330" s="42"/>
       <c r="J330" s="42"/>
@@ -13301,13 +13379,13 @@
       <c r="T333" s="36"/>
     </row>
     <row r="334" spans="1:20" ht="18" customHeight="1">
-      <c r="A334" s="55"/>
-      <c r="B334" s="92"/>
-      <c r="C334" s="93"/>
-      <c r="D334" s="93"/>
-      <c r="E334" s="93"/>
-      <c r="F334" s="91"/>
-      <c r="G334" s="95"/>
+      <c r="A334" s="42"/>
+      <c r="B334" s="55"/>
+      <c r="C334" s="55"/>
+      <c r="D334" s="55"/>
+      <c r="E334" s="55"/>
+      <c r="F334" s="55"/>
+      <c r="G334" s="31"/>
       <c r="H334" s="42"/>
       <c r="I334" s="42"/>
       <c r="J334" s="42"/>
@@ -13420,7 +13498,7 @@
       <c r="G339" s="31"/>
       <c r="H339" s="42"/>
       <c r="I339" s="42"/>
-      <c r="J339" s="42"/>
+      <c r="J339" s="46"/>
       <c r="K339" s="46"/>
       <c r="L339" s="55"/>
       <c r="M339" s="55"/>
@@ -13440,7 +13518,7 @@
       <c r="E340" s="55"/>
       <c r="F340" s="55"/>
       <c r="G340" s="31"/>
-      <c r="H340" s="42"/>
+      <c r="H340" s="55"/>
       <c r="I340" s="42"/>
       <c r="J340" s="46"/>
       <c r="K340" s="46"/>
@@ -13506,7 +13584,7 @@
       <c r="E343" s="55"/>
       <c r="F343" s="55"/>
       <c r="G343" s="31"/>
-      <c r="H343" s="55"/>
+      <c r="H343" s="42"/>
       <c r="I343" s="42"/>
       <c r="J343" s="46"/>
       <c r="K343" s="46"/>
@@ -13619,7 +13697,7 @@
       <c r="H348" s="42"/>
       <c r="I348" s="42"/>
       <c r="J348" s="46"/>
-      <c r="K348" s="46"/>
+      <c r="K348" s="42"/>
       <c r="L348" s="55"/>
       <c r="M348" s="55"/>
       <c r="N348" s="55"/>
@@ -13685,7 +13763,7 @@
       <c r="H351" s="42"/>
       <c r="I351" s="42"/>
       <c r="J351" s="46"/>
-      <c r="K351" s="42"/>
+      <c r="K351" s="55"/>
       <c r="L351" s="55"/>
       <c r="M351" s="55"/>
       <c r="N351" s="55"/>
@@ -13707,7 +13785,7 @@
       <c r="H352" s="42"/>
       <c r="I352" s="42"/>
       <c r="J352" s="46"/>
-      <c r="K352" s="55"/>
+      <c r="K352" s="42"/>
       <c r="L352" s="55"/>
       <c r="M352" s="55"/>
       <c r="N352" s="55"/>
@@ -13882,8 +13960,8 @@
       <c r="G360" s="31"/>
       <c r="H360" s="42"/>
       <c r="I360" s="42"/>
-      <c r="J360" s="46"/>
-      <c r="K360" s="42"/>
+      <c r="J360" s="42"/>
+      <c r="K360" s="46"/>
       <c r="L360" s="55"/>
       <c r="M360" s="55"/>
       <c r="N360" s="55"/>
@@ -13949,7 +14027,7 @@
       <c r="H363" s="42"/>
       <c r="I363" s="42"/>
       <c r="J363" s="42"/>
-      <c r="K363" s="46"/>
+      <c r="K363" s="42"/>
       <c r="L363" s="55"/>
       <c r="M363" s="55"/>
       <c r="N363" s="55"/>
@@ -14343,8 +14421,8 @@
       <c r="F381" s="55"/>
       <c r="G381" s="31"/>
       <c r="H381" s="42"/>
-      <c r="I381" s="42"/>
-      <c r="J381" s="42"/>
+      <c r="I381" s="55"/>
+      <c r="J381" s="46"/>
       <c r="K381" s="42"/>
       <c r="L381" s="55"/>
       <c r="M381" s="55"/>
@@ -14763,7 +14841,7 @@
       <c r="H400" s="42"/>
       <c r="I400" s="55"/>
       <c r="J400" s="46"/>
-      <c r="K400" s="42"/>
+      <c r="K400" s="56"/>
       <c r="L400" s="55"/>
       <c r="M400" s="55"/>
       <c r="N400" s="55"/>
@@ -14781,10 +14859,10 @@
       <c r="D401" s="55"/>
       <c r="E401" s="55"/>
       <c r="F401" s="55"/>
-      <c r="G401" s="31"/>
-      <c r="H401" s="42"/>
-      <c r="I401" s="55"/>
-      <c r="J401" s="46"/>
+      <c r="G401" s="55"/>
+      <c r="H401" s="55"/>
+      <c r="I401" s="42"/>
+      <c r="J401" s="56"/>
       <c r="K401" s="56"/>
       <c r="L401" s="55"/>
       <c r="M401" s="55"/>
@@ -14872,8 +14950,8 @@
       <c r="G405" s="55"/>
       <c r="H405" s="55"/>
       <c r="I405" s="42"/>
-      <c r="J405" s="56"/>
-      <c r="K405" s="56"/>
+      <c r="J405" s="42"/>
+      <c r="K405" s="46"/>
       <c r="L405" s="55"/>
       <c r="M405" s="55"/>
       <c r="N405" s="55"/>
@@ -14952,14 +15030,14 @@
     </row>
     <row r="409" spans="1:20" ht="18" customHeight="1">
       <c r="A409" s="42"/>
-      <c r="B409" s="55"/>
-      <c r="C409" s="55"/>
-      <c r="D409" s="55"/>
-      <c r="E409" s="55"/>
-      <c r="F409" s="55"/>
-      <c r="G409" s="55"/>
-      <c r="H409" s="55"/>
-      <c r="I409" s="42"/>
+      <c r="B409" s="90"/>
+      <c r="C409" s="91"/>
+      <c r="D409" s="91"/>
+      <c r="E409" s="91"/>
+      <c r="F409" s="91"/>
+      <c r="G409" s="91"/>
+      <c r="H409" s="91"/>
+      <c r="I409" s="91"/>
       <c r="J409" s="42"/>
       <c r="K409" s="46"/>
       <c r="L409" s="55"/>
@@ -14974,16 +15052,16 @@
     </row>
     <row r="410" spans="1:20" ht="18" customHeight="1">
       <c r="A410" s="42"/>
-      <c r="B410" s="90"/>
-      <c r="C410" s="91"/>
-      <c r="D410" s="91"/>
-      <c r="E410" s="91"/>
+      <c r="B410" s="92"/>
+      <c r="C410" s="93"/>
+      <c r="D410" s="93"/>
+      <c r="E410" s="93"/>
       <c r="F410" s="91"/>
-      <c r="G410" s="91"/>
-      <c r="H410" s="91"/>
-      <c r="I410" s="91"/>
+      <c r="G410" s="93"/>
+      <c r="H410" s="93"/>
+      <c r="I410" s="93"/>
       <c r="J410" s="42"/>
-      <c r="K410" s="46"/>
+      <c r="K410" s="42"/>
       <c r="L410" s="55"/>
       <c r="M410" s="55"/>
       <c r="N410" s="55"/>
@@ -15040,15 +15118,15 @@
     </row>
     <row r="413" spans="1:20" ht="18" customHeight="1">
       <c r="A413" s="42"/>
-      <c r="B413" s="92"/>
-      <c r="C413" s="93"/>
-      <c r="D413" s="93"/>
-      <c r="E413" s="93"/>
-      <c r="F413" s="91"/>
+      <c r="B413" s="55"/>
+      <c r="C413" s="55"/>
+      <c r="D413" s="55"/>
+      <c r="E413" s="55"/>
+      <c r="F413" s="55"/>
       <c r="G413" s="93"/>
       <c r="H413" s="93"/>
       <c r="I413" s="93"/>
-      <c r="J413" s="42"/>
+      <c r="J413" s="56"/>
       <c r="K413" s="42"/>
       <c r="L413" s="55"/>
       <c r="M413" s="55"/>
@@ -15071,7 +15149,7 @@
       <c r="H414" s="93"/>
       <c r="I414" s="93"/>
       <c r="J414" s="56"/>
-      <c r="K414" s="42"/>
+      <c r="K414" s="56"/>
       <c r="L414" s="55"/>
       <c r="M414" s="55"/>
       <c r="N414" s="55"/>
@@ -15171,10 +15249,10 @@
       <c r="T418" s="36"/>
     </row>
     <row r="419" spans="1:20" ht="18" customHeight="1">
-      <c r="A419" s="42"/>
-      <c r="B419" s="55"/>
-      <c r="C419" s="55"/>
-      <c r="D419" s="55"/>
+      <c r="A419" s="55"/>
+      <c r="B419" s="90"/>
+      <c r="C419" s="91"/>
+      <c r="D419" s="91"/>
       <c r="E419" s="55"/>
       <c r="F419" s="55"/>
       <c r="G419" s="93"/>
@@ -15194,9 +15272,9 @@
     </row>
     <row r="420" spans="1:20" ht="18" customHeight="1">
       <c r="A420" s="55"/>
-      <c r="B420" s="90"/>
-      <c r="C420" s="91"/>
-      <c r="D420" s="91"/>
+      <c r="B420" s="92"/>
+      <c r="C420" s="93"/>
+      <c r="D420" s="93"/>
       <c r="E420" s="55"/>
       <c r="F420" s="55"/>
       <c r="G420" s="93"/>
@@ -15238,16 +15316,16 @@
     </row>
     <row r="422" spans="1:20" ht="18" customHeight="1">
       <c r="A422" s="55"/>
-      <c r="B422" s="92"/>
-      <c r="C422" s="93"/>
-      <c r="D422" s="93"/>
+      <c r="B422" s="55"/>
+      <c r="C422" s="55"/>
+      <c r="D422" s="55"/>
       <c r="E422" s="55"/>
       <c r="F422" s="55"/>
       <c r="G422" s="93"/>
       <c r="H422" s="93"/>
       <c r="I422" s="93"/>
       <c r="J422" s="56"/>
-      <c r="K422" s="56"/>
+      <c r="K422" s="42"/>
       <c r="L422" s="55"/>
       <c r="M422" s="55"/>
       <c r="N422" s="55"/>
@@ -15334,7 +15412,7 @@
       <c r="G426" s="93"/>
       <c r="H426" s="93"/>
       <c r="I426" s="93"/>
-      <c r="J426" s="56"/>
+      <c r="J426" s="42"/>
       <c r="K426" s="42"/>
       <c r="L426" s="55"/>
       <c r="M426" s="55"/>
@@ -15375,9 +15453,9 @@
       <c r="D428" s="55"/>
       <c r="E428" s="55"/>
       <c r="F428" s="55"/>
-      <c r="G428" s="93"/>
-      <c r="H428" s="93"/>
-      <c r="I428" s="93"/>
+      <c r="G428" s="55"/>
+      <c r="H428" s="42"/>
+      <c r="I428" s="42"/>
       <c r="J428" s="42"/>
       <c r="K428" s="42"/>
       <c r="L428" s="55"/>
@@ -15422,7 +15500,7 @@
       <c r="G430" s="55"/>
       <c r="H430" s="42"/>
       <c r="I430" s="42"/>
-      <c r="J430" s="42"/>
+      <c r="J430" s="56"/>
       <c r="K430" s="42"/>
       <c r="L430" s="55"/>
       <c r="M430" s="55"/>
@@ -15444,7 +15522,7 @@
       <c r="G431" s="55"/>
       <c r="H431" s="42"/>
       <c r="I431" s="42"/>
-      <c r="J431" s="56"/>
+      <c r="J431" s="42"/>
       <c r="K431" s="42"/>
       <c r="L431" s="55"/>
       <c r="M431" s="55"/>
@@ -15655,14 +15733,14 @@
       <c r="T440" s="36"/>
     </row>
     <row r="441" spans="1:20" ht="15" customHeight="1">
-      <c r="A441" s="55"/>
+      <c r="A441" s="42"/>
       <c r="B441" s="55"/>
       <c r="C441" s="55"/>
       <c r="D441" s="55"/>
       <c r="E441" s="55"/>
       <c r="F441" s="55"/>
       <c r="G441" s="55"/>
-      <c r="H441" s="42"/>
+      <c r="H441" s="55"/>
       <c r="I441" s="42"/>
       <c r="J441" s="42"/>
       <c r="K441" s="42"/>
@@ -15854,10 +15932,10 @@
     </row>
     <row r="450" spans="1:20" ht="15" customHeight="1">
       <c r="A450" s="42"/>
-      <c r="B450" s="55"/>
-      <c r="C450" s="55"/>
-      <c r="D450" s="55"/>
-      <c r="E450" s="55"/>
+      <c r="B450" s="90"/>
+      <c r="C450" s="91"/>
+      <c r="D450" s="91"/>
+      <c r="E450" s="91"/>
       <c r="F450" s="55"/>
       <c r="G450" s="55"/>
       <c r="H450" s="55"/>
@@ -15876,10 +15954,10 @@
     </row>
     <row r="451" spans="1:20" ht="15" customHeight="1">
       <c r="A451" s="42"/>
-      <c r="B451" s="90"/>
-      <c r="C451" s="91"/>
-      <c r="D451" s="91"/>
-      <c r="E451" s="91"/>
+      <c r="B451" s="92"/>
+      <c r="C451" s="93"/>
+      <c r="D451" s="93"/>
+      <c r="E451" s="93"/>
       <c r="F451" s="55"/>
       <c r="G451" s="55"/>
       <c r="H451" s="55"/>
@@ -16052,10 +16130,10 @@
     </row>
     <row r="459" spans="1:20" ht="15" customHeight="1">
       <c r="A459" s="42"/>
-      <c r="B459" s="92"/>
-      <c r="C459" s="93"/>
-      <c r="D459" s="93"/>
-      <c r="E459" s="93"/>
+      <c r="B459" s="90"/>
+      <c r="C459" s="91"/>
+      <c r="D459" s="91"/>
+      <c r="E459" s="91"/>
       <c r="F459" s="55"/>
       <c r="G459" s="55"/>
       <c r="H459" s="55"/>
@@ -16074,10 +16152,10 @@
     </row>
     <row r="460" spans="1:20" ht="15" customHeight="1">
       <c r="A460" s="42"/>
-      <c r="B460" s="90"/>
-      <c r="C460" s="91"/>
-      <c r="D460" s="91"/>
-      <c r="E460" s="91"/>
+      <c r="B460" s="92"/>
+      <c r="C460" s="93"/>
+      <c r="D460" s="93"/>
+      <c r="E460" s="93"/>
       <c r="F460" s="55"/>
       <c r="G460" s="55"/>
       <c r="H460" s="55"/>
@@ -16250,13 +16328,13 @@
     </row>
     <row r="468" spans="1:20" ht="15" customHeight="1">
       <c r="A468" s="42"/>
-      <c r="B468" s="92"/>
-      <c r="C468" s="93"/>
-      <c r="D468" s="93"/>
-      <c r="E468" s="93"/>
+      <c r="B468" s="90"/>
+      <c r="C468" s="91"/>
+      <c r="D468" s="91"/>
+      <c r="E468" s="91"/>
       <c r="F468" s="55"/>
       <c r="G468" s="55"/>
-      <c r="H468" s="55"/>
+      <c r="H468" s="42"/>
       <c r="I468" s="42"/>
       <c r="J468" s="42"/>
       <c r="K468" s="42"/>
@@ -16272,10 +16350,10 @@
     </row>
     <row r="469" spans="1:20" ht="15" customHeight="1">
       <c r="A469" s="42"/>
-      <c r="B469" s="90"/>
-      <c r="C469" s="91"/>
-      <c r="D469" s="91"/>
-      <c r="E469" s="91"/>
+      <c r="B469" s="92"/>
+      <c r="C469" s="93"/>
+      <c r="D469" s="93"/>
+      <c r="E469" s="93"/>
       <c r="F469" s="55"/>
       <c r="G469" s="55"/>
       <c r="H469" s="42"/>
@@ -16360,10 +16438,10 @@
     </row>
     <row r="473" spans="1:20" ht="15" customHeight="1">
       <c r="A473" s="42"/>
-      <c r="B473" s="92"/>
-      <c r="C473" s="93"/>
-      <c r="D473" s="93"/>
-      <c r="E473" s="93"/>
+      <c r="B473" s="90"/>
+      <c r="C473" s="91"/>
+      <c r="D473" s="91"/>
+      <c r="E473" s="91"/>
       <c r="F473" s="55"/>
       <c r="G473" s="55"/>
       <c r="H473" s="42"/>
@@ -16382,10 +16460,10 @@
     </row>
     <row r="474" spans="1:20" ht="15" customHeight="1">
       <c r="A474" s="42"/>
-      <c r="B474" s="90"/>
-      <c r="C474" s="91"/>
-      <c r="D474" s="91"/>
-      <c r="E474" s="91"/>
+      <c r="B474" s="92"/>
+      <c r="C474" s="93"/>
+      <c r="D474" s="93"/>
+      <c r="E474" s="93"/>
       <c r="F474" s="55"/>
       <c r="G474" s="55"/>
       <c r="H474" s="42"/>
@@ -16470,10 +16548,10 @@
     </row>
     <row r="478" spans="1:20" ht="15" customHeight="1">
       <c r="A478" s="42"/>
-      <c r="B478" s="92"/>
-      <c r="C478" s="93"/>
-      <c r="D478" s="93"/>
-      <c r="E478" s="93"/>
+      <c r="B478" s="90"/>
+      <c r="C478" s="91"/>
+      <c r="D478" s="91"/>
+      <c r="E478" s="91"/>
       <c r="F478" s="55"/>
       <c r="G478" s="55"/>
       <c r="H478" s="42"/>
@@ -16492,10 +16570,10 @@
     </row>
     <row r="479" spans="1:20" ht="15" customHeight="1">
       <c r="A479" s="42"/>
-      <c r="B479" s="90"/>
-      <c r="C479" s="91"/>
-      <c r="D479" s="91"/>
-      <c r="E479" s="91"/>
+      <c r="B479" s="92"/>
+      <c r="C479" s="93"/>
+      <c r="D479" s="93"/>
+      <c r="E479" s="93"/>
       <c r="F479" s="55"/>
       <c r="G479" s="55"/>
       <c r="H479" s="42"/>
@@ -16668,12 +16746,12 @@
     </row>
     <row r="487" spans="1:20" ht="15" customHeight="1">
       <c r="A487" s="42"/>
-      <c r="B487" s="92"/>
-      <c r="C487" s="93"/>
-      <c r="D487" s="93"/>
-      <c r="E487" s="93"/>
+      <c r="B487" s="55"/>
+      <c r="C487" s="55"/>
+      <c r="D487" s="55"/>
+      <c r="E487" s="55"/>
       <c r="F487" s="55"/>
-      <c r="G487" s="55"/>
+      <c r="G487" s="31"/>
       <c r="H487" s="42"/>
       <c r="I487" s="42"/>
       <c r="J487" s="42"/>
@@ -16975,17 +17053,17 @@
       <c r="T500" s="36"/>
     </row>
     <row r="501" spans="1:20" ht="15" customHeight="1">
-      <c r="A501" s="42"/>
-      <c r="B501" s="55"/>
-      <c r="C501" s="55"/>
-      <c r="D501" s="55"/>
-      <c r="E501" s="55"/>
-      <c r="F501" s="55"/>
-      <c r="G501" s="31"/>
-      <c r="H501" s="42"/>
-      <c r="I501" s="42"/>
+      <c r="A501" s="90"/>
+      <c r="B501" s="91"/>
+      <c r="C501" s="91"/>
+      <c r="D501" s="91"/>
+      <c r="E501" s="91"/>
+      <c r="F501" s="91"/>
+      <c r="G501" s="94"/>
+      <c r="H501" s="91"/>
+      <c r="I501" s="91"/>
       <c r="J501" s="42"/>
-      <c r="K501" s="42"/>
+      <c r="K501" s="91"/>
       <c r="L501" s="55"/>
       <c r="M501" s="55"/>
       <c r="N501" s="55"/>
@@ -16997,17 +17075,17 @@
       <c r="T501" s="36"/>
     </row>
     <row r="502" spans="1:20" ht="15" customHeight="1">
-      <c r="A502" s="90"/>
-      <c r="B502" s="91"/>
-      <c r="C502" s="91"/>
-      <c r="D502" s="91"/>
-      <c r="E502" s="91"/>
+      <c r="A502" s="92"/>
+      <c r="B502" s="93"/>
+      <c r="C502" s="93"/>
+      <c r="D502" s="93"/>
+      <c r="E502" s="93"/>
       <c r="F502" s="91"/>
-      <c r="G502" s="94"/>
-      <c r="H502" s="91"/>
-      <c r="I502" s="91"/>
+      <c r="G502" s="95"/>
+      <c r="H502" s="93"/>
+      <c r="I502" s="93"/>
       <c r="J502" s="42"/>
-      <c r="K502" s="91"/>
+      <c r="K502" s="93"/>
       <c r="L502" s="91"/>
       <c r="M502" s="91"/>
       <c r="N502" s="91"/>
@@ -17029,7 +17107,7 @@
       <c r="H503" s="93"/>
       <c r="I503" s="93"/>
       <c r="J503" s="42"/>
-      <c r="K503" s="93"/>
+      <c r="K503" s="96"/>
       <c r="L503" s="91"/>
       <c r="M503" s="91"/>
       <c r="N503" s="93"/>
@@ -17437,17 +17515,17 @@
       <c r="T521" s="36"/>
     </row>
     <row r="522" spans="1:20" ht="15" customHeight="1">
-      <c r="A522" s="92"/>
-      <c r="B522" s="93"/>
-      <c r="C522" s="93"/>
-      <c r="D522" s="93"/>
-      <c r="E522" s="93"/>
-      <c r="F522" s="91"/>
+      <c r="A522" s="42"/>
+      <c r="B522" s="55"/>
+      <c r="C522" s="55"/>
+      <c r="D522" s="55"/>
+      <c r="E522" s="42"/>
+      <c r="F522" s="55"/>
       <c r="G522" s="95"/>
-      <c r="H522" s="93"/>
-      <c r="I522" s="93"/>
+      <c r="H522" s="55"/>
+      <c r="I522" s="42"/>
       <c r="J522" s="42"/>
-      <c r="K522" s="96"/>
+      <c r="K522" s="42"/>
       <c r="L522" s="91"/>
       <c r="M522" s="91"/>
       <c r="N522" s="93"/>
@@ -17619,7 +17697,7 @@
       <c r="E530" s="42"/>
       <c r="F530" s="55"/>
       <c r="G530" s="95"/>
-      <c r="H530" s="55"/>
+      <c r="H530" s="42"/>
       <c r="I530" s="42"/>
       <c r="J530" s="42"/>
       <c r="K530" s="42"/>
@@ -17832,11 +17910,11 @@
       <c r="T539" s="36"/>
     </row>
     <row r="540" spans="1:20" ht="15" customHeight="1">
-      <c r="A540" s="42"/>
+      <c r="A540" s="55"/>
       <c r="B540" s="55"/>
       <c r="C540" s="55"/>
       <c r="D540" s="55"/>
-      <c r="E540" s="42"/>
+      <c r="E540" s="55"/>
       <c r="F540" s="55"/>
       <c r="G540" s="95"/>
       <c r="H540" s="42"/>
@@ -18096,15 +18174,15 @@
       <c r="T551" s="36"/>
     </row>
     <row r="552" spans="1:20" ht="15" customHeight="1">
-      <c r="A552" s="55"/>
-      <c r="B552" s="55"/>
-      <c r="C552" s="55"/>
-      <c r="D552" s="55"/>
-      <c r="E552" s="55"/>
-      <c r="F552" s="55"/>
+      <c r="A552" s="90"/>
+      <c r="B552" s="91"/>
+      <c r="C552" s="91"/>
+      <c r="D552" s="91"/>
+      <c r="E552" s="91"/>
+      <c r="F552" s="91"/>
       <c r="G552" s="95"/>
-      <c r="H552" s="42"/>
-      <c r="I552" s="42"/>
+      <c r="H552" s="91"/>
+      <c r="I552" s="91"/>
       <c r="J552" s="42"/>
       <c r="K552" s="42"/>
       <c r="L552" s="55"/>
@@ -18118,15 +18196,15 @@
       <c r="T552" s="36"/>
     </row>
     <row r="553" spans="1:20" ht="15" customHeight="1">
-      <c r="A553" s="90"/>
-      <c r="B553" s="91"/>
-      <c r="C553" s="91"/>
-      <c r="D553" s="91"/>
-      <c r="E553" s="91"/>
+      <c r="A553" s="92"/>
+      <c r="B553" s="93"/>
+      <c r="C553" s="93"/>
+      <c r="D553" s="93"/>
+      <c r="E553" s="93"/>
       <c r="F553" s="91"/>
       <c r="G553" s="95"/>
-      <c r="H553" s="91"/>
-      <c r="I553" s="91"/>
+      <c r="H553" s="93"/>
+      <c r="I553" s="93"/>
       <c r="J553" s="42"/>
       <c r="K553" s="42"/>
       <c r="L553" s="55"/>
@@ -18228,17 +18306,17 @@
       <c r="T557" s="36"/>
     </row>
     <row r="558" spans="1:20" ht="15" customHeight="1">
-      <c r="A558" s="92"/>
-      <c r="B558" s="93"/>
-      <c r="C558" s="93"/>
-      <c r="D558" s="93"/>
-      <c r="E558" s="93"/>
+      <c r="A558" s="90"/>
+      <c r="B558" s="91"/>
+      <c r="C558" s="91"/>
+      <c r="D558" s="91"/>
+      <c r="E558" s="91"/>
       <c r="F558" s="91"/>
       <c r="G558" s="95"/>
-      <c r="H558" s="93"/>
-      <c r="I558" s="93"/>
-      <c r="J558" s="42"/>
-      <c r="K558" s="42"/>
+      <c r="H558" s="42"/>
+      <c r="I558" s="42"/>
+      <c r="J558" s="86"/>
+      <c r="K558" s="86"/>
       <c r="L558" s="55"/>
       <c r="M558" s="55"/>
       <c r="N558" s="55"/>
@@ -18250,11 +18328,11 @@
       <c r="T558" s="36"/>
     </row>
     <row r="559" spans="1:20" ht="15" customHeight="1">
-      <c r="A559" s="90"/>
-      <c r="B559" s="91"/>
-      <c r="C559" s="91"/>
-      <c r="D559" s="91"/>
-      <c r="E559" s="91"/>
+      <c r="A559" s="92"/>
+      <c r="B559" s="93"/>
+      <c r="C559" s="93"/>
+      <c r="D559" s="93"/>
+      <c r="E559" s="93"/>
       <c r="F559" s="91"/>
       <c r="G559" s="95"/>
       <c r="H559" s="42"/>
@@ -18360,17 +18438,17 @@
       <c r="T563" s="36"/>
     </row>
     <row r="564" spans="1:20" ht="15" customHeight="1">
-      <c r="A564" s="92"/>
-      <c r="B564" s="93"/>
-      <c r="C564" s="93"/>
-      <c r="D564" s="93"/>
-      <c r="E564" s="93"/>
-      <c r="F564" s="91"/>
+      <c r="A564" s="42"/>
+      <c r="B564" s="55"/>
+      <c r="C564" s="55"/>
+      <c r="D564" s="55"/>
+      <c r="E564" s="55"/>
+      <c r="F564" s="55"/>
       <c r="G564" s="95"/>
-      <c r="H564" s="42"/>
+      <c r="H564" s="55"/>
       <c r="I564" s="42"/>
-      <c r="J564" s="86"/>
-      <c r="K564" s="86"/>
+      <c r="J564" s="42"/>
+      <c r="K564" s="42"/>
       <c r="L564" s="55"/>
       <c r="M564" s="55"/>
       <c r="N564" s="55"/>
@@ -18757,10 +18835,10 @@
     </row>
     <row r="582" spans="1:20" ht="15" customHeight="1">
       <c r="A582" s="42"/>
-      <c r="B582" s="55"/>
-      <c r="C582" s="55"/>
-      <c r="D582" s="55"/>
-      <c r="E582" s="55"/>
+      <c r="B582" s="90"/>
+      <c r="C582" s="91"/>
+      <c r="D582" s="91"/>
+      <c r="E582" s="91"/>
       <c r="F582" s="55"/>
       <c r="G582" s="95"/>
       <c r="H582" s="55"/>
@@ -18779,10 +18857,10 @@
     </row>
     <row r="583" spans="1:20" ht="15" customHeight="1">
       <c r="A583" s="42"/>
-      <c r="B583" s="90"/>
-      <c r="C583" s="91"/>
-      <c r="D583" s="91"/>
-      <c r="E583" s="91"/>
+      <c r="B583" s="92"/>
+      <c r="C583" s="93"/>
+      <c r="D583" s="93"/>
+      <c r="E583" s="93"/>
       <c r="F583" s="55"/>
       <c r="G583" s="95"/>
       <c r="H583" s="55"/>
@@ -18888,11 +18966,11 @@
       <c r="T587" s="36"/>
     </row>
     <row r="588" spans="1:20" ht="15" customHeight="1">
-      <c r="A588" s="42"/>
-      <c r="B588" s="92"/>
-      <c r="C588" s="93"/>
-      <c r="D588" s="93"/>
-      <c r="E588" s="93"/>
+      <c r="A588" s="55"/>
+      <c r="B588" s="55"/>
+      <c r="C588" s="55"/>
+      <c r="D588" s="55"/>
+      <c r="E588" s="42"/>
       <c r="F588" s="55"/>
       <c r="G588" s="95"/>
       <c r="H588" s="55"/>
@@ -18910,14 +18988,14 @@
       <c r="T588" s="36"/>
     </row>
     <row r="589" spans="1:20" ht="15" customHeight="1">
-      <c r="A589" s="55"/>
-      <c r="B589" s="55"/>
+      <c r="A589" s="97"/>
+      <c r="B589" s="97"/>
       <c r="C589" s="55"/>
       <c r="D589" s="55"/>
-      <c r="E589" s="42"/>
+      <c r="E589" s="55"/>
       <c r="F589" s="55"/>
       <c r="G589" s="95"/>
-      <c r="H589" s="55"/>
+      <c r="H589" s="42"/>
       <c r="I589" s="42"/>
       <c r="J589" s="42"/>
       <c r="K589" s="42"/>
@@ -18932,13 +19010,13 @@
       <c r="T589" s="36"/>
     </row>
     <row r="590" spans="1:20" ht="15" customHeight="1">
-      <c r="A590" s="97"/>
-      <c r="B590" s="97"/>
+      <c r="A590" s="42"/>
+      <c r="B590" s="55"/>
       <c r="C590" s="55"/>
       <c r="D590" s="55"/>
       <c r="E590" s="55"/>
-      <c r="F590" s="55"/>
-      <c r="G590" s="95"/>
+      <c r="F590" s="42"/>
+      <c r="G590" s="42"/>
       <c r="H590" s="42"/>
       <c r="I590" s="42"/>
       <c r="J590" s="42"/>
@@ -19047,12 +19125,12 @@
       <c r="C595" s="55"/>
       <c r="D595" s="55"/>
       <c r="E595" s="55"/>
-      <c r="F595" s="42"/>
-      <c r="G595" s="42"/>
+      <c r="F595" s="55"/>
+      <c r="G595" s="55"/>
       <c r="H595" s="42"/>
       <c r="I595" s="42"/>
-      <c r="J595" s="42"/>
-      <c r="K595" s="42"/>
+      <c r="J595" s="86"/>
+      <c r="K595" s="86"/>
       <c r="L595" s="42"/>
       <c r="M595" s="55"/>
       <c r="N595" s="55"/>
@@ -19159,10 +19237,10 @@
       <c r="E600" s="55"/>
       <c r="F600" s="55"/>
       <c r="G600" s="55"/>
-      <c r="H600" s="42"/>
+      <c r="H600" s="55"/>
       <c r="I600" s="42"/>
-      <c r="J600" s="86"/>
-      <c r="K600" s="86"/>
+      <c r="J600" s="56"/>
+      <c r="K600" s="56"/>
       <c r="L600" s="55"/>
       <c r="M600" s="55"/>
       <c r="N600" s="55"/>
@@ -19205,8 +19283,8 @@
       <c r="G602" s="55"/>
       <c r="H602" s="55"/>
       <c r="I602" s="42"/>
-      <c r="J602" s="56"/>
-      <c r="K602" s="56"/>
+      <c r="J602" s="42"/>
+      <c r="K602" s="42"/>
       <c r="L602" s="55"/>
       <c r="M602" s="55"/>
       <c r="N602" s="55"/>
@@ -19244,10 +19322,10 @@
       <c r="B604" s="55"/>
       <c r="C604" s="55"/>
       <c r="D604" s="55"/>
-      <c r="E604" s="55"/>
-      <c r="F604" s="55"/>
-      <c r="G604" s="55"/>
-      <c r="H604" s="55"/>
+      <c r="E604" s="42"/>
+      <c r="F604" s="42"/>
+      <c r="G604" s="42"/>
+      <c r="H604" s="42"/>
       <c r="I604" s="42"/>
       <c r="J604" s="42"/>
       <c r="K604" s="42"/>
@@ -19288,13 +19366,13 @@
       <c r="B606" s="55"/>
       <c r="C606" s="55"/>
       <c r="D606" s="55"/>
-      <c r="E606" s="42"/>
-      <c r="F606" s="42"/>
-      <c r="G606" s="42"/>
+      <c r="E606" s="55"/>
+      <c r="F606" s="55"/>
+      <c r="G606" s="55"/>
       <c r="H606" s="42"/>
       <c r="I606" s="42"/>
-      <c r="J606" s="42"/>
-      <c r="K606" s="42"/>
+      <c r="J606" s="86"/>
+      <c r="K606" s="86"/>
       <c r="L606" s="42"/>
       <c r="M606" s="42"/>
       <c r="N606" s="55"/>
@@ -19338,7 +19416,7 @@
       <c r="H608" s="42"/>
       <c r="I608" s="42"/>
       <c r="J608" s="86"/>
-      <c r="K608" s="86"/>
+      <c r="K608" s="42"/>
       <c r="L608" s="55"/>
       <c r="M608" s="55"/>
       <c r="N608" s="55"/>
@@ -19447,7 +19525,7 @@
       <c r="G613" s="55"/>
       <c r="H613" s="42"/>
       <c r="I613" s="42"/>
-      <c r="J613" s="86"/>
+      <c r="J613" s="42"/>
       <c r="K613" s="42"/>
       <c r="L613" s="55"/>
       <c r="M613" s="55"/>
@@ -19557,7 +19635,7 @@
       <c r="G618" s="55"/>
       <c r="H618" s="42"/>
       <c r="I618" s="42"/>
-      <c r="J618" s="42"/>
+      <c r="J618" s="56"/>
       <c r="K618" s="42"/>
       <c r="L618" s="55"/>
       <c r="M618" s="55"/>
@@ -19659,12 +19737,12 @@
     </row>
     <row r="623" spans="1:20" ht="15" customHeight="1">
       <c r="A623" s="42"/>
-      <c r="B623" s="55"/>
-      <c r="C623" s="55"/>
-      <c r="D623" s="55"/>
-      <c r="E623" s="55"/>
-      <c r="F623" s="55"/>
-      <c r="G623" s="55"/>
+      <c r="B623" s="90"/>
+      <c r="C623" s="91"/>
+      <c r="D623" s="91"/>
+      <c r="E623" s="91"/>
+      <c r="F623" s="91"/>
+      <c r="G623" s="91"/>
       <c r="H623" s="42"/>
       <c r="I623" s="42"/>
       <c r="J623" s="56"/>
@@ -19681,12 +19759,12 @@
     </row>
     <row r="624" spans="1:20" ht="16" customHeight="1">
       <c r="A624" s="42"/>
-      <c r="B624" s="90"/>
-      <c r="C624" s="91"/>
-      <c r="D624" s="91"/>
-      <c r="E624" s="91"/>
+      <c r="B624" s="92"/>
+      <c r="C624" s="93"/>
+      <c r="D624" s="93"/>
+      <c r="E624" s="93"/>
       <c r="F624" s="91"/>
-      <c r="G624" s="91"/>
+      <c r="G624" s="93"/>
       <c r="H624" s="42"/>
       <c r="I624" s="42"/>
       <c r="J624" s="56"/>
@@ -19769,12 +19847,12 @@
     </row>
     <row r="628" spans="1:20" ht="16" customHeight="1">
       <c r="A628" s="42"/>
-      <c r="B628" s="92"/>
-      <c r="C628" s="93"/>
-      <c r="D628" s="93"/>
-      <c r="E628" s="93"/>
+      <c r="B628" s="90"/>
+      <c r="C628" s="91"/>
+      <c r="D628" s="91"/>
+      <c r="E628" s="91"/>
       <c r="F628" s="91"/>
-      <c r="G628" s="93"/>
+      <c r="G628" s="91"/>
       <c r="H628" s="42"/>
       <c r="I628" s="42"/>
       <c r="J628" s="56"/>
@@ -19791,12 +19869,12 @@
     </row>
     <row r="629" spans="1:20" ht="16" customHeight="1">
       <c r="A629" s="42"/>
-      <c r="B629" s="90"/>
-      <c r="C629" s="91"/>
-      <c r="D629" s="91"/>
-      <c r="E629" s="91"/>
+      <c r="B629" s="92"/>
+      <c r="C629" s="93"/>
+      <c r="D629" s="93"/>
+      <c r="E629" s="93"/>
       <c r="F629" s="91"/>
-      <c r="G629" s="91"/>
+      <c r="G629" s="93"/>
       <c r="H629" s="42"/>
       <c r="I629" s="42"/>
       <c r="J629" s="56"/>
@@ -19879,15 +19957,15 @@
     </row>
     <row r="633" spans="1:20" ht="16" customHeight="1">
       <c r="A633" s="42"/>
-      <c r="B633" s="92"/>
-      <c r="C633" s="93"/>
-      <c r="D633" s="93"/>
-      <c r="E633" s="93"/>
+      <c r="B633" s="90"/>
+      <c r="C633" s="91"/>
+      <c r="D633" s="91"/>
+      <c r="E633" s="91"/>
       <c r="F633" s="91"/>
-      <c r="G633" s="93"/>
+      <c r="G633" s="91"/>
       <c r="H633" s="42"/>
       <c r="I633" s="42"/>
-      <c r="J633" s="56"/>
+      <c r="J633" s="42"/>
       <c r="K633" s="42"/>
       <c r="L633" s="55"/>
       <c r="M633" s="55"/>
@@ -19901,12 +19979,12 @@
     </row>
     <row r="634" spans="1:20" ht="16" customHeight="1">
       <c r="A634" s="42"/>
-      <c r="B634" s="90"/>
-      <c r="C634" s="91"/>
-      <c r="D634" s="91"/>
-      <c r="E634" s="91"/>
+      <c r="B634" s="92"/>
+      <c r="C634" s="93"/>
+      <c r="D634" s="93"/>
+      <c r="E634" s="93"/>
       <c r="F634" s="91"/>
-      <c r="G634" s="91"/>
+      <c r="G634" s="93"/>
       <c r="H634" s="42"/>
       <c r="I634" s="42"/>
       <c r="J634" s="42"/>
@@ -20010,17 +20088,17 @@
       <c r="T638" s="36"/>
     </row>
     <row r="639" spans="1:20" ht="16" customHeight="1">
-      <c r="A639" s="42"/>
-      <c r="B639" s="92"/>
-      <c r="C639" s="93"/>
-      <c r="D639" s="93"/>
-      <c r="E639" s="93"/>
-      <c r="F639" s="91"/>
-      <c r="G639" s="93"/>
+      <c r="A639" s="55"/>
+      <c r="B639" s="55"/>
+      <c r="C639" s="55"/>
+      <c r="D639" s="55"/>
+      <c r="E639" s="55"/>
+      <c r="F639" s="55"/>
+      <c r="G639" s="55"/>
       <c r="H639" s="42"/>
       <c r="I639" s="42"/>
-      <c r="J639" s="42"/>
-      <c r="K639" s="42"/>
+      <c r="J639" s="86"/>
+      <c r="K639" s="86"/>
       <c r="L639" s="55"/>
       <c r="M639" s="55"/>
       <c r="N639" s="55"/>
@@ -20107,8 +20185,8 @@
       <c r="G643" s="55"/>
       <c r="H643" s="42"/>
       <c r="I643" s="42"/>
-      <c r="J643" s="86"/>
-      <c r="K643" s="86"/>
+      <c r="J643" s="42"/>
+      <c r="K643" s="42"/>
       <c r="L643" s="55"/>
       <c r="M643" s="55"/>
       <c r="N643" s="55"/>
@@ -20193,10 +20271,10 @@
       <c r="E647" s="55"/>
       <c r="F647" s="55"/>
       <c r="G647" s="55"/>
-      <c r="H647" s="42"/>
+      <c r="H647" s="55"/>
       <c r="I647" s="42"/>
-      <c r="J647" s="42"/>
-      <c r="K647" s="42"/>
+      <c r="J647" s="86"/>
+      <c r="K647" s="86"/>
       <c r="L647" s="55"/>
       <c r="M647" s="42"/>
       <c r="N647" s="55"/>
@@ -20283,8 +20361,8 @@
       <c r="G651" s="55"/>
       <c r="H651" s="55"/>
       <c r="I651" s="42"/>
-      <c r="J651" s="86"/>
-      <c r="K651" s="86"/>
+      <c r="J651" s="56"/>
+      <c r="K651" s="42"/>
       <c r="L651" s="55"/>
       <c r="M651" s="55"/>
       <c r="N651" s="55"/>
@@ -20322,13 +20400,13 @@
       <c r="B653" s="55"/>
       <c r="C653" s="55"/>
       <c r="D653" s="55"/>
-      <c r="E653" s="55"/>
+      <c r="E653" s="42"/>
       <c r="F653" s="55"/>
       <c r="G653" s="55"/>
       <c r="H653" s="55"/>
       <c r="I653" s="42"/>
-      <c r="J653" s="56"/>
-      <c r="K653" s="42"/>
+      <c r="J653" s="86"/>
+      <c r="K653" s="86"/>
       <c r="L653" s="42"/>
       <c r="M653" s="42"/>
       <c r="N653" s="55"/>
@@ -20366,7 +20444,7 @@
       <c r="B655" s="55"/>
       <c r="C655" s="55"/>
       <c r="D655" s="55"/>
-      <c r="E655" s="42"/>
+      <c r="E655" s="55"/>
       <c r="F655" s="55"/>
       <c r="G655" s="55"/>
       <c r="H655" s="55"/>
@@ -20410,13 +20488,13 @@
       <c r="B657" s="55"/>
       <c r="C657" s="55"/>
       <c r="D657" s="55"/>
-      <c r="E657" s="55"/>
+      <c r="E657" s="42"/>
       <c r="F657" s="55"/>
       <c r="G657" s="55"/>
       <c r="H657" s="55"/>
       <c r="I657" s="42"/>
-      <c r="J657" s="86"/>
-      <c r="K657" s="86"/>
+      <c r="J657" s="56"/>
+      <c r="K657" s="42"/>
       <c r="L657" s="55"/>
       <c r="M657" s="55"/>
       <c r="N657" s="55"/>
@@ -20454,7 +20532,7 @@
       <c r="B659" s="55"/>
       <c r="C659" s="55"/>
       <c r="D659" s="55"/>
-      <c r="E659" s="42"/>
+      <c r="E659" s="55"/>
       <c r="F659" s="55"/>
       <c r="G659" s="55"/>
       <c r="H659" s="55"/>
@@ -20498,7 +20576,7 @@
       <c r="B661" s="55"/>
       <c r="C661" s="55"/>
       <c r="D661" s="55"/>
-      <c r="E661" s="55"/>
+      <c r="E661" s="42"/>
       <c r="F661" s="55"/>
       <c r="G661" s="55"/>
       <c r="H661" s="55"/>
@@ -20542,7 +20620,7 @@
       <c r="B663" s="55"/>
       <c r="C663" s="55"/>
       <c r="D663" s="55"/>
-      <c r="E663" s="42"/>
+      <c r="E663" s="55"/>
       <c r="F663" s="55"/>
       <c r="G663" s="55"/>
       <c r="H663" s="55"/>
@@ -20586,7 +20664,7 @@
       <c r="B665" s="55"/>
       <c r="C665" s="55"/>
       <c r="D665" s="55"/>
-      <c r="E665" s="55"/>
+      <c r="E665" s="42"/>
       <c r="F665" s="55"/>
       <c r="G665" s="55"/>
       <c r="H665" s="55"/>
@@ -20630,7 +20708,7 @@
       <c r="B667" s="55"/>
       <c r="C667" s="55"/>
       <c r="D667" s="55"/>
-      <c r="E667" s="42"/>
+      <c r="E667" s="55"/>
       <c r="F667" s="55"/>
       <c r="G667" s="55"/>
       <c r="H667" s="55"/>
@@ -20652,7 +20730,7 @@
       <c r="B668" s="55"/>
       <c r="C668" s="55"/>
       <c r="D668" s="55"/>
-      <c r="E668" s="55"/>
+      <c r="E668" s="42"/>
       <c r="F668" s="55"/>
       <c r="G668" s="55"/>
       <c r="H668" s="55"/>
@@ -20696,7 +20774,7 @@
       <c r="B670" s="55"/>
       <c r="C670" s="55"/>
       <c r="D670" s="55"/>
-      <c r="E670" s="42"/>
+      <c r="E670" s="55"/>
       <c r="F670" s="55"/>
       <c r="G670" s="55"/>
       <c r="H670" s="55"/>
@@ -20736,7 +20814,7 @@
       <c r="T671" s="36"/>
     </row>
     <row r="672" spans="1:20" ht="16" customHeight="1">
-      <c r="A672" s="55"/>
+      <c r="A672" s="42"/>
       <c r="B672" s="55"/>
       <c r="C672" s="55"/>
       <c r="D672" s="55"/>
@@ -20745,7 +20823,7 @@
       <c r="G672" s="55"/>
       <c r="H672" s="55"/>
       <c r="I672" s="42"/>
-      <c r="J672" s="56"/>
+      <c r="J672" s="86"/>
       <c r="K672" s="42"/>
       <c r="L672" s="55"/>
       <c r="M672" s="55"/>
@@ -20765,7 +20843,7 @@
       <c r="E673" s="55"/>
       <c r="F673" s="55"/>
       <c r="G673" s="55"/>
-      <c r="H673" s="55"/>
+      <c r="H673" s="42"/>
       <c r="I673" s="42"/>
       <c r="J673" s="86"/>
       <c r="K673" s="42"/>
@@ -20787,7 +20865,7 @@
       <c r="E674" s="55"/>
       <c r="F674" s="55"/>
       <c r="G674" s="55"/>
-      <c r="H674" s="42"/>
+      <c r="H674" s="55"/>
       <c r="I674" s="42"/>
       <c r="J674" s="86"/>
       <c r="K674" s="42"/>
@@ -20809,7 +20887,7 @@
       <c r="E675" s="55"/>
       <c r="F675" s="55"/>
       <c r="G675" s="55"/>
-      <c r="H675" s="55"/>
+      <c r="H675" s="42"/>
       <c r="I675" s="42"/>
       <c r="J675" s="86"/>
       <c r="K675" s="42"/>
@@ -20831,7 +20909,7 @@
       <c r="E676" s="55"/>
       <c r="F676" s="55"/>
       <c r="G676" s="55"/>
-      <c r="H676" s="42"/>
+      <c r="H676" s="55"/>
       <c r="I676" s="42"/>
       <c r="J676" s="86"/>
       <c r="K676" s="42"/>
@@ -20853,7 +20931,7 @@
       <c r="E677" s="55"/>
       <c r="F677" s="55"/>
       <c r="G677" s="55"/>
-      <c r="H677" s="55"/>
+      <c r="H677" s="42"/>
       <c r="I677" s="42"/>
       <c r="J677" s="86"/>
       <c r="K677" s="42"/>
@@ -20872,12 +20950,12 @@
       <c r="B678" s="55"/>
       <c r="C678" s="55"/>
       <c r="D678" s="55"/>
-      <c r="E678" s="55"/>
+      <c r="E678" s="42"/>
       <c r="F678" s="55"/>
       <c r="G678" s="55"/>
       <c r="H678" s="42"/>
       <c r="I678" s="42"/>
-      <c r="J678" s="86"/>
+      <c r="J678" s="56"/>
       <c r="K678" s="42"/>
       <c r="L678" s="55"/>
       <c r="M678" s="55"/>
@@ -20913,16 +20991,16 @@
     </row>
     <row r="680" spans="1:20" ht="16" customHeight="1">
       <c r="A680" s="42"/>
-      <c r="B680" s="55"/>
+      <c r="B680" s="98"/>
       <c r="C680" s="55"/>
       <c r="D680" s="55"/>
-      <c r="E680" s="42"/>
+      <c r="E680" s="55"/>
       <c r="F680" s="55"/>
       <c r="G680" s="55"/>
       <c r="H680" s="42"/>
       <c r="I680" s="42"/>
-      <c r="J680" s="56"/>
-      <c r="K680" s="42"/>
+      <c r="J680" s="86"/>
+      <c r="K680" s="86"/>
       <c r="L680" s="55"/>
       <c r="M680" s="42"/>
       <c r="N680" s="55"/>
@@ -20965,8 +21043,8 @@
       <c r="G682" s="55"/>
       <c r="H682" s="42"/>
       <c r="I682" s="42"/>
-      <c r="J682" s="86"/>
-      <c r="K682" s="86"/>
+      <c r="J682" s="56"/>
+      <c r="K682" s="56"/>
       <c r="L682" s="55"/>
       <c r="M682" s="55"/>
       <c r="N682" s="55"/>
@@ -21045,16 +21123,16 @@
     </row>
     <row r="686" spans="1:20" ht="16" customHeight="1">
       <c r="A686" s="42"/>
-      <c r="B686" s="98"/>
-      <c r="C686" s="55"/>
-      <c r="D686" s="55"/>
-      <c r="E686" s="55"/>
-      <c r="F686" s="55"/>
-      <c r="G686" s="55"/>
+      <c r="B686" s="42"/>
+      <c r="C686" s="42"/>
+      <c r="D686" s="42"/>
+      <c r="E686" s="42"/>
+      <c r="F686" s="42"/>
+      <c r="G686" s="42"/>
       <c r="H686" s="42"/>
       <c r="I686" s="42"/>
-      <c r="J686" s="56"/>
-      <c r="K686" s="56"/>
+      <c r="J686" s="42"/>
+      <c r="K686" s="42"/>
       <c r="L686" s="55"/>
       <c r="M686" s="55"/>
       <c r="N686" s="55"/>
@@ -26589,7 +26667,6 @@
     </row>
     <row r="938" spans="1:20" ht="15" customHeight="1">
       <c r="A938" s="42"/>
-      <c r="B938" s="42"/>
       <c r="C938" s="42"/>
       <c r="D938" s="42"/>
       <c r="E938" s="42"/>
@@ -26716,7 +26793,6 @@
     </row>
     <row r="944" spans="1:20" ht="15" customHeight="1">
       <c r="A944" s="42"/>
-      <c r="C944" s="42"/>
       <c r="D944" s="42"/>
       <c r="E944" s="42"/>
       <c r="F944" s="42"/>
@@ -26742,9 +26818,6 @@
       <c r="F945" s="42"/>
       <c r="G945" s="42"/>
       <c r="H945" s="42"/>
-      <c r="I945" s="42"/>
-      <c r="J945" s="42"/>
-      <c r="K945" s="42"/>
       <c r="L945" s="42"/>
       <c r="M945" s="42"/>
       <c r="N945" s="42"/>
@@ -26910,12 +26983,6 @@
       <c r="T955" s="42"/>
     </row>
     <row r="956" spans="1:20" ht="15" customHeight="1">
-      <c r="A956" s="42"/>
-      <c r="D956" s="42"/>
-      <c r="E956" s="42"/>
-      <c r="F956" s="42"/>
-      <c r="G956" s="42"/>
-      <c r="H956" s="42"/>
       <c r="M956" s="42"/>
       <c r="N956" s="42"/>
       <c r="O956" s="42"/>
@@ -26946,6 +27013,11 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="O5:O7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="P8:T8"/>
     <mergeCell ref="D2:E3"/>
     <mergeCell ref="F2:N3"/>
     <mergeCell ref="C5:C6"/>
@@ -26960,11 +27032,6 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
-    <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="P8:T8"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
- parsed data from `10.1109/ACCESS.2026.3693781`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010B7EF2-4B12-8945-802B-53C9FE7C4A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65F2DE9-AB28-DD45-9F39-4068C0DBF4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="164">
   <si>
     <r>
       <rPr>
@@ -616,6 +616,12 @@
   </si>
   <si>
     <t>10.1016/j.jmrt.2026.05.105</t>
+  </si>
+  <si>
+    <t>MoNiSiTiV</t>
+  </si>
+  <si>
+    <t>10.1109/ACCESS.2026.3693781</t>
   </si>
 </sst>
 </file>
@@ -8687,7 +8693,7 @@
         <v>298</v>
       </c>
       <c r="J121" s="86">
-        <f t="shared" ref="J121:K121" si="3">P121*9807000</f>
+        <f t="shared" ref="J121:K122" si="3">P121*9807000</f>
         <v>5285973000</v>
       </c>
       <c r="K121" s="86">
@@ -8716,22 +8722,48 @@
     </row>
     <row r="122" spans="1:20" ht="18" customHeight="1">
       <c r="A122" s="29"/>
-      <c r="B122" s="30"/>
-      <c r="C122" s="29"/>
-      <c r="D122" s="29"/>
+      <c r="B122" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="C122" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D122" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E122" s="29"/>
-      <c r="F122" s="31"/>
-      <c r="G122" s="31"/>
+      <c r="F122" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G122" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H122" s="32"/>
-      <c r="I122" s="38"/>
-      <c r="J122" s="86"/>
-      <c r="K122" s="34"/>
-      <c r="L122" s="31"/>
+      <c r="I122" s="108">
+        <v>298</v>
+      </c>
+      <c r="J122" s="86">
+        <f t="shared" si="3"/>
+        <v>8679195000</v>
+      </c>
+      <c r="K122" s="86">
+        <f t="shared" si="3"/>
+        <v>98070000</v>
+      </c>
+      <c r="L122" s="31" t="s">
+        <v>32</v>
+      </c>
       <c r="M122" s="39"/>
-      <c r="N122" s="35"/>
+      <c r="N122" s="35" t="s">
+        <v>163</v>
+      </c>
       <c r="O122" s="43"/>
-      <c r="P122" s="43"/>
-      <c r="Q122" s="37"/>
+      <c r="P122" s="43">
+        <v>885</v>
+      </c>
+      <c r="Q122" s="37">
+        <v>10</v>
+      </c>
       <c r="R122" s="43"/>
       <c r="S122" s="36"/>
       <c r="T122" s="36"/>

</xml_diff>

<commit_message>
- parsed data from `10.1080/10667857.2026.2674815`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65F2DE9-AB28-DD45-9F39-4068C0DBF4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5BB2AB-AD9B-3C4C-AF41-7C162BDCFCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="181">
   <si>
     <r>
       <rPr>
@@ -622,6 +622,57 @@
   </si>
   <si>
     <t>10.1109/ACCESS.2026.3693781</t>
+  </si>
+  <si>
+    <t>AAM</t>
+  </si>
+  <si>
+    <t>W0.4 Mo Nb1.3 Ta Ti</t>
+  </si>
+  <si>
+    <t>Cr0</t>
+  </si>
+  <si>
+    <t>W0.4 Mo Nb1.3 Ta Ti Cr0.25</t>
+  </si>
+  <si>
+    <t>W0.4 Mo Nb1.3 Ta Ti Cr0.5</t>
+  </si>
+  <si>
+    <t>W0.4 Mo Nb1.3 Ta Ti Cr0.75</t>
+  </si>
+  <si>
+    <t>Cr0.25</t>
+  </si>
+  <si>
+    <t>Cr0.5</t>
+  </si>
+  <si>
+    <t>Cr.075</t>
+  </si>
+  <si>
+    <t>BCC+laves</t>
+  </si>
+  <si>
+    <t>minor laves phase content around 10%</t>
+  </si>
+  <si>
+    <t>very minor laves phase content around 2%</t>
+  </si>
+  <si>
+    <t>very minor laves phase content around 5%</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>T7</t>
+  </si>
+  <si>
+    <t>F7</t>
+  </si>
+  <si>
+    <t>10.1080/10667857.2026.2674815</t>
   </si>
 </sst>
 </file>
@@ -8693,7 +8744,7 @@
         <v>298</v>
       </c>
       <c r="J121" s="86">
-        <f t="shared" ref="J121:K122" si="3">P121*9807000</f>
+        <f t="shared" ref="J121:K126" si="3">P121*9807000</f>
         <v>5285973000</v>
       </c>
       <c r="K121" s="86">
@@ -8769,108 +8820,256 @@
       <c r="T122" s="36"/>
     </row>
     <row r="123" spans="1:20" ht="18" customHeight="1">
-      <c r="A123" s="29"/>
-      <c r="B123" s="30"/>
-      <c r="C123" s="29"/>
-      <c r="D123" s="29"/>
+      <c r="A123" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B123" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="C123" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D123" s="29" t="s">
+        <v>164</v>
+      </c>
       <c r="E123" s="29"/>
-      <c r="F123" s="31"/>
-      <c r="G123" s="31"/>
+      <c r="F123" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G123" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H123" s="32"/>
-      <c r="I123" s="38"/>
-      <c r="J123" s="86"/>
-      <c r="K123" s="34"/>
-      <c r="L123" s="31"/>
-      <c r="M123" s="39"/>
-      <c r="N123" s="35"/>
+      <c r="I123" s="108">
+        <v>298</v>
+      </c>
+      <c r="J123" s="86">
+        <f t="shared" si="3"/>
+        <v>4522007700</v>
+      </c>
+      <c r="K123" s="86">
+        <f t="shared" si="3"/>
+        <v>68649000</v>
+      </c>
+      <c r="L123" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M123" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="N123" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O123" s="43"/>
-      <c r="P123" s="43"/>
-      <c r="Q123" s="37"/>
+      <c r="P123" s="43">
+        <v>461.1</v>
+      </c>
+      <c r="Q123" s="37">
+        <v>7</v>
+      </c>
       <c r="R123" s="43"/>
       <c r="S123" s="36"/>
       <c r="T123" s="36"/>
     </row>
     <row r="124" spans="1:20" ht="18" customHeight="1">
-      <c r="A124" s="29"/>
-      <c r="B124" s="30"/>
-      <c r="C124" s="29"/>
-      <c r="D124" s="29"/>
-      <c r="E124" s="29"/>
-      <c r="F124" s="31"/>
-      <c r="G124" s="31"/>
+      <c r="A124" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="B124" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="C124" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D124" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E124" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="F124" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G124" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H124" s="32"/>
-      <c r="I124" s="38"/>
-      <c r="J124" s="86"/>
-      <c r="K124" s="34"/>
-      <c r="L124" s="31"/>
-      <c r="M124" s="39"/>
-      <c r="N124" s="35"/>
+      <c r="I124" s="108">
+        <v>298</v>
+      </c>
+      <c r="J124" s="86">
+        <f t="shared" si="3"/>
+        <v>4954496400</v>
+      </c>
+      <c r="K124" s="86">
+        <f t="shared" si="3"/>
+        <v>107877000</v>
+      </c>
+      <c r="L124" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M124" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="N124" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O124" s="43"/>
-      <c r="P124" s="36"/>
-      <c r="Q124" s="37"/>
+      <c r="P124" s="36">
+        <v>505.2</v>
+      </c>
+      <c r="Q124" s="37">
+        <v>11</v>
+      </c>
       <c r="R124" s="43"/>
       <c r="S124" s="36"/>
       <c r="T124" s="36"/>
     </row>
     <row r="125" spans="1:20" ht="18" customHeight="1">
-      <c r="A125" s="29"/>
-      <c r="B125" s="30"/>
-      <c r="C125" s="29"/>
-      <c r="D125" s="29"/>
-      <c r="E125" s="29"/>
-      <c r="F125" s="31"/>
-      <c r="G125" s="31"/>
+      <c r="A125" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B125" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C125" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D125" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E125" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="F125" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G125" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H125" s="32"/>
-      <c r="I125" s="38"/>
-      <c r="J125" s="86"/>
-      <c r="K125" s="34"/>
-      <c r="L125" s="31"/>
-      <c r="M125" s="39"/>
-      <c r="N125" s="35"/>
+      <c r="I125" s="108">
+        <v>298</v>
+      </c>
+      <c r="J125" s="86">
+        <f t="shared" si="3"/>
+        <v>5497804200</v>
+      </c>
+      <c r="K125" s="86">
+        <f t="shared" si="3"/>
+        <v>117684000</v>
+      </c>
+      <c r="L125" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M125" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="N125" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O125" s="36"/>
-      <c r="P125" s="36"/>
-      <c r="Q125" s="37"/>
+      <c r="P125" s="36">
+        <v>560.6</v>
+      </c>
+      <c r="Q125" s="37">
+        <v>12</v>
+      </c>
       <c r="R125" s="43"/>
       <c r="S125" s="36"/>
       <c r="T125" s="36"/>
     </row>
     <row r="126" spans="1:20" ht="18" customHeight="1">
-      <c r="A126" s="29"/>
-      <c r="B126" s="30"/>
-      <c r="C126" s="29"/>
-      <c r="D126" s="29"/>
-      <c r="E126" s="29"/>
-      <c r="F126" s="31"/>
-      <c r="G126" s="31"/>
+      <c r="A126" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="B126" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="C126" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D126" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E126" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="F126" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G126" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H126" s="32"/>
-      <c r="I126" s="38"/>
-      <c r="J126" s="86"/>
-      <c r="K126" s="34"/>
-      <c r="L126" s="31"/>
-      <c r="M126" s="39"/>
-      <c r="N126" s="35"/>
+      <c r="I126" s="108">
+        <v>298</v>
+      </c>
+      <c r="J126" s="86">
+        <f t="shared" si="3"/>
+        <v>6004826100</v>
+      </c>
+      <c r="K126" s="86">
+        <f t="shared" si="3"/>
+        <v>88263000</v>
+      </c>
+      <c r="L126" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M126" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="N126" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O126" s="36"/>
-      <c r="P126" s="36"/>
-      <c r="Q126" s="37"/>
+      <c r="P126" s="36">
+        <v>612.29999999999995</v>
+      </c>
+      <c r="Q126" s="37">
+        <v>9</v>
+      </c>
       <c r="R126" s="43"/>
       <c r="S126" s="36"/>
       <c r="T126" s="36"/>
     </row>
     <row r="127" spans="1:20" ht="18" customHeight="1">
-      <c r="A127" s="29"/>
-      <c r="B127" s="30"/>
-      <c r="C127" s="29"/>
-      <c r="D127" s="29"/>
+      <c r="A127" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B127" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="C127" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D127" s="29" t="s">
+        <v>164</v>
+      </c>
       <c r="E127" s="29"/>
-      <c r="F127" s="31"/>
-      <c r="G127" s="31"/>
+      <c r="F127" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G127" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H127" s="32"/>
-      <c r="I127" s="38"/>
-      <c r="J127" s="86"/>
+      <c r="I127" s="108">
+        <v>298</v>
+      </c>
+      <c r="J127" s="86">
+        <v>1400000000</v>
+      </c>
       <c r="K127" s="34"/>
-      <c r="L127" s="31"/>
-      <c r="M127" s="39"/>
-      <c r="N127" s="35"/>
+      <c r="L127" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M127" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N127" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O127" s="36"/>
       <c r="P127" s="36"/>
       <c r="Q127" s="37"/>
@@ -8879,20 +9078,44 @@
       <c r="T127" s="36"/>
     </row>
     <row r="128" spans="1:20" ht="18" customHeight="1">
-      <c r="A128" s="29"/>
-      <c r="B128" s="30"/>
-      <c r="C128" s="29"/>
-      <c r="D128" s="29"/>
-      <c r="E128" s="29"/>
-      <c r="F128" s="31"/>
-      <c r="G128" s="31"/>
+      <c r="A128" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="B128" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="C128" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D128" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E128" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="F128" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G128" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H128" s="32"/>
-      <c r="I128" s="33"/>
-      <c r="J128" s="86"/>
+      <c r="I128" s="108">
+        <v>298</v>
+      </c>
+      <c r="J128" s="86">
+        <v>1460000000</v>
+      </c>
       <c r="K128" s="34"/>
-      <c r="L128" s="31"/>
-      <c r="M128" s="39"/>
-      <c r="N128" s="35"/>
+      <c r="L128" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M128" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N128" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O128" s="36"/>
       <c r="P128" s="36"/>
       <c r="Q128" s="37"/>
@@ -8901,20 +9124,44 @@
       <c r="T128" s="36"/>
     </row>
     <row r="129" spans="1:20" ht="18" customHeight="1">
-      <c r="A129" s="29"/>
-      <c r="B129" s="30"/>
-      <c r="C129" s="29"/>
-      <c r="D129" s="29"/>
-      <c r="E129" s="29"/>
-      <c r="F129" s="31"/>
-      <c r="G129" s="31"/>
+      <c r="A129" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B129" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C129" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D129" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E129" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="F129" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G129" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H129" s="32"/>
-      <c r="I129" s="33"/>
-      <c r="J129" s="86"/>
+      <c r="I129" s="108">
+        <v>298</v>
+      </c>
+      <c r="J129" s="86">
+        <v>1500000000</v>
+      </c>
       <c r="K129" s="34"/>
-      <c r="L129" s="31"/>
-      <c r="M129" s="31"/>
-      <c r="N129" s="35"/>
+      <c r="L129" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M129" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N129" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O129" s="36"/>
       <c r="P129" s="36"/>
       <c r="Q129" s="37"/>
@@ -8923,20 +9170,44 @@
       <c r="T129" s="36"/>
     </row>
     <row r="130" spans="1:20" ht="18" customHeight="1">
-      <c r="A130" s="29"/>
-      <c r="B130" s="30"/>
-      <c r="C130" s="29"/>
-      <c r="D130" s="29"/>
-      <c r="E130" s="29"/>
-      <c r="F130" s="31"/>
-      <c r="G130" s="31"/>
+      <c r="A130" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="B130" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="C130" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="D130" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E130" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="F130" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G130" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H130" s="32"/>
-      <c r="I130" s="33"/>
-      <c r="J130" s="86"/>
+      <c r="I130" s="108">
+        <v>298</v>
+      </c>
+      <c r="J130" s="86">
+        <v>1550000000</v>
+      </c>
       <c r="K130" s="34"/>
-      <c r="L130" s="31"/>
-      <c r="M130" s="31"/>
-      <c r="N130" s="35"/>
+      <c r="L130" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M130" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N130" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O130" s="36"/>
       <c r="P130" s="36"/>
       <c r="Q130" s="37"/>
@@ -8945,20 +9216,42 @@
       <c r="T130" s="36"/>
     </row>
     <row r="131" spans="1:20" ht="18" customHeight="1">
-      <c r="A131" s="29"/>
-      <c r="B131" s="30"/>
-      <c r="C131" s="29"/>
-      <c r="D131" s="29"/>
-      <c r="E131" s="29"/>
-      <c r="F131" s="31"/>
-      <c r="G131" s="31"/>
-      <c r="H131" s="32"/>
-      <c r="I131" s="33"/>
-      <c r="J131" s="86"/>
+      <c r="A131" s="114" t="s">
+        <v>166</v>
+      </c>
+      <c r="B131" s="100" t="s">
+        <v>165</v>
+      </c>
+      <c r="C131" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D131" s="87" t="s">
+        <v>164</v>
+      </c>
+      <c r="E131" s="87"/>
+      <c r="F131" s="94" t="s">
+        <v>125</v>
+      </c>
+      <c r="G131" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H131" s="118"/>
+      <c r="I131" s="108">
+        <v>298</v>
+      </c>
+      <c r="J131" s="86">
+        <v>1980000000</v>
+      </c>
       <c r="K131" s="34"/>
-      <c r="L131" s="31"/>
-      <c r="M131" s="31"/>
-      <c r="N131" s="35"/>
+      <c r="L131" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M131" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N131" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O131" s="36"/>
       <c r="P131" s="36"/>
       <c r="Q131" s="37"/>
@@ -8967,20 +9260,44 @@
       <c r="T131" s="36"/>
     </row>
     <row r="132" spans="1:20" ht="18" customHeight="1">
-      <c r="A132" s="29"/>
-      <c r="B132" s="30"/>
-      <c r="C132" s="29"/>
-      <c r="D132" s="29"/>
-      <c r="E132" s="29"/>
-      <c r="F132" s="31"/>
-      <c r="G132" s="31"/>
-      <c r="H132" s="32"/>
-      <c r="I132" s="33"/>
-      <c r="J132" s="43"/>
+      <c r="A132" s="115" t="s">
+        <v>170</v>
+      </c>
+      <c r="B132" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="C132" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D132" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E132" s="88" t="s">
+        <v>175</v>
+      </c>
+      <c r="F132" s="94" t="s">
+        <v>125</v>
+      </c>
+      <c r="G132" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H132" s="119"/>
+      <c r="I132" s="108">
+        <v>298</v>
+      </c>
+      <c r="J132" s="116">
+        <v>2070000000</v>
+      </c>
       <c r="K132" s="34"/>
-      <c r="L132" s="31"/>
-      <c r="M132" s="31"/>
-      <c r="N132" s="35"/>
+      <c r="L132" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M132" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N132" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O132" s="36"/>
       <c r="P132" s="36"/>
       <c r="Q132" s="37"/>
@@ -8989,20 +9306,44 @@
       <c r="T132" s="36"/>
     </row>
     <row r="133" spans="1:20" ht="18" customHeight="1">
-      <c r="A133" s="29"/>
-      <c r="B133" s="30"/>
-      <c r="C133" s="29"/>
-      <c r="D133" s="29"/>
-      <c r="E133" s="29"/>
-      <c r="F133" s="31"/>
-      <c r="G133" s="31"/>
-      <c r="H133" s="32"/>
-      <c r="I133" s="33"/>
-      <c r="J133" s="43"/>
+      <c r="A133" s="115" t="s">
+        <v>171</v>
+      </c>
+      <c r="B133" s="102" t="s">
+        <v>168</v>
+      </c>
+      <c r="C133" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D133" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E133" s="88" t="s">
+        <v>176</v>
+      </c>
+      <c r="F133" s="94" t="s">
+        <v>125</v>
+      </c>
+      <c r="G133" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H133" s="119"/>
+      <c r="I133" s="108">
+        <v>298</v>
+      </c>
+      <c r="J133" s="116">
+        <v>2120000000</v>
+      </c>
       <c r="K133" s="34"/>
-      <c r="L133" s="31"/>
-      <c r="M133" s="31"/>
-      <c r="N133" s="35"/>
+      <c r="L133" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M133" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N133" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O133" s="36"/>
       <c r="P133" s="36"/>
       <c r="Q133" s="36"/>
@@ -9011,20 +9352,44 @@
       <c r="T133" s="36"/>
     </row>
     <row r="134" spans="1:20" ht="18" customHeight="1">
-      <c r="A134" s="29"/>
-      <c r="B134" s="30"/>
-      <c r="C134" s="29"/>
-      <c r="D134" s="29"/>
-      <c r="E134" s="29"/>
-      <c r="F134" s="31"/>
-      <c r="G134" s="31"/>
-      <c r="H134" s="32"/>
-      <c r="I134" s="33"/>
-      <c r="J134" s="43"/>
+      <c r="A134" s="115" t="s">
+        <v>172</v>
+      </c>
+      <c r="B134" s="102" t="s">
+        <v>169</v>
+      </c>
+      <c r="C134" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D134" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E134" s="88" t="s">
+        <v>174</v>
+      </c>
+      <c r="F134" s="94" t="s">
+        <v>125</v>
+      </c>
+      <c r="G134" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H134" s="119"/>
+      <c r="I134" s="108">
+        <v>298</v>
+      </c>
+      <c r="J134" s="116">
+        <v>2200000000</v>
+      </c>
       <c r="K134" s="34"/>
-      <c r="L134" s="31"/>
-      <c r="M134" s="31"/>
-      <c r="N134" s="35"/>
+      <c r="L134" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M134" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N134" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O134" s="36"/>
       <c r="P134" s="36"/>
       <c r="Q134" s="36"/>
@@ -9033,20 +9398,42 @@
       <c r="T134" s="36"/>
     </row>
     <row r="135" spans="1:20" ht="18" customHeight="1">
-      <c r="A135" s="29"/>
-      <c r="B135" s="30"/>
-      <c r="C135" s="29"/>
-      <c r="D135" s="29"/>
-      <c r="E135" s="29"/>
-      <c r="F135" s="31"/>
-      <c r="G135" s="31"/>
-      <c r="H135" s="32"/>
-      <c r="I135" s="33"/>
-      <c r="J135" s="43"/>
+      <c r="A135" s="114" t="s">
+        <v>166</v>
+      </c>
+      <c r="B135" s="100" t="s">
+        <v>165</v>
+      </c>
+      <c r="C135" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D135" s="87" t="s">
+        <v>164</v>
+      </c>
+      <c r="E135" s="87"/>
+      <c r="F135" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G135" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H135" s="118"/>
+      <c r="I135" s="108">
+        <v>298</v>
+      </c>
+      <c r="J135" s="43">
+        <v>41.1</v>
+      </c>
       <c r="K135" s="34"/>
-      <c r="L135" s="31"/>
-      <c r="M135" s="31"/>
-      <c r="N135" s="35"/>
+      <c r="L135" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M135" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N135" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O135" s="36"/>
       <c r="P135" s="36"/>
       <c r="Q135" s="36"/>
@@ -9055,20 +9442,44 @@
       <c r="T135" s="36"/>
     </row>
     <row r="136" spans="1:20" ht="18" customHeight="1">
-      <c r="A136" s="29"/>
-      <c r="B136" s="30"/>
-      <c r="C136" s="29"/>
-      <c r="D136" s="29"/>
-      <c r="E136" s="29"/>
-      <c r="F136" s="31"/>
-      <c r="G136" s="31"/>
-      <c r="H136" s="32"/>
-      <c r="I136" s="33"/>
-      <c r="J136" s="43"/>
+      <c r="A136" s="115" t="s">
+        <v>170</v>
+      </c>
+      <c r="B136" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="C136" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D136" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E136" s="88" t="s">
+        <v>175</v>
+      </c>
+      <c r="F136" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G136" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H136" s="119"/>
+      <c r="I136" s="108">
+        <v>298</v>
+      </c>
+      <c r="J136" s="43">
+        <v>35.4</v>
+      </c>
       <c r="K136" s="34"/>
-      <c r="L136" s="31"/>
-      <c r="M136" s="31"/>
-      <c r="N136" s="35"/>
+      <c r="L136" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M136" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N136" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O136" s="36"/>
       <c r="P136" s="36"/>
       <c r="Q136" s="36"/>
@@ -9077,20 +9488,44 @@
       <c r="T136" s="36"/>
     </row>
     <row r="137" spans="1:20" ht="18" customHeight="1">
-      <c r="A137" s="29"/>
-      <c r="B137" s="30"/>
-      <c r="C137" s="29"/>
-      <c r="D137" s="29"/>
-      <c r="E137" s="29"/>
-      <c r="F137" s="31"/>
-      <c r="G137" s="31"/>
-      <c r="H137" s="32"/>
-      <c r="I137" s="33"/>
-      <c r="J137" s="43"/>
+      <c r="A137" s="115" t="s">
+        <v>171</v>
+      </c>
+      <c r="B137" s="102" t="s">
+        <v>168</v>
+      </c>
+      <c r="C137" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D137" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E137" s="88" t="s">
+        <v>176</v>
+      </c>
+      <c r="F137" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G137" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H137" s="119"/>
+      <c r="I137" s="108">
+        <v>298</v>
+      </c>
+      <c r="J137" s="43">
+        <v>28.2</v>
+      </c>
       <c r="K137" s="34"/>
-      <c r="L137" s="31"/>
-      <c r="M137" s="31"/>
-      <c r="N137" s="35"/>
+      <c r="L137" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M137" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N137" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O137" s="36"/>
       <c r="P137" s="36"/>
       <c r="Q137" s="36"/>
@@ -9099,20 +9534,44 @@
       <c r="T137" s="36"/>
     </row>
     <row r="138" spans="1:20" ht="18" customHeight="1">
-      <c r="A138" s="29"/>
-      <c r="B138" s="30"/>
-      <c r="C138" s="29"/>
-      <c r="D138" s="29"/>
-      <c r="E138" s="29"/>
-      <c r="F138" s="31"/>
-      <c r="G138" s="31"/>
-      <c r="H138" s="32"/>
-      <c r="I138" s="33"/>
-      <c r="J138" s="34"/>
+      <c r="A138" s="115" t="s">
+        <v>172</v>
+      </c>
+      <c r="B138" s="102" t="s">
+        <v>169</v>
+      </c>
+      <c r="C138" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D138" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E138" s="88" t="s">
+        <v>174</v>
+      </c>
+      <c r="F138" s="94" t="s">
+        <v>114</v>
+      </c>
+      <c r="G138" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H138" s="119"/>
+      <c r="I138" s="108">
+        <v>298</v>
+      </c>
+      <c r="J138" s="34">
+        <v>10.4</v>
+      </c>
       <c r="K138" s="34"/>
-      <c r="L138" s="31"/>
-      <c r="M138" s="31"/>
-      <c r="N138" s="35"/>
+      <c r="L138" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M138" s="39" t="s">
+        <v>178</v>
+      </c>
+      <c r="N138" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O138" s="36"/>
       <c r="P138" s="36"/>
       <c r="Q138" s="36"/>
@@ -9121,20 +9580,44 @@
       <c r="T138" s="36"/>
     </row>
     <row r="139" spans="1:20" ht="18" customHeight="1">
-      <c r="A139" s="29"/>
-      <c r="B139" s="30"/>
-      <c r="C139" s="29"/>
-      <c r="D139" s="29"/>
-      <c r="E139" s="29"/>
-      <c r="F139" s="31"/>
-      <c r="G139" s="31"/>
-      <c r="H139" s="32"/>
-      <c r="I139" s="33"/>
-      <c r="J139" s="34"/>
+      <c r="A139" s="114" t="s">
+        <v>166</v>
+      </c>
+      <c r="B139" s="100" t="s">
+        <v>165</v>
+      </c>
+      <c r="C139" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D139" s="87" t="s">
+        <v>164</v>
+      </c>
+      <c r="E139" s="87"/>
+      <c r="F139" s="94" t="s">
+        <v>153</v>
+      </c>
+      <c r="G139" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H139" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I139" s="108">
+        <v>298</v>
+      </c>
+      <c r="J139" s="34">
+        <v>-0.42248999999999998</v>
+      </c>
       <c r="K139" s="34"/>
-      <c r="L139" s="31"/>
-      <c r="M139" s="31"/>
-      <c r="N139" s="35"/>
+      <c r="L139" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M139" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="N139" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O139" s="36"/>
       <c r="P139" s="37"/>
       <c r="Q139" s="37"/>
@@ -9143,20 +9626,46 @@
       <c r="T139" s="36"/>
     </row>
     <row r="140" spans="1:20" ht="18" customHeight="1">
-      <c r="A140" s="48"/>
-      <c r="B140" s="30"/>
-      <c r="C140" s="88"/>
-      <c r="D140" s="29"/>
-      <c r="E140" s="30"/>
-      <c r="F140" s="31"/>
-      <c r="G140" s="31"/>
-      <c r="H140" s="32"/>
-      <c r="I140" s="33"/>
-      <c r="J140" s="34"/>
+      <c r="A140" s="115" t="s">
+        <v>170</v>
+      </c>
+      <c r="B140" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="C140" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D140" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E140" s="88" t="s">
+        <v>175</v>
+      </c>
+      <c r="F140" s="94" t="s">
+        <v>153</v>
+      </c>
+      <c r="G140" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H140" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I140" s="108">
+        <v>298</v>
+      </c>
+      <c r="J140" s="34">
+        <v>-0.37193999999999999</v>
+      </c>
       <c r="K140" s="34"/>
-      <c r="L140" s="31"/>
-      <c r="M140" s="31"/>
-      <c r="N140" s="35"/>
+      <c r="L140" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M140" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="N140" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O140" s="36"/>
       <c r="P140" s="37"/>
       <c r="Q140" s="37"/>
@@ -9165,20 +9674,46 @@
       <c r="T140" s="36"/>
     </row>
     <row r="141" spans="1:20" ht="18" customHeight="1">
-      <c r="A141" s="48"/>
-      <c r="B141" s="30"/>
-      <c r="C141" s="88"/>
-      <c r="D141" s="29"/>
-      <c r="E141" s="30"/>
-      <c r="F141" s="31"/>
-      <c r="G141" s="31"/>
-      <c r="H141" s="32"/>
-      <c r="I141" s="33"/>
-      <c r="J141" s="34"/>
+      <c r="A141" s="115" t="s">
+        <v>171</v>
+      </c>
+      <c r="B141" s="102" t="s">
+        <v>168</v>
+      </c>
+      <c r="C141" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D141" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E141" s="88" t="s">
+        <v>176</v>
+      </c>
+      <c r="F141" s="94" t="s">
+        <v>153</v>
+      </c>
+      <c r="G141" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H141" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I141" s="108">
+        <v>298</v>
+      </c>
+      <c r="J141" s="34">
+        <v>-0.34039999999999998</v>
+      </c>
       <c r="K141" s="34"/>
-      <c r="L141" s="31"/>
-      <c r="M141" s="31"/>
-      <c r="N141" s="35"/>
+      <c r="L141" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M141" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="N141" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O141" s="36"/>
       <c r="P141" s="37"/>
       <c r="Q141" s="37"/>
@@ -9187,20 +9722,46 @@
       <c r="T141" s="36"/>
     </row>
     <row r="142" spans="1:20" ht="18" customHeight="1">
-      <c r="A142" s="48"/>
-      <c r="B142" s="30"/>
-      <c r="C142" s="29"/>
-      <c r="D142" s="29"/>
-      <c r="E142" s="30"/>
-      <c r="F142" s="31"/>
-      <c r="G142" s="31"/>
-      <c r="H142" s="32"/>
-      <c r="I142" s="33"/>
-      <c r="J142" s="34"/>
+      <c r="A142" s="115" t="s">
+        <v>172</v>
+      </c>
+      <c r="B142" s="102" t="s">
+        <v>169</v>
+      </c>
+      <c r="C142" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="D142" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="E142" s="88" t="s">
+        <v>174</v>
+      </c>
+      <c r="F142" s="94" t="s">
+        <v>153</v>
+      </c>
+      <c r="G142" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H142" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="I142" s="108">
+        <v>298</v>
+      </c>
+      <c r="J142" s="34">
+        <v>-0.30552000000000001</v>
+      </c>
       <c r="K142" s="34"/>
-      <c r="L142" s="31"/>
-      <c r="M142" s="31"/>
-      <c r="N142" s="35"/>
+      <c r="L142" s="31" t="s">
+        <v>156</v>
+      </c>
+      <c r="M142" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="N142" s="35" t="s">
+        <v>180</v>
+      </c>
       <c r="O142" s="36"/>
       <c r="P142" s="37"/>
       <c r="Q142" s="37"/>
@@ -9284,7 +9845,7 @@
       <c r="G146" s="31"/>
       <c r="H146" s="32"/>
       <c r="I146" s="33"/>
-      <c r="J146" s="34"/>
+      <c r="J146" s="56"/>
       <c r="K146" s="34"/>
       <c r="L146" s="31"/>
       <c r="M146" s="31"/>
@@ -9372,7 +9933,7 @@
       <c r="G150" s="31"/>
       <c r="H150" s="32"/>
       <c r="I150" s="33"/>
-      <c r="J150" s="56"/>
+      <c r="J150" s="46"/>
       <c r="K150" s="46"/>
       <c r="L150" s="31"/>
       <c r="M150" s="47"/>
@@ -9680,7 +10241,7 @@
       <c r="G164" s="31"/>
       <c r="H164" s="32"/>
       <c r="I164" s="33"/>
-      <c r="J164" s="46"/>
+      <c r="J164" s="34"/>
       <c r="K164" s="37"/>
       <c r="L164" s="31"/>
       <c r="M164" s="47"/>
@@ -9768,7 +10329,7 @@
       <c r="G168" s="31"/>
       <c r="H168" s="32"/>
       <c r="I168" s="33"/>
-      <c r="J168" s="34"/>
+      <c r="J168" s="46"/>
       <c r="K168" s="37"/>
       <c r="L168" s="31"/>
       <c r="M168" s="47"/>
@@ -9922,7 +10483,7 @@
       <c r="G175" s="95"/>
       <c r="H175" s="32"/>
       <c r="I175" s="108"/>
-      <c r="J175" s="46"/>
+      <c r="J175" s="34"/>
       <c r="K175" s="37"/>
       <c r="L175" s="31"/>
       <c r="M175" s="47"/>
@@ -10032,7 +10593,7 @@
       <c r="G180" s="95"/>
       <c r="H180" s="32"/>
       <c r="I180" s="108"/>
-      <c r="J180" s="34"/>
+      <c r="J180" s="49"/>
       <c r="K180" s="37"/>
       <c r="L180" s="31"/>
       <c r="M180" s="47"/>
@@ -10296,7 +10857,7 @@
       <c r="G192" s="95"/>
       <c r="H192" s="54"/>
       <c r="I192" s="52"/>
-      <c r="J192" s="49"/>
+      <c r="J192" s="37"/>
       <c r="K192" s="37"/>
       <c r="L192" s="47"/>
       <c r="M192" s="47"/>
@@ -10428,7 +10989,7 @@
       <c r="G198" s="95"/>
       <c r="H198" s="45"/>
       <c r="I198" s="52"/>
-      <c r="J198" s="37"/>
+      <c r="J198" s="34"/>
       <c r="K198" s="37"/>
       <c r="L198" s="47"/>
       <c r="M198" s="39"/>
@@ -10494,7 +11055,7 @@
       <c r="G201" s="31"/>
       <c r="H201" s="54"/>
       <c r="I201" s="52"/>
-      <c r="J201" s="34"/>
+      <c r="J201" s="56"/>
       <c r="K201" s="34"/>
       <c r="L201" s="39"/>
       <c r="M201" s="39"/>
@@ -10758,7 +11319,7 @@
       <c r="G213" s="31"/>
       <c r="H213" s="54"/>
       <c r="I213" s="52"/>
-      <c r="J213" s="56"/>
+      <c r="J213" s="86"/>
       <c r="K213" s="37"/>
       <c r="L213" s="39"/>
       <c r="M213" s="39"/>
@@ -10890,7 +11451,7 @@
       <c r="G219" s="31"/>
       <c r="H219" s="54"/>
       <c r="I219" s="52"/>
-      <c r="J219" s="86"/>
+      <c r="J219" s="42"/>
       <c r="K219" s="37"/>
       <c r="L219" s="39"/>
       <c r="M219" s="39"/>
@@ -11154,7 +11715,7 @@
       <c r="G231" s="31"/>
       <c r="H231" s="54"/>
       <c r="I231" s="52"/>
-      <c r="J231" s="42"/>
+      <c r="J231" s="34"/>
       <c r="K231" s="37"/>
       <c r="L231" s="39"/>
       <c r="M231" s="39"/>
@@ -11330,7 +11891,7 @@
       <c r="G239" s="31"/>
       <c r="H239" s="54"/>
       <c r="I239" s="52"/>
-      <c r="J239" s="34"/>
+      <c r="J239" s="39"/>
       <c r="K239" s="37"/>
       <c r="L239" s="39"/>
       <c r="M239" s="39"/>
@@ -11858,7 +12419,7 @@
       <c r="G263" s="31"/>
       <c r="H263" s="54"/>
       <c r="I263" s="52"/>
-      <c r="J263" s="39"/>
+      <c r="J263" s="112"/>
       <c r="K263" s="37"/>
       <c r="L263" s="39"/>
       <c r="M263" s="39"/>
@@ -11946,7 +12507,7 @@
       <c r="G267" s="31"/>
       <c r="H267" s="54"/>
       <c r="I267" s="52"/>
-      <c r="J267" s="112"/>
+      <c r="J267" s="34"/>
       <c r="K267" s="37"/>
       <c r="L267" s="39"/>
       <c r="M267" s="39"/>
@@ -11990,7 +12551,7 @@
       <c r="G269" s="31"/>
       <c r="H269" s="54"/>
       <c r="I269" s="52"/>
-      <c r="J269" s="34"/>
+      <c r="J269" s="49"/>
       <c r="K269" s="37"/>
       <c r="L269" s="39"/>
       <c r="M269" s="39"/>
@@ -12166,7 +12727,7 @@
       <c r="G277" s="31"/>
       <c r="H277" s="54"/>
       <c r="I277" s="52"/>
-      <c r="J277" s="49"/>
+      <c r="J277" s="42"/>
       <c r="K277" s="42"/>
       <c r="L277" s="55"/>
       <c r="M277" s="55"/>
@@ -12254,7 +12815,7 @@
       <c r="G281" s="31"/>
       <c r="H281" s="54"/>
       <c r="I281" s="52"/>
-      <c r="J281" s="42"/>
+      <c r="J281" s="56"/>
       <c r="K281" s="42"/>
       <c r="L281" s="55"/>
       <c r="M281" s="55"/>
@@ -12408,7 +12969,7 @@
       <c r="G288" s="31"/>
       <c r="H288" s="55"/>
       <c r="I288" s="52"/>
-      <c r="J288" s="56"/>
+      <c r="J288" s="49"/>
       <c r="K288" s="42"/>
       <c r="L288" s="55"/>
       <c r="M288" s="55"/>
@@ -12430,7 +12991,7 @@
       <c r="G289" s="31"/>
       <c r="H289" s="55"/>
       <c r="I289" s="52"/>
-      <c r="J289" s="49"/>
+      <c r="J289" s="42"/>
       <c r="K289" s="42"/>
       <c r="L289" s="55"/>
       <c r="M289" s="55"/>
@@ -12628,7 +13189,7 @@
       <c r="G298" s="31"/>
       <c r="H298" s="55"/>
       <c r="I298" s="37"/>
-      <c r="J298" s="42"/>
+      <c r="J298" s="56"/>
       <c r="K298" s="42"/>
       <c r="L298" s="55"/>
       <c r="M298" s="55"/>
@@ -12848,7 +13409,7 @@
       <c r="G308" s="31"/>
       <c r="H308" s="55"/>
       <c r="I308" s="37"/>
-      <c r="J308" s="56"/>
+      <c r="J308" s="42"/>
       <c r="K308" s="42"/>
       <c r="L308" s="55"/>
       <c r="M308" s="55"/>
@@ -12958,7 +13519,7 @@
       <c r="G313" s="31"/>
       <c r="H313" s="55"/>
       <c r="I313" s="37"/>
-      <c r="J313" s="42"/>
+      <c r="J313" s="34"/>
       <c r="K313" s="42"/>
       <c r="L313" s="55"/>
       <c r="M313" s="55"/>
@@ -13068,7 +13629,7 @@
       <c r="G318" s="31"/>
       <c r="H318" s="55"/>
       <c r="I318" s="37"/>
-      <c r="J318" s="34"/>
+      <c r="J318" s="42"/>
       <c r="K318" s="34"/>
       <c r="L318" s="55"/>
       <c r="M318" s="55"/>
@@ -13178,7 +13739,7 @@
       <c r="G323" s="31"/>
       <c r="H323" s="42"/>
       <c r="I323" s="42"/>
-      <c r="J323" s="42"/>
+      <c r="J323" s="56"/>
       <c r="K323" s="46"/>
       <c r="L323" s="55"/>
       <c r="M323" s="55"/>
@@ -13288,7 +13849,7 @@
       <c r="G328" s="31"/>
       <c r="H328" s="42"/>
       <c r="I328" s="42"/>
-      <c r="J328" s="56"/>
+      <c r="J328" s="42"/>
       <c r="K328" s="46"/>
       <c r="L328" s="55"/>
       <c r="M328" s="55"/>
@@ -13508,7 +14069,7 @@
       <c r="G338" s="31"/>
       <c r="H338" s="42"/>
       <c r="I338" s="42"/>
-      <c r="J338" s="42"/>
+      <c r="J338" s="46"/>
       <c r="K338" s="46"/>
       <c r="L338" s="55"/>
       <c r="M338" s="55"/>
@@ -13970,7 +14531,7 @@
       <c r="G359" s="31"/>
       <c r="H359" s="42"/>
       <c r="I359" s="42"/>
-      <c r="J359" s="46"/>
+      <c r="J359" s="42"/>
       <c r="K359" s="42"/>
       <c r="L359" s="55"/>
       <c r="M359" s="55"/>
@@ -14432,7 +14993,7 @@
       <c r="G380" s="31"/>
       <c r="H380" s="42"/>
       <c r="I380" s="42"/>
-      <c r="J380" s="42"/>
+      <c r="J380" s="46"/>
       <c r="K380" s="42"/>
       <c r="L380" s="55"/>
       <c r="M380" s="55"/>
@@ -14872,7 +15433,7 @@
       <c r="G400" s="31"/>
       <c r="H400" s="42"/>
       <c r="I400" s="55"/>
-      <c r="J400" s="46"/>
+      <c r="J400" s="56"/>
       <c r="K400" s="56"/>
       <c r="L400" s="55"/>
       <c r="M400" s="55"/>
@@ -14960,7 +15521,7 @@
       <c r="G404" s="55"/>
       <c r="H404" s="55"/>
       <c r="I404" s="42"/>
-      <c r="J404" s="56"/>
+      <c r="J404" s="42"/>
       <c r="K404" s="56"/>
       <c r="L404" s="55"/>
       <c r="M404" s="55"/>
@@ -15136,7 +15697,7 @@
       <c r="G412" s="93"/>
       <c r="H412" s="93"/>
       <c r="I412" s="93"/>
-      <c r="J412" s="42"/>
+      <c r="J412" s="56"/>
       <c r="K412" s="42"/>
       <c r="L412" s="55"/>
       <c r="M412" s="55"/>
@@ -15422,7 +15983,7 @@
       <c r="G425" s="93"/>
       <c r="H425" s="93"/>
       <c r="I425" s="93"/>
-      <c r="J425" s="56"/>
+      <c r="J425" s="42"/>
       <c r="K425" s="42"/>
       <c r="L425" s="55"/>
       <c r="M425" s="55"/>
@@ -15510,7 +16071,7 @@
       <c r="G429" s="55"/>
       <c r="H429" s="42"/>
       <c r="I429" s="42"/>
-      <c r="J429" s="42"/>
+      <c r="J429" s="56"/>
       <c r="K429" s="42"/>
       <c r="L429" s="55"/>
       <c r="M429" s="55"/>
@@ -15532,7 +16093,7 @@
       <c r="G430" s="55"/>
       <c r="H430" s="42"/>
       <c r="I430" s="42"/>
-      <c r="J430" s="56"/>
+      <c r="J430" s="42"/>
       <c r="K430" s="42"/>
       <c r="L430" s="55"/>
       <c r="M430" s="55"/>
@@ -18325,7 +18886,7 @@
       <c r="G557" s="95"/>
       <c r="H557" s="93"/>
       <c r="I557" s="93"/>
-      <c r="J557" s="42"/>
+      <c r="J557" s="86"/>
       <c r="K557" s="42"/>
       <c r="L557" s="55"/>
       <c r="M557" s="55"/>
@@ -18457,7 +19018,7 @@
       <c r="G563" s="95"/>
       <c r="H563" s="42"/>
       <c r="I563" s="42"/>
-      <c r="J563" s="86"/>
+      <c r="J563" s="42"/>
       <c r="K563" s="86"/>
       <c r="L563" s="55"/>
       <c r="M563" s="55"/>
@@ -19139,7 +19700,7 @@
       <c r="G594" s="42"/>
       <c r="H594" s="42"/>
       <c r="I594" s="42"/>
-      <c r="J594" s="42"/>
+      <c r="J594" s="86"/>
       <c r="K594" s="42"/>
       <c r="L594" s="42"/>
       <c r="M594" s="55"/>
@@ -19249,7 +19810,7 @@
       <c r="G599" s="55"/>
       <c r="H599" s="42"/>
       <c r="I599" s="42"/>
-      <c r="J599" s="86"/>
+      <c r="J599" s="56"/>
       <c r="K599" s="86"/>
       <c r="L599" s="55"/>
       <c r="M599" s="55"/>
@@ -19293,7 +19854,7 @@
       <c r="G601" s="55"/>
       <c r="H601" s="55"/>
       <c r="I601" s="42"/>
-      <c r="J601" s="56"/>
+      <c r="J601" s="42"/>
       <c r="K601" s="56"/>
       <c r="L601" s="55"/>
       <c r="M601" s="55"/>
@@ -19381,7 +19942,7 @@
       <c r="G605" s="42"/>
       <c r="H605" s="42"/>
       <c r="I605" s="42"/>
-      <c r="J605" s="42"/>
+      <c r="J605" s="86"/>
       <c r="K605" s="42"/>
       <c r="L605" s="42"/>
       <c r="M605" s="42"/>
@@ -19535,7 +20096,7 @@
       <c r="G612" s="55"/>
       <c r="H612" s="42"/>
       <c r="I612" s="42"/>
-      <c r="J612" s="86"/>
+      <c r="J612" s="42"/>
       <c r="K612" s="42"/>
       <c r="L612" s="55"/>
       <c r="M612" s="55"/>
@@ -19645,7 +20206,7 @@
       <c r="G617" s="55"/>
       <c r="H617" s="42"/>
       <c r="I617" s="42"/>
-      <c r="J617" s="42"/>
+      <c r="J617" s="56"/>
       <c r="K617" s="42"/>
       <c r="L617" s="55"/>
       <c r="M617" s="55"/>
@@ -19975,7 +20536,7 @@
       <c r="G632" s="93"/>
       <c r="H632" s="42"/>
       <c r="I632" s="42"/>
-      <c r="J632" s="56"/>
+      <c r="J632" s="42"/>
       <c r="K632" s="42"/>
       <c r="L632" s="55"/>
       <c r="M632" s="55"/>
@@ -20107,7 +20668,7 @@
       <c r="G638" s="93"/>
       <c r="H638" s="42"/>
       <c r="I638" s="42"/>
-      <c r="J638" s="42"/>
+      <c r="J638" s="86"/>
       <c r="K638" s="42"/>
       <c r="L638" s="55"/>
       <c r="M638" s="55"/>
@@ -20195,7 +20756,7 @@
       <c r="G642" s="55"/>
       <c r="H642" s="42"/>
       <c r="I642" s="42"/>
-      <c r="J642" s="86"/>
+      <c r="J642" s="42"/>
       <c r="K642" s="86"/>
       <c r="L642" s="55"/>
       <c r="M642" s="55"/>
@@ -20283,7 +20844,7 @@
       <c r="G646" s="55"/>
       <c r="H646" s="42"/>
       <c r="I646" s="42"/>
-      <c r="J646" s="42"/>
+      <c r="J646" s="86"/>
       <c r="K646" s="42"/>
       <c r="L646" s="55"/>
       <c r="M646" s="42"/>
@@ -20371,7 +20932,7 @@
       <c r="G650" s="55"/>
       <c r="H650" s="55"/>
       <c r="I650" s="42"/>
-      <c r="J650" s="86"/>
+      <c r="J650" s="56"/>
       <c r="K650" s="86"/>
       <c r="L650" s="55"/>
       <c r="M650" s="55"/>
@@ -20415,7 +20976,7 @@
       <c r="G652" s="55"/>
       <c r="H652" s="55"/>
       <c r="I652" s="42"/>
-      <c r="J652" s="56"/>
+      <c r="J652" s="86"/>
       <c r="K652" s="42"/>
       <c r="L652" s="42"/>
       <c r="M652" s="42"/>
@@ -20503,7 +21064,7 @@
       <c r="G656" s="55"/>
       <c r="H656" s="55"/>
       <c r="I656" s="42"/>
-      <c r="J656" s="86"/>
+      <c r="J656" s="56"/>
       <c r="K656" s="86"/>
       <c r="L656" s="55"/>
       <c r="M656" s="55"/>
@@ -20833,7 +21394,7 @@
       <c r="G671" s="55"/>
       <c r="H671" s="55"/>
       <c r="I671" s="42"/>
-      <c r="J671" s="56"/>
+      <c r="J671" s="86"/>
       <c r="K671" s="42"/>
       <c r="L671" s="55"/>
       <c r="M671" s="55"/>
@@ -20965,7 +21526,7 @@
       <c r="G677" s="55"/>
       <c r="H677" s="42"/>
       <c r="I677" s="42"/>
-      <c r="J677" s="86"/>
+      <c r="J677" s="56"/>
       <c r="K677" s="42"/>
       <c r="L677" s="55"/>
       <c r="M677" s="55"/>
@@ -21009,7 +21570,7 @@
       <c r="G679" s="55"/>
       <c r="H679" s="42"/>
       <c r="I679" s="42"/>
-      <c r="J679" s="56"/>
+      <c r="J679" s="86"/>
       <c r="K679" s="42"/>
       <c r="L679" s="55"/>
       <c r="M679" s="42"/>
@@ -21053,7 +21614,7 @@
       <c r="G681" s="55"/>
       <c r="H681" s="42"/>
       <c r="I681" s="42"/>
-      <c r="J681" s="86"/>
+      <c r="J681" s="56"/>
       <c r="K681" s="86"/>
       <c r="L681" s="55"/>
       <c r="M681" s="55"/>
@@ -21141,7 +21702,7 @@
       <c r="G685" s="55"/>
       <c r="H685" s="42"/>
       <c r="I685" s="42"/>
-      <c r="J685" s="56"/>
+      <c r="J685" s="42"/>
       <c r="K685" s="56"/>
       <c r="L685" s="55"/>
       <c r="M685" s="55"/>
@@ -26831,7 +27392,6 @@
       <c r="G944" s="42"/>
       <c r="H944" s="42"/>
       <c r="I944" s="42"/>
-      <c r="J944" s="42"/>
       <c r="K944" s="42"/>
       <c r="L944" s="42"/>
       <c r="M944" s="42"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.ijrmhm.2026.107918`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5BB2AB-AD9B-3C4C-AF41-7C162BDCFCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0563E99-876F-864E-86F1-9BF767CC4561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="186">
   <si>
     <r>
       <rPr>
@@ -673,6 +673,21 @@
   </si>
   <si>
     <t>10.1080/10667857.2026.2674815</t>
+  </si>
+  <si>
+    <t>10.1016/j.ijrmhm.2026.107918</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>MA+DED</t>
+  </si>
+  <si>
+    <t>Al39 Mo10 (Nb0.333 Ta0.333 Ti0.333)51</t>
+  </si>
+  <si>
+    <t>ball milled for 12h and laser DED with 2mm diameter spot and 500W power; some minor possible sigma observed but not XRD-detected; the compressive nature of the test not stated in text but inferred from the sample geometry</t>
   </si>
 </sst>
 </file>
@@ -8744,11 +8759,11 @@
         <v>298</v>
       </c>
       <c r="J121" s="86">
-        <f t="shared" ref="J121:K126" si="3">P121*9807000</f>
+        <f>P121*9807000</f>
         <v>5285973000</v>
       </c>
       <c r="K121" s="86">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="J121:K126" si="3">Q121*9807000</f>
         <v>117684000</v>
       </c>
       <c r="L121" s="31" t="s">
@@ -9771,19 +9786,41 @@
     </row>
     <row r="143" spans="1:20" ht="18" customHeight="1">
       <c r="A143" s="48"/>
-      <c r="B143" s="30"/>
-      <c r="C143" s="88"/>
-      <c r="D143" s="29"/>
-      <c r="E143" s="30"/>
-      <c r="F143" s="31"/>
-      <c r="G143" s="31"/>
+      <c r="B143" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="C143" s="88" t="s">
+        <v>63</v>
+      </c>
+      <c r="D143" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="E143" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="F143" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G143" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H143" s="32"/>
-      <c r="I143" s="33"/>
-      <c r="J143" s="34"/>
+      <c r="I143" s="108">
+        <v>298</v>
+      </c>
+      <c r="J143" s="34">
+        <v>1452000000</v>
+      </c>
       <c r="K143" s="34"/>
-      <c r="L143" s="31"/>
-      <c r="M143" s="31"/>
-      <c r="N143" s="35"/>
+      <c r="L143" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M143" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="N143" s="35" t="s">
+        <v>181</v>
+      </c>
       <c r="O143" s="36"/>
       <c r="P143" s="37"/>
       <c r="Q143" s="37"/>
@@ -9793,19 +9830,41 @@
     </row>
     <row r="144" spans="1:20" ht="18" customHeight="1">
       <c r="A144" s="48"/>
-      <c r="B144" s="30"/>
-      <c r="C144" s="88"/>
-      <c r="D144" s="29"/>
-      <c r="E144" s="30"/>
-      <c r="F144" s="31"/>
-      <c r="G144" s="31"/>
+      <c r="B144" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="C144" s="88" t="s">
+        <v>63</v>
+      </c>
+      <c r="D144" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="E144" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="F144" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="G144" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H144" s="32"/>
-      <c r="I144" s="33"/>
-      <c r="J144" s="34"/>
+      <c r="I144" s="108">
+        <v>298</v>
+      </c>
+      <c r="J144" s="34">
+        <v>7.8</v>
+      </c>
       <c r="K144" s="34"/>
-      <c r="L144" s="31"/>
-      <c r="M144" s="31"/>
-      <c r="N144" s="35"/>
+      <c r="L144" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M144" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="N144" s="35" t="s">
+        <v>181</v>
+      </c>
       <c r="O144" s="36"/>
       <c r="P144" s="37"/>
       <c r="Q144" s="37"/>
@@ -9815,19 +9874,42 @@
     </row>
     <row r="145" spans="1:20" ht="18" customHeight="1">
       <c r="A145" s="48"/>
-      <c r="B145" s="30"/>
-      <c r="C145" s="88"/>
-      <c r="D145" s="29"/>
-      <c r="E145" s="30"/>
-      <c r="F145" s="31"/>
-      <c r="G145" s="31"/>
+      <c r="B145" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="C145" s="88" t="s">
+        <v>63</v>
+      </c>
+      <c r="D145" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="E145" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="F145" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="G145" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H145" s="32"/>
-      <c r="I145" s="33"/>
-      <c r="J145" s="34"/>
+      <c r="I145" s="108">
+        <v>298</v>
+      </c>
+      <c r="J145" s="34">
+        <f>656.16*9807000</f>
+        <v>6434961120</v>
+      </c>
       <c r="K145" s="34"/>
-      <c r="L145" s="31"/>
-      <c r="M145" s="31"/>
-      <c r="N145" s="35"/>
+      <c r="L145" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M145" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="N145" s="35" t="s">
+        <v>181</v>
+      </c>
       <c r="O145" s="36"/>
       <c r="P145" s="37"/>
       <c r="Q145" s="37"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.ijrmhm.2026.107917`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0563E99-876F-864E-86F1-9BF767CC4561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02C1B91-0FC0-9F4C-B151-550639987956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="8500" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="280" yWindow="8180" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="190">
   <si>
     <r>
       <rPr>
@@ -688,6 +688,18 @@
   </si>
   <si>
     <t>ball milled for 12h and laser DED with 2mm diameter spot and 500W power; some minor possible sigma observed but not XRD-detected; the compressive nature of the test not stated in text but inferred from the sample geometry</t>
+  </si>
+  <si>
+    <t>10.1016/j.ijrmhm.2026.107917</t>
+  </si>
+  <si>
+    <t>Ti30V20Al30Nb10Ta10</t>
+  </si>
+  <si>
+    <t>elastic modulus</t>
+  </si>
+  <si>
+    <t>F8</t>
   </si>
 </sst>
 </file>
@@ -9919,19 +9931,41 @@
     </row>
     <row r="146" spans="1:20" ht="18" customHeight="1">
       <c r="A146" s="48"/>
-      <c r="B146" s="30"/>
-      <c r="C146" s="29"/>
-      <c r="D146" s="29"/>
+      <c r="B146" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C146" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D146" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E146" s="30"/>
-      <c r="F146" s="31"/>
-      <c r="G146" s="31"/>
+      <c r="F146" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G146" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H146" s="32"/>
-      <c r="I146" s="33"/>
-      <c r="J146" s="56"/>
-      <c r="K146" s="34"/>
-      <c r="L146" s="31"/>
-      <c r="M146" s="31"/>
-      <c r="N146" s="35"/>
+      <c r="I146" s="108">
+        <v>298</v>
+      </c>
+      <c r="J146" s="56">
+        <v>1610000000</v>
+      </c>
+      <c r="K146" s="34">
+        <v>20000000</v>
+      </c>
+      <c r="L146" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M146" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="N146" s="35" t="s">
+        <v>186</v>
+      </c>
       <c r="O146" s="36"/>
       <c r="P146" s="37"/>
       <c r="Q146" s="37"/>
@@ -9941,19 +9975,43 @@
     </row>
     <row r="147" spans="1:20" ht="18" customHeight="1">
       <c r="A147" s="48"/>
-      <c r="B147" s="30"/>
-      <c r="C147" s="88"/>
-      <c r="D147" s="29"/>
+      <c r="B147" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C147" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D147" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E147" s="30"/>
-      <c r="F147" s="50"/>
-      <c r="G147" s="31"/>
+      <c r="F147" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="G147" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H147" s="32"/>
-      <c r="I147" s="33"/>
-      <c r="J147" s="56"/>
-      <c r="K147" s="49"/>
-      <c r="L147" s="31"/>
-      <c r="M147" s="31"/>
-      <c r="N147" s="29"/>
+      <c r="I147" s="108">
+        <v>298</v>
+      </c>
+      <c r="J147" s="56">
+        <f>((1831+1745)*1000000)/2</f>
+        <v>1788000000</v>
+      </c>
+      <c r="K147" s="56">
+        <f>((1831-1745)*1000000)/2</f>
+        <v>43000000</v>
+      </c>
+      <c r="L147" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M147" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="N147" s="35" t="s">
+        <v>186</v>
+      </c>
       <c r="O147" s="36"/>
       <c r="P147" s="37"/>
       <c r="Q147" s="37"/>
@@ -9963,19 +10021,43 @@
     </row>
     <row r="148" spans="1:20" ht="18" customHeight="1">
       <c r="A148" s="48"/>
-      <c r="B148" s="30"/>
-      <c r="C148" s="29"/>
-      <c r="D148" s="29"/>
+      <c r="B148" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C148" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D148" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E148" s="30"/>
-      <c r="F148" s="50"/>
-      <c r="G148" s="31"/>
+      <c r="F148" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="G148" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H148" s="32"/>
-      <c r="I148" s="33"/>
-      <c r="J148" s="56"/>
-      <c r="K148" s="49"/>
-      <c r="L148" s="31"/>
-      <c r="M148" s="47"/>
-      <c r="N148" s="29"/>
+      <c r="I148" s="108">
+        <v>298</v>
+      </c>
+      <c r="J148" s="56">
+        <f>(15.5+18)/2</f>
+        <v>16.75</v>
+      </c>
+      <c r="K148" s="56">
+        <f>(18-15.5)/2</f>
+        <v>1.25</v>
+      </c>
+      <c r="L148" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M148" s="47" t="s">
+        <v>189</v>
+      </c>
+      <c r="N148" s="35" t="s">
+        <v>186</v>
+      </c>
       <c r="O148" s="36"/>
       <c r="P148" s="37"/>
       <c r="Q148" s="37"/>
@@ -9985,19 +10067,39 @@
     </row>
     <row r="149" spans="1:20" ht="18" customHeight="1">
       <c r="A149" s="48"/>
-      <c r="B149" s="30"/>
-      <c r="C149" s="29"/>
-      <c r="D149" s="29"/>
+      <c r="B149" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C149" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D149" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E149" s="30"/>
-      <c r="F149" s="50"/>
-      <c r="G149" s="31"/>
+      <c r="F149" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="G149" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H149" s="32"/>
-      <c r="I149" s="33"/>
-      <c r="J149" s="56"/>
+      <c r="I149" s="108">
+        <v>298</v>
+      </c>
+      <c r="J149" s="56">
+        <v>145000000000</v>
+      </c>
       <c r="K149" s="46"/>
-      <c r="L149" s="31"/>
-      <c r="M149" s="47"/>
-      <c r="N149" s="29"/>
+      <c r="L149" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M149" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N149" s="35" t="s">
+        <v>186</v>
+      </c>
       <c r="O149" s="36"/>
       <c r="P149" s="37"/>
       <c r="Q149" s="37"/>
@@ -10007,19 +10109,43 @@
     </row>
     <row r="150" spans="1:20" ht="18" customHeight="1">
       <c r="A150" s="48"/>
-      <c r="B150" s="30"/>
-      <c r="C150" s="29"/>
-      <c r="D150" s="29"/>
+      <c r="B150" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="C150" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D150" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E150" s="30"/>
-      <c r="F150" s="50"/>
-      <c r="G150" s="31"/>
+      <c r="F150" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="G150" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H150" s="32"/>
-      <c r="I150" s="33"/>
-      <c r="J150" s="46"/>
-      <c r="K150" s="46"/>
-      <c r="L150" s="31"/>
-      <c r="M150" s="47"/>
-      <c r="N150" s="29"/>
+      <c r="I150" s="108">
+        <v>298</v>
+      </c>
+      <c r="J150" s="46">
+        <f>520*9807000</f>
+        <v>5099640000</v>
+      </c>
+      <c r="K150" s="46">
+        <f>14*9807000</f>
+        <v>137298000</v>
+      </c>
+      <c r="L150" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M150" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N150" s="35" t="s">
+        <v>186</v>
+      </c>
       <c r="O150" s="36"/>
       <c r="P150" s="37"/>
       <c r="Q150" s="37"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.ijrmhm.2025.107571`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02C1B91-0FC0-9F4C-B151-550639987956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F20A4DC-4606-FD47-8429-B646DD615893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="8180" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="8180" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="197">
   <si>
     <r>
       <rPr>
@@ -700,6 +700,27 @@
   </si>
   <si>
     <t>F8</t>
+  </si>
+  <si>
+    <t>Mo Ti Zr Cr0.5 Nb</t>
+  </si>
+  <si>
+    <t>BCC+C15</t>
+  </si>
+  <si>
+    <t>VAM+BM+SPS</t>
+  </si>
+  <si>
+    <t>high energy ball milling with 304 SS balls at 350rpm for 70h and SPS at 1773K under 30MPa for 10min</t>
+  </si>
+  <si>
+    <t>S2.3</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>10.1016/j.ijrmhm.2025.107571</t>
   </si>
 </sst>
 </file>
@@ -10155,19 +10176,41 @@
     </row>
     <row r="151" spans="1:20" ht="18" customHeight="1">
       <c r="A151" s="48"/>
-      <c r="B151" s="30"/>
-      <c r="C151" s="29"/>
-      <c r="D151" s="29"/>
+      <c r="B151" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C151" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D151" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E151" s="30"/>
-      <c r="F151" s="50"/>
-      <c r="G151" s="31"/>
+      <c r="F151" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="G151" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H151" s="32"/>
-      <c r="I151" s="33"/>
-      <c r="J151" s="46"/>
-      <c r="K151" s="46"/>
-      <c r="L151" s="31"/>
-      <c r="M151" s="47"/>
-      <c r="N151" s="29"/>
+      <c r="I151" s="108">
+        <v>298</v>
+      </c>
+      <c r="J151" s="46">
+        <v>7410</v>
+      </c>
+      <c r="K151" s="46">
+        <v>57</v>
+      </c>
+      <c r="L151" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="M151" s="47" t="s">
+        <v>194</v>
+      </c>
+      <c r="N151" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O151" s="36"/>
       <c r="P151" s="37"/>
       <c r="Q151" s="37"/>
@@ -10177,19 +10220,43 @@
     </row>
     <row r="152" spans="1:20" ht="18" customHeight="1">
       <c r="A152" s="48"/>
-      <c r="B152" s="30"/>
-      <c r="C152" s="29"/>
-      <c r="D152" s="29"/>
-      <c r="E152" s="30"/>
-      <c r="F152" s="50"/>
-      <c r="G152" s="31"/>
+      <c r="B152" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C152" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D152" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E152" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F152" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="G152" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H152" s="32"/>
-      <c r="I152" s="33"/>
-      <c r="J152" s="46"/>
-      <c r="K152" s="46"/>
-      <c r="L152" s="31"/>
-      <c r="M152" s="47"/>
-      <c r="N152" s="29"/>
+      <c r="I152" s="108">
+        <v>298</v>
+      </c>
+      <c r="J152" s="46">
+        <v>7100</v>
+      </c>
+      <c r="K152" s="46">
+        <v>82</v>
+      </c>
+      <c r="L152" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="M152" s="47" t="s">
+        <v>194</v>
+      </c>
+      <c r="N152" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O152" s="36"/>
       <c r="P152" s="37"/>
       <c r="Q152" s="37"/>
@@ -10199,21 +10266,44 @@
     </row>
     <row r="153" spans="1:20" ht="18" customHeight="1">
       <c r="A153" s="48"/>
-      <c r="B153" s="30"/>
-      <c r="C153" s="29"/>
-      <c r="D153" s="29"/>
+      <c r="B153" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C153" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D153" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E153" s="30"/>
-      <c r="F153" s="50"/>
-      <c r="G153" s="31"/>
+      <c r="F153" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="G153" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H153" s="32"/>
-      <c r="I153" s="33"/>
-      <c r="J153" s="46"/>
+      <c r="I153" s="108">
+        <v>298</v>
+      </c>
+      <c r="J153" s="86">
+        <f t="shared" ref="J153:J154" si="4">P153*9807000</f>
+        <v>5623529940</v>
+      </c>
       <c r="K153" s="46"/>
-      <c r="L153" s="31"/>
-      <c r="M153" s="47"/>
-      <c r="N153" s="29"/>
+      <c r="L153" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M153" s="47" t="s">
+        <v>195</v>
+      </c>
+      <c r="N153" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O153" s="36"/>
-      <c r="P153" s="38"/>
+      <c r="P153" s="38">
+        <v>573.41999999999996</v>
+      </c>
       <c r="Q153" s="37"/>
       <c r="R153" s="36"/>
       <c r="S153" s="36"/>
@@ -10221,21 +10311,46 @@
     </row>
     <row r="154" spans="1:20" ht="18" customHeight="1">
       <c r="A154" s="48"/>
-      <c r="B154" s="30"/>
-      <c r="C154" s="29"/>
-      <c r="D154" s="29"/>
-      <c r="E154" s="30"/>
-      <c r="F154" s="50"/>
-      <c r="G154" s="31"/>
+      <c r="B154" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C154" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D154" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E154" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F154" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="G154" s="95" t="s">
+        <v>28</v>
+      </c>
       <c r="H154" s="32"/>
-      <c r="I154" s="33"/>
-      <c r="J154" s="46"/>
+      <c r="I154" s="108">
+        <v>298</v>
+      </c>
+      <c r="J154" s="86">
+        <f t="shared" si="4"/>
+        <v>15891753150</v>
+      </c>
       <c r="K154" s="46"/>
-      <c r="L154" s="31"/>
-      <c r="M154" s="47"/>
-      <c r="N154" s="29"/>
+      <c r="L154" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M154" s="47" t="s">
+        <v>195</v>
+      </c>
+      <c r="N154" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O154" s="36"/>
-      <c r="P154" s="44"/>
+      <c r="P154" s="44">
+        <v>1620.45</v>
+      </c>
       <c r="Q154" s="37"/>
       <c r="R154" s="36"/>
       <c r="S154" s="36"/>
@@ -10243,19 +10358,41 @@
     </row>
     <row r="155" spans="1:20" ht="18" customHeight="1">
       <c r="A155" s="48"/>
-      <c r="B155" s="30"/>
-      <c r="C155" s="29"/>
-      <c r="D155" s="29"/>
+      <c r="B155" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C155" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D155" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E155" s="30"/>
-      <c r="F155" s="50"/>
-      <c r="G155" s="31"/>
-      <c r="H155" s="32"/>
-      <c r="I155" s="33"/>
-      <c r="J155" s="46"/>
+      <c r="F155" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="G155" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H155" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I155" s="108">
+        <v>298</v>
+      </c>
+      <c r="J155" s="46">
+        <v>2310.6</v>
+      </c>
       <c r="K155" s="37"/>
-      <c r="L155" s="31"/>
-      <c r="M155" s="47"/>
-      <c r="N155" s="29"/>
+      <c r="L155" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M155" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N155" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O155" s="36"/>
       <c r="P155" s="44"/>
       <c r="Q155" s="37"/>
@@ -10265,19 +10402,43 @@
     </row>
     <row r="156" spans="1:20" ht="18" customHeight="1">
       <c r="A156" s="48"/>
-      <c r="B156" s="30"/>
-      <c r="C156" s="29"/>
-      <c r="D156" s="29"/>
-      <c r="E156" s="30"/>
-      <c r="F156" s="50"/>
-      <c r="G156" s="31"/>
-      <c r="H156" s="32"/>
-      <c r="I156" s="33"/>
-      <c r="J156" s="46"/>
+      <c r="B156" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C156" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D156" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E156" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F156" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="G156" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H156" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I156" s="108">
+        <v>298</v>
+      </c>
+      <c r="J156" s="46">
+        <v>1918.3</v>
+      </c>
       <c r="K156" s="37"/>
-      <c r="L156" s="31"/>
-      <c r="M156" s="47"/>
-      <c r="N156" s="29"/>
+      <c r="L156" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M156" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N156" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O156" s="36"/>
       <c r="P156" s="44"/>
       <c r="Q156" s="37"/>
@@ -10287,19 +10448,41 @@
     </row>
     <row r="157" spans="1:20" ht="18" customHeight="1">
       <c r="A157" s="48"/>
-      <c r="B157" s="30"/>
-      <c r="C157" s="29"/>
-      <c r="D157" s="29"/>
+      <c r="B157" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C157" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D157" s="29" t="s">
+        <v>108</v>
+      </c>
       <c r="E157" s="30"/>
-      <c r="F157" s="50"/>
-      <c r="G157" s="31"/>
-      <c r="H157" s="32"/>
-      <c r="I157" s="33"/>
-      <c r="J157" s="46"/>
+      <c r="F157" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="G157" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H157" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I157" s="108">
+        <v>298</v>
+      </c>
+      <c r="J157" s="46">
+        <v>17.95</v>
+      </c>
       <c r="K157" s="37"/>
-      <c r="L157" s="31"/>
-      <c r="M157" s="47"/>
-      <c r="N157" s="29"/>
+      <c r="L157" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M157" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N157" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O157" s="36"/>
       <c r="P157" s="44"/>
       <c r="Q157" s="37"/>
@@ -10309,19 +10492,43 @@
     </row>
     <row r="158" spans="1:20" ht="18" customHeight="1">
       <c r="A158" s="48"/>
-      <c r="B158" s="30"/>
-      <c r="C158" s="29"/>
-      <c r="D158" s="29"/>
-      <c r="E158" s="30"/>
-      <c r="F158" s="50"/>
-      <c r="G158" s="31"/>
-      <c r="H158" s="32"/>
-      <c r="I158" s="33"/>
-      <c r="J158" s="46"/>
+      <c r="B158" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C158" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D158" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E158" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F158" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="G158" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H158" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I158" s="108">
+        <v>298</v>
+      </c>
+      <c r="J158" s="46">
+        <v>10.09</v>
+      </c>
       <c r="K158" s="37"/>
-      <c r="L158" s="31"/>
-      <c r="M158" s="47"/>
-      <c r="N158" s="29"/>
+      <c r="L158" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M158" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N158" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O158" s="36"/>
       <c r="P158" s="44"/>
       <c r="Q158" s="37"/>
@@ -10331,19 +10538,41 @@
     </row>
     <row r="159" spans="1:20" ht="18" customHeight="1">
       <c r="A159" s="48"/>
-      <c r="B159" s="99"/>
-      <c r="C159" s="87"/>
-      <c r="D159" s="87"/>
-      <c r="E159" s="100"/>
-      <c r="F159" s="50"/>
-      <c r="G159" s="31"/>
-      <c r="H159" s="32"/>
-      <c r="I159" s="33"/>
-      <c r="J159" s="46"/>
+      <c r="B159" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C159" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D159" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="E159" s="30"/>
+      <c r="F159" s="50" t="s">
+        <v>112</v>
+      </c>
+      <c r="G159" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H159" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I159" s="108">
+        <v>298</v>
+      </c>
+      <c r="J159" s="46">
+        <v>2238</v>
+      </c>
       <c r="K159" s="37"/>
-      <c r="L159" s="31"/>
-      <c r="M159" s="47"/>
-      <c r="N159" s="29"/>
+      <c r="L159" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M159" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N159" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O159" s="36"/>
       <c r="P159" s="44"/>
       <c r="Q159" s="37"/>
@@ -10353,19 +10582,43 @@
     </row>
     <row r="160" spans="1:20" ht="18" customHeight="1">
       <c r="A160" s="48"/>
-      <c r="B160" s="101"/>
-      <c r="C160" s="88"/>
-      <c r="D160" s="88"/>
-      <c r="E160" s="102"/>
-      <c r="F160" s="50"/>
-      <c r="G160" s="31"/>
-      <c r="H160" s="32"/>
-      <c r="I160" s="33"/>
-      <c r="J160" s="46"/>
+      <c r="B160" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="C160" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D160" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="E160" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="F160" s="50" t="s">
+        <v>112</v>
+      </c>
+      <c r="G160" s="95" t="s">
+        <v>28</v>
+      </c>
+      <c r="H160" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="I160" s="108">
+        <v>298</v>
+      </c>
+      <c r="J160" s="46">
+        <v>1918</v>
+      </c>
       <c r="K160" s="49"/>
-      <c r="L160" s="31"/>
-      <c r="M160" s="47"/>
-      <c r="N160" s="29"/>
+      <c r="L160" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M160" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="N160" s="29" t="s">
+        <v>196</v>
+      </c>
       <c r="O160" s="36"/>
       <c r="P160" s="44"/>
       <c r="Q160" s="37"/>

</xml_diff>

<commit_message>
- parsed data from `10.1038/s41524-026-02189-5`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44BBF86E-76CA-944C-8F6E-B80A0D8450A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DEADD6-06B1-7E44-A2D2-5CAE20E7FE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="8180" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="320" yWindow="12140" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1622" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1676" uniqueCount="216">
   <si>
     <r>
       <rPr>
@@ -760,6 +760,24 @@
   </si>
   <si>
     <t>10.1016/j.ijrmhm.2024.106572</t>
+  </si>
+  <si>
+    <t>Ti19 Nb29 Hf25 Mo18 Al2 Ni3</t>
+  </si>
+  <si>
+    <t>Ti Ta Nb Hf Ni0.5</t>
+  </si>
+  <si>
+    <t>Ti Ta Nb Hf Ni0.25</t>
+  </si>
+  <si>
+    <t>designed with ML; phase information scattered around the paper so less reliable</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>10.1038/s41524-026-02189-5</t>
   </si>
 </sst>
 </file>
@@ -1794,7 +1812,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1983,7 +2001,6 @@
     <xf numFmtId="3" fontId="13" fillId="10" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="13" fillId="10" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -3332,19 +3349,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="12"/>
-      <c r="D2" s="118" t="s">
+      <c r="D2" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="119"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="123"/>
-      <c r="H2" s="123"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="125"/>
-      <c r="K2" s="125"/>
-      <c r="L2" s="123"/>
-      <c r="M2" s="123"/>
-      <c r="N2" s="126"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="124"/>
+      <c r="K2" s="124"/>
+      <c r="L2" s="122"/>
+      <c r="M2" s="122"/>
+      <c r="N2" s="125"/>
       <c r="O2" s="13"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -3356,21 +3373,21 @@
       <c r="A3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="110" t="s">
         <v>72</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="120"/>
-      <c r="E3" s="121"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="129"/>
-      <c r="K3" s="129"/>
-      <c r="L3" s="127"/>
-      <c r="M3" s="127"/>
-      <c r="N3" s="130"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="120"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="127"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="128"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="129"/>
       <c r="O3" s="13"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -3411,43 +3428,43 @@
       <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="131" t="s">
+      <c r="C5" s="130" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="133" t="s">
+      <c r="D5" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="133" t="s">
+      <c r="E5" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="133" t="s">
+      <c r="F5" s="132" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="133" t="s">
+      <c r="G5" s="132" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="134" t="s">
+      <c r="H5" s="133" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="133" t="s">
+      <c r="I5" s="132" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="133" t="s">
+      <c r="J5" s="132" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="133" t="s">
+      <c r="K5" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="133" t="s">
+      <c r="L5" s="132" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="133" t="s">
+      <c r="M5" s="132" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="133" t="s">
+      <c r="N5" s="132" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="138" t="s">
+      <c r="O5" s="137" t="s">
         <v>19</v>
       </c>
       <c r="P5" s="24"/>
@@ -3463,19 +3480,19 @@
       <c r="B6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="132"/>
-      <c r="D6" s="132"/>
-      <c r="E6" s="132"/>
-      <c r="F6" s="132"/>
-      <c r="G6" s="132"/>
-      <c r="H6" s="135"/>
-      <c r="I6" s="136"/>
-      <c r="J6" s="137"/>
-      <c r="K6" s="137"/>
-      <c r="L6" s="132"/>
-      <c r="M6" s="132"/>
-      <c r="N6" s="132"/>
-      <c r="O6" s="139"/>
+      <c r="C6" s="131"/>
+      <c r="D6" s="131"/>
+      <c r="E6" s="131"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="131"/>
+      <c r="H6" s="134"/>
+      <c r="I6" s="135"/>
+      <c r="J6" s="136"/>
+      <c r="K6" s="136"/>
+      <c r="L6" s="131"/>
+      <c r="M6" s="131"/>
+      <c r="N6" s="131"/>
+      <c r="O6" s="138"/>
       <c r="P6" s="24"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="9"/>
@@ -3525,7 +3542,7 @@
       <c r="N7" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="O7" s="140"/>
+      <c r="O7" s="139"/>
       <c r="P7" s="61" t="s">
         <v>61</v>
       </c>
@@ -3540,35 +3557,35 @@
     </row>
     <row r="8" spans="1:20" ht="20.25" customHeight="1" thickBot="1">
       <c r="A8" s="56"/>
-      <c r="B8" s="141" t="s">
+      <c r="B8" s="140" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="142"/>
-      <c r="D8" s="142"/>
-      <c r="E8" s="143"/>
-      <c r="F8" s="144" t="s">
+      <c r="C8" s="141"/>
+      <c r="D8" s="141"/>
+      <c r="E8" s="142"/>
+      <c r="F8" s="143" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="145"/>
-      <c r="H8" s="145"/>
-      <c r="I8" s="146"/>
-      <c r="J8" s="147"/>
-      <c r="K8" s="147"/>
-      <c r="L8" s="148"/>
-      <c r="M8" s="149" t="s">
+      <c r="G8" s="144"/>
+      <c r="H8" s="144"/>
+      <c r="I8" s="145"/>
+      <c r="J8" s="146"/>
+      <c r="K8" s="146"/>
+      <c r="L8" s="147"/>
+      <c r="M8" s="148" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="150"/>
+      <c r="N8" s="149"/>
       <c r="O8" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="P8" s="151" t="s">
+      <c r="P8" s="150" t="s">
         <v>41</v>
       </c>
-      <c r="Q8" s="152"/>
-      <c r="R8" s="153"/>
-      <c r="S8" s="153"/>
-      <c r="T8" s="154"/>
+      <c r="Q8" s="151"/>
+      <c r="R8" s="152"/>
+      <c r="S8" s="152"/>
+      <c r="T8" s="153"/>
     </row>
     <row r="9" spans="1:20" ht="21" customHeight="1" thickBot="1">
       <c r="A9" s="57" t="s">
@@ -3940,7 +3957,7 @@
         <v>83</v>
       </c>
       <c r="I16" s="68"/>
-      <c r="J16" s="110">
+      <c r="J16" s="109">
         <v>0.64600000000000002</v>
       </c>
       <c r="K16" s="38"/>
@@ -4212,10 +4229,10 @@
       <c r="I22" s="68">
         <v>298</v>
       </c>
-      <c r="J22" s="110">
+      <c r="J22" s="109">
         <v>1490000000</v>
       </c>
-      <c r="K22" s="110">
+      <c r="K22" s="109">
         <v>15000000</v>
       </c>
       <c r="L22" s="66" t="s">
@@ -5101,7 +5118,7 @@
       <c r="T41" s="35"/>
     </row>
     <row r="42" spans="1:20" ht="18.75" customHeight="1">
-      <c r="A42" s="112" t="s">
+      <c r="A42" s="111" t="s">
         <v>103</v>
       </c>
       <c r="B42" s="98" t="s">
@@ -5147,7 +5164,7 @@
       <c r="T42" s="35"/>
     </row>
     <row r="43" spans="1:20" ht="18" customHeight="1">
-      <c r="A43" s="113" t="s">
+      <c r="A43" s="112" t="s">
         <v>104</v>
       </c>
       <c r="B43" s="100" t="s">
@@ -5195,7 +5212,7 @@
       <c r="T43" s="35"/>
     </row>
     <row r="44" spans="1:20" ht="18" customHeight="1">
-      <c r="A44" s="113" t="s">
+      <c r="A44" s="112" t="s">
         <v>105</v>
       </c>
       <c r="B44" s="100" t="s">
@@ -5241,7 +5258,7 @@
       <c r="T44" s="35"/>
     </row>
     <row r="45" spans="1:20" ht="18" customHeight="1">
-      <c r="A45" s="113" t="s">
+      <c r="A45" s="112" t="s">
         <v>106</v>
       </c>
       <c r="B45" s="100" t="s">
@@ -5287,7 +5304,7 @@
       <c r="T45" s="35"/>
     </row>
     <row r="46" spans="1:20" ht="18" customHeight="1">
-      <c r="A46" s="113" t="s">
+      <c r="A46" s="112" t="s">
         <v>107</v>
       </c>
       <c r="B46" s="100" t="s">
@@ -5358,10 +5375,10 @@
       <c r="I47" s="68">
         <v>298</v>
       </c>
-      <c r="J47" s="114">
+      <c r="J47" s="113">
         <v>1597000000</v>
       </c>
-      <c r="K47" s="115">
+      <c r="K47" s="114">
         <v>18000000</v>
       </c>
       <c r="L47" s="31" t="s">
@@ -5406,10 +5423,10 @@
       <c r="I48" s="68">
         <v>298</v>
       </c>
-      <c r="J48" s="114">
+      <c r="J48" s="113">
         <v>1794000000</v>
       </c>
-      <c r="K48" s="115">
+      <c r="K48" s="114">
         <v>44000000</v>
       </c>
       <c r="L48" s="31" t="s">
@@ -5454,10 +5471,10 @@
       <c r="I49" s="68">
         <v>298</v>
       </c>
-      <c r="J49" s="114">
+      <c r="J49" s="113">
         <v>1764000000</v>
       </c>
-      <c r="K49" s="115">
+      <c r="K49" s="114">
         <v>41000000</v>
       </c>
       <c r="L49" s="31" t="s">
@@ -5505,7 +5522,7 @@
       <c r="J50" s="85">
         <v>2032000000</v>
       </c>
-      <c r="K50" s="115">
+      <c r="K50" s="114">
         <v>17000000</v>
       </c>
       <c r="L50" s="31" t="s">
@@ -5621,7 +5638,7 @@
       <c r="T52" s="35"/>
     </row>
     <row r="53" spans="1:20" ht="18" customHeight="1">
-      <c r="A53" s="112" t="s">
+      <c r="A53" s="111" t="s">
         <v>121</v>
       </c>
       <c r="B53" s="98" t="s">
@@ -5669,7 +5686,7 @@
       <c r="T53" s="35"/>
     </row>
     <row r="54" spans="1:20" ht="18" customHeight="1">
-      <c r="A54" s="113" t="s">
+      <c r="A54" s="112" t="s">
         <v>122</v>
       </c>
       <c r="B54" s="100" t="s">
@@ -5717,7 +5734,7 @@
       <c r="T54" s="35"/>
     </row>
     <row r="55" spans="1:20" ht="18" customHeight="1">
-      <c r="A55" s="113" t="s">
+      <c r="A55" s="112" t="s">
         <v>123</v>
       </c>
       <c r="B55" s="100" t="s">
@@ -7039,7 +7056,7 @@
       <c r="T83" s="35"/>
     </row>
     <row r="84" spans="1:20" ht="18" customHeight="1">
-      <c r="A84" s="112" t="s">
+      <c r="A84" s="111" t="s">
         <v>128</v>
       </c>
       <c r="B84" s="100" t="s">
@@ -7058,8 +7075,8 @@
       <c r="G84" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H84" s="116"/>
-      <c r="I84" s="106">
+      <c r="H84" s="115"/>
+      <c r="I84" s="105">
         <v>298</v>
       </c>
       <c r="J84" s="85">
@@ -7083,7 +7100,7 @@
       <c r="T84" s="35"/>
     </row>
     <row r="85" spans="1:20" ht="18" customHeight="1">
-      <c r="A85" s="113" t="s">
+      <c r="A85" s="112" t="s">
         <v>131</v>
       </c>
       <c r="B85" s="100" t="s">
@@ -7102,8 +7119,8 @@
       <c r="G85" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H85" s="117"/>
-      <c r="I85" s="106">
+      <c r="H85" s="116"/>
+      <c r="I85" s="105">
         <v>298</v>
       </c>
       <c r="J85" s="85">
@@ -7127,7 +7144,7 @@
       <c r="T85" s="35"/>
     </row>
     <row r="86" spans="1:20" ht="18" customHeight="1">
-      <c r="A86" s="113" t="s">
+      <c r="A86" s="112" t="s">
         <v>134</v>
       </c>
       <c r="B86" s="100" t="s">
@@ -7146,8 +7163,8 @@
       <c r="G86" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H86" s="117"/>
-      <c r="I86" s="106">
+      <c r="H86" s="116"/>
+      <c r="I86" s="105">
         <v>298</v>
       </c>
       <c r="J86" s="85">
@@ -7171,7 +7188,7 @@
       <c r="T86" s="35"/>
     </row>
     <row r="87" spans="1:20" ht="18" customHeight="1">
-      <c r="A87" s="113" t="s">
+      <c r="A87" s="112" t="s">
         <v>138</v>
       </c>
       <c r="B87" s="100" t="s">
@@ -7190,8 +7207,8 @@
       <c r="G87" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H87" s="117"/>
-      <c r="I87" s="106">
+      <c r="H87" s="116"/>
+      <c r="I87" s="105">
         <v>298</v>
       </c>
       <c r="J87" s="85">
@@ -7215,7 +7232,7 @@
       <c r="T87" s="35"/>
     </row>
     <row r="88" spans="1:20" ht="18" customHeight="1">
-      <c r="A88" s="113" t="s">
+      <c r="A88" s="112" t="s">
         <v>142</v>
       </c>
       <c r="B88" s="100" t="s">
@@ -7234,8 +7251,8 @@
       <c r="G88" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H88" s="117"/>
-      <c r="I88" s="106">
+      <c r="H88" s="116"/>
+      <c r="I88" s="105">
         <v>298</v>
       </c>
       <c r="J88" s="85">
@@ -7259,7 +7276,7 @@
       <c r="T88" s="35"/>
     </row>
     <row r="89" spans="1:20" ht="18" customHeight="1">
-      <c r="A89" s="113" t="s">
+      <c r="A89" s="112" t="s">
         <v>144</v>
       </c>
       <c r="B89" s="100" t="s">
@@ -7278,8 +7295,8 @@
       <c r="G89" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H89" s="117"/>
-      <c r="I89" s="106">
+      <c r="H89" s="116"/>
+      <c r="I89" s="105">
         <v>298</v>
       </c>
       <c r="J89" s="85">
@@ -7303,7 +7320,7 @@
       <c r="T89" s="35"/>
     </row>
     <row r="90" spans="1:20" ht="18" customHeight="1">
-      <c r="A90" s="113" t="s">
+      <c r="A90" s="112" t="s">
         <v>146</v>
       </c>
       <c r="B90" s="100" t="s">
@@ -7322,8 +7339,8 @@
       <c r="G90" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H90" s="117"/>
-      <c r="I90" s="106">
+      <c r="H90" s="116"/>
+      <c r="I90" s="105">
         <v>298</v>
       </c>
       <c r="J90" s="85">
@@ -7369,7 +7386,7 @@
       <c r="H91" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I91" s="106">
+      <c r="I91" s="105">
         <v>298</v>
       </c>
       <c r="J91" s="85">
@@ -7418,7 +7435,7 @@
       <c r="H92" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I92" s="106">
+      <c r="I92" s="105">
         <v>298</v>
       </c>
       <c r="J92" s="85">
@@ -7467,7 +7484,7 @@
       <c r="H93" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I93" s="106">
+      <c r="I93" s="105">
         <v>298</v>
       </c>
       <c r="J93" s="85">
@@ -7516,7 +7533,7 @@
       <c r="H94" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I94" s="106">
+      <c r="I94" s="105">
         <v>298</v>
       </c>
       <c r="J94" s="85">
@@ -7565,7 +7582,7 @@
       <c r="H95" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I95" s="106">
+      <c r="I95" s="105">
         <v>298</v>
       </c>
       <c r="J95" s="85">
@@ -7614,7 +7631,7 @@
       <c r="H96" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I96" s="106">
+      <c r="I96" s="105">
         <v>298</v>
       </c>
       <c r="J96" s="85">
@@ -7663,7 +7680,7 @@
       <c r="H97" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I97" s="106">
+      <c r="I97" s="105">
         <v>298</v>
       </c>
       <c r="J97" s="85">
@@ -7712,7 +7729,7 @@
       <c r="H98" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I98" s="106">
+      <c r="I98" s="105">
         <v>298</v>
       </c>
       <c r="J98" s="85">
@@ -7761,7 +7778,7 @@
       <c r="H99" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I99" s="106">
+      <c r="I99" s="105">
         <v>298</v>
       </c>
       <c r="J99" s="85">
@@ -7810,7 +7827,7 @@
       <c r="H100" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I100" s="106">
+      <c r="I100" s="105">
         <v>298</v>
       </c>
       <c r="J100" s="85">
@@ -7859,7 +7876,7 @@
       <c r="H101" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I101" s="106">
+      <c r="I101" s="105">
         <v>298</v>
       </c>
       <c r="J101" s="85">
@@ -7908,7 +7925,7 @@
       <c r="H102" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I102" s="106">
+      <c r="I102" s="105">
         <v>298</v>
       </c>
       <c r="J102" s="85">
@@ -7957,7 +7974,7 @@
       <c r="H103" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I103" s="106">
+      <c r="I103" s="105">
         <v>298</v>
       </c>
       <c r="J103" s="85">
@@ -8006,7 +8023,7 @@
       <c r="H104" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I104" s="106">
+      <c r="I104" s="105">
         <v>298</v>
       </c>
       <c r="J104" s="85">
@@ -8055,7 +8072,7 @@
       <c r="H105" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I105" s="106">
+      <c r="I105" s="105">
         <v>298</v>
       </c>
       <c r="J105" s="85">
@@ -8104,7 +8121,7 @@
       <c r="H106" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I106" s="106">
+      <c r="I106" s="105">
         <v>298</v>
       </c>
       <c r="J106" s="85">
@@ -8153,7 +8170,7 @@
       <c r="H107" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I107" s="106">
+      <c r="I107" s="105">
         <v>298</v>
       </c>
       <c r="J107" s="85">
@@ -8202,7 +8219,7 @@
       <c r="H108" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I108" s="106">
+      <c r="I108" s="105">
         <v>298</v>
       </c>
       <c r="J108" s="85">
@@ -8251,7 +8268,7 @@
       <c r="H109" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I109" s="106">
+      <c r="I109" s="105">
         <v>298</v>
       </c>
       <c r="J109" s="85">
@@ -8300,7 +8317,7 @@
       <c r="H110" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I110" s="106">
+      <c r="I110" s="105">
         <v>298</v>
       </c>
       <c r="J110" s="85">
@@ -8349,7 +8366,7 @@
       <c r="H111" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I111" s="106">
+      <c r="I111" s="105">
         <v>298</v>
       </c>
       <c r="J111" s="85">
@@ -8398,7 +8415,7 @@
       <c r="H112" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I112" s="106">
+      <c r="I112" s="105">
         <v>298</v>
       </c>
       <c r="J112" s="85">
@@ -8447,7 +8464,7 @@
       <c r="H113" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I113" s="106">
+      <c r="I113" s="105">
         <v>298</v>
       </c>
       <c r="J113" s="85">
@@ -8496,7 +8513,7 @@
       <c r="H114" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I114" s="106">
+      <c r="I114" s="105">
         <v>298</v>
       </c>
       <c r="J114" s="85">
@@ -8545,7 +8562,7 @@
       <c r="H115" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I115" s="106">
+      <c r="I115" s="105">
         <v>298</v>
       </c>
       <c r="J115" s="85">
@@ -8594,7 +8611,7 @@
       <c r="H116" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I116" s="106">
+      <c r="I116" s="105">
         <v>298</v>
       </c>
       <c r="J116" s="85">
@@ -8643,7 +8660,7 @@
       <c r="H117" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I117" s="106">
+      <c r="I117" s="105">
         <v>298</v>
       </c>
       <c r="J117" s="85">
@@ -8692,7 +8709,7 @@
       <c r="H118" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I118" s="106">
+      <c r="I118" s="105">
         <v>298</v>
       </c>
       <c r="J118" s="85">
@@ -8737,7 +8754,7 @@
         <v>28</v>
       </c>
       <c r="H119" s="32"/>
-      <c r="I119" s="106">
+      <c r="I119" s="105">
         <v>298</v>
       </c>
       <c r="J119" s="85">
@@ -8781,7 +8798,7 @@
         <v>28</v>
       </c>
       <c r="H120" s="32"/>
-      <c r="I120" s="106">
+      <c r="I120" s="105">
         <v>298</v>
       </c>
       <c r="J120" s="85">
@@ -8825,7 +8842,7 @@
         <v>28</v>
       </c>
       <c r="H121" s="32"/>
-      <c r="I121" s="106">
+      <c r="I121" s="105">
         <v>298</v>
       </c>
       <c r="J121" s="85">
@@ -8875,7 +8892,7 @@
         <v>28</v>
       </c>
       <c r="H122" s="32"/>
-      <c r="I122" s="106">
+      <c r="I122" s="105">
         <v>298</v>
       </c>
       <c r="J122" s="85">
@@ -8925,7 +8942,7 @@
         <v>28</v>
       </c>
       <c r="H123" s="32"/>
-      <c r="I123" s="106">
+      <c r="I123" s="105">
         <v>298</v>
       </c>
       <c r="J123" s="85">
@@ -8979,7 +8996,7 @@
         <v>28</v>
       </c>
       <c r="H124" s="32"/>
-      <c r="I124" s="106">
+      <c r="I124" s="105">
         <v>298</v>
       </c>
       <c r="J124" s="85">
@@ -9033,7 +9050,7 @@
         <v>28</v>
       </c>
       <c r="H125" s="32"/>
-      <c r="I125" s="106">
+      <c r="I125" s="105">
         <v>298</v>
       </c>
       <c r="J125" s="85">
@@ -9087,7 +9104,7 @@
         <v>28</v>
       </c>
       <c r="H126" s="32"/>
-      <c r="I126" s="106">
+      <c r="I126" s="105">
         <v>298</v>
       </c>
       <c r="J126" s="85">
@@ -9139,7 +9156,7 @@
         <v>28</v>
       </c>
       <c r="H127" s="32"/>
-      <c r="I127" s="106">
+      <c r="I127" s="105">
         <v>298</v>
       </c>
       <c r="J127" s="85">
@@ -9185,7 +9202,7 @@
         <v>28</v>
       </c>
       <c r="H128" s="32"/>
-      <c r="I128" s="106">
+      <c r="I128" s="105">
         <v>298</v>
       </c>
       <c r="J128" s="85">
@@ -9231,7 +9248,7 @@
         <v>28</v>
       </c>
       <c r="H129" s="32"/>
-      <c r="I129" s="106">
+      <c r="I129" s="105">
         <v>298</v>
       </c>
       <c r="J129" s="85">
@@ -9277,7 +9294,7 @@
         <v>28</v>
       </c>
       <c r="H130" s="32"/>
-      <c r="I130" s="106">
+      <c r="I130" s="105">
         <v>298</v>
       </c>
       <c r="J130" s="85">
@@ -9301,7 +9318,7 @@
       <c r="T130" s="35"/>
     </row>
     <row r="131" spans="1:20" ht="18" customHeight="1">
-      <c r="A131" s="112" t="s">
+      <c r="A131" s="111" t="s">
         <v>166</v>
       </c>
       <c r="B131" s="98" t="s">
@@ -9320,8 +9337,8 @@
       <c r="G131" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H131" s="116"/>
-      <c r="I131" s="106">
+      <c r="H131" s="115"/>
+      <c r="I131" s="105">
         <v>298</v>
       </c>
       <c r="J131" s="85">
@@ -9345,7 +9362,7 @@
       <c r="T131" s="35"/>
     </row>
     <row r="132" spans="1:20" ht="18" customHeight="1">
-      <c r="A132" s="113" t="s">
+      <c r="A132" s="112" t="s">
         <v>170</v>
       </c>
       <c r="B132" s="100" t="s">
@@ -9366,11 +9383,11 @@
       <c r="G132" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H132" s="117"/>
-      <c r="I132" s="106">
+      <c r="H132" s="116"/>
+      <c r="I132" s="105">
         <v>298</v>
       </c>
-      <c r="J132" s="114">
+      <c r="J132" s="113">
         <v>2070000000</v>
       </c>
       <c r="K132" s="33"/>
@@ -9391,7 +9408,7 @@
       <c r="T132" s="35"/>
     </row>
     <row r="133" spans="1:20" ht="18" customHeight="1">
-      <c r="A133" s="113" t="s">
+      <c r="A133" s="112" t="s">
         <v>171</v>
       </c>
       <c r="B133" s="100" t="s">
@@ -9412,11 +9429,11 @@
       <c r="G133" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H133" s="117"/>
-      <c r="I133" s="106">
+      <c r="H133" s="116"/>
+      <c r="I133" s="105">
         <v>298</v>
       </c>
-      <c r="J133" s="114">
+      <c r="J133" s="113">
         <v>2120000000</v>
       </c>
       <c r="K133" s="33"/>
@@ -9437,7 +9454,7 @@
       <c r="T133" s="35"/>
     </row>
     <row r="134" spans="1:20" ht="18" customHeight="1">
-      <c r="A134" s="113" t="s">
+      <c r="A134" s="112" t="s">
         <v>172</v>
       </c>
       <c r="B134" s="100" t="s">
@@ -9458,11 +9475,11 @@
       <c r="G134" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H134" s="117"/>
-      <c r="I134" s="106">
+      <c r="H134" s="116"/>
+      <c r="I134" s="105">
         <v>298</v>
       </c>
-      <c r="J134" s="114">
+      <c r="J134" s="113">
         <v>2200000000</v>
       </c>
       <c r="K134" s="33"/>
@@ -9483,7 +9500,7 @@
       <c r="T134" s="35"/>
     </row>
     <row r="135" spans="1:20" ht="18" customHeight="1">
-      <c r="A135" s="112" t="s">
+      <c r="A135" s="111" t="s">
         <v>166</v>
       </c>
       <c r="B135" s="98" t="s">
@@ -9502,8 +9519,8 @@
       <c r="G135" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H135" s="116"/>
-      <c r="I135" s="106">
+      <c r="H135" s="115"/>
+      <c r="I135" s="105">
         <v>298</v>
       </c>
       <c r="J135" s="42">
@@ -9527,7 +9544,7 @@
       <c r="T135" s="35"/>
     </row>
     <row r="136" spans="1:20" ht="18" customHeight="1">
-      <c r="A136" s="113" t="s">
+      <c r="A136" s="112" t="s">
         <v>170</v>
       </c>
       <c r="B136" s="100" t="s">
@@ -9548,8 +9565,8 @@
       <c r="G136" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H136" s="117"/>
-      <c r="I136" s="106">
+      <c r="H136" s="116"/>
+      <c r="I136" s="105">
         <v>298</v>
       </c>
       <c r="J136" s="42">
@@ -9573,7 +9590,7 @@
       <c r="T136" s="35"/>
     </row>
     <row r="137" spans="1:20" ht="18" customHeight="1">
-      <c r="A137" s="113" t="s">
+      <c r="A137" s="112" t="s">
         <v>171</v>
       </c>
       <c r="B137" s="100" t="s">
@@ -9594,8 +9611,8 @@
       <c r="G137" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H137" s="117"/>
-      <c r="I137" s="106">
+      <c r="H137" s="116"/>
+      <c r="I137" s="105">
         <v>298</v>
       </c>
       <c r="J137" s="42">
@@ -9619,7 +9636,7 @@
       <c r="T137" s="35"/>
     </row>
     <row r="138" spans="1:20" ht="18" customHeight="1">
-      <c r="A138" s="113" t="s">
+      <c r="A138" s="112" t="s">
         <v>172</v>
       </c>
       <c r="B138" s="100" t="s">
@@ -9640,8 +9657,8 @@
       <c r="G138" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H138" s="117"/>
-      <c r="I138" s="106">
+      <c r="H138" s="116"/>
+      <c r="I138" s="105">
         <v>298</v>
       </c>
       <c r="J138" s="33">
@@ -9665,7 +9682,7 @@
       <c r="T138" s="35"/>
     </row>
     <row r="139" spans="1:20" ht="18" customHeight="1">
-      <c r="A139" s="112" t="s">
+      <c r="A139" s="111" t="s">
         <v>166</v>
       </c>
       <c r="B139" s="98" t="s">
@@ -9687,7 +9704,7 @@
       <c r="H139" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I139" s="106">
+      <c r="I139" s="105">
         <v>298</v>
       </c>
       <c r="J139" s="33">
@@ -9711,7 +9728,7 @@
       <c r="T139" s="35"/>
     </row>
     <row r="140" spans="1:20" ht="18" customHeight="1">
-      <c r="A140" s="113" t="s">
+      <c r="A140" s="112" t="s">
         <v>170</v>
       </c>
       <c r="B140" s="100" t="s">
@@ -9735,7 +9752,7 @@
       <c r="H140" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I140" s="106">
+      <c r="I140" s="105">
         <v>298</v>
       </c>
       <c r="J140" s="33">
@@ -9759,7 +9776,7 @@
       <c r="T140" s="35"/>
     </row>
     <row r="141" spans="1:20" ht="18" customHeight="1">
-      <c r="A141" s="113" t="s">
+      <c r="A141" s="112" t="s">
         <v>171</v>
       </c>
       <c r="B141" s="100" t="s">
@@ -9783,7 +9800,7 @@
       <c r="H141" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I141" s="106">
+      <c r="I141" s="105">
         <v>298</v>
       </c>
       <c r="J141" s="33">
@@ -9807,7 +9824,7 @@
       <c r="T141" s="35"/>
     </row>
     <row r="142" spans="1:20" ht="18" customHeight="1">
-      <c r="A142" s="113" t="s">
+      <c r="A142" s="112" t="s">
         <v>172</v>
       </c>
       <c r="B142" s="100" t="s">
@@ -9831,7 +9848,7 @@
       <c r="H142" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="I142" s="106">
+      <c r="I142" s="105">
         <v>298</v>
       </c>
       <c r="J142" s="33">
@@ -9875,7 +9892,7 @@
         <v>28</v>
       </c>
       <c r="H143" s="32"/>
-      <c r="I143" s="106">
+      <c r="I143" s="105">
         <v>298</v>
       </c>
       <c r="J143" s="33">
@@ -9919,7 +9936,7 @@
         <v>28</v>
       </c>
       <c r="H144" s="32"/>
-      <c r="I144" s="106">
+      <c r="I144" s="105">
         <v>298</v>
       </c>
       <c r="J144" s="33">
@@ -9963,7 +9980,7 @@
         <v>28</v>
       </c>
       <c r="H145" s="32"/>
-      <c r="I145" s="106">
+      <c r="I145" s="105">
         <v>298</v>
       </c>
       <c r="J145" s="33">
@@ -10006,7 +10023,7 @@
         <v>28</v>
       </c>
       <c r="H146" s="32"/>
-      <c r="I146" s="106">
+      <c r="I146" s="105">
         <v>298</v>
       </c>
       <c r="J146" s="55">
@@ -10050,7 +10067,7 @@
         <v>28</v>
       </c>
       <c r="H147" s="32"/>
-      <c r="I147" s="106">
+      <c r="I147" s="105">
         <v>298</v>
       </c>
       <c r="J147" s="55">
@@ -10096,7 +10113,7 @@
         <v>28</v>
       </c>
       <c r="H148" s="32"/>
-      <c r="I148" s="106">
+      <c r="I148" s="105">
         <v>298</v>
       </c>
       <c r="J148" s="55">
@@ -10142,7 +10159,7 @@
         <v>28</v>
       </c>
       <c r="H149" s="32"/>
-      <c r="I149" s="106">
+      <c r="I149" s="105">
         <v>298</v>
       </c>
       <c r="J149" s="55">
@@ -10184,7 +10201,7 @@
         <v>28</v>
       </c>
       <c r="H150" s="32"/>
-      <c r="I150" s="106">
+      <c r="I150" s="105">
         <v>298</v>
       </c>
       <c r="J150" s="45">
@@ -10230,7 +10247,7 @@
         <v>28</v>
       </c>
       <c r="H151" s="32"/>
-      <c r="I151" s="106">
+      <c r="I151" s="105">
         <v>298</v>
       </c>
       <c r="J151" s="45">
@@ -10276,7 +10293,7 @@
         <v>28</v>
       </c>
       <c r="H152" s="32"/>
-      <c r="I152" s="106">
+      <c r="I152" s="105">
         <v>298</v>
       </c>
       <c r="J152" s="45">
@@ -10320,7 +10337,7 @@
         <v>28</v>
       </c>
       <c r="H153" s="32"/>
-      <c r="I153" s="106">
+      <c r="I153" s="105">
         <v>298</v>
       </c>
       <c r="J153" s="85">
@@ -10367,7 +10384,7 @@
         <v>28</v>
       </c>
       <c r="H154" s="32"/>
-      <c r="I154" s="106">
+      <c r="I154" s="105">
         <v>298</v>
       </c>
       <c r="J154" s="85">
@@ -10414,7 +10431,7 @@
       <c r="H155" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I155" s="106">
+      <c r="I155" s="105">
         <v>298</v>
       </c>
       <c r="J155" s="45">
@@ -10460,7 +10477,7 @@
       <c r="H156" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I156" s="106">
+      <c r="I156" s="105">
         <v>298</v>
       </c>
       <c r="J156" s="45">
@@ -10504,7 +10521,7 @@
       <c r="H157" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I157" s="106">
+      <c r="I157" s="105">
         <v>298</v>
       </c>
       <c r="J157" s="45">
@@ -10550,7 +10567,7 @@
       <c r="H158" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I158" s="106">
+      <c r="I158" s="105">
         <v>298</v>
       </c>
       <c r="J158" s="45">
@@ -10594,7 +10611,7 @@
       <c r="H159" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I159" s="106">
+      <c r="I159" s="105">
         <v>298</v>
       </c>
       <c r="J159" s="45">
@@ -10640,7 +10657,7 @@
       <c r="H160" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I160" s="106">
+      <c r="I160" s="105">
         <v>298</v>
       </c>
       <c r="J160" s="45">
@@ -10686,7 +10703,7 @@
       <c r="H161" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I161" s="106">
+      <c r="I161" s="105">
         <v>298</v>
       </c>
       <c r="J161" s="45">
@@ -10732,7 +10749,7 @@
       <c r="H162" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I162" s="106">
+      <c r="I162" s="105">
         <v>298</v>
       </c>
       <c r="J162" s="45">
@@ -10778,7 +10795,7 @@
       <c r="H163" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I163" s="106">
+      <c r="I163" s="105">
         <v>298</v>
       </c>
       <c r="J163" s="45">
@@ -10824,7 +10841,7 @@
       <c r="H164" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I164" s="106">
+      <c r="I164" s="105">
         <v>298</v>
       </c>
       <c r="J164" s="33">
@@ -10870,7 +10887,7 @@
       <c r="H165" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I165" s="106">
+      <c r="I165" s="105">
         <v>298</v>
       </c>
       <c r="J165" s="33">
@@ -10916,7 +10933,7 @@
       <c r="H166" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I166" s="106">
+      <c r="I166" s="105">
         <v>298</v>
       </c>
       <c r="J166" s="33">
@@ -10962,7 +10979,7 @@
       <c r="H167" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I167" s="106">
+      <c r="I167" s="105">
         <v>298</v>
       </c>
       <c r="J167" s="33">
@@ -11008,7 +11025,7 @@
       <c r="H168" s="32" t="s">
         <v>206</v>
       </c>
-      <c r="I168" s="106">
+      <c r="I168" s="105">
         <v>298</v>
       </c>
       <c r="J168" s="45">
@@ -11051,10 +11068,10 @@
       <c r="G169" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H169" s="116" t="s">
+      <c r="H169" s="115" t="s">
         <v>206</v>
       </c>
-      <c r="I169" s="106">
+      <c r="I169" s="105">
         <v>298</v>
       </c>
       <c r="J169" s="85">
@@ -11100,10 +11117,10 @@
       <c r="G170" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H170" s="117" t="s">
+      <c r="H170" s="116" t="s">
         <v>206</v>
       </c>
-      <c r="I170" s="106">
+      <c r="I170" s="105">
         <v>298</v>
       </c>
       <c r="J170" s="85">
@@ -11149,10 +11166,10 @@
       <c r="G171" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H171" s="117" t="s">
+      <c r="H171" s="116" t="s">
         <v>206</v>
       </c>
-      <c r="I171" s="106">
+      <c r="I171" s="105">
         <v>298</v>
       </c>
       <c r="J171" s="85">
@@ -11198,10 +11215,10 @@
       <c r="G172" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="H172" s="117" t="s">
+      <c r="H172" s="116" t="s">
         <v>206</v>
       </c>
-      <c r="I172" s="106">
+      <c r="I172" s="105">
         <v>298</v>
       </c>
       <c r="J172" s="85">
@@ -11229,19 +11246,41 @@
     </row>
     <row r="173" spans="1:20" ht="18" customHeight="1">
       <c r="A173" s="103"/>
-      <c r="B173" s="98"/>
-      <c r="C173" s="86"/>
-      <c r="D173" s="86"/>
-      <c r="E173" s="98"/>
-      <c r="F173" s="93"/>
-      <c r="G173" s="93"/>
+      <c r="B173" s="98" t="s">
+        <v>210</v>
+      </c>
+      <c r="C173" s="86" t="s">
+        <v>173</v>
+      </c>
+      <c r="D173" s="86" t="s">
+        <v>108</v>
+      </c>
+      <c r="E173" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F173" s="93" t="s">
+        <v>112</v>
+      </c>
+      <c r="G173" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H173" s="32"/>
-      <c r="I173" s="104"/>
-      <c r="J173" s="45"/>
+      <c r="I173" s="105">
+        <v>298</v>
+      </c>
+      <c r="J173" s="45">
+        <v>1479000000</v>
+      </c>
       <c r="K173" s="36"/>
-      <c r="L173" s="31"/>
-      <c r="M173" s="46"/>
-      <c r="N173" s="29"/>
+      <c r="L173" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M173" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N173" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O173" s="35"/>
       <c r="P173" s="36"/>
       <c r="Q173" s="36"/>
@@ -11250,20 +11289,42 @@
       <c r="T173" s="35"/>
     </row>
     <row r="174" spans="1:20" ht="18" customHeight="1">
-      <c r="A174" s="105"/>
-      <c r="B174" s="100"/>
-      <c r="C174" s="87"/>
-      <c r="D174" s="87"/>
-      <c r="E174" s="100"/>
-      <c r="F174" s="93"/>
-      <c r="G174" s="94"/>
+      <c r="A174" s="104"/>
+      <c r="B174" s="100" t="s">
+        <v>212</v>
+      </c>
+      <c r="C174" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D174" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E174" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F174" s="93" t="s">
+        <v>112</v>
+      </c>
+      <c r="G174" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H174" s="32"/>
-      <c r="I174" s="106"/>
-      <c r="J174" s="45"/>
+      <c r="I174" s="105">
+        <v>298</v>
+      </c>
+      <c r="J174" s="45">
+        <v>1230000000</v>
+      </c>
       <c r="K174" s="36"/>
-      <c r="L174" s="31"/>
-      <c r="M174" s="46"/>
-      <c r="N174" s="29"/>
+      <c r="L174" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M174" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N174" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O174" s="35"/>
       <c r="P174" s="36"/>
       <c r="Q174" s="36"/>
@@ -11272,20 +11333,42 @@
       <c r="T174" s="35"/>
     </row>
     <row r="175" spans="1:20" ht="18" customHeight="1">
-      <c r="A175" s="105"/>
-      <c r="B175" s="100"/>
-      <c r="C175" s="87"/>
-      <c r="D175" s="87"/>
-      <c r="E175" s="100"/>
-      <c r="F175" s="93"/>
-      <c r="G175" s="94"/>
+      <c r="A175" s="104"/>
+      <c r="B175" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="C175" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D175" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E175" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F175" s="93" t="s">
+        <v>112</v>
+      </c>
+      <c r="G175" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H175" s="32"/>
-      <c r="I175" s="106"/>
-      <c r="J175" s="33"/>
+      <c r="I175" s="105">
+        <v>298</v>
+      </c>
+      <c r="J175" s="33">
+        <v>1311000000</v>
+      </c>
       <c r="K175" s="36"/>
-      <c r="L175" s="31"/>
-      <c r="M175" s="46"/>
-      <c r="N175" s="29"/>
+      <c r="L175" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="M175" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N175" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O175" s="35"/>
       <c r="P175" s="36"/>
       <c r="Q175" s="36"/>
@@ -11294,20 +11377,42 @@
       <c r="T175" s="35"/>
     </row>
     <row r="176" spans="1:20" ht="18" customHeight="1">
-      <c r="A176" s="105"/>
-      <c r="B176" s="100"/>
-      <c r="C176" s="87"/>
-      <c r="D176" s="87"/>
-      <c r="E176" s="100"/>
-      <c r="F176" s="93"/>
-      <c r="G176" s="94"/>
+      <c r="A176" s="104"/>
+      <c r="B176" s="98" t="s">
+        <v>210</v>
+      </c>
+      <c r="C176" s="86" t="s">
+        <v>173</v>
+      </c>
+      <c r="D176" s="86" t="s">
+        <v>108</v>
+      </c>
+      <c r="E176" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F176" s="93" t="s">
+        <v>114</v>
+      </c>
+      <c r="G176" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H176" s="32"/>
-      <c r="I176" s="106"/>
-      <c r="J176" s="33"/>
+      <c r="I176" s="105">
+        <v>298</v>
+      </c>
+      <c r="J176" s="33">
+        <v>20.100000000000001</v>
+      </c>
       <c r="K176" s="36"/>
-      <c r="L176" s="31"/>
-      <c r="M176" s="46"/>
-      <c r="N176" s="29"/>
+      <c r="L176" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M176" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N176" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O176" s="35"/>
       <c r="P176" s="35"/>
       <c r="Q176" s="36"/>
@@ -11317,19 +11422,41 @@
     </row>
     <row r="177" spans="1:20" ht="18" customHeight="1">
       <c r="A177" s="103"/>
-      <c r="B177" s="98"/>
-      <c r="C177" s="86"/>
-      <c r="D177" s="86"/>
-      <c r="E177" s="98"/>
-      <c r="F177" s="93"/>
-      <c r="G177" s="93"/>
+      <c r="B177" s="100" t="s">
+        <v>212</v>
+      </c>
+      <c r="C177" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D177" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E177" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F177" s="93" t="s">
+        <v>114</v>
+      </c>
+      <c r="G177" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H177" s="32"/>
-      <c r="I177" s="104"/>
-      <c r="J177" s="33"/>
+      <c r="I177" s="105">
+        <v>298</v>
+      </c>
+      <c r="J177" s="33">
+        <v>47.7</v>
+      </c>
       <c r="K177" s="36"/>
-      <c r="L177" s="31"/>
-      <c r="M177" s="46"/>
-      <c r="N177" s="29"/>
+      <c r="L177" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M177" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N177" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O177" s="35"/>
       <c r="P177" s="35"/>
       <c r="Q177" s="36"/>
@@ -11338,20 +11465,42 @@
       <c r="T177" s="35"/>
     </row>
     <row r="178" spans="1:20" ht="18" customHeight="1">
-      <c r="A178" s="105"/>
-      <c r="B178" s="100"/>
-      <c r="C178" s="87"/>
-      <c r="D178" s="87"/>
-      <c r="E178" s="100"/>
-      <c r="F178" s="93"/>
-      <c r="G178" s="94"/>
+      <c r="A178" s="104"/>
+      <c r="B178" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="C178" s="87" t="s">
+        <v>63</v>
+      </c>
+      <c r="D178" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E178" s="98" t="s">
+        <v>213</v>
+      </c>
+      <c r="F178" s="93" t="s">
+        <v>114</v>
+      </c>
+      <c r="G178" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H178" s="32"/>
-      <c r="I178" s="106"/>
-      <c r="J178" s="33"/>
+      <c r="I178" s="105">
+        <v>298</v>
+      </c>
+      <c r="J178" s="33">
+        <v>21.7</v>
+      </c>
       <c r="K178" s="36"/>
-      <c r="L178" s="31"/>
-      <c r="M178" s="46"/>
-      <c r="N178" s="29"/>
+      <c r="L178" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="M178" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N178" s="29" t="s">
+        <v>215</v>
+      </c>
       <c r="O178" s="35"/>
       <c r="P178" s="35"/>
       <c r="Q178" s="36"/>
@@ -11360,7 +11509,7 @@
       <c r="T178" s="35"/>
     </row>
     <row r="179" spans="1:20" ht="18" customHeight="1">
-      <c r="A179" s="105"/>
+      <c r="A179" s="104"/>
       <c r="B179" s="100"/>
       <c r="C179" s="87"/>
       <c r="D179" s="87"/>
@@ -11368,7 +11517,7 @@
       <c r="F179" s="93"/>
       <c r="G179" s="94"/>
       <c r="H179" s="32"/>
-      <c r="I179" s="106"/>
+      <c r="I179" s="105"/>
       <c r="J179" s="33"/>
       <c r="K179" s="36"/>
       <c r="L179" s="31"/>
@@ -11382,7 +11531,7 @@
       <c r="T179" s="35"/>
     </row>
     <row r="180" spans="1:20" ht="18" customHeight="1">
-      <c r="A180" s="105"/>
+      <c r="A180" s="104"/>
       <c r="B180" s="100"/>
       <c r="C180" s="87"/>
       <c r="D180" s="87"/>
@@ -11390,7 +11539,7 @@
       <c r="F180" s="93"/>
       <c r="G180" s="94"/>
       <c r="H180" s="32"/>
-      <c r="I180" s="106"/>
+      <c r="I180" s="105"/>
       <c r="J180" s="48"/>
       <c r="K180" s="36"/>
       <c r="L180" s="31"/>
@@ -11514,7 +11663,7 @@
       <c r="T185" s="35"/>
     </row>
     <row r="186" spans="1:20" ht="18" customHeight="1">
-      <c r="A186" s="105"/>
+      <c r="A186" s="104"/>
       <c r="B186" s="100"/>
       <c r="C186" s="87"/>
       <c r="D186" s="87"/>
@@ -11536,7 +11685,7 @@
       <c r="T186" s="35"/>
     </row>
     <row r="187" spans="1:20" ht="18" customHeight="1">
-      <c r="A187" s="105"/>
+      <c r="A187" s="104"/>
       <c r="B187" s="100"/>
       <c r="C187" s="87"/>
       <c r="D187" s="87"/>
@@ -11558,7 +11707,7 @@
       <c r="T187" s="35"/>
     </row>
     <row r="188" spans="1:20" ht="18" customHeight="1">
-      <c r="A188" s="105"/>
+      <c r="A188" s="104"/>
       <c r="B188" s="100"/>
       <c r="C188" s="87"/>
       <c r="D188" s="87"/>
@@ -11602,7 +11751,7 @@
       <c r="T189" s="35"/>
     </row>
     <row r="190" spans="1:20" ht="18" customHeight="1">
-      <c r="A190" s="105"/>
+      <c r="A190" s="104"/>
       <c r="B190" s="100"/>
       <c r="C190" s="87"/>
       <c r="D190" s="87"/>
@@ -11624,7 +11773,7 @@
       <c r="T190" s="35"/>
     </row>
     <row r="191" spans="1:20" ht="18" customHeight="1">
-      <c r="A191" s="105"/>
+      <c r="A191" s="104"/>
       <c r="B191" s="100"/>
       <c r="C191" s="87"/>
       <c r="D191" s="87"/>
@@ -11646,7 +11795,7 @@
       <c r="T191" s="35"/>
     </row>
     <row r="192" spans="1:20" ht="18" customHeight="1">
-      <c r="A192" s="105"/>
+      <c r="A192" s="104"/>
       <c r="B192" s="100"/>
       <c r="C192" s="87"/>
       <c r="D192" s="87"/>
@@ -11805,7 +11954,7 @@
       <c r="C199" s="29"/>
       <c r="D199" s="29"/>
       <c r="E199" s="30"/>
-      <c r="F199" s="107"/>
+      <c r="F199" s="106"/>
       <c r="G199" s="31"/>
       <c r="H199" s="53"/>
       <c r="I199" s="51"/>
@@ -12174,7 +12323,7 @@
       <c r="T215" s="35"/>
     </row>
     <row r="216" spans="1:20" ht="18" customHeight="1">
-      <c r="A216" s="108"/>
+      <c r="A216" s="107"/>
       <c r="B216" s="98"/>
       <c r="C216" s="86"/>
       <c r="D216" s="86"/>
@@ -12196,7 +12345,7 @@
       <c r="T216" s="35"/>
     </row>
     <row r="217" spans="1:20" ht="18" customHeight="1">
-      <c r="A217" s="109"/>
+      <c r="A217" s="108"/>
       <c r="B217" s="100"/>
       <c r="C217" s="87"/>
       <c r="D217" s="87"/>
@@ -12218,7 +12367,7 @@
       <c r="T217" s="35"/>
     </row>
     <row r="218" spans="1:20" ht="18" customHeight="1">
-      <c r="A218" s="109"/>
+      <c r="A218" s="108"/>
       <c r="B218" s="100"/>
       <c r="C218" s="87"/>
       <c r="D218" s="87"/>
@@ -12240,7 +12389,7 @@
       <c r="T218" s="35"/>
     </row>
     <row r="219" spans="1:20" ht="18" customHeight="1">
-      <c r="A219" s="109"/>
+      <c r="A219" s="108"/>
       <c r="B219" s="100"/>
       <c r="C219" s="87"/>
       <c r="D219" s="87"/>
@@ -12262,7 +12411,7 @@
       <c r="T219" s="35"/>
     </row>
     <row r="220" spans="1:20" ht="18" customHeight="1">
-      <c r="A220" s="109"/>
+      <c r="A220" s="108"/>
       <c r="B220" s="100"/>
       <c r="C220" s="87"/>
       <c r="D220" s="87"/>
@@ -12284,7 +12433,7 @@
       <c r="T220" s="35"/>
     </row>
     <row r="221" spans="1:20" ht="18" customHeight="1">
-      <c r="A221" s="109"/>
+      <c r="A221" s="108"/>
       <c r="B221" s="100"/>
       <c r="C221" s="87"/>
       <c r="D221" s="87"/>
@@ -12306,7 +12455,7 @@
       <c r="T221" s="35"/>
     </row>
     <row r="222" spans="1:20" ht="18" customHeight="1">
-      <c r="A222" s="109"/>
+      <c r="A222" s="108"/>
       <c r="B222" s="100"/>
       <c r="C222" s="87"/>
       <c r="D222" s="87"/>
@@ -12328,7 +12477,7 @@
       <c r="T222" s="35"/>
     </row>
     <row r="223" spans="1:20" ht="18" customHeight="1">
-      <c r="A223" s="109"/>
+      <c r="A223" s="108"/>
       <c r="B223" s="100"/>
       <c r="C223" s="87"/>
       <c r="D223" s="87"/>
@@ -12350,7 +12499,7 @@
       <c r="T223" s="35"/>
     </row>
     <row r="224" spans="1:20" ht="18" customHeight="1">
-      <c r="A224" s="108"/>
+      <c r="A224" s="107"/>
       <c r="B224" s="98"/>
       <c r="C224" s="86"/>
       <c r="D224" s="86"/>
@@ -12372,7 +12521,7 @@
       <c r="T224" s="35"/>
     </row>
     <row r="225" spans="1:20" ht="18" customHeight="1">
-      <c r="A225" s="109"/>
+      <c r="A225" s="108"/>
       <c r="B225" s="100"/>
       <c r="C225" s="87"/>
       <c r="D225" s="87"/>
@@ -12394,7 +12543,7 @@
       <c r="T225" s="35"/>
     </row>
     <row r="226" spans="1:20" ht="18" customHeight="1">
-      <c r="A226" s="109"/>
+      <c r="A226" s="108"/>
       <c r="B226" s="100"/>
       <c r="C226" s="87"/>
       <c r="D226" s="87"/>
@@ -12416,7 +12565,7 @@
       <c r="T226" s="35"/>
     </row>
     <row r="227" spans="1:20" ht="18" customHeight="1">
-      <c r="A227" s="109"/>
+      <c r="A227" s="108"/>
       <c r="B227" s="100"/>
       <c r="C227" s="87"/>
       <c r="D227" s="87"/>
@@ -12438,7 +12587,7 @@
       <c r="T227" s="35"/>
     </row>
     <row r="228" spans="1:20" ht="18" customHeight="1">
-      <c r="A228" s="109"/>
+      <c r="A228" s="108"/>
       <c r="B228" s="100"/>
       <c r="C228" s="87"/>
       <c r="D228" s="87"/>
@@ -12460,7 +12609,7 @@
       <c r="T228" s="35"/>
     </row>
     <row r="229" spans="1:20" ht="18" customHeight="1">
-      <c r="A229" s="109"/>
+      <c r="A229" s="108"/>
       <c r="B229" s="100"/>
       <c r="C229" s="87"/>
       <c r="D229" s="87"/>
@@ -12482,7 +12631,7 @@
       <c r="T229" s="35"/>
     </row>
     <row r="230" spans="1:20" ht="18" customHeight="1">
-      <c r="A230" s="109"/>
+      <c r="A230" s="108"/>
       <c r="B230" s="100"/>
       <c r="C230" s="87"/>
       <c r="D230" s="87"/>
@@ -12504,7 +12653,7 @@
       <c r="T230" s="35"/>
     </row>
     <row r="231" spans="1:20" ht="18" customHeight="1">
-      <c r="A231" s="109"/>
+      <c r="A231" s="108"/>
       <c r="B231" s="100"/>
       <c r="C231" s="87"/>
       <c r="D231" s="87"/>
@@ -12526,7 +12675,7 @@
       <c r="T231" s="35"/>
     </row>
     <row r="232" spans="1:20" ht="18" customHeight="1">
-      <c r="A232" s="108"/>
+      <c r="A232" s="107"/>
       <c r="B232" s="98"/>
       <c r="C232" s="86"/>
       <c r="D232" s="86"/>
@@ -12548,7 +12697,7 @@
       <c r="T232" s="35"/>
     </row>
     <row r="233" spans="1:20" ht="18" customHeight="1">
-      <c r="A233" s="109"/>
+      <c r="A233" s="108"/>
       <c r="B233" s="100"/>
       <c r="C233" s="87"/>
       <c r="D233" s="87"/>
@@ -12570,7 +12719,7 @@
       <c r="T233" s="35"/>
     </row>
     <row r="234" spans="1:20" ht="18" customHeight="1">
-      <c r="A234" s="109"/>
+      <c r="A234" s="108"/>
       <c r="B234" s="100"/>
       <c r="C234" s="87"/>
       <c r="D234" s="87"/>
@@ -12592,7 +12741,7 @@
       <c r="T234" s="35"/>
     </row>
     <row r="235" spans="1:20" ht="18" customHeight="1">
-      <c r="A235" s="109"/>
+      <c r="A235" s="108"/>
       <c r="B235" s="100"/>
       <c r="C235" s="87"/>
       <c r="D235" s="87"/>
@@ -12614,7 +12763,7 @@
       <c r="T235" s="35"/>
     </row>
     <row r="236" spans="1:20" ht="18" customHeight="1">
-      <c r="A236" s="109"/>
+      <c r="A236" s="108"/>
       <c r="B236" s="100"/>
       <c r="C236" s="87"/>
       <c r="D236" s="87"/>
@@ -12636,7 +12785,7 @@
       <c r="T236" s="35"/>
     </row>
     <row r="237" spans="1:20" ht="18" customHeight="1">
-      <c r="A237" s="109"/>
+      <c r="A237" s="108"/>
       <c r="B237" s="100"/>
       <c r="C237" s="87"/>
       <c r="D237" s="87"/>
@@ -12658,7 +12807,7 @@
       <c r="T237" s="35"/>
     </row>
     <row r="238" spans="1:20" ht="18" customHeight="1">
-      <c r="A238" s="109"/>
+      <c r="A238" s="108"/>
       <c r="B238" s="100"/>
       <c r="C238" s="87"/>
       <c r="D238" s="87"/>
@@ -12680,7 +12829,7 @@
       <c r="T238" s="35"/>
     </row>
     <row r="239" spans="1:20" ht="18" customHeight="1">
-      <c r="A239" s="109"/>
+      <c r="A239" s="108"/>
       <c r="B239" s="100"/>
       <c r="C239" s="87"/>
       <c r="D239" s="87"/>
@@ -12702,7 +12851,7 @@
       <c r="T239" s="35"/>
     </row>
     <row r="240" spans="1:20" ht="18" customHeight="1">
-      <c r="A240" s="108"/>
+      <c r="A240" s="107"/>
       <c r="B240" s="98"/>
       <c r="C240" s="86"/>
       <c r="D240" s="86"/>
@@ -12724,7 +12873,7 @@
       <c r="T240" s="35"/>
     </row>
     <row r="241" spans="1:20" ht="18" customHeight="1">
-      <c r="A241" s="109"/>
+      <c r="A241" s="108"/>
       <c r="B241" s="100"/>
       <c r="C241" s="87"/>
       <c r="D241" s="87"/>
@@ -12746,7 +12895,7 @@
       <c r="T241" s="35"/>
     </row>
     <row r="242" spans="1:20" ht="18" customHeight="1">
-      <c r="A242" s="109"/>
+      <c r="A242" s="108"/>
       <c r="B242" s="100"/>
       <c r="C242" s="87"/>
       <c r="D242" s="87"/>
@@ -12768,7 +12917,7 @@
       <c r="T242" s="35"/>
     </row>
     <row r="243" spans="1:20" ht="18" customHeight="1">
-      <c r="A243" s="109"/>
+      <c r="A243" s="108"/>
       <c r="B243" s="100"/>
       <c r="C243" s="87"/>
       <c r="D243" s="87"/>
@@ -12790,7 +12939,7 @@
       <c r="T243" s="35"/>
     </row>
     <row r="244" spans="1:20" ht="18" customHeight="1">
-      <c r="A244" s="109"/>
+      <c r="A244" s="108"/>
       <c r="B244" s="100"/>
       <c r="C244" s="87"/>
       <c r="D244" s="87"/>
@@ -12812,7 +12961,7 @@
       <c r="T244" s="35"/>
     </row>
     <row r="245" spans="1:20" ht="18" customHeight="1">
-      <c r="A245" s="109"/>
+      <c r="A245" s="108"/>
       <c r="B245" s="100"/>
       <c r="C245" s="87"/>
       <c r="D245" s="87"/>
@@ -12834,7 +12983,7 @@
       <c r="T245" s="35"/>
     </row>
     <row r="246" spans="1:20" ht="18" customHeight="1">
-      <c r="A246" s="109"/>
+      <c r="A246" s="108"/>
       <c r="B246" s="100"/>
       <c r="C246" s="87"/>
       <c r="D246" s="87"/>
@@ -12856,7 +13005,7 @@
       <c r="T246" s="35"/>
     </row>
     <row r="247" spans="1:20" ht="18" customHeight="1">
-      <c r="A247" s="109"/>
+      <c r="A247" s="108"/>
       <c r="B247" s="100"/>
       <c r="C247" s="87"/>
       <c r="D247" s="87"/>
@@ -12878,7 +13027,7 @@
       <c r="T247" s="41"/>
     </row>
     <row r="248" spans="1:20" ht="18" customHeight="1">
-      <c r="A248" s="108"/>
+      <c r="A248" s="107"/>
       <c r="B248" s="98"/>
       <c r="C248" s="86"/>
       <c r="D248" s="86"/>
@@ -12900,7 +13049,7 @@
       <c r="T248" s="41"/>
     </row>
     <row r="249" spans="1:20" ht="18" customHeight="1">
-      <c r="A249" s="109"/>
+      <c r="A249" s="108"/>
       <c r="B249" s="100"/>
       <c r="C249" s="87"/>
       <c r="D249" s="87"/>
@@ -12922,7 +13071,7 @@
       <c r="T249" s="41"/>
     </row>
     <row r="250" spans="1:20" ht="18" customHeight="1">
-      <c r="A250" s="109"/>
+      <c r="A250" s="108"/>
       <c r="B250" s="100"/>
       <c r="C250" s="87"/>
       <c r="D250" s="87"/>
@@ -12944,7 +13093,7 @@
       <c r="T250" s="35"/>
     </row>
     <row r="251" spans="1:20" ht="18" customHeight="1">
-      <c r="A251" s="109"/>
+      <c r="A251" s="108"/>
       <c r="B251" s="100"/>
       <c r="C251" s="87"/>
       <c r="D251" s="87"/>
@@ -12966,7 +13115,7 @@
       <c r="T251" s="35"/>
     </row>
     <row r="252" spans="1:20" ht="18" customHeight="1">
-      <c r="A252" s="109"/>
+      <c r="A252" s="108"/>
       <c r="B252" s="100"/>
       <c r="C252" s="87"/>
       <c r="D252" s="87"/>
@@ -12988,7 +13137,7 @@
       <c r="T252" s="35"/>
     </row>
     <row r="253" spans="1:20" ht="18" customHeight="1">
-      <c r="A253" s="109"/>
+      <c r="A253" s="108"/>
       <c r="B253" s="100"/>
       <c r="C253" s="87"/>
       <c r="D253" s="87"/>
@@ -13010,7 +13159,7 @@
       <c r="T253" s="35"/>
     </row>
     <row r="254" spans="1:20" ht="18" customHeight="1">
-      <c r="A254" s="109"/>
+      <c r="A254" s="108"/>
       <c r="B254" s="100"/>
       <c r="C254" s="87"/>
       <c r="D254" s="87"/>
@@ -13032,7 +13181,7 @@
       <c r="T254" s="35"/>
     </row>
     <row r="255" spans="1:20" ht="18" customHeight="1">
-      <c r="A255" s="109"/>
+      <c r="A255" s="108"/>
       <c r="B255" s="100"/>
       <c r="C255" s="87"/>
       <c r="D255" s="87"/>
@@ -13054,7 +13203,7 @@
       <c r="T255" s="35"/>
     </row>
     <row r="256" spans="1:20" ht="18" customHeight="1">
-      <c r="A256" s="108"/>
+      <c r="A256" s="107"/>
       <c r="B256" s="98"/>
       <c r="C256" s="86"/>
       <c r="D256" s="86"/>
@@ -13076,7 +13225,7 @@
       <c r="T256" s="35"/>
     </row>
     <row r="257" spans="1:20" ht="18" customHeight="1">
-      <c r="A257" s="109"/>
+      <c r="A257" s="108"/>
       <c r="B257" s="100"/>
       <c r="C257" s="87"/>
       <c r="D257" s="87"/>
@@ -13098,7 +13247,7 @@
       <c r="T257" s="35"/>
     </row>
     <row r="258" spans="1:20" ht="18" customHeight="1">
-      <c r="A258" s="109"/>
+      <c r="A258" s="108"/>
       <c r="B258" s="100"/>
       <c r="C258" s="87"/>
       <c r="D258" s="87"/>
@@ -13120,7 +13269,7 @@
       <c r="T258" s="35"/>
     </row>
     <row r="259" spans="1:20" ht="18" customHeight="1">
-      <c r="A259" s="109"/>
+      <c r="A259" s="108"/>
       <c r="B259" s="100"/>
       <c r="C259" s="87"/>
       <c r="D259" s="87"/>
@@ -13142,7 +13291,7 @@
       <c r="T259" s="35"/>
     </row>
     <row r="260" spans="1:20" ht="18" customHeight="1">
-      <c r="A260" s="109"/>
+      <c r="A260" s="108"/>
       <c r="B260" s="100"/>
       <c r="C260" s="87"/>
       <c r="D260" s="87"/>
@@ -13164,7 +13313,7 @@
       <c r="T260" s="35"/>
     </row>
     <row r="261" spans="1:20" ht="18" customHeight="1">
-      <c r="A261" s="109"/>
+      <c r="A261" s="108"/>
       <c r="B261" s="100"/>
       <c r="C261" s="87"/>
       <c r="D261" s="87"/>
@@ -13186,7 +13335,7 @@
       <c r="T261" s="35"/>
     </row>
     <row r="262" spans="1:20" ht="18" customHeight="1">
-      <c r="A262" s="109"/>
+      <c r="A262" s="108"/>
       <c r="B262" s="100"/>
       <c r="C262" s="87"/>
       <c r="D262" s="87"/>
@@ -13208,7 +13357,7 @@
       <c r="T262" s="35"/>
     </row>
     <row r="263" spans="1:20" ht="18" customHeight="1">
-      <c r="A263" s="109"/>
+      <c r="A263" s="108"/>
       <c r="B263" s="100"/>
       <c r="C263" s="87"/>
       <c r="D263" s="87"/>
@@ -13217,7 +13366,7 @@
       <c r="G263" s="31"/>
       <c r="H263" s="53"/>
       <c r="I263" s="51"/>
-      <c r="J263" s="110"/>
+      <c r="J263" s="109"/>
       <c r="K263" s="36"/>
       <c r="L263" s="38"/>
       <c r="M263" s="38"/>
@@ -13239,7 +13388,7 @@
       <c r="G264" s="31"/>
       <c r="H264" s="53"/>
       <c r="I264" s="51"/>
-      <c r="J264" s="110"/>
+      <c r="J264" s="109"/>
       <c r="K264" s="36"/>
       <c r="L264" s="38"/>
       <c r="M264" s="38"/>
@@ -13261,7 +13410,7 @@
       <c r="G265" s="31"/>
       <c r="H265" s="53"/>
       <c r="I265" s="51"/>
-      <c r="J265" s="110"/>
+      <c r="J265" s="109"/>
       <c r="K265" s="36"/>
       <c r="L265" s="38"/>
       <c r="M265" s="38"/>
@@ -13283,7 +13432,7 @@
       <c r="G266" s="31"/>
       <c r="H266" s="53"/>
       <c r="I266" s="51"/>
-      <c r="J266" s="110"/>
+      <c r="J266" s="109"/>
       <c r="K266" s="36"/>
       <c r="L266" s="38"/>
       <c r="M266" s="38"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jnoncrysol.2025.123838`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DEADD6-06B1-7E44-A2D2-5CAE20E7FE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F777AC3E-9E49-834F-AD3B-8D92A7B0C910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="12140" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1676" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="228">
   <si>
     <r>
       <rPr>
@@ -778,6 +778,42 @@
   </si>
   <si>
     <t>10.1038/s41524-026-02189-5</t>
+  </si>
+  <si>
+    <t>Gd36 Dy20 Ni20 Al24</t>
+  </si>
+  <si>
+    <t>Gd36 Ho20 Ni20 Al24</t>
+  </si>
+  <si>
+    <t>Gd36 Er20 Ni20 Al24</t>
+  </si>
+  <si>
+    <t>amorphous</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>melt spun into amorphous state verified with XRD</t>
+  </si>
+  <si>
+    <t>curie temperature</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>peak magnetic entropy change</t>
+  </si>
+  <si>
+    <t>J/kgK</t>
+  </si>
+  <si>
+    <t>10.1016/j.jnoncrysol.2025.123838</t>
+  </si>
+  <si>
+    <t>5T</t>
   </si>
 </sst>
 </file>
@@ -11510,19 +11546,39 @@
     </row>
     <row r="179" spans="1:20" ht="18" customHeight="1">
       <c r="A179" s="104"/>
-      <c r="B179" s="100"/>
-      <c r="C179" s="87"/>
-      <c r="D179" s="87"/>
-      <c r="E179" s="100"/>
-      <c r="F179" s="93"/>
-      <c r="G179" s="94"/>
+      <c r="B179" s="100" t="s">
+        <v>216</v>
+      </c>
+      <c r="C179" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D179" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E179" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F179" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="G179" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H179" s="32"/>
       <c r="I179" s="105"/>
-      <c r="J179" s="33"/>
+      <c r="J179" s="33">
+        <v>50</v>
+      </c>
       <c r="K179" s="36"/>
-      <c r="L179" s="31"/>
-      <c r="M179" s="46"/>
-      <c r="N179" s="29"/>
+      <c r="L179" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="M179" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N179" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O179" s="35"/>
       <c r="P179" s="35"/>
       <c r="Q179" s="36"/>
@@ -11532,19 +11588,39 @@
     </row>
     <row r="180" spans="1:20" ht="18" customHeight="1">
       <c r="A180" s="104"/>
-      <c r="B180" s="100"/>
-      <c r="C180" s="87"/>
-      <c r="D180" s="87"/>
-      <c r="E180" s="100"/>
-      <c r="F180" s="93"/>
-      <c r="G180" s="94"/>
+      <c r="B180" s="100" t="s">
+        <v>217</v>
+      </c>
+      <c r="C180" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D180" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E180" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F180" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="G180" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H180" s="32"/>
       <c r="I180" s="105"/>
-      <c r="J180" s="48"/>
+      <c r="J180" s="48">
+        <v>45</v>
+      </c>
       <c r="K180" s="36"/>
-      <c r="L180" s="31"/>
-      <c r="M180" s="46"/>
-      <c r="N180" s="29"/>
+      <c r="L180" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="M180" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N180" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O180" s="35"/>
       <c r="P180" s="35"/>
       <c r="Q180" s="36"/>
@@ -11554,19 +11630,39 @@
     </row>
     <row r="181" spans="1:20" ht="18" customHeight="1">
       <c r="A181" s="47"/>
-      <c r="B181" s="30"/>
-      <c r="C181" s="29"/>
-      <c r="D181" s="29"/>
-      <c r="E181" s="30"/>
-      <c r="F181" s="49"/>
-      <c r="G181" s="31"/>
+      <c r="B181" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="C181" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D181" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E181" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F181" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="G181" s="94" t="s">
+        <v>28</v>
+      </c>
       <c r="H181" s="53"/>
       <c r="I181" s="51"/>
-      <c r="J181" s="48"/>
+      <c r="J181" s="48">
+        <v>40</v>
+      </c>
       <c r="K181" s="36"/>
-      <c r="L181" s="31"/>
-      <c r="M181" s="46"/>
-      <c r="N181" s="29"/>
+      <c r="L181" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="M181" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N181" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O181" s="35"/>
       <c r="P181" s="35"/>
       <c r="Q181" s="36"/>
@@ -11576,19 +11672,41 @@
     </row>
     <row r="182" spans="1:20" ht="18" customHeight="1">
       <c r="A182" s="47"/>
-      <c r="B182" s="30"/>
-      <c r="C182" s="29"/>
-      <c r="D182" s="29"/>
-      <c r="E182" s="30"/>
-      <c r="F182" s="49"/>
-      <c r="G182" s="31"/>
-      <c r="H182" s="53"/>
+      <c r="B182" s="100" t="s">
+        <v>216</v>
+      </c>
+      <c r="C182" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D182" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E182" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F182" s="93" t="s">
+        <v>224</v>
+      </c>
+      <c r="G182" s="94" t="s">
+        <v>28</v>
+      </c>
+      <c r="H182" s="53" t="s">
+        <v>227</v>
+      </c>
       <c r="I182" s="51"/>
-      <c r="J182" s="48"/>
+      <c r="J182" s="48">
+        <v>7.79</v>
+      </c>
       <c r="K182" s="36"/>
-      <c r="L182" s="31"/>
-      <c r="M182" s="46"/>
-      <c r="N182" s="29"/>
+      <c r="L182" s="31" t="s">
+        <v>225</v>
+      </c>
+      <c r="M182" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N182" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O182" s="35"/>
       <c r="P182" s="35"/>
       <c r="Q182" s="36"/>
@@ -11598,19 +11716,41 @@
     </row>
     <row r="183" spans="1:20" ht="18" customHeight="1">
       <c r="A183" s="47"/>
-      <c r="B183" s="30"/>
-      <c r="C183" s="29"/>
-      <c r="D183" s="29"/>
-      <c r="E183" s="30"/>
-      <c r="F183" s="49"/>
-      <c r="G183" s="31"/>
-      <c r="H183" s="53"/>
+      <c r="B183" s="100" t="s">
+        <v>217</v>
+      </c>
+      <c r="C183" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D183" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E183" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F183" s="93" t="s">
+        <v>224</v>
+      </c>
+      <c r="G183" s="94" t="s">
+        <v>28</v>
+      </c>
+      <c r="H183" s="53" t="s">
+        <v>227</v>
+      </c>
       <c r="I183" s="51"/>
-      <c r="J183" s="48"/>
+      <c r="J183" s="48">
+        <v>8.75</v>
+      </c>
       <c r="K183" s="36"/>
-      <c r="L183" s="31"/>
-      <c r="M183" s="46"/>
-      <c r="N183" s="29"/>
+      <c r="L183" s="31" t="s">
+        <v>225</v>
+      </c>
+      <c r="M183" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N183" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O183" s="35"/>
       <c r="P183" s="35"/>
       <c r="Q183" s="36"/>
@@ -11620,19 +11760,41 @@
     </row>
     <row r="184" spans="1:20" ht="18" customHeight="1">
       <c r="A184" s="47"/>
-      <c r="B184" s="30"/>
-      <c r="C184" s="29"/>
-      <c r="D184" s="29"/>
-      <c r="E184" s="30"/>
-      <c r="F184" s="49"/>
-      <c r="G184" s="31"/>
-      <c r="H184" s="53"/>
+      <c r="B184" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="C184" s="87" t="s">
+        <v>219</v>
+      </c>
+      <c r="D184" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="E184" s="100" t="s">
+        <v>221</v>
+      </c>
+      <c r="F184" s="93" t="s">
+        <v>224</v>
+      </c>
+      <c r="G184" s="94" t="s">
+        <v>28</v>
+      </c>
+      <c r="H184" s="53" t="s">
+        <v>227</v>
+      </c>
       <c r="I184" s="51"/>
-      <c r="J184" s="48"/>
+      <c r="J184" s="48">
+        <v>8.5500000000000007</v>
+      </c>
       <c r="K184" s="36"/>
-      <c r="L184" s="31"/>
-      <c r="M184" s="46"/>
-      <c r="N184" s="29"/>
+      <c r="L184" s="31" t="s">
+        <v>225</v>
+      </c>
+      <c r="M184" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="N184" s="29" t="s">
+        <v>226</v>
+      </c>
       <c r="O184" s="35"/>
       <c r="P184" s="35"/>
       <c r="Q184" s="36"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.actbio.2013.01.029`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A81F2B0C-72B6-3A44-B636-B4DDDDF72737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5531EBD3-9BF8-9048-BA9C-38413339DCCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="12140" windowWidth="34560" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2063" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="254">
   <si>
     <r>
       <rPr>
@@ -868,6 +868,30 @@
   </si>
   <si>
     <t>10.1016/j.ijrmhm.2026.107954</t>
+  </si>
+  <si>
+    <t>Ca20 Mg20 Zn20 Sr20 Yb20</t>
+  </si>
+  <si>
+    <t>VIM+RS</t>
+  </si>
+  <si>
+    <t>BMG designed for biocompatibility</t>
+  </si>
+  <si>
+    <t>1e-4 strain rate</t>
+  </si>
+  <si>
+    <t>youngs modulus</t>
+  </si>
+  <si>
+    <t>shear modulus</t>
+  </si>
+  <si>
+    <t>bulk modulus</t>
+  </si>
+  <si>
+    <t>10.1016/j.actbio.2013.01.029</t>
   </si>
 </sst>
 </file>
@@ -13303,19 +13327,45 @@
     </row>
     <row r="215" spans="1:20" ht="18" customHeight="1">
       <c r="A215" s="38"/>
-      <c r="B215" s="30"/>
-      <c r="C215" s="29"/>
-      <c r="D215" s="29"/>
-      <c r="E215" s="30"/>
-      <c r="F215" s="92"/>
-      <c r="G215" s="31"/>
-      <c r="H215" s="52"/>
-      <c r="I215" s="50"/>
-      <c r="J215" s="84"/>
-      <c r="K215" s="47"/>
-      <c r="L215" s="38"/>
-      <c r="M215" s="38"/>
-      <c r="N215" s="29"/>
+      <c r="B215" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="C215" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D215" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="E215" s="30" t="s">
+        <v>248</v>
+      </c>
+      <c r="F215" s="92" t="s">
+        <v>125</v>
+      </c>
+      <c r="G215" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H215" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="I215" s="50">
+        <v>298</v>
+      </c>
+      <c r="J215" s="84">
+        <v>370700000</v>
+      </c>
+      <c r="K215" s="47">
+        <v>25400000</v>
+      </c>
+      <c r="L215" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M215" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N215" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O215" s="35"/>
       <c r="P215" s="41"/>
       <c r="Q215" s="41"/>
@@ -13325,19 +13375,45 @@
     </row>
     <row r="216" spans="1:20" ht="18" customHeight="1">
       <c r="A216" s="105"/>
-      <c r="B216" s="97"/>
-      <c r="C216" s="85"/>
-      <c r="D216" s="85"/>
-      <c r="E216" s="97"/>
-      <c r="F216" s="49"/>
-      <c r="G216" s="31"/>
-      <c r="H216" s="52"/>
-      <c r="I216" s="50"/>
-      <c r="J216" s="84"/>
-      <c r="K216" s="47"/>
-      <c r="L216" s="38"/>
-      <c r="M216" s="38"/>
-      <c r="N216" s="29"/>
+      <c r="B216" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="C216" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D216" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="E216" s="30" t="s">
+        <v>248</v>
+      </c>
+      <c r="F216" s="49" t="s">
+        <v>250</v>
+      </c>
+      <c r="G216" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H216" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="I216" s="50">
+        <v>298</v>
+      </c>
+      <c r="J216" s="84">
+        <v>19400000000</v>
+      </c>
+      <c r="K216" s="47">
+        <v>3400000000</v>
+      </c>
+      <c r="L216" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M216" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N216" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O216" s="35"/>
       <c r="P216" s="41"/>
       <c r="Q216" s="41"/>
@@ -13347,19 +13423,45 @@
     </row>
     <row r="217" spans="1:20" ht="18" customHeight="1">
       <c r="A217" s="106"/>
-      <c r="B217" s="99"/>
-      <c r="C217" s="86"/>
-      <c r="D217" s="86"/>
-      <c r="E217" s="99"/>
-      <c r="F217" s="49"/>
-      <c r="G217" s="31"/>
-      <c r="H217" s="52"/>
-      <c r="I217" s="50"/>
-      <c r="J217" s="84"/>
-      <c r="K217" s="47"/>
-      <c r="L217" s="38"/>
-      <c r="M217" s="38"/>
-      <c r="N217" s="29"/>
+      <c r="B217" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="C217" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D217" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="E217" s="30" t="s">
+        <v>248</v>
+      </c>
+      <c r="F217" s="49" t="s">
+        <v>251</v>
+      </c>
+      <c r="G217" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H217" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="I217" s="50">
+        <v>298</v>
+      </c>
+      <c r="J217" s="84">
+        <v>7600000000</v>
+      </c>
+      <c r="K217" s="47">
+        <v>1300000000</v>
+      </c>
+      <c r="L217" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M217" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N217" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O217" s="41"/>
       <c r="P217" s="41"/>
       <c r="Q217" s="41"/>
@@ -13369,19 +13471,45 @@
     </row>
     <row r="218" spans="1:20" ht="18" customHeight="1">
       <c r="A218" s="106"/>
-      <c r="B218" s="99"/>
-      <c r="C218" s="86"/>
-      <c r="D218" s="86"/>
-      <c r="E218" s="99"/>
-      <c r="F218" s="49"/>
-      <c r="G218" s="31"/>
-      <c r="H218" s="52"/>
-      <c r="I218" s="50"/>
-      <c r="J218" s="84"/>
-      <c r="K218" s="36"/>
-      <c r="L218" s="38"/>
-      <c r="M218" s="38"/>
-      <c r="N218" s="29"/>
+      <c r="B218" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="C218" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D218" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="E218" s="30" t="s">
+        <v>248</v>
+      </c>
+      <c r="F218" s="49" t="s">
+        <v>252</v>
+      </c>
+      <c r="G218" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H218" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="I218" s="50">
+        <v>298</v>
+      </c>
+      <c r="J218" s="84">
+        <v>15000000000</v>
+      </c>
+      <c r="K218" s="47">
+        <v>2600000000</v>
+      </c>
+      <c r="L218" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M218" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N218" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O218" s="41"/>
       <c r="P218" s="41"/>
       <c r="Q218" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.cjph.2024.09.021`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5531EBD3-9BF8-9048-BA9C-38413339DCCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C7FFE8-5747-9B41-BDFB-6E2B0D44319C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2103" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="259">
   <si>
     <r>
       <rPr>
@@ -876,9 +876,6 @@
     <t>VIM+RS</t>
   </si>
   <si>
-    <t>BMG designed for biocompatibility</t>
-  </si>
-  <si>
     <t>1e-4 strain rate</t>
   </si>
   <si>
@@ -892,6 +889,24 @@
   </si>
   <si>
     <t>10.1016/j.actbio.2013.01.029</t>
+  </si>
+  <si>
+    <t>10.1016/j.cjph.2024.09.021</t>
+  </si>
+  <si>
+    <t>Gd20 Tb20 Er20 Al20 Fe20</t>
+  </si>
+  <si>
+    <t>Gd20 Tb20 Er20 Al20 Co20</t>
+  </si>
+  <si>
+    <t>VAM+VIM+MS</t>
+  </si>
+  <si>
+    <t>BMG designed for magnetocaloric applications; surface layer of ingot removed and then melt spun at 30m/s onto copper resulting in 4mm width and 30um thickness</t>
+  </si>
+  <si>
+    <t>BMG designed for biocompatibility; rapidly solidified into liquid nitrogen copper mold</t>
   </si>
 </sst>
 </file>
@@ -13337,7 +13352,7 @@
         <v>247</v>
       </c>
       <c r="E215" s="30" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="F215" s="92" t="s">
         <v>125</v>
@@ -13346,7 +13361,7 @@
         <v>28</v>
       </c>
       <c r="H215" s="52" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I215" s="50">
         <v>298</v>
@@ -13364,7 +13379,7 @@
         <v>214</v>
       </c>
       <c r="N215" s="29" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O215" s="35"/>
       <c r="P215" s="41"/>
@@ -13385,16 +13400,16 @@
         <v>247</v>
       </c>
       <c r="E216" s="30" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="F216" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G216" s="31" t="s">
         <v>28</v>
       </c>
       <c r="H216" s="52" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I216" s="50">
         <v>298</v>
@@ -13412,7 +13427,7 @@
         <v>214</v>
       </c>
       <c r="N216" s="29" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O216" s="35"/>
       <c r="P216" s="41"/>
@@ -13433,16 +13448,16 @@
         <v>247</v>
       </c>
       <c r="E217" s="30" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="F217" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G217" s="31" t="s">
         <v>28</v>
       </c>
       <c r="H217" s="52" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I217" s="50">
         <v>298</v>
@@ -13460,7 +13475,7 @@
         <v>214</v>
       </c>
       <c r="N217" s="29" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O217" s="41"/>
       <c r="P217" s="41"/>
@@ -13481,16 +13496,16 @@
         <v>247</v>
       </c>
       <c r="E218" s="30" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="F218" s="49" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G218" s="31" t="s">
         <v>28</v>
       </c>
       <c r="H218" s="52" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I218" s="50">
         <v>298</v>
@@ -13508,7 +13523,7 @@
         <v>214</v>
       </c>
       <c r="N218" s="29" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="O218" s="41"/>
       <c r="P218" s="41"/>
@@ -13519,19 +13534,41 @@
     </row>
     <row r="219" spans="1:20" ht="18" customHeight="1">
       <c r="A219" s="106"/>
-      <c r="B219" s="99"/>
-      <c r="C219" s="86"/>
-      <c r="D219" s="86"/>
-      <c r="E219" s="99"/>
-      <c r="F219" s="49"/>
-      <c r="G219" s="31"/>
-      <c r="H219" s="52"/>
+      <c r="B219" s="99" t="s">
+        <v>254</v>
+      </c>
+      <c r="C219" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D219" s="86" t="s">
+        <v>256</v>
+      </c>
+      <c r="E219" s="99" t="s">
+        <v>257</v>
+      </c>
+      <c r="F219" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G219" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H219" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I219" s="50"/>
-      <c r="J219" s="41"/>
+      <c r="J219" s="41">
+        <v>92</v>
+      </c>
       <c r="K219" s="36"/>
-      <c r="L219" s="38"/>
-      <c r="M219" s="38"/>
-      <c r="N219" s="29"/>
+      <c r="L219" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M219" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N219" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O219" s="41"/>
       <c r="P219" s="41"/>
       <c r="Q219" s="41"/>
@@ -13541,19 +13578,41 @@
     </row>
     <row r="220" spans="1:20" ht="18" customHeight="1">
       <c r="A220" s="106"/>
-      <c r="B220" s="99"/>
-      <c r="C220" s="86"/>
-      <c r="D220" s="86"/>
-      <c r="E220" s="99"/>
-      <c r="F220" s="49"/>
-      <c r="G220" s="31"/>
-      <c r="H220" s="52"/>
+      <c r="B220" s="99" t="s">
+        <v>255</v>
+      </c>
+      <c r="C220" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D220" s="86" t="s">
+        <v>256</v>
+      </c>
+      <c r="E220" s="99" t="s">
+        <v>257</v>
+      </c>
+      <c r="F220" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G220" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H220" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I220" s="50"/>
-      <c r="J220" s="41"/>
+      <c r="J220" s="41">
+        <v>51</v>
+      </c>
       <c r="K220" s="36"/>
-      <c r="L220" s="38"/>
-      <c r="M220" s="38"/>
-      <c r="N220" s="29"/>
+      <c r="L220" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M220" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N220" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O220" s="41"/>
       <c r="P220" s="41"/>
       <c r="Q220" s="41"/>
@@ -13563,19 +13622,41 @@
     </row>
     <row r="221" spans="1:20" ht="18" customHeight="1">
       <c r="A221" s="106"/>
-      <c r="B221" s="99"/>
-      <c r="C221" s="86"/>
-      <c r="D221" s="86"/>
-      <c r="E221" s="99"/>
-      <c r="F221" s="49"/>
-      <c r="G221" s="31"/>
-      <c r="H221" s="52"/>
+      <c r="B221" s="99" t="s">
+        <v>254</v>
+      </c>
+      <c r="C221" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D221" s="86" t="s">
+        <v>256</v>
+      </c>
+      <c r="E221" s="99" t="s">
+        <v>257</v>
+      </c>
+      <c r="F221" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G221" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H221" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I221" s="50"/>
-      <c r="J221" s="41"/>
+      <c r="J221" s="41">
+        <v>5.87</v>
+      </c>
       <c r="K221" s="36"/>
-      <c r="L221" s="38"/>
-      <c r="M221" s="38"/>
-      <c r="N221" s="29"/>
+      <c r="L221" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M221" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N221" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O221" s="41"/>
       <c r="P221" s="41"/>
       <c r="Q221" s="41"/>
@@ -13585,19 +13666,41 @@
     </row>
     <row r="222" spans="1:20" ht="18" customHeight="1">
       <c r="A222" s="106"/>
-      <c r="B222" s="99"/>
-      <c r="C222" s="86"/>
-      <c r="D222" s="86"/>
-      <c r="E222" s="99"/>
-      <c r="F222" s="49"/>
-      <c r="G222" s="31"/>
-      <c r="H222" s="52"/>
+      <c r="B222" s="99" t="s">
+        <v>255</v>
+      </c>
+      <c r="C222" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D222" s="86" t="s">
+        <v>256</v>
+      </c>
+      <c r="E222" s="99" t="s">
+        <v>257</v>
+      </c>
+      <c r="F222" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G222" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H222" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I222" s="50"/>
-      <c r="J222" s="41"/>
+      <c r="J222" s="41">
+        <v>7.66</v>
+      </c>
       <c r="K222" s="36"/>
-      <c r="L222" s="38"/>
-      <c r="M222" s="38"/>
-      <c r="N222" s="29"/>
+      <c r="L222" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M222" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N222" s="29" t="s">
+        <v>253</v>
+      </c>
       <c r="O222" s="41"/>
       <c r="P222" s="41"/>
       <c r="Q222" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.intermet.2018.03.002`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C7FFE8-5747-9B41-BDFB-6E2B0D44319C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA67AF5-17FA-8B46-96E8-A7031DF230BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2233" uniqueCount="267">
   <si>
     <r>
       <rPr>
@@ -907,6 +907,30 @@
   </si>
   <si>
     <t>BMG designed for biocompatibility; rapidly solidified into liquid nitrogen copper mold</t>
+  </si>
+  <si>
+    <t>AAM+SC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAM and scution cast into 1.5mm diameter copper mold </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAM and scution cast into 1mm diameter copper mold </t>
+  </si>
+  <si>
+    <t>Er20 Dy20 Co20 Al20 Gd20</t>
+  </si>
+  <si>
+    <t>Er20 Dy20 Co20 Al20 Tb20</t>
+  </si>
+  <si>
+    <t>Er20 Dy20 Co20 Al20 Tm20</t>
+  </si>
+  <si>
+    <t>glass transition temperature</t>
+  </si>
+  <si>
+    <t>10.1016/j.intermet.2018.03.002</t>
   </si>
 </sst>
 </file>
@@ -13710,19 +13734,41 @@
     </row>
     <row r="223" spans="1:20" ht="18" customHeight="1">
       <c r="A223" s="106"/>
-      <c r="B223" s="99"/>
-      <c r="C223" s="86"/>
-      <c r="D223" s="86"/>
-      <c r="E223" s="99"/>
-      <c r="F223" s="49"/>
-      <c r="G223" s="31"/>
-      <c r="H223" s="52"/>
+      <c r="B223" s="99" t="s">
+        <v>262</v>
+      </c>
+      <c r="C223" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D223" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E223" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F223" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G223" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H223" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I223" s="50"/>
-      <c r="J223" s="41"/>
+      <c r="J223" s="41">
+        <v>43</v>
+      </c>
       <c r="K223" s="36"/>
-      <c r="L223" s="38"/>
-      <c r="M223" s="38"/>
-      <c r="N223" s="29"/>
+      <c r="L223" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M223" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N223" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O223" s="41"/>
       <c r="P223" s="41"/>
       <c r="Q223" s="41"/>
@@ -13732,19 +13778,41 @@
     </row>
     <row r="224" spans="1:20" ht="18" customHeight="1">
       <c r="A224" s="105"/>
-      <c r="B224" s="97"/>
-      <c r="C224" s="85"/>
-      <c r="D224" s="85"/>
-      <c r="E224" s="97"/>
-      <c r="F224" s="49"/>
-      <c r="G224" s="31"/>
-      <c r="H224" s="52"/>
+      <c r="B224" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="C224" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D224" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E224" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F224" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G224" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H224" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I224" s="50"/>
-      <c r="J224" s="41"/>
+      <c r="J224" s="41">
+        <v>29</v>
+      </c>
       <c r="K224" s="36"/>
-      <c r="L224" s="38"/>
-      <c r="M224" s="38"/>
-      <c r="N224" s="29"/>
+      <c r="L224" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M224" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N224" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O224" s="41"/>
       <c r="P224" s="41"/>
       <c r="Q224" s="41"/>
@@ -13754,19 +13822,41 @@
     </row>
     <row r="225" spans="1:20" ht="18" customHeight="1">
       <c r="A225" s="106"/>
-      <c r="B225" s="99"/>
-      <c r="C225" s="86"/>
-      <c r="D225" s="86"/>
-      <c r="E225" s="99"/>
-      <c r="F225" s="49"/>
-      <c r="G225" s="31"/>
-      <c r="H225" s="52"/>
+      <c r="B225" s="99" t="s">
+        <v>264</v>
+      </c>
+      <c r="C225" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D225" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E225" s="99" t="s">
+        <v>261</v>
+      </c>
+      <c r="F225" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G225" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H225" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I225" s="50"/>
-      <c r="J225" s="41"/>
+      <c r="J225" s="41">
+        <v>13</v>
+      </c>
       <c r="K225" s="36"/>
-      <c r="L225" s="38"/>
-      <c r="M225" s="38"/>
-      <c r="N225" s="29"/>
+      <c r="L225" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M225" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N225" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O225" s="41"/>
       <c r="P225" s="41"/>
       <c r="Q225" s="41"/>
@@ -13776,19 +13866,41 @@
     </row>
     <row r="226" spans="1:20" ht="18" customHeight="1">
       <c r="A226" s="106"/>
-      <c r="B226" s="99"/>
-      <c r="C226" s="86"/>
-      <c r="D226" s="86"/>
-      <c r="E226" s="99"/>
-      <c r="F226" s="49"/>
-      <c r="G226" s="31"/>
-      <c r="H226" s="52"/>
+      <c r="B226" s="99" t="s">
+        <v>262</v>
+      </c>
+      <c r="C226" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D226" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E226" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F226" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G226" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H226" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I226" s="50"/>
-      <c r="J226" s="41"/>
+      <c r="J226" s="41">
+        <v>610</v>
+      </c>
       <c r="K226" s="36"/>
-      <c r="L226" s="38"/>
-      <c r="M226" s="38"/>
-      <c r="N226" s="29"/>
+      <c r="L226" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M226" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N226" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O226" s="41"/>
       <c r="P226" s="41"/>
       <c r="Q226" s="41"/>
@@ -13798,19 +13910,41 @@
     </row>
     <row r="227" spans="1:20" ht="18" customHeight="1">
       <c r="A227" s="106"/>
-      <c r="B227" s="99"/>
-      <c r="C227" s="86"/>
-      <c r="D227" s="86"/>
-      <c r="E227" s="99"/>
-      <c r="F227" s="49"/>
-      <c r="G227" s="31"/>
-      <c r="H227" s="52"/>
+      <c r="B227" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="C227" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D227" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E227" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F227" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G227" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H227" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I227" s="50"/>
-      <c r="J227" s="41"/>
+      <c r="J227" s="41">
+        <v>623</v>
+      </c>
       <c r="K227" s="36"/>
-      <c r="L227" s="38"/>
-      <c r="M227" s="38"/>
-      <c r="N227" s="29"/>
+      <c r="L227" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M227" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N227" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O227" s="41"/>
       <c r="P227" s="41"/>
       <c r="Q227" s="41"/>
@@ -13820,19 +13954,41 @@
     </row>
     <row r="228" spans="1:20" ht="18" customHeight="1">
       <c r="A228" s="106"/>
-      <c r="B228" s="99"/>
-      <c r="C228" s="86"/>
-      <c r="D228" s="86"/>
-      <c r="E228" s="99"/>
-      <c r="F228" s="49"/>
-      <c r="G228" s="31"/>
-      <c r="H228" s="52"/>
+      <c r="B228" s="99" t="s">
+        <v>264</v>
+      </c>
+      <c r="C228" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D228" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E228" s="99" t="s">
+        <v>261</v>
+      </c>
+      <c r="F228" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G228" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H228" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I228" s="50"/>
-      <c r="J228" s="41"/>
+      <c r="J228" s="41">
+        <v>645</v>
+      </c>
       <c r="K228" s="36"/>
-      <c r="L228" s="38"/>
-      <c r="M228" s="38"/>
-      <c r="N228" s="29"/>
+      <c r="L228" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M228" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N228" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O228" s="41"/>
       <c r="P228" s="41"/>
       <c r="Q228" s="41"/>
@@ -13842,19 +13998,41 @@
     </row>
     <row r="229" spans="1:20" ht="18" customHeight="1">
       <c r="A229" s="106"/>
-      <c r="B229" s="99"/>
-      <c r="C229" s="86"/>
-      <c r="D229" s="86"/>
-      <c r="E229" s="99"/>
-      <c r="F229" s="49"/>
-      <c r="G229" s="31"/>
-      <c r="H229" s="52"/>
+      <c r="B229" s="99" t="s">
+        <v>262</v>
+      </c>
+      <c r="C229" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D229" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E229" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F229" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G229" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H229" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I229" s="50"/>
-      <c r="J229" s="41"/>
+      <c r="J229" s="41">
+        <v>9.1</v>
+      </c>
       <c r="K229" s="36"/>
-      <c r="L229" s="38"/>
-      <c r="M229" s="38"/>
-      <c r="N229" s="29"/>
+      <c r="L229" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M229" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N229" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O229" s="41"/>
       <c r="P229" s="41"/>
       <c r="Q229" s="41"/>
@@ -13864,19 +14042,41 @@
     </row>
     <row r="230" spans="1:20" ht="18" customHeight="1">
       <c r="A230" s="106"/>
-      <c r="B230" s="99"/>
-      <c r="C230" s="86"/>
-      <c r="D230" s="86"/>
-      <c r="E230" s="99"/>
-      <c r="F230" s="49"/>
-      <c r="G230" s="31"/>
-      <c r="H230" s="52"/>
+      <c r="B230" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="C230" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D230" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E230" s="99" t="s">
+        <v>260</v>
+      </c>
+      <c r="F230" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G230" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H230" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I230" s="50"/>
-      <c r="J230" s="41"/>
+      <c r="J230" s="41">
+        <v>8.6</v>
+      </c>
       <c r="K230" s="36"/>
-      <c r="L230" s="38"/>
-      <c r="M230" s="38"/>
-      <c r="N230" s="29"/>
+      <c r="L230" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M230" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N230" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O230" s="41"/>
       <c r="P230" s="41"/>
       <c r="Q230" s="41"/>
@@ -13886,19 +14086,41 @@
     </row>
     <row r="231" spans="1:20" ht="18" customHeight="1">
       <c r="A231" s="106"/>
-      <c r="B231" s="99"/>
-      <c r="C231" s="86"/>
-      <c r="D231" s="86"/>
-      <c r="E231" s="99"/>
-      <c r="F231" s="49"/>
-      <c r="G231" s="31"/>
-      <c r="H231" s="52"/>
+      <c r="B231" s="99" t="s">
+        <v>264</v>
+      </c>
+      <c r="C231" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="D231" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E231" s="99" t="s">
+        <v>261</v>
+      </c>
+      <c r="F231" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G231" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H231" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I231" s="50"/>
-      <c r="J231" s="33"/>
+      <c r="J231" s="33">
+        <v>11.9</v>
+      </c>
       <c r="K231" s="36"/>
-      <c r="L231" s="38"/>
-      <c r="M231" s="38"/>
-      <c r="N231" s="29"/>
+      <c r="L231" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M231" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N231" s="29" t="s">
+        <v>266</v>
+      </c>
       <c r="O231" s="41"/>
       <c r="P231" s="41"/>
       <c r="Q231" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jallcom.2018.10.328`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA67AF5-17FA-8B46-96E8-A7031DF230BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C945E070-B66B-EB4E-A4E5-037413A81728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2233" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2263" uniqueCount="271">
   <si>
     <r>
       <rPr>
@@ -931,6 +931,18 @@
   </si>
   <si>
     <t>10.1016/j.intermet.2018.03.002</t>
+  </si>
+  <si>
+    <t>Gd10 Tb10 Dy10 Ho10 Er10 Y10 Ni10 Co10 Ag10 Al10</t>
+  </si>
+  <si>
+    <t>AAM+MS</t>
+  </si>
+  <si>
+    <t>denary HEMG</t>
+  </si>
+  <si>
+    <t>10.1016/j.jallcom.2018.10.328</t>
   </si>
 </sst>
 </file>
@@ -14130,19 +14142,41 @@
     </row>
     <row r="232" spans="1:20" ht="18" customHeight="1">
       <c r="A232" s="105"/>
-      <c r="B232" s="97"/>
-      <c r="C232" s="85"/>
-      <c r="D232" s="85"/>
-      <c r="E232" s="97"/>
-      <c r="F232" s="49"/>
-      <c r="G232" s="31"/>
-      <c r="H232" s="52"/>
+      <c r="B232" s="97" t="s">
+        <v>267</v>
+      </c>
+      <c r="C232" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D232" s="85" t="s">
+        <v>268</v>
+      </c>
+      <c r="E232" s="97" t="s">
+        <v>269</v>
+      </c>
+      <c r="F232" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G232" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H232" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I232" s="50"/>
-      <c r="J232" s="33"/>
+      <c r="J232" s="33">
+        <v>29</v>
+      </c>
       <c r="K232" s="36"/>
-      <c r="L232" s="38"/>
-      <c r="M232" s="38"/>
-      <c r="N232" s="29"/>
+      <c r="L232" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M232" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N232" s="29" t="s">
+        <v>270</v>
+      </c>
       <c r="O232" s="41"/>
       <c r="P232" s="41"/>
       <c r="Q232" s="41"/>
@@ -14152,19 +14186,41 @@
     </row>
     <row r="233" spans="1:20" ht="18" customHeight="1">
       <c r="A233" s="106"/>
-      <c r="B233" s="99"/>
-      <c r="C233" s="86"/>
-      <c r="D233" s="86"/>
-      <c r="E233" s="99"/>
-      <c r="F233" s="49"/>
-      <c r="G233" s="31"/>
-      <c r="H233" s="52"/>
+      <c r="B233" s="97" t="s">
+        <v>267</v>
+      </c>
+      <c r="C233" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D233" s="85" t="s">
+        <v>268</v>
+      </c>
+      <c r="E233" s="97" t="s">
+        <v>269</v>
+      </c>
+      <c r="F233" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G233" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H233" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I233" s="50"/>
-      <c r="J233" s="33"/>
+      <c r="J233" s="33">
+        <v>597</v>
+      </c>
       <c r="K233" s="36"/>
-      <c r="L233" s="38"/>
-      <c r="M233" s="38"/>
-      <c r="N233" s="29"/>
+      <c r="L233" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M233" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N233" s="29" t="s">
+        <v>270</v>
+      </c>
       <c r="O233" s="41"/>
       <c r="P233" s="41"/>
       <c r="Q233" s="41"/>
@@ -14174,19 +14230,41 @@
     </row>
     <row r="234" spans="1:20" ht="18" customHeight="1">
       <c r="A234" s="106"/>
-      <c r="B234" s="99"/>
-      <c r="C234" s="86"/>
-      <c r="D234" s="86"/>
-      <c r="E234" s="99"/>
-      <c r="F234" s="49"/>
-      <c r="G234" s="31"/>
-      <c r="H234" s="52"/>
+      <c r="B234" s="97" t="s">
+        <v>267</v>
+      </c>
+      <c r="C234" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D234" s="85" t="s">
+        <v>268</v>
+      </c>
+      <c r="E234" s="97" t="s">
+        <v>269</v>
+      </c>
+      <c r="F234" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="G234" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H234" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I234" s="50"/>
-      <c r="J234" s="33"/>
+      <c r="J234" s="33">
+        <v>10.64</v>
+      </c>
       <c r="K234" s="36"/>
-      <c r="L234" s="38"/>
-      <c r="M234" s="38"/>
-      <c r="N234" s="29"/>
+      <c r="L234" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M234" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N234" s="29" t="s">
+        <v>270</v>
+      </c>
       <c r="O234" s="41"/>
       <c r="P234" s="41"/>
       <c r="Q234" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jallcom.2020.154101`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C945E070-B66B-EB4E-A4E5-037413A81728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A021E5C2-0366-2742-BA67-1FA45D7DF366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2263" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="278">
   <si>
     <r>
       <rPr>
@@ -943,6 +943,27 @@
   </si>
   <si>
     <t>10.1016/j.jallcom.2018.10.328</t>
+  </si>
+  <si>
+    <t>Gd25 Co25 Al25 Y25</t>
+  </si>
+  <si>
+    <t>Gd25 Co25 Al25 Y15 Dy10</t>
+  </si>
+  <si>
+    <t>Gd25 Co25 Al25 Y15 Ho10</t>
+  </si>
+  <si>
+    <t>Gd25 Co25 Al25 Y15 Er10</t>
+  </si>
+  <si>
+    <t>melt spun into 2mm ribbons with 30um thickness</t>
+  </si>
+  <si>
+    <t>suction cast into 1mm diameter rods; made and tested with XRD to contrast structure with ribbons finding no major changes but dual peak DSC curve</t>
+  </si>
+  <si>
+    <t>10.1016/j.jallcom.2020.154101</t>
   </si>
 </sst>
 </file>
@@ -1966,7 +1987,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2282,6 +2303,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3444,7 +3468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T960"/>
+  <dimension ref="A1:T959"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.1640625" style="1" customWidth="1"/>
@@ -14274,10 +14298,18 @@
     </row>
     <row r="235" spans="1:20" ht="18" customHeight="1">
       <c r="A235" s="106"/>
-      <c r="B235" s="99"/>
-      <c r="C235" s="86"/>
-      <c r="D235" s="86"/>
-      <c r="E235" s="99"/>
+      <c r="B235" s="99" t="s">
+        <v>272</v>
+      </c>
+      <c r="C235" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D235" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E235" s="99" t="s">
+        <v>276</v>
+      </c>
       <c r="F235" s="49"/>
       <c r="G235" s="31"/>
       <c r="H235" s="52"/>
@@ -14286,7 +14318,9 @@
       <c r="K235" s="36"/>
       <c r="L235" s="38"/>
       <c r="M235" s="38"/>
-      <c r="N235" s="29"/>
+      <c r="N235" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O235" s="41"/>
       <c r="P235" s="41"/>
       <c r="Q235" s="41"/>
@@ -14296,10 +14330,18 @@
     </row>
     <row r="236" spans="1:20" ht="18" customHeight="1">
       <c r="A236" s="106"/>
-      <c r="B236" s="99"/>
-      <c r="C236" s="86"/>
-      <c r="D236" s="86"/>
-      <c r="E236" s="99"/>
+      <c r="B236" s="99" t="s">
+        <v>273</v>
+      </c>
+      <c r="C236" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D236" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E236" s="99" t="s">
+        <v>276</v>
+      </c>
       <c r="F236" s="49"/>
       <c r="G236" s="31"/>
       <c r="H236" s="52"/>
@@ -14308,7 +14350,9 @@
       <c r="K236" s="36"/>
       <c r="L236" s="38"/>
       <c r="M236" s="38"/>
-      <c r="N236" s="29"/>
+      <c r="N236" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O236" s="41"/>
       <c r="P236" s="41"/>
       <c r="Q236" s="41"/>
@@ -14318,10 +14362,18 @@
     </row>
     <row r="237" spans="1:20" ht="18" customHeight="1">
       <c r="A237" s="106"/>
-      <c r="B237" s="99"/>
-      <c r="C237" s="86"/>
-      <c r="D237" s="86"/>
-      <c r="E237" s="99"/>
+      <c r="B237" s="99" t="s">
+        <v>274</v>
+      </c>
+      <c r="C237" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D237" s="86" t="s">
+        <v>259</v>
+      </c>
+      <c r="E237" s="99" t="s">
+        <v>276</v>
+      </c>
       <c r="F237" s="49"/>
       <c r="G237" s="31"/>
       <c r="H237" s="52"/>
@@ -14330,29 +14382,53 @@
       <c r="K237" s="36"/>
       <c r="L237" s="38"/>
       <c r="M237" s="38"/>
-      <c r="N237" s="29"/>
+      <c r="N237" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O237" s="41"/>
       <c r="P237" s="41"/>
       <c r="Q237" s="41"/>
-      <c r="R237" s="35"/>
+      <c r="R237" s="41"/>
       <c r="S237" s="35"/>
       <c r="T237" s="35"/>
     </row>
     <row r="238" spans="1:20" ht="18" customHeight="1">
       <c r="A238" s="106"/>
-      <c r="B238" s="99"/>
-      <c r="C238" s="86"/>
-      <c r="D238" s="86"/>
-      <c r="E238" s="99"/>
-      <c r="F238" s="49"/>
-      <c r="G238" s="31"/>
-      <c r="H238" s="52"/>
+      <c r="B238" s="99" t="s">
+        <v>271</v>
+      </c>
+      <c r="C238" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D238" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E238" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F238" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G238" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H238" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I238" s="50"/>
-      <c r="J238" s="33"/>
+      <c r="J238" s="38">
+        <v>39</v>
+      </c>
       <c r="K238" s="36"/>
-      <c r="L238" s="38"/>
-      <c r="M238" s="38"/>
-      <c r="N238" s="29"/>
+      <c r="L238" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M238" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N238" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O238" s="41"/>
       <c r="P238" s="41"/>
       <c r="Q238" s="41"/>
@@ -14361,20 +14437,42 @@
       <c r="T238" s="35"/>
     </row>
     <row r="239" spans="1:20" ht="18" customHeight="1">
-      <c r="A239" s="106"/>
-      <c r="B239" s="99"/>
-      <c r="C239" s="86"/>
-      <c r="D239" s="86"/>
-      <c r="E239" s="99"/>
-      <c r="F239" s="49"/>
-      <c r="G239" s="31"/>
-      <c r="H239" s="52"/>
+      <c r="A239" s="105"/>
+      <c r="B239" s="99" t="s">
+        <v>272</v>
+      </c>
+      <c r="C239" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D239" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E239" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F239" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G239" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H239" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I239" s="50"/>
-      <c r="J239" s="38"/>
+      <c r="J239" s="38">
+        <v>44</v>
+      </c>
       <c r="K239" s="36"/>
-      <c r="L239" s="38"/>
-      <c r="M239" s="38"/>
-      <c r="N239" s="29"/>
+      <c r="L239" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M239" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N239" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O239" s="41"/>
       <c r="P239" s="41"/>
       <c r="Q239" s="41"/>
@@ -14383,20 +14481,42 @@
       <c r="T239" s="35"/>
     </row>
     <row r="240" spans="1:20" ht="18" customHeight="1">
-      <c r="A240" s="105"/>
-      <c r="B240" s="97"/>
-      <c r="C240" s="85"/>
-      <c r="D240" s="85"/>
-      <c r="E240" s="97"/>
-      <c r="F240" s="49"/>
-      <c r="G240" s="31"/>
-      <c r="H240" s="52"/>
+      <c r="A240" s="106"/>
+      <c r="B240" s="99" t="s">
+        <v>273</v>
+      </c>
+      <c r="C240" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D240" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E240" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F240" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G240" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H240" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I240" s="50"/>
-      <c r="J240" s="38"/>
+      <c r="J240" s="38">
+        <v>41</v>
+      </c>
       <c r="K240" s="36"/>
-      <c r="L240" s="38"/>
-      <c r="M240" s="38"/>
-      <c r="N240" s="29"/>
+      <c r="L240" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M240" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N240" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O240" s="41"/>
       <c r="P240" s="41"/>
       <c r="Q240" s="41"/>
@@ -14406,19 +14526,41 @@
     </row>
     <row r="241" spans="1:20" ht="18" customHeight="1">
       <c r="A241" s="106"/>
-      <c r="B241" s="99"/>
-      <c r="C241" s="86"/>
-      <c r="D241" s="86"/>
-      <c r="E241" s="99"/>
-      <c r="F241" s="49"/>
-      <c r="G241" s="31"/>
-      <c r="H241" s="52"/>
+      <c r="B241" s="99" t="s">
+        <v>274</v>
+      </c>
+      <c r="C241" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D241" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E241" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F241" s="49" t="s">
+        <v>222</v>
+      </c>
+      <c r="G241" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H241" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I241" s="50"/>
-      <c r="J241" s="38"/>
+      <c r="J241" s="38">
+        <v>43</v>
+      </c>
       <c r="K241" s="36"/>
-      <c r="L241" s="38"/>
-      <c r="M241" s="38"/>
-      <c r="N241" s="29"/>
+      <c r="L241" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M241" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N241" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O241" s="41"/>
       <c r="P241" s="41"/>
       <c r="Q241" s="41"/>
@@ -14428,19 +14570,41 @@
     </row>
     <row r="242" spans="1:20" ht="18" customHeight="1">
       <c r="A242" s="106"/>
-      <c r="B242" s="99"/>
-      <c r="C242" s="86"/>
-      <c r="D242" s="86"/>
-      <c r="E242" s="99"/>
-      <c r="F242" s="49"/>
-      <c r="G242" s="31"/>
-      <c r="H242" s="52"/>
+      <c r="B242" s="99" t="s">
+        <v>271</v>
+      </c>
+      <c r="C242" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D242" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E242" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F242" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G242" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H242" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I242" s="50"/>
-      <c r="J242" s="38"/>
+      <c r="J242" s="38">
+        <v>626</v>
+      </c>
       <c r="K242" s="36"/>
-      <c r="L242" s="38"/>
-      <c r="M242" s="38"/>
-      <c r="N242" s="29"/>
+      <c r="L242" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M242" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N242" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O242" s="41"/>
       <c r="P242" s="41"/>
       <c r="Q242" s="41"/>
@@ -14450,19 +14614,41 @@
     </row>
     <row r="243" spans="1:20" ht="18" customHeight="1">
       <c r="A243" s="106"/>
-      <c r="B243" s="99"/>
-      <c r="C243" s="86"/>
-      <c r="D243" s="86"/>
-      <c r="E243" s="99"/>
-      <c r="F243" s="49"/>
-      <c r="G243" s="31"/>
-      <c r="H243" s="52"/>
+      <c r="B243" s="99" t="s">
+        <v>272</v>
+      </c>
+      <c r="C243" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D243" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E243" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F243" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G243" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H243" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I243" s="50"/>
-      <c r="J243" s="38"/>
+      <c r="J243" s="38">
+        <v>628</v>
+      </c>
       <c r="K243" s="36"/>
-      <c r="L243" s="38"/>
-      <c r="M243" s="38"/>
-      <c r="N243" s="29"/>
+      <c r="L243" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M243" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N243" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O243" s="41"/>
       <c r="P243" s="41"/>
       <c r="Q243" s="41"/>
@@ -14472,19 +14658,41 @@
     </row>
     <row r="244" spans="1:20" ht="18" customHeight="1">
       <c r="A244" s="106"/>
-      <c r="B244" s="99"/>
-      <c r="C244" s="86"/>
-      <c r="D244" s="86"/>
-      <c r="E244" s="99"/>
-      <c r="F244" s="49"/>
-      <c r="G244" s="31"/>
-      <c r="H244" s="52"/>
+      <c r="B244" s="99" t="s">
+        <v>273</v>
+      </c>
+      <c r="C244" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D244" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E244" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F244" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G244" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H244" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I244" s="50"/>
-      <c r="J244" s="38"/>
+      <c r="J244" s="38">
+        <v>626</v>
+      </c>
       <c r="K244" s="36"/>
-      <c r="L244" s="38"/>
-      <c r="M244" s="38"/>
-      <c r="N244" s="29"/>
+      <c r="L244" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M244" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N244" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O244" s="41"/>
       <c r="P244" s="41"/>
       <c r="Q244" s="41"/>
@@ -14494,19 +14702,41 @@
     </row>
     <row r="245" spans="1:20" ht="18" customHeight="1">
       <c r="A245" s="106"/>
-      <c r="B245" s="99"/>
-      <c r="C245" s="86"/>
-      <c r="D245" s="86"/>
-      <c r="E245" s="99"/>
-      <c r="F245" s="49"/>
-      <c r="G245" s="31"/>
-      <c r="H245" s="52"/>
+      <c r="B245" s="99" t="s">
+        <v>274</v>
+      </c>
+      <c r="C245" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D245" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E245" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F245" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G245" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H245" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I245" s="50"/>
-      <c r="J245" s="38"/>
+      <c r="J245" s="38">
+        <v>628</v>
+      </c>
       <c r="K245" s="36"/>
-      <c r="L245" s="38"/>
-      <c r="M245" s="38"/>
-      <c r="N245" s="29"/>
+      <c r="L245" s="38" t="s">
+        <v>223</v>
+      </c>
+      <c r="M245" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N245" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O245" s="41"/>
       <c r="P245" s="41"/>
       <c r="Q245" s="41"/>
@@ -14516,41 +14746,85 @@
     </row>
     <row r="246" spans="1:20" ht="18" customHeight="1">
       <c r="A246" s="106"/>
-      <c r="B246" s="99"/>
-      <c r="C246" s="86"/>
-      <c r="D246" s="86"/>
-      <c r="E246" s="99"/>
-      <c r="F246" s="49"/>
-      <c r="G246" s="31"/>
-      <c r="H246" s="52"/>
+      <c r="B246" s="99" t="s">
+        <v>271</v>
+      </c>
+      <c r="C246" s="85" t="s">
+        <v>219</v>
+      </c>
+      <c r="D246" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E246" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F246" s="152" t="s">
+        <v>224</v>
+      </c>
+      <c r="G246" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H246" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I246" s="50"/>
-      <c r="J246" s="38"/>
+      <c r="J246" s="38">
+        <v>6.02</v>
+      </c>
       <c r="K246" s="36"/>
-      <c r="L246" s="38"/>
-      <c r="M246" s="38"/>
-      <c r="N246" s="29"/>
+      <c r="L246" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M246" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N246" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O246" s="41"/>
       <c r="P246" s="41"/>
       <c r="Q246" s="41"/>
       <c r="R246" s="41"/>
       <c r="S246" s="35"/>
-      <c r="T246" s="35"/>
+      <c r="T246" s="41"/>
     </row>
     <row r="247" spans="1:20" ht="18" customHeight="1">
-      <c r="A247" s="106"/>
-      <c r="B247" s="99"/>
-      <c r="C247" s="86"/>
-      <c r="D247" s="86"/>
-      <c r="E247" s="99"/>
-      <c r="F247" s="49"/>
-      <c r="G247" s="31"/>
-      <c r="H247" s="52"/>
+      <c r="A247" s="105"/>
+      <c r="B247" s="99" t="s">
+        <v>272</v>
+      </c>
+      <c r="C247" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D247" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E247" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F247" s="152" t="s">
+        <v>224</v>
+      </c>
+      <c r="G247" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H247" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I247" s="50"/>
-      <c r="J247" s="38"/>
+      <c r="J247" s="38">
+        <v>6.76</v>
+      </c>
       <c r="K247" s="36"/>
-      <c r="L247" s="38"/>
-      <c r="M247" s="38"/>
-      <c r="N247" s="29"/>
+      <c r="L247" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M247" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N247" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O247" s="41"/>
       <c r="P247" s="41"/>
       <c r="Q247" s="41"/>
@@ -14559,20 +14833,42 @@
       <c r="T247" s="41"/>
     </row>
     <row r="248" spans="1:20" ht="18" customHeight="1">
-      <c r="A248" s="105"/>
-      <c r="B248" s="97"/>
-      <c r="C248" s="85"/>
-      <c r="D248" s="85"/>
-      <c r="E248" s="97"/>
-      <c r="F248" s="49"/>
-      <c r="G248" s="31"/>
-      <c r="H248" s="52"/>
+      <c r="A248" s="106"/>
+      <c r="B248" s="99" t="s">
+        <v>273</v>
+      </c>
+      <c r="C248" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D248" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E248" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F248" s="152" t="s">
+        <v>224</v>
+      </c>
+      <c r="G248" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H248" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I248" s="50"/>
-      <c r="J248" s="38"/>
+      <c r="J248" s="38">
+        <v>7.35</v>
+      </c>
       <c r="K248" s="36"/>
-      <c r="L248" s="38"/>
-      <c r="M248" s="38"/>
-      <c r="N248" s="29"/>
+      <c r="L248" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M248" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N248" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O248" s="41"/>
       <c r="P248" s="41"/>
       <c r="Q248" s="41"/>
@@ -14582,25 +14878,47 @@
     </row>
     <row r="249" spans="1:20" ht="18" customHeight="1">
       <c r="A249" s="106"/>
-      <c r="B249" s="99"/>
-      <c r="C249" s="86"/>
-      <c r="D249" s="86"/>
-      <c r="E249" s="99"/>
-      <c r="F249" s="49"/>
-      <c r="G249" s="31"/>
-      <c r="H249" s="52"/>
+      <c r="B249" s="99" t="s">
+        <v>274</v>
+      </c>
+      <c r="C249" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D249" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E249" s="99" t="s">
+        <v>275</v>
+      </c>
+      <c r="F249" s="152" t="s">
+        <v>224</v>
+      </c>
+      <c r="G249" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H249" s="52" t="s">
+        <v>227</v>
+      </c>
       <c r="I249" s="50"/>
-      <c r="J249" s="38"/>
+      <c r="J249" s="38">
+        <v>6.96</v>
+      </c>
       <c r="K249" s="36"/>
-      <c r="L249" s="38"/>
-      <c r="M249" s="38"/>
-      <c r="N249" s="29"/>
+      <c r="L249" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="M249" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="N249" s="29" t="s">
+        <v>277</v>
+      </c>
       <c r="O249" s="41"/>
       <c r="P249" s="41"/>
       <c r="Q249" s="41"/>
       <c r="R249" s="41"/>
       <c r="S249" s="35"/>
-      <c r="T249" s="41"/>
+      <c r="T249" s="35"/>
     </row>
     <row r="250" spans="1:20" ht="18" customHeight="1">
       <c r="A250" s="106"/>
@@ -14713,11 +15031,11 @@
       <c r="T254" s="35"/>
     </row>
     <row r="255" spans="1:20" ht="18" customHeight="1">
-      <c r="A255" s="106"/>
-      <c r="B255" s="99"/>
-      <c r="C255" s="86"/>
-      <c r="D255" s="86"/>
-      <c r="E255" s="99"/>
+      <c r="A255" s="105"/>
+      <c r="B255" s="97"/>
+      <c r="C255" s="85"/>
+      <c r="D255" s="85"/>
+      <c r="E255" s="97"/>
       <c r="F255" s="49"/>
       <c r="G255" s="31"/>
       <c r="H255" s="52"/>
@@ -14735,11 +15053,11 @@
       <c r="T255" s="35"/>
     </row>
     <row r="256" spans="1:20" ht="18" customHeight="1">
-      <c r="A256" s="105"/>
-      <c r="B256" s="97"/>
-      <c r="C256" s="85"/>
-      <c r="D256" s="85"/>
-      <c r="E256" s="97"/>
+      <c r="A256" s="106"/>
+      <c r="B256" s="99"/>
+      <c r="C256" s="86"/>
+      <c r="D256" s="86"/>
+      <c r="E256" s="99"/>
       <c r="F256" s="49"/>
       <c r="G256" s="31"/>
       <c r="H256" s="52"/>
@@ -14876,7 +15194,7 @@
       <c r="G262" s="31"/>
       <c r="H262" s="52"/>
       <c r="I262" s="50"/>
-      <c r="J262" s="38"/>
+      <c r="J262" s="107"/>
       <c r="K262" s="36"/>
       <c r="L262" s="38"/>
       <c r="M262" s="38"/>
@@ -14889,11 +15207,11 @@
       <c r="T262" s="35"/>
     </row>
     <row r="263" spans="1:20" ht="18" customHeight="1">
-      <c r="A263" s="106"/>
-      <c r="B263" s="99"/>
-      <c r="C263" s="86"/>
-      <c r="D263" s="86"/>
-      <c r="E263" s="99"/>
+      <c r="A263" s="53"/>
+      <c r="B263" s="39"/>
+      <c r="C263" s="29"/>
+      <c r="D263" s="29"/>
+      <c r="E263" s="30"/>
       <c r="F263" s="49"/>
       <c r="G263" s="31"/>
       <c r="H263" s="52"/>
@@ -14924,7 +15242,7 @@
       <c r="K264" s="36"/>
       <c r="L264" s="38"/>
       <c r="M264" s="38"/>
-      <c r="N264" s="29"/>
+      <c r="N264" s="38"/>
       <c r="O264" s="41"/>
       <c r="P264" s="41"/>
       <c r="Q264" s="41"/>
@@ -14964,7 +15282,7 @@
       <c r="G266" s="31"/>
       <c r="H266" s="52"/>
       <c r="I266" s="50"/>
-      <c r="J266" s="107"/>
+      <c r="J266" s="33"/>
       <c r="K266" s="36"/>
       <c r="L266" s="38"/>
       <c r="M266" s="38"/>
@@ -14981,7 +15299,7 @@
       <c r="B267" s="39"/>
       <c r="C267" s="29"/>
       <c r="D267" s="29"/>
-      <c r="E267" s="30"/>
+      <c r="E267" s="51"/>
       <c r="F267" s="49"/>
       <c r="G267" s="31"/>
       <c r="H267" s="52"/>
@@ -15008,7 +15326,7 @@
       <c r="G268" s="31"/>
       <c r="H268" s="52"/>
       <c r="I268" s="50"/>
-      <c r="J268" s="33"/>
+      <c r="J268" s="47"/>
       <c r="K268" s="36"/>
       <c r="L268" s="38"/>
       <c r="M268" s="38"/>
@@ -15026,7 +15344,7 @@
       <c r="C269" s="29"/>
       <c r="D269" s="29"/>
       <c r="E269" s="51"/>
-      <c r="F269" s="49"/>
+      <c r="F269" s="53"/>
       <c r="G269" s="31"/>
       <c r="H269" s="52"/>
       <c r="I269" s="50"/>
@@ -15053,7 +15371,7 @@
       <c r="H270" s="52"/>
       <c r="I270" s="50"/>
       <c r="J270" s="47"/>
-      <c r="K270" s="36"/>
+      <c r="K270" s="47"/>
       <c r="L270" s="38"/>
       <c r="M270" s="38"/>
       <c r="N270" s="38"/>
@@ -15097,7 +15415,7 @@
       <c r="H272" s="52"/>
       <c r="I272" s="50"/>
       <c r="J272" s="47"/>
-      <c r="K272" s="47"/>
+      <c r="K272" s="36"/>
       <c r="L272" s="38"/>
       <c r="M272" s="38"/>
       <c r="N272" s="38"/>
@@ -15141,7 +15459,7 @@
       <c r="H274" s="52"/>
       <c r="I274" s="50"/>
       <c r="J274" s="47"/>
-      <c r="K274" s="36"/>
+      <c r="K274" s="41"/>
       <c r="L274" s="38"/>
       <c r="M274" s="38"/>
       <c r="N274" s="38"/>
@@ -15153,10 +15471,10 @@
       <c r="T274" s="35"/>
     </row>
     <row r="275" spans="1:20" ht="18" customHeight="1">
-      <c r="A275" s="53"/>
-      <c r="B275" s="39"/>
-      <c r="C275" s="29"/>
-      <c r="D275" s="29"/>
+      <c r="A275" s="88"/>
+      <c r="B275" s="97"/>
+      <c r="C275" s="85"/>
+      <c r="D275" s="85"/>
       <c r="E275" s="51"/>
       <c r="F275" s="53"/>
       <c r="G275" s="31"/>
@@ -15175,21 +15493,21 @@
       <c r="T275" s="35"/>
     </row>
     <row r="276" spans="1:20" ht="18" customHeight="1">
-      <c r="A276" s="88"/>
-      <c r="B276" s="97"/>
-      <c r="C276" s="85"/>
-      <c r="D276" s="85"/>
+      <c r="A276" s="90"/>
+      <c r="B276" s="99"/>
+      <c r="C276" s="86"/>
+      <c r="D276" s="86"/>
       <c r="E276" s="51"/>
       <c r="F276" s="53"/>
       <c r="G276" s="31"/>
       <c r="H276" s="52"/>
       <c r="I276" s="50"/>
-      <c r="J276" s="47"/>
+      <c r="J276" s="41"/>
       <c r="K276" s="41"/>
-      <c r="L276" s="38"/>
-      <c r="M276" s="38"/>
+      <c r="L276" s="53"/>
+      <c r="M276" s="53"/>
       <c r="N276" s="38"/>
-      <c r="O276" s="41"/>
+      <c r="O276" s="87"/>
       <c r="P276" s="41"/>
       <c r="Q276" s="41"/>
       <c r="R276" s="41"/>
@@ -15211,7 +15529,7 @@
       <c r="L277" s="53"/>
       <c r="M277" s="53"/>
       <c r="N277" s="38"/>
-      <c r="O277" s="87"/>
+      <c r="O277" s="41"/>
       <c r="P277" s="41"/>
       <c r="Q277" s="41"/>
       <c r="R277" s="41"/>
@@ -15272,7 +15590,7 @@
       <c r="G280" s="31"/>
       <c r="H280" s="52"/>
       <c r="I280" s="50"/>
-      <c r="J280" s="41"/>
+      <c r="J280" s="54"/>
       <c r="K280" s="41"/>
       <c r="L280" s="53"/>
       <c r="M280" s="53"/>
@@ -15285,17 +15603,17 @@
       <c r="T280" s="35"/>
     </row>
     <row r="281" spans="1:20" ht="18" customHeight="1">
-      <c r="A281" s="90"/>
-      <c r="B281" s="99"/>
-      <c r="C281" s="86"/>
-      <c r="D281" s="86"/>
-      <c r="E281" s="51"/>
+      <c r="A281" s="53"/>
+      <c r="B281" s="53"/>
+      <c r="C281" s="53"/>
+      <c r="D281" s="53"/>
+      <c r="E281" s="53"/>
       <c r="F281" s="53"/>
       <c r="G281" s="31"/>
-      <c r="H281" s="52"/>
+      <c r="H281" s="53"/>
       <c r="I281" s="50"/>
       <c r="J281" s="54"/>
-      <c r="K281" s="41"/>
+      <c r="K281" s="44"/>
       <c r="L281" s="53"/>
       <c r="M281" s="53"/>
       <c r="N281" s="38"/>
@@ -15317,7 +15635,7 @@
       <c r="H282" s="53"/>
       <c r="I282" s="50"/>
       <c r="J282" s="54"/>
-      <c r="K282" s="44"/>
+      <c r="K282" s="54"/>
       <c r="L282" s="53"/>
       <c r="M282" s="53"/>
       <c r="N282" s="38"/>
@@ -15361,7 +15679,7 @@
       <c r="H284" s="53"/>
       <c r="I284" s="50"/>
       <c r="J284" s="54"/>
-      <c r="K284" s="54"/>
+      <c r="K284" s="41"/>
       <c r="L284" s="53"/>
       <c r="M284" s="53"/>
       <c r="N284" s="38"/>
@@ -15405,7 +15723,7 @@
       <c r="H286" s="53"/>
       <c r="I286" s="50"/>
       <c r="J286" s="54"/>
-      <c r="K286" s="41"/>
+      <c r="K286" s="54"/>
       <c r="L286" s="53"/>
       <c r="M286" s="53"/>
       <c r="N286" s="38"/>
@@ -15426,8 +15744,8 @@
       <c r="G287" s="31"/>
       <c r="H287" s="53"/>
       <c r="I287" s="50"/>
-      <c r="J287" s="54"/>
-      <c r="K287" s="54"/>
+      <c r="J287" s="47"/>
+      <c r="K287" s="41"/>
       <c r="L287" s="53"/>
       <c r="M287" s="53"/>
       <c r="N287" s="38"/>
@@ -15448,7 +15766,7 @@
       <c r="G288" s="31"/>
       <c r="H288" s="53"/>
       <c r="I288" s="50"/>
-      <c r="J288" s="47"/>
+      <c r="J288" s="41"/>
       <c r="K288" s="41"/>
       <c r="L288" s="53"/>
       <c r="M288" s="53"/>
@@ -15553,11 +15871,11 @@
       <c r="B293" s="53"/>
       <c r="C293" s="53"/>
       <c r="D293" s="53"/>
-      <c r="E293" s="53"/>
+      <c r="E293" s="51"/>
       <c r="F293" s="53"/>
       <c r="G293" s="31"/>
       <c r="H293" s="53"/>
-      <c r="I293" s="50"/>
+      <c r="I293" s="36"/>
       <c r="J293" s="41"/>
       <c r="K293" s="41"/>
       <c r="L293" s="53"/>
@@ -15646,7 +15964,7 @@
       <c r="G297" s="31"/>
       <c r="H297" s="53"/>
       <c r="I297" s="36"/>
-      <c r="J297" s="41"/>
+      <c r="J297" s="54"/>
       <c r="K297" s="41"/>
       <c r="L297" s="53"/>
       <c r="M297" s="53"/>
@@ -15725,7 +16043,7 @@
       <c r="T300" s="35"/>
     </row>
     <row r="301" spans="1:20" ht="18" customHeight="1">
-      <c r="A301" s="53"/>
+      <c r="A301" s="88"/>
       <c r="B301" s="53"/>
       <c r="C301" s="53"/>
       <c r="D301" s="53"/>
@@ -15747,7 +16065,7 @@
       <c r="T301" s="35"/>
     </row>
     <row r="302" spans="1:20" ht="18" customHeight="1">
-      <c r="A302" s="88"/>
+      <c r="A302" s="90"/>
       <c r="B302" s="53"/>
       <c r="C302" s="53"/>
       <c r="D302" s="53"/>
@@ -15774,7 +16092,7 @@
       <c r="C303" s="53"/>
       <c r="D303" s="53"/>
       <c r="E303" s="51"/>
-      <c r="F303" s="53"/>
+      <c r="F303" s="89"/>
       <c r="G303" s="31"/>
       <c r="H303" s="53"/>
       <c r="I303" s="36"/>
@@ -15791,7 +16109,7 @@
       <c r="T303" s="35"/>
     </row>
     <row r="304" spans="1:20" ht="18" customHeight="1">
-      <c r="A304" s="90"/>
+      <c r="A304" s="88"/>
       <c r="B304" s="53"/>
       <c r="C304" s="53"/>
       <c r="D304" s="53"/>
@@ -15813,7 +16131,7 @@
       <c r="T304" s="35"/>
     </row>
     <row r="305" spans="1:20" ht="18" customHeight="1">
-      <c r="A305" s="88"/>
+      <c r="A305" s="90"/>
       <c r="B305" s="53"/>
       <c r="C305" s="53"/>
       <c r="D305" s="53"/>
@@ -15857,7 +16175,7 @@
       <c r="T306" s="35"/>
     </row>
     <row r="307" spans="1:20" ht="18" customHeight="1">
-      <c r="A307" s="90"/>
+      <c r="A307" s="53"/>
       <c r="B307" s="53"/>
       <c r="C307" s="53"/>
       <c r="D307" s="53"/>
@@ -15866,7 +16184,7 @@
       <c r="G307" s="31"/>
       <c r="H307" s="53"/>
       <c r="I307" s="36"/>
-      <c r="J307" s="54"/>
+      <c r="J307" s="41"/>
       <c r="K307" s="41"/>
       <c r="L307" s="53"/>
       <c r="M307" s="53"/>
@@ -15880,11 +16198,11 @@
     </row>
     <row r="308" spans="1:20" ht="18" customHeight="1">
       <c r="A308" s="53"/>
-      <c r="B308" s="53"/>
-      <c r="C308" s="53"/>
-      <c r="D308" s="53"/>
-      <c r="E308" s="51"/>
-      <c r="F308" s="89"/>
+      <c r="B308" s="88"/>
+      <c r="C308" s="89"/>
+      <c r="D308" s="89"/>
+      <c r="E308" s="100"/>
+      <c r="F308" s="53"/>
       <c r="G308" s="31"/>
       <c r="H308" s="53"/>
       <c r="I308" s="36"/>
@@ -15902,10 +16220,10 @@
     </row>
     <row r="309" spans="1:20" ht="18" customHeight="1">
       <c r="A309" s="53"/>
-      <c r="B309" s="88"/>
-      <c r="C309" s="89"/>
-      <c r="D309" s="89"/>
-      <c r="E309" s="100"/>
+      <c r="B309" s="90"/>
+      <c r="C309" s="91"/>
+      <c r="D309" s="91"/>
+      <c r="E309" s="101"/>
       <c r="F309" s="53"/>
       <c r="G309" s="31"/>
       <c r="H309" s="53"/>
@@ -15976,7 +16294,7 @@
       <c r="G312" s="31"/>
       <c r="H312" s="53"/>
       <c r="I312" s="36"/>
-      <c r="J312" s="41"/>
+      <c r="J312" s="33"/>
       <c r="K312" s="41"/>
       <c r="L312" s="53"/>
       <c r="M312" s="53"/>
@@ -15990,16 +16308,16 @@
     </row>
     <row r="313" spans="1:20" ht="18" customHeight="1">
       <c r="A313" s="53"/>
-      <c r="B313" s="90"/>
-      <c r="C313" s="91"/>
-      <c r="D313" s="91"/>
-      <c r="E313" s="101"/>
+      <c r="B313" s="88"/>
+      <c r="C313" s="89"/>
+      <c r="D313" s="89"/>
+      <c r="E313" s="100"/>
       <c r="F313" s="53"/>
       <c r="G313" s="31"/>
       <c r="H313" s="53"/>
       <c r="I313" s="36"/>
       <c r="J313" s="33"/>
-      <c r="K313" s="41"/>
+      <c r="K313" s="33"/>
       <c r="L313" s="53"/>
       <c r="M313" s="53"/>
       <c r="N313" s="38"/>
@@ -16012,10 +16330,10 @@
     </row>
     <row r="314" spans="1:20" ht="18" customHeight="1">
       <c r="A314" s="53"/>
-      <c r="B314" s="88"/>
-      <c r="C314" s="89"/>
-      <c r="D314" s="89"/>
-      <c r="E314" s="100"/>
+      <c r="B314" s="90"/>
+      <c r="C314" s="91"/>
+      <c r="D314" s="91"/>
+      <c r="E314" s="101"/>
       <c r="F314" s="53"/>
       <c r="G314" s="31"/>
       <c r="H314" s="53"/>
@@ -16086,7 +16404,7 @@
       <c r="G317" s="31"/>
       <c r="H317" s="53"/>
       <c r="I317" s="36"/>
-      <c r="J317" s="33"/>
+      <c r="J317" s="41"/>
       <c r="K317" s="33"/>
       <c r="L317" s="53"/>
       <c r="M317" s="53"/>
@@ -16100,16 +16418,16 @@
     </row>
     <row r="318" spans="1:20" ht="18" customHeight="1">
       <c r="A318" s="53"/>
-      <c r="B318" s="90"/>
-      <c r="C318" s="91"/>
-      <c r="D318" s="91"/>
-      <c r="E318" s="101"/>
+      <c r="B318" s="88"/>
+      <c r="C318" s="89"/>
+      <c r="D318" s="53"/>
+      <c r="E318" s="53"/>
       <c r="F318" s="53"/>
       <c r="G318" s="31"/>
       <c r="H318" s="53"/>
-      <c r="I318" s="36"/>
+      <c r="I318" s="41"/>
       <c r="J318" s="41"/>
-      <c r="K318" s="33"/>
+      <c r="K318" s="41"/>
       <c r="L318" s="53"/>
       <c r="M318" s="53"/>
       <c r="N318" s="38"/>
@@ -16122,8 +16440,8 @@
     </row>
     <row r="319" spans="1:20" ht="18" customHeight="1">
       <c r="A319" s="53"/>
-      <c r="B319" s="88"/>
-      <c r="C319" s="89"/>
+      <c r="B319" s="90"/>
+      <c r="C319" s="91"/>
       <c r="D319" s="53"/>
       <c r="E319" s="53"/>
       <c r="F319" s="53"/>
@@ -16131,7 +16449,7 @@
       <c r="H319" s="53"/>
       <c r="I319" s="41"/>
       <c r="J319" s="41"/>
-      <c r="K319" s="41"/>
+      <c r="K319" s="44"/>
       <c r="L319" s="53"/>
       <c r="M319" s="53"/>
       <c r="N319" s="38"/>
@@ -16172,7 +16490,7 @@
       <c r="E321" s="53"/>
       <c r="F321" s="53"/>
       <c r="G321" s="31"/>
-      <c r="H321" s="53"/>
+      <c r="H321" s="41"/>
       <c r="I321" s="41"/>
       <c r="J321" s="41"/>
       <c r="K321" s="44"/>
@@ -16196,7 +16514,7 @@
       <c r="G322" s="31"/>
       <c r="H322" s="41"/>
       <c r="I322" s="41"/>
-      <c r="J322" s="41"/>
+      <c r="J322" s="54"/>
       <c r="K322" s="44"/>
       <c r="L322" s="53"/>
       <c r="M322" s="53"/>
@@ -16210,8 +16528,8 @@
     </row>
     <row r="323" spans="1:20" ht="18" customHeight="1">
       <c r="A323" s="53"/>
-      <c r="B323" s="90"/>
-      <c r="C323" s="91"/>
+      <c r="B323" s="88"/>
+      <c r="C323" s="89"/>
       <c r="D323" s="53"/>
       <c r="E323" s="53"/>
       <c r="F323" s="53"/>
@@ -16232,8 +16550,8 @@
     </row>
     <row r="324" spans="1:20" ht="18" customHeight="1">
       <c r="A324" s="53"/>
-      <c r="B324" s="88"/>
-      <c r="C324" s="89"/>
+      <c r="B324" s="90"/>
+      <c r="C324" s="91"/>
       <c r="D324" s="53"/>
       <c r="E324" s="53"/>
       <c r="F324" s="53"/>
@@ -16306,7 +16624,7 @@
       <c r="G327" s="31"/>
       <c r="H327" s="41"/>
       <c r="I327" s="41"/>
-      <c r="J327" s="54"/>
+      <c r="J327" s="41"/>
       <c r="K327" s="44"/>
       <c r="L327" s="53"/>
       <c r="M327" s="53"/>
@@ -16320,12 +16638,12 @@
     </row>
     <row r="328" spans="1:20" ht="18" customHeight="1">
       <c r="A328" s="53"/>
-      <c r="B328" s="90"/>
-      <c r="C328" s="91"/>
-      <c r="D328" s="53"/>
-      <c r="E328" s="53"/>
-      <c r="F328" s="53"/>
-      <c r="G328" s="31"/>
+      <c r="B328" s="88"/>
+      <c r="C328" s="89"/>
+      <c r="D328" s="89"/>
+      <c r="E328" s="89"/>
+      <c r="F328" s="89"/>
+      <c r="G328" s="92"/>
       <c r="H328" s="41"/>
       <c r="I328" s="41"/>
       <c r="J328" s="41"/>
@@ -16342,12 +16660,12 @@
     </row>
     <row r="329" spans="1:20" ht="18" customHeight="1">
       <c r="A329" s="53"/>
-      <c r="B329" s="88"/>
-      <c r="C329" s="89"/>
-      <c r="D329" s="89"/>
-      <c r="E329" s="89"/>
+      <c r="B329" s="90"/>
+      <c r="C329" s="91"/>
+      <c r="D329" s="91"/>
+      <c r="E329" s="91"/>
       <c r="F329" s="89"/>
-      <c r="G329" s="92"/>
+      <c r="G329" s="93"/>
       <c r="H329" s="41"/>
       <c r="I329" s="41"/>
       <c r="J329" s="41"/>
@@ -16429,13 +16747,13 @@
       <c r="T332" s="35"/>
     </row>
     <row r="333" spans="1:20" ht="18" customHeight="1">
-      <c r="A333" s="53"/>
-      <c r="B333" s="90"/>
-      <c r="C333" s="91"/>
-      <c r="D333" s="91"/>
-      <c r="E333" s="91"/>
-      <c r="F333" s="89"/>
-      <c r="G333" s="93"/>
+      <c r="A333" s="41"/>
+      <c r="B333" s="53"/>
+      <c r="C333" s="53"/>
+      <c r="D333" s="53"/>
+      <c r="E333" s="53"/>
+      <c r="F333" s="53"/>
+      <c r="G333" s="31"/>
       <c r="H333" s="41"/>
       <c r="I333" s="41"/>
       <c r="J333" s="41"/>
@@ -16464,7 +16782,7 @@
       <c r="K334" s="44"/>
       <c r="L334" s="53"/>
       <c r="M334" s="53"/>
-      <c r="N334" s="38"/>
+      <c r="N334" s="53"/>
       <c r="O334" s="41"/>
       <c r="P334" s="41"/>
       <c r="Q334" s="41"/>
@@ -16526,7 +16844,7 @@
       <c r="G337" s="31"/>
       <c r="H337" s="41"/>
       <c r="I337" s="41"/>
-      <c r="J337" s="41"/>
+      <c r="J337" s="44"/>
       <c r="K337" s="44"/>
       <c r="L337" s="53"/>
       <c r="M337" s="53"/>
@@ -16568,7 +16886,7 @@
       <c r="E339" s="53"/>
       <c r="F339" s="53"/>
       <c r="G339" s="31"/>
-      <c r="H339" s="41"/>
+      <c r="H339" s="53"/>
       <c r="I339" s="41"/>
       <c r="J339" s="44"/>
       <c r="K339" s="44"/>
@@ -16634,7 +16952,7 @@
       <c r="E342" s="53"/>
       <c r="F342" s="53"/>
       <c r="G342" s="31"/>
-      <c r="H342" s="53"/>
+      <c r="H342" s="41"/>
       <c r="I342" s="41"/>
       <c r="J342" s="44"/>
       <c r="K342" s="44"/>
@@ -16747,7 +17065,7 @@
       <c r="H347" s="41"/>
       <c r="I347" s="41"/>
       <c r="J347" s="44"/>
-      <c r="K347" s="44"/>
+      <c r="K347" s="41"/>
       <c r="L347" s="53"/>
       <c r="M347" s="53"/>
       <c r="N347" s="53"/>
@@ -16813,7 +17131,7 @@
       <c r="H350" s="41"/>
       <c r="I350" s="41"/>
       <c r="J350" s="44"/>
-      <c r="K350" s="41"/>
+      <c r="K350" s="53"/>
       <c r="L350" s="53"/>
       <c r="M350" s="53"/>
       <c r="N350" s="53"/>
@@ -16835,7 +17153,7 @@
       <c r="H351" s="41"/>
       <c r="I351" s="41"/>
       <c r="J351" s="44"/>
-      <c r="K351" s="53"/>
+      <c r="K351" s="41"/>
       <c r="L351" s="53"/>
       <c r="M351" s="53"/>
       <c r="N351" s="53"/>
@@ -16988,7 +17306,7 @@
       <c r="G358" s="31"/>
       <c r="H358" s="41"/>
       <c r="I358" s="41"/>
-      <c r="J358" s="44"/>
+      <c r="J358" s="41"/>
       <c r="K358" s="41"/>
       <c r="L358" s="53"/>
       <c r="M358" s="53"/>
@@ -17011,7 +17329,7 @@
       <c r="H359" s="41"/>
       <c r="I359" s="41"/>
       <c r="J359" s="41"/>
-      <c r="K359" s="41"/>
+      <c r="K359" s="44"/>
       <c r="L359" s="53"/>
       <c r="M359" s="53"/>
       <c r="N359" s="53"/>
@@ -17077,7 +17395,7 @@
       <c r="H362" s="41"/>
       <c r="I362" s="41"/>
       <c r="J362" s="41"/>
-      <c r="K362" s="44"/>
+      <c r="K362" s="41"/>
       <c r="L362" s="53"/>
       <c r="M362" s="53"/>
       <c r="N362" s="53"/>
@@ -17450,7 +17768,7 @@
       <c r="G379" s="31"/>
       <c r="H379" s="41"/>
       <c r="I379" s="41"/>
-      <c r="J379" s="41"/>
+      <c r="J379" s="44"/>
       <c r="K379" s="41"/>
       <c r="L379" s="53"/>
       <c r="M379" s="53"/>
@@ -17471,7 +17789,7 @@
       <c r="F380" s="53"/>
       <c r="G380" s="31"/>
       <c r="H380" s="41"/>
-      <c r="I380" s="41"/>
+      <c r="I380" s="53"/>
       <c r="J380" s="44"/>
       <c r="K380" s="41"/>
       <c r="L380" s="53"/>
@@ -17890,8 +18208,8 @@
       <c r="G399" s="31"/>
       <c r="H399" s="41"/>
       <c r="I399" s="53"/>
-      <c r="J399" s="44"/>
-      <c r="K399" s="41"/>
+      <c r="J399" s="54"/>
+      <c r="K399" s="54"/>
       <c r="L399" s="53"/>
       <c r="M399" s="53"/>
       <c r="N399" s="53"/>
@@ -17909,9 +18227,9 @@
       <c r="D400" s="53"/>
       <c r="E400" s="53"/>
       <c r="F400" s="53"/>
-      <c r="G400" s="31"/>
-      <c r="H400" s="41"/>
-      <c r="I400" s="53"/>
+      <c r="G400" s="53"/>
+      <c r="H400" s="53"/>
+      <c r="I400" s="41"/>
       <c r="J400" s="54"/>
       <c r="K400" s="54"/>
       <c r="L400" s="53"/>
@@ -17978,7 +18296,7 @@
       <c r="G403" s="53"/>
       <c r="H403" s="53"/>
       <c r="I403" s="41"/>
-      <c r="J403" s="54"/>
+      <c r="J403" s="41"/>
       <c r="K403" s="54"/>
       <c r="L403" s="53"/>
       <c r="M403" s="53"/>
@@ -18001,7 +18319,7 @@
       <c r="H404" s="53"/>
       <c r="I404" s="41"/>
       <c r="J404" s="41"/>
-      <c r="K404" s="54"/>
+      <c r="K404" s="44"/>
       <c r="L404" s="53"/>
       <c r="M404" s="53"/>
       <c r="N404" s="53"/>
@@ -18080,14 +18398,14 @@
     </row>
     <row r="408" spans="1:20" ht="18" customHeight="1">
       <c r="A408" s="41"/>
-      <c r="B408" s="53"/>
-      <c r="C408" s="53"/>
-      <c r="D408" s="53"/>
-      <c r="E408" s="53"/>
-      <c r="F408" s="53"/>
-      <c r="G408" s="53"/>
-      <c r="H408" s="53"/>
-      <c r="I408" s="41"/>
+      <c r="B408" s="88"/>
+      <c r="C408" s="89"/>
+      <c r="D408" s="89"/>
+      <c r="E408" s="89"/>
+      <c r="F408" s="89"/>
+      <c r="G408" s="89"/>
+      <c r="H408" s="89"/>
+      <c r="I408" s="89"/>
       <c r="J408" s="41"/>
       <c r="K408" s="44"/>
       <c r="L408" s="53"/>
@@ -18102,16 +18420,16 @@
     </row>
     <row r="409" spans="1:20" ht="18" customHeight="1">
       <c r="A409" s="41"/>
-      <c r="B409" s="88"/>
-      <c r="C409" s="89"/>
-      <c r="D409" s="89"/>
-      <c r="E409" s="89"/>
+      <c r="B409" s="90"/>
+      <c r="C409" s="91"/>
+      <c r="D409" s="91"/>
+      <c r="E409" s="91"/>
       <c r="F409" s="89"/>
-      <c r="G409" s="89"/>
-      <c r="H409" s="89"/>
-      <c r="I409" s="89"/>
+      <c r="G409" s="91"/>
+      <c r="H409" s="91"/>
+      <c r="I409" s="91"/>
       <c r="J409" s="41"/>
-      <c r="K409" s="44"/>
+      <c r="K409" s="41"/>
       <c r="L409" s="53"/>
       <c r="M409" s="53"/>
       <c r="N409" s="53"/>
@@ -18154,7 +18472,7 @@
       <c r="G411" s="91"/>
       <c r="H411" s="91"/>
       <c r="I411" s="91"/>
-      <c r="J411" s="41"/>
+      <c r="J411" s="54"/>
       <c r="K411" s="41"/>
       <c r="L411" s="53"/>
       <c r="M411" s="53"/>
@@ -18168,11 +18486,11 @@
     </row>
     <row r="412" spans="1:20" ht="18" customHeight="1">
       <c r="A412" s="41"/>
-      <c r="B412" s="90"/>
-      <c r="C412" s="91"/>
-      <c r="D412" s="91"/>
-      <c r="E412" s="91"/>
-      <c r="F412" s="89"/>
+      <c r="B412" s="53"/>
+      <c r="C412" s="53"/>
+      <c r="D412" s="53"/>
+      <c r="E412" s="53"/>
+      <c r="F412" s="53"/>
       <c r="G412" s="91"/>
       <c r="H412" s="91"/>
       <c r="I412" s="91"/>
@@ -18199,7 +18517,7 @@
       <c r="H413" s="91"/>
       <c r="I413" s="91"/>
       <c r="J413" s="54"/>
-      <c r="K413" s="41"/>
+      <c r="K413" s="54"/>
       <c r="L413" s="53"/>
       <c r="M413" s="53"/>
       <c r="N413" s="53"/>
@@ -18299,10 +18617,10 @@
       <c r="T417" s="35"/>
     </row>
     <row r="418" spans="1:20" ht="18" customHeight="1">
-      <c r="A418" s="41"/>
-      <c r="B418" s="53"/>
-      <c r="C418" s="53"/>
-      <c r="D418" s="53"/>
+      <c r="A418" s="53"/>
+      <c r="B418" s="88"/>
+      <c r="C418" s="89"/>
+      <c r="D418" s="89"/>
       <c r="E418" s="53"/>
       <c r="F418" s="53"/>
       <c r="G418" s="91"/>
@@ -18322,9 +18640,9 @@
     </row>
     <row r="419" spans="1:20" ht="18" customHeight="1">
       <c r="A419" s="53"/>
-      <c r="B419" s="88"/>
-      <c r="C419" s="89"/>
-      <c r="D419" s="89"/>
+      <c r="B419" s="90"/>
+      <c r="C419" s="91"/>
+      <c r="D419" s="91"/>
       <c r="E419" s="53"/>
       <c r="F419" s="53"/>
       <c r="G419" s="91"/>
@@ -18366,16 +18684,16 @@
     </row>
     <row r="421" spans="1:20" ht="18" customHeight="1">
       <c r="A421" s="53"/>
-      <c r="B421" s="90"/>
-      <c r="C421" s="91"/>
-      <c r="D421" s="91"/>
+      <c r="B421" s="53"/>
+      <c r="C421" s="53"/>
+      <c r="D421" s="53"/>
       <c r="E421" s="53"/>
       <c r="F421" s="53"/>
       <c r="G421" s="91"/>
       <c r="H421" s="91"/>
       <c r="I421" s="91"/>
       <c r="J421" s="54"/>
-      <c r="K421" s="54"/>
+      <c r="K421" s="41"/>
       <c r="L421" s="53"/>
       <c r="M421" s="53"/>
       <c r="N421" s="53"/>
@@ -18386,7 +18704,7 @@
       <c r="S421" s="35"/>
       <c r="T421" s="35"/>
     </row>
-    <row r="422" spans="1:20" ht="18" customHeight="1">
+    <row r="422" spans="1:20" ht="15" customHeight="1">
       <c r="A422" s="53"/>
       <c r="B422" s="53"/>
       <c r="C422" s="53"/>
@@ -18440,7 +18758,7 @@
       <c r="G424" s="91"/>
       <c r="H424" s="91"/>
       <c r="I424" s="91"/>
-      <c r="J424" s="54"/>
+      <c r="J424" s="41"/>
       <c r="K424" s="41"/>
       <c r="L424" s="53"/>
       <c r="M424" s="53"/>
@@ -18503,9 +18821,9 @@
       <c r="D427" s="53"/>
       <c r="E427" s="53"/>
       <c r="F427" s="53"/>
-      <c r="G427" s="91"/>
-      <c r="H427" s="91"/>
-      <c r="I427" s="91"/>
+      <c r="G427" s="53"/>
+      <c r="H427" s="41"/>
+      <c r="I427" s="41"/>
       <c r="J427" s="41"/>
       <c r="K427" s="41"/>
       <c r="L427" s="53"/>
@@ -18528,7 +18846,7 @@
       <c r="G428" s="53"/>
       <c r="H428" s="41"/>
       <c r="I428" s="41"/>
-      <c r="J428" s="41"/>
+      <c r="J428" s="54"/>
       <c r="K428" s="41"/>
       <c r="L428" s="53"/>
       <c r="M428" s="53"/>
@@ -18550,7 +18868,7 @@
       <c r="G429" s="53"/>
       <c r="H429" s="41"/>
       <c r="I429" s="41"/>
-      <c r="J429" s="54"/>
+      <c r="J429" s="41"/>
       <c r="K429" s="41"/>
       <c r="L429" s="53"/>
       <c r="M429" s="53"/>
@@ -18783,14 +19101,14 @@
       <c r="T439" s="35"/>
     </row>
     <row r="440" spans="1:20" ht="15" customHeight="1">
-      <c r="A440" s="53"/>
+      <c r="A440" s="41"/>
       <c r="B440" s="53"/>
       <c r="C440" s="53"/>
       <c r="D440" s="53"/>
       <c r="E440" s="53"/>
       <c r="F440" s="53"/>
       <c r="G440" s="53"/>
-      <c r="H440" s="41"/>
+      <c r="H440" s="53"/>
       <c r="I440" s="41"/>
       <c r="J440" s="41"/>
       <c r="K440" s="41"/>
@@ -18982,10 +19300,10 @@
     </row>
     <row r="449" spans="1:20" ht="15" customHeight="1">
       <c r="A449" s="41"/>
-      <c r="B449" s="53"/>
-      <c r="C449" s="53"/>
-      <c r="D449" s="53"/>
-      <c r="E449" s="53"/>
+      <c r="B449" s="88"/>
+      <c r="C449" s="89"/>
+      <c r="D449" s="89"/>
+      <c r="E449" s="89"/>
       <c r="F449" s="53"/>
       <c r="G449" s="53"/>
       <c r="H449" s="53"/>
@@ -19004,10 +19322,10 @@
     </row>
     <row r="450" spans="1:20" ht="15" customHeight="1">
       <c r="A450" s="41"/>
-      <c r="B450" s="88"/>
-      <c r="C450" s="89"/>
-      <c r="D450" s="89"/>
-      <c r="E450" s="89"/>
+      <c r="B450" s="90"/>
+      <c r="C450" s="91"/>
+      <c r="D450" s="91"/>
+      <c r="E450" s="91"/>
       <c r="F450" s="53"/>
       <c r="G450" s="53"/>
       <c r="H450" s="53"/>
@@ -19180,10 +19498,10 @@
     </row>
     <row r="458" spans="1:20" ht="15" customHeight="1">
       <c r="A458" s="41"/>
-      <c r="B458" s="90"/>
-      <c r="C458" s="91"/>
-      <c r="D458" s="91"/>
-      <c r="E458" s="91"/>
+      <c r="B458" s="88"/>
+      <c r="C458" s="89"/>
+      <c r="D458" s="89"/>
+      <c r="E458" s="89"/>
       <c r="F458" s="53"/>
       <c r="G458" s="53"/>
       <c r="H458" s="53"/>
@@ -19202,10 +19520,10 @@
     </row>
     <row r="459" spans="1:20" ht="15" customHeight="1">
       <c r="A459" s="41"/>
-      <c r="B459" s="88"/>
-      <c r="C459" s="89"/>
-      <c r="D459" s="89"/>
-      <c r="E459" s="89"/>
+      <c r="B459" s="90"/>
+      <c r="C459" s="91"/>
+      <c r="D459" s="91"/>
+      <c r="E459" s="91"/>
       <c r="F459" s="53"/>
       <c r="G459" s="53"/>
       <c r="H459" s="53"/>
@@ -19378,13 +19696,13 @@
     </row>
     <row r="467" spans="1:20" ht="15" customHeight="1">
       <c r="A467" s="41"/>
-      <c r="B467" s="90"/>
-      <c r="C467" s="91"/>
-      <c r="D467" s="91"/>
-      <c r="E467" s="91"/>
+      <c r="B467" s="88"/>
+      <c r="C467" s="89"/>
+      <c r="D467" s="89"/>
+      <c r="E467" s="89"/>
       <c r="F467" s="53"/>
       <c r="G467" s="53"/>
-      <c r="H467" s="53"/>
+      <c r="H467" s="41"/>
       <c r="I467" s="41"/>
       <c r="J467" s="41"/>
       <c r="K467" s="41"/>
@@ -19400,10 +19718,10 @@
     </row>
     <row r="468" spans="1:20" ht="15" customHeight="1">
       <c r="A468" s="41"/>
-      <c r="B468" s="88"/>
-      <c r="C468" s="89"/>
-      <c r="D468" s="89"/>
-      <c r="E468" s="89"/>
+      <c r="B468" s="90"/>
+      <c r="C468" s="91"/>
+      <c r="D468" s="91"/>
+      <c r="E468" s="91"/>
       <c r="F468" s="53"/>
       <c r="G468" s="53"/>
       <c r="H468" s="41"/>
@@ -19488,10 +19806,10 @@
     </row>
     <row r="472" spans="1:20" ht="15" customHeight="1">
       <c r="A472" s="41"/>
-      <c r="B472" s="90"/>
-      <c r="C472" s="91"/>
-      <c r="D472" s="91"/>
-      <c r="E472" s="91"/>
+      <c r="B472" s="88"/>
+      <c r="C472" s="89"/>
+      <c r="D472" s="89"/>
+      <c r="E472" s="89"/>
       <c r="F472" s="53"/>
       <c r="G472" s="53"/>
       <c r="H472" s="41"/>
@@ -19510,10 +19828,10 @@
     </row>
     <row r="473" spans="1:20" ht="15" customHeight="1">
       <c r="A473" s="41"/>
-      <c r="B473" s="88"/>
-      <c r="C473" s="89"/>
-      <c r="D473" s="89"/>
-      <c r="E473" s="89"/>
+      <c r="B473" s="90"/>
+      <c r="C473" s="91"/>
+      <c r="D473" s="91"/>
+      <c r="E473" s="91"/>
       <c r="F473" s="53"/>
       <c r="G473" s="53"/>
       <c r="H473" s="41"/>
@@ -19598,10 +19916,10 @@
     </row>
     <row r="477" spans="1:20" ht="15" customHeight="1">
       <c r="A477" s="41"/>
-      <c r="B477" s="90"/>
-      <c r="C477" s="91"/>
-      <c r="D477" s="91"/>
-      <c r="E477" s="91"/>
+      <c r="B477" s="88"/>
+      <c r="C477" s="89"/>
+      <c r="D477" s="89"/>
+      <c r="E477" s="89"/>
       <c r="F477" s="53"/>
       <c r="G477" s="53"/>
       <c r="H477" s="41"/>
@@ -19620,10 +19938,10 @@
     </row>
     <row r="478" spans="1:20" ht="15" customHeight="1">
       <c r="A478" s="41"/>
-      <c r="B478" s="88"/>
-      <c r="C478" s="89"/>
-      <c r="D478" s="89"/>
-      <c r="E478" s="89"/>
+      <c r="B478" s="90"/>
+      <c r="C478" s="91"/>
+      <c r="D478" s="91"/>
+      <c r="E478" s="91"/>
       <c r="F478" s="53"/>
       <c r="G478" s="53"/>
       <c r="H478" s="41"/>
@@ -19796,12 +20114,12 @@
     </row>
     <row r="486" spans="1:20" ht="15" customHeight="1">
       <c r="A486" s="41"/>
-      <c r="B486" s="90"/>
-      <c r="C486" s="91"/>
-      <c r="D486" s="91"/>
-      <c r="E486" s="91"/>
+      <c r="B486" s="53"/>
+      <c r="C486" s="53"/>
+      <c r="D486" s="53"/>
+      <c r="E486" s="53"/>
       <c r="F486" s="53"/>
-      <c r="G486" s="53"/>
+      <c r="G486" s="31"/>
       <c r="H486" s="41"/>
       <c r="I486" s="41"/>
       <c r="J486" s="41"/>
@@ -20103,17 +20421,17 @@
       <c r="T499" s="35"/>
     </row>
     <row r="500" spans="1:20" ht="15" customHeight="1">
-      <c r="A500" s="41"/>
-      <c r="B500" s="53"/>
-      <c r="C500" s="53"/>
-      <c r="D500" s="53"/>
-      <c r="E500" s="53"/>
-      <c r="F500" s="53"/>
-      <c r="G500" s="31"/>
-      <c r="H500" s="41"/>
-      <c r="I500" s="41"/>
+      <c r="A500" s="88"/>
+      <c r="B500" s="89"/>
+      <c r="C500" s="89"/>
+      <c r="D500" s="89"/>
+      <c r="E500" s="89"/>
+      <c r="F500" s="89"/>
+      <c r="G500" s="92"/>
+      <c r="H500" s="89"/>
+      <c r="I500" s="89"/>
       <c r="J500" s="41"/>
-      <c r="K500" s="41"/>
+      <c r="K500" s="89"/>
       <c r="L500" s="53"/>
       <c r="M500" s="53"/>
       <c r="N500" s="53"/>
@@ -20125,20 +20443,20 @@
       <c r="T500" s="35"/>
     </row>
     <row r="501" spans="1:20" ht="15" customHeight="1">
-      <c r="A501" s="88"/>
-      <c r="B501" s="89"/>
-      <c r="C501" s="89"/>
-      <c r="D501" s="89"/>
-      <c r="E501" s="89"/>
+      <c r="A501" s="90"/>
+      <c r="B501" s="91"/>
+      <c r="C501" s="91"/>
+      <c r="D501" s="91"/>
+      <c r="E501" s="91"/>
       <c r="F501" s="89"/>
-      <c r="G501" s="92"/>
-      <c r="H501" s="89"/>
-      <c r="I501" s="89"/>
+      <c r="G501" s="93"/>
+      <c r="H501" s="91"/>
+      <c r="I501" s="91"/>
       <c r="J501" s="41"/>
-      <c r="K501" s="89"/>
-      <c r="L501" s="53"/>
-      <c r="M501" s="53"/>
-      <c r="N501" s="53"/>
+      <c r="K501" s="91"/>
+      <c r="L501" s="89"/>
+      <c r="M501" s="89"/>
+      <c r="N501" s="89"/>
       <c r="O501" s="41"/>
       <c r="P501" s="41"/>
       <c r="Q501" s="41"/>
@@ -20157,10 +20475,10 @@
       <c r="H502" s="91"/>
       <c r="I502" s="91"/>
       <c r="J502" s="41"/>
-      <c r="K502" s="91"/>
+      <c r="K502" s="94"/>
       <c r="L502" s="89"/>
       <c r="M502" s="89"/>
-      <c r="N502" s="89"/>
+      <c r="N502" s="91"/>
       <c r="O502" s="41"/>
       <c r="P502" s="41"/>
       <c r="Q502" s="41"/>
@@ -20565,17 +20883,17 @@
       <c r="T520" s="35"/>
     </row>
     <row r="521" spans="1:20" ht="15" customHeight="1">
-      <c r="A521" s="90"/>
-      <c r="B521" s="91"/>
-      <c r="C521" s="91"/>
-      <c r="D521" s="91"/>
-      <c r="E521" s="91"/>
-      <c r="F521" s="89"/>
+      <c r="A521" s="41"/>
+      <c r="B521" s="53"/>
+      <c r="C521" s="53"/>
+      <c r="D521" s="53"/>
+      <c r="E521" s="41"/>
+      <c r="F521" s="53"/>
       <c r="G521" s="93"/>
-      <c r="H521" s="91"/>
-      <c r="I521" s="91"/>
+      <c r="H521" s="53"/>
+      <c r="I521" s="41"/>
       <c r="J521" s="41"/>
-      <c r="K521" s="94"/>
+      <c r="K521" s="41"/>
       <c r="L521" s="89"/>
       <c r="M521" s="89"/>
       <c r="N521" s="91"/>
@@ -20598,9 +20916,9 @@
       <c r="I522" s="41"/>
       <c r="J522" s="41"/>
       <c r="K522" s="41"/>
-      <c r="L522" s="89"/>
-      <c r="M522" s="89"/>
-      <c r="N522" s="91"/>
+      <c r="L522" s="53"/>
+      <c r="M522" s="53"/>
+      <c r="N522" s="53"/>
       <c r="O522" s="41"/>
       <c r="P522" s="41"/>
       <c r="Q522" s="41"/>
@@ -20734,7 +21052,6 @@
       <c r="M528" s="53"/>
       <c r="N528" s="53"/>
       <c r="O528" s="41"/>
-      <c r="P528" s="41"/>
       <c r="Q528" s="41"/>
       <c r="R528" s="41"/>
       <c r="S528" s="35"/>
@@ -20748,7 +21065,7 @@
       <c r="E529" s="41"/>
       <c r="F529" s="53"/>
       <c r="G529" s="93"/>
-      <c r="H529" s="53"/>
+      <c r="H529" s="41"/>
       <c r="I529" s="41"/>
       <c r="J529" s="41"/>
       <c r="K529" s="41"/>
@@ -20756,6 +21073,7 @@
       <c r="M529" s="53"/>
       <c r="N529" s="53"/>
       <c r="O529" s="41"/>
+      <c r="P529" s="41"/>
       <c r="Q529" s="41"/>
       <c r="R529" s="41"/>
       <c r="S529" s="35"/>
@@ -20960,11 +21278,11 @@
       <c r="T538" s="35"/>
     </row>
     <row r="539" spans="1:20" ht="15" customHeight="1">
-      <c r="A539" s="41"/>
+      <c r="A539" s="53"/>
       <c r="B539" s="53"/>
       <c r="C539" s="53"/>
       <c r="D539" s="53"/>
-      <c r="E539" s="41"/>
+      <c r="E539" s="53"/>
       <c r="F539" s="53"/>
       <c r="G539" s="93"/>
       <c r="H539" s="41"/>
@@ -21224,15 +21542,15 @@
       <c r="T550" s="35"/>
     </row>
     <row r="551" spans="1:20" ht="15" customHeight="1">
-      <c r="A551" s="53"/>
-      <c r="B551" s="53"/>
-      <c r="C551" s="53"/>
-      <c r="D551" s="53"/>
-      <c r="E551" s="53"/>
-      <c r="F551" s="53"/>
+      <c r="A551" s="88"/>
+      <c r="B551" s="89"/>
+      <c r="C551" s="89"/>
+      <c r="D551" s="89"/>
+      <c r="E551" s="89"/>
+      <c r="F551" s="89"/>
       <c r="G551" s="93"/>
-      <c r="H551" s="41"/>
-      <c r="I551" s="41"/>
+      <c r="H551" s="89"/>
+      <c r="I551" s="89"/>
       <c r="J551" s="41"/>
       <c r="K551" s="41"/>
       <c r="L551" s="53"/>
@@ -21246,15 +21564,15 @@
       <c r="T551" s="35"/>
     </row>
     <row r="552" spans="1:20" ht="15" customHeight="1">
-      <c r="A552" s="88"/>
-      <c r="B552" s="89"/>
-      <c r="C552" s="89"/>
-      <c r="D552" s="89"/>
-      <c r="E552" s="89"/>
+      <c r="A552" s="90"/>
+      <c r="B552" s="91"/>
+      <c r="C552" s="91"/>
+      <c r="D552" s="91"/>
+      <c r="E552" s="91"/>
       <c r="F552" s="89"/>
       <c r="G552" s="93"/>
-      <c r="H552" s="89"/>
-      <c r="I552" s="89"/>
+      <c r="H552" s="91"/>
+      <c r="I552" s="91"/>
       <c r="J552" s="41"/>
       <c r="K552" s="41"/>
       <c r="L552" s="53"/>
@@ -21343,7 +21661,7 @@
       <c r="G556" s="93"/>
       <c r="H556" s="91"/>
       <c r="I556" s="91"/>
-      <c r="J556" s="41"/>
+      <c r="J556" s="84"/>
       <c r="K556" s="41"/>
       <c r="L556" s="53"/>
       <c r="M556" s="53"/>
@@ -21356,17 +21674,17 @@
       <c r="T556" s="35"/>
     </row>
     <row r="557" spans="1:20" ht="15" customHeight="1">
-      <c r="A557" s="90"/>
-      <c r="B557" s="91"/>
-      <c r="C557" s="91"/>
-      <c r="D557" s="91"/>
-      <c r="E557" s="91"/>
+      <c r="A557" s="88"/>
+      <c r="B557" s="89"/>
+      <c r="C557" s="89"/>
+      <c r="D557" s="89"/>
+      <c r="E557" s="89"/>
       <c r="F557" s="89"/>
       <c r="G557" s="93"/>
-      <c r="H557" s="91"/>
-      <c r="I557" s="91"/>
+      <c r="H557" s="41"/>
+      <c r="I557" s="41"/>
       <c r="J557" s="84"/>
-      <c r="K557" s="41"/>
+      <c r="K557" s="84"/>
       <c r="L557" s="53"/>
       <c r="M557" s="53"/>
       <c r="N557" s="53"/>
@@ -21378,11 +21696,11 @@
       <c r="T557" s="35"/>
     </row>
     <row r="558" spans="1:20" ht="15" customHeight="1">
-      <c r="A558" s="88"/>
-      <c r="B558" s="89"/>
-      <c r="C558" s="89"/>
-      <c r="D558" s="89"/>
-      <c r="E558" s="89"/>
+      <c r="A558" s="90"/>
+      <c r="B558" s="91"/>
+      <c r="C558" s="91"/>
+      <c r="D558" s="91"/>
+      <c r="E558" s="91"/>
       <c r="F558" s="89"/>
       <c r="G558" s="93"/>
       <c r="H558" s="41"/>
@@ -21475,7 +21793,7 @@
       <c r="G562" s="93"/>
       <c r="H562" s="41"/>
       <c r="I562" s="41"/>
-      <c r="J562" s="84"/>
+      <c r="J562" s="41"/>
       <c r="K562" s="84"/>
       <c r="L562" s="53"/>
       <c r="M562" s="53"/>
@@ -21488,17 +21806,17 @@
       <c r="T562" s="35"/>
     </row>
     <row r="563" spans="1:20" ht="15" customHeight="1">
-      <c r="A563" s="90"/>
-      <c r="B563" s="91"/>
-      <c r="C563" s="91"/>
-      <c r="D563" s="91"/>
-      <c r="E563" s="91"/>
-      <c r="F563" s="89"/>
+      <c r="A563" s="41"/>
+      <c r="B563" s="53"/>
+      <c r="C563" s="53"/>
+      <c r="D563" s="53"/>
+      <c r="E563" s="53"/>
+      <c r="F563" s="53"/>
       <c r="G563" s="93"/>
-      <c r="H563" s="41"/>
+      <c r="H563" s="53"/>
       <c r="I563" s="41"/>
       <c r="J563" s="41"/>
-      <c r="K563" s="84"/>
+      <c r="K563" s="41"/>
       <c r="L563" s="53"/>
       <c r="M563" s="53"/>
       <c r="N563" s="53"/>
@@ -21885,10 +22203,10 @@
     </row>
     <row r="581" spans="1:20" ht="15" customHeight="1">
       <c r="A581" s="41"/>
-      <c r="B581" s="53"/>
-      <c r="C581" s="53"/>
-      <c r="D581" s="53"/>
-      <c r="E581" s="53"/>
+      <c r="B581" s="88"/>
+      <c r="C581" s="89"/>
+      <c r="D581" s="89"/>
+      <c r="E581" s="89"/>
       <c r="F581" s="53"/>
       <c r="G581" s="93"/>
       <c r="H581" s="53"/>
@@ -21907,10 +22225,10 @@
     </row>
     <row r="582" spans="1:20" ht="15" customHeight="1">
       <c r="A582" s="41"/>
-      <c r="B582" s="88"/>
-      <c r="C582" s="89"/>
-      <c r="D582" s="89"/>
-      <c r="E582" s="89"/>
+      <c r="B582" s="90"/>
+      <c r="C582" s="91"/>
+      <c r="D582" s="91"/>
+      <c r="E582" s="91"/>
       <c r="F582" s="53"/>
       <c r="G582" s="93"/>
       <c r="H582" s="53"/>
@@ -22016,11 +22334,11 @@
       <c r="T586" s="35"/>
     </row>
     <row r="587" spans="1:20" ht="15" customHeight="1">
-      <c r="A587" s="41"/>
-      <c r="B587" s="90"/>
-      <c r="C587" s="91"/>
-      <c r="D587" s="91"/>
-      <c r="E587" s="91"/>
+      <c r="A587" s="53"/>
+      <c r="B587" s="53"/>
+      <c r="C587" s="53"/>
+      <c r="D587" s="53"/>
+      <c r="E587" s="41"/>
       <c r="F587" s="53"/>
       <c r="G587" s="93"/>
       <c r="H587" s="53"/>
@@ -22038,14 +22356,14 @@
       <c r="T587" s="35"/>
     </row>
     <row r="588" spans="1:20" ht="15" customHeight="1">
-      <c r="A588" s="53"/>
-      <c r="B588" s="53"/>
+      <c r="A588" s="95"/>
+      <c r="B588" s="95"/>
       <c r="C588" s="53"/>
       <c r="D588" s="53"/>
-      <c r="E588" s="41"/>
+      <c r="E588" s="53"/>
       <c r="F588" s="53"/>
       <c r="G588" s="93"/>
-      <c r="H588" s="53"/>
+      <c r="H588" s="41"/>
       <c r="I588" s="41"/>
       <c r="J588" s="41"/>
       <c r="K588" s="41"/>
@@ -22060,13 +22378,13 @@
       <c r="T588" s="35"/>
     </row>
     <row r="589" spans="1:20" ht="15" customHeight="1">
-      <c r="A589" s="95"/>
-      <c r="B589" s="95"/>
+      <c r="A589" s="41"/>
+      <c r="B589" s="53"/>
       <c r="C589" s="53"/>
       <c r="D589" s="53"/>
       <c r="E589" s="53"/>
-      <c r="F589" s="53"/>
-      <c r="G589" s="93"/>
+      <c r="F589" s="41"/>
+      <c r="G589" s="41"/>
       <c r="H589" s="41"/>
       <c r="I589" s="41"/>
       <c r="J589" s="41"/>
@@ -22093,7 +22411,7 @@
       <c r="I590" s="41"/>
       <c r="J590" s="41"/>
       <c r="K590" s="41"/>
-      <c r="L590" s="53"/>
+      <c r="L590" s="41"/>
       <c r="M590" s="53"/>
       <c r="N590" s="53"/>
       <c r="O590" s="41"/>
@@ -22157,7 +22475,7 @@
       <c r="G593" s="41"/>
       <c r="H593" s="41"/>
       <c r="I593" s="41"/>
-      <c r="J593" s="41"/>
+      <c r="J593" s="84"/>
       <c r="K593" s="41"/>
       <c r="L593" s="41"/>
       <c r="M593" s="53"/>
@@ -22175,12 +22493,12 @@
       <c r="C594" s="53"/>
       <c r="D594" s="53"/>
       <c r="E594" s="53"/>
-      <c r="F594" s="41"/>
-      <c r="G594" s="41"/>
+      <c r="F594" s="53"/>
+      <c r="G594" s="53"/>
       <c r="H594" s="41"/>
       <c r="I594" s="41"/>
       <c r="J594" s="84"/>
-      <c r="K594" s="41"/>
+      <c r="K594" s="84"/>
       <c r="L594" s="41"/>
       <c r="M594" s="53"/>
       <c r="N594" s="53"/>
@@ -22203,7 +22521,7 @@
       <c r="I595" s="41"/>
       <c r="J595" s="84"/>
       <c r="K595" s="84"/>
-      <c r="L595" s="41"/>
+      <c r="L595" s="53"/>
       <c r="M595" s="53"/>
       <c r="N595" s="53"/>
       <c r="O595" s="41"/>
@@ -22267,7 +22585,7 @@
       <c r="G598" s="53"/>
       <c r="H598" s="41"/>
       <c r="I598" s="41"/>
-      <c r="J598" s="84"/>
+      <c r="J598" s="54"/>
       <c r="K598" s="84"/>
       <c r="L598" s="53"/>
       <c r="M598" s="53"/>
@@ -22287,10 +22605,10 @@
       <c r="E599" s="53"/>
       <c r="F599" s="53"/>
       <c r="G599" s="53"/>
-      <c r="H599" s="41"/>
+      <c r="H599" s="53"/>
       <c r="I599" s="41"/>
       <c r="J599" s="54"/>
-      <c r="K599" s="84"/>
+      <c r="K599" s="54"/>
       <c r="L599" s="53"/>
       <c r="M599" s="53"/>
       <c r="N599" s="53"/>
@@ -22311,7 +22629,7 @@
       <c r="G600" s="53"/>
       <c r="H600" s="53"/>
       <c r="I600" s="41"/>
-      <c r="J600" s="54"/>
+      <c r="J600" s="41"/>
       <c r="K600" s="54"/>
       <c r="L600" s="53"/>
       <c r="M600" s="53"/>
@@ -22334,7 +22652,7 @@
       <c r="H601" s="53"/>
       <c r="I601" s="41"/>
       <c r="J601" s="41"/>
-      <c r="K601" s="54"/>
+      <c r="K601" s="41"/>
       <c r="L601" s="53"/>
       <c r="M601" s="53"/>
       <c r="N601" s="53"/>
@@ -22372,10 +22690,10 @@
       <c r="B603" s="53"/>
       <c r="C603" s="53"/>
       <c r="D603" s="53"/>
-      <c r="E603" s="53"/>
-      <c r="F603" s="53"/>
-      <c r="G603" s="53"/>
-      <c r="H603" s="53"/>
+      <c r="E603" s="41"/>
+      <c r="F603" s="41"/>
+      <c r="G603" s="41"/>
+      <c r="H603" s="41"/>
       <c r="I603" s="41"/>
       <c r="J603" s="41"/>
       <c r="K603" s="41"/>
@@ -22399,10 +22717,10 @@
       <c r="G604" s="41"/>
       <c r="H604" s="41"/>
       <c r="I604" s="41"/>
-      <c r="J604" s="41"/>
+      <c r="J604" s="84"/>
       <c r="K604" s="41"/>
-      <c r="L604" s="53"/>
-      <c r="M604" s="53"/>
+      <c r="L604" s="41"/>
+      <c r="M604" s="41"/>
       <c r="N604" s="53"/>
       <c r="O604" s="41"/>
       <c r="P604" s="41"/>
@@ -22416,13 +22734,13 @@
       <c r="B605" s="53"/>
       <c r="C605" s="53"/>
       <c r="D605" s="53"/>
-      <c r="E605" s="41"/>
-      <c r="F605" s="41"/>
-      <c r="G605" s="41"/>
+      <c r="E605" s="53"/>
+      <c r="F605" s="53"/>
+      <c r="G605" s="53"/>
       <c r="H605" s="41"/>
       <c r="I605" s="41"/>
       <c r="J605" s="84"/>
-      <c r="K605" s="41"/>
+      <c r="K605" s="84"/>
       <c r="L605" s="41"/>
       <c r="M605" s="41"/>
       <c r="N605" s="53"/>
@@ -22445,8 +22763,8 @@
       <c r="I606" s="41"/>
       <c r="J606" s="84"/>
       <c r="K606" s="84"/>
-      <c r="L606" s="41"/>
-      <c r="M606" s="41"/>
+      <c r="L606" s="53"/>
+      <c r="M606" s="53"/>
       <c r="N606" s="53"/>
       <c r="O606" s="41"/>
       <c r="P606" s="41"/>
@@ -22466,7 +22784,7 @@
       <c r="H607" s="41"/>
       <c r="I607" s="41"/>
       <c r="J607" s="84"/>
-      <c r="K607" s="84"/>
+      <c r="K607" s="41"/>
       <c r="L607" s="53"/>
       <c r="M607" s="53"/>
       <c r="N607" s="53"/>
@@ -22553,7 +22871,7 @@
       <c r="G611" s="53"/>
       <c r="H611" s="41"/>
       <c r="I611" s="41"/>
-      <c r="J611" s="84"/>
+      <c r="J611" s="41"/>
       <c r="K611" s="41"/>
       <c r="L611" s="53"/>
       <c r="M611" s="53"/>
@@ -22663,7 +22981,7 @@
       <c r="G616" s="53"/>
       <c r="H616" s="41"/>
       <c r="I616" s="41"/>
-      <c r="J616" s="41"/>
+      <c r="J616" s="54"/>
       <c r="K616" s="41"/>
       <c r="L616" s="53"/>
       <c r="M616" s="53"/>
@@ -22787,12 +23105,12 @@
     </row>
     <row r="622" spans="1:20" ht="15" customHeight="1">
       <c r="A622" s="41"/>
-      <c r="B622" s="53"/>
-      <c r="C622" s="53"/>
-      <c r="D622" s="53"/>
-      <c r="E622" s="53"/>
-      <c r="F622" s="53"/>
-      <c r="G622" s="53"/>
+      <c r="B622" s="88"/>
+      <c r="C622" s="89"/>
+      <c r="D622" s="89"/>
+      <c r="E622" s="89"/>
+      <c r="F622" s="89"/>
+      <c r="G622" s="89"/>
       <c r="H622" s="41"/>
       <c r="I622" s="41"/>
       <c r="J622" s="54"/>
@@ -22807,14 +23125,14 @@
       <c r="S622" s="35"/>
       <c r="T622" s="35"/>
     </row>
-    <row r="623" spans="1:20" ht="15" customHeight="1">
+    <row r="623" spans="1:20" ht="16" customHeight="1">
       <c r="A623" s="41"/>
-      <c r="B623" s="88"/>
-      <c r="C623" s="89"/>
-      <c r="D623" s="89"/>
-      <c r="E623" s="89"/>
+      <c r="B623" s="90"/>
+      <c r="C623" s="91"/>
+      <c r="D623" s="91"/>
+      <c r="E623" s="91"/>
       <c r="F623" s="89"/>
-      <c r="G623" s="89"/>
+      <c r="G623" s="91"/>
       <c r="H623" s="41"/>
       <c r="I623" s="41"/>
       <c r="J623" s="54"/>
@@ -22897,12 +23215,12 @@
     </row>
     <row r="627" spans="1:20" ht="16" customHeight="1">
       <c r="A627" s="41"/>
-      <c r="B627" s="90"/>
-      <c r="C627" s="91"/>
-      <c r="D627" s="91"/>
-      <c r="E627" s="91"/>
+      <c r="B627" s="88"/>
+      <c r="C627" s="89"/>
+      <c r="D627" s="89"/>
+      <c r="E627" s="89"/>
       <c r="F627" s="89"/>
-      <c r="G627" s="91"/>
+      <c r="G627" s="89"/>
       <c r="H627" s="41"/>
       <c r="I627" s="41"/>
       <c r="J627" s="54"/>
@@ -22919,12 +23237,12 @@
     </row>
     <row r="628" spans="1:20" ht="16" customHeight="1">
       <c r="A628" s="41"/>
-      <c r="B628" s="88"/>
-      <c r="C628" s="89"/>
-      <c r="D628" s="89"/>
-      <c r="E628" s="89"/>
+      <c r="B628" s="90"/>
+      <c r="C628" s="91"/>
+      <c r="D628" s="91"/>
+      <c r="E628" s="91"/>
       <c r="F628" s="89"/>
-      <c r="G628" s="89"/>
+      <c r="G628" s="91"/>
       <c r="H628" s="41"/>
       <c r="I628" s="41"/>
       <c r="J628" s="54"/>
@@ -22993,7 +23311,7 @@
       <c r="G631" s="91"/>
       <c r="H631" s="41"/>
       <c r="I631" s="41"/>
-      <c r="J631" s="54"/>
+      <c r="J631" s="41"/>
       <c r="K631" s="41"/>
       <c r="L631" s="53"/>
       <c r="M631" s="53"/>
@@ -23007,12 +23325,12 @@
     </row>
     <row r="632" spans="1:20" ht="16" customHeight="1">
       <c r="A632" s="41"/>
-      <c r="B632" s="90"/>
-      <c r="C632" s="91"/>
-      <c r="D632" s="91"/>
-      <c r="E632" s="91"/>
+      <c r="B632" s="88"/>
+      <c r="C632" s="89"/>
+      <c r="D632" s="89"/>
+      <c r="E632" s="89"/>
       <c r="F632" s="89"/>
-      <c r="G632" s="91"/>
+      <c r="G632" s="89"/>
       <c r="H632" s="41"/>
       <c r="I632" s="41"/>
       <c r="J632" s="41"/>
@@ -23029,12 +23347,12 @@
     </row>
     <row r="633" spans="1:20" ht="16" customHeight="1">
       <c r="A633" s="41"/>
-      <c r="B633" s="88"/>
-      <c r="C633" s="89"/>
-      <c r="D633" s="89"/>
-      <c r="E633" s="89"/>
+      <c r="B633" s="90"/>
+      <c r="C633" s="91"/>
+      <c r="D633" s="91"/>
+      <c r="E633" s="91"/>
       <c r="F633" s="89"/>
-      <c r="G633" s="89"/>
+      <c r="G633" s="91"/>
       <c r="H633" s="41"/>
       <c r="I633" s="41"/>
       <c r="J633" s="41"/>
@@ -23125,7 +23443,7 @@
       <c r="G637" s="91"/>
       <c r="H637" s="41"/>
       <c r="I637" s="41"/>
-      <c r="J637" s="41"/>
+      <c r="J637" s="84"/>
       <c r="K637" s="41"/>
       <c r="L637" s="53"/>
       <c r="M637" s="53"/>
@@ -23138,17 +23456,17 @@
       <c r="T637" s="35"/>
     </row>
     <row r="638" spans="1:20" ht="16" customHeight="1">
-      <c r="A638" s="41"/>
-      <c r="B638" s="90"/>
-      <c r="C638" s="91"/>
-      <c r="D638" s="91"/>
-      <c r="E638" s="91"/>
-      <c r="F638" s="89"/>
-      <c r="G638" s="91"/>
+      <c r="A638" s="53"/>
+      <c r="B638" s="53"/>
+      <c r="C638" s="53"/>
+      <c r="D638" s="53"/>
+      <c r="E638" s="53"/>
+      <c r="F638" s="53"/>
+      <c r="G638" s="53"/>
       <c r="H638" s="41"/>
       <c r="I638" s="41"/>
       <c r="J638" s="84"/>
-      <c r="K638" s="41"/>
+      <c r="K638" s="84"/>
       <c r="L638" s="53"/>
       <c r="M638" s="53"/>
       <c r="N638" s="53"/>
@@ -23213,7 +23531,7 @@
       <c r="G641" s="53"/>
       <c r="H641" s="41"/>
       <c r="I641" s="41"/>
-      <c r="J641" s="84"/>
+      <c r="J641" s="41"/>
       <c r="K641" s="84"/>
       <c r="L641" s="53"/>
       <c r="M641" s="53"/>
@@ -23236,7 +23554,7 @@
       <c r="H642" s="41"/>
       <c r="I642" s="41"/>
       <c r="J642" s="41"/>
-      <c r="K642" s="84"/>
+      <c r="K642" s="41"/>
       <c r="L642" s="53"/>
       <c r="M642" s="53"/>
       <c r="N642" s="53"/>
@@ -23301,10 +23619,10 @@
       <c r="G645" s="53"/>
       <c r="H645" s="41"/>
       <c r="I645" s="41"/>
-      <c r="J645" s="41"/>
+      <c r="J645" s="84"/>
       <c r="K645" s="41"/>
       <c r="L645" s="53"/>
-      <c r="M645" s="53"/>
+      <c r="M645" s="41"/>
       <c r="N645" s="53"/>
       <c r="O645" s="41"/>
       <c r="P645" s="41"/>
@@ -23321,10 +23639,10 @@
       <c r="E646" s="53"/>
       <c r="F646" s="53"/>
       <c r="G646" s="53"/>
-      <c r="H646" s="41"/>
+      <c r="H646" s="53"/>
       <c r="I646" s="41"/>
       <c r="J646" s="84"/>
-      <c r="K646" s="41"/>
+      <c r="K646" s="84"/>
       <c r="L646" s="53"/>
       <c r="M646" s="41"/>
       <c r="N646" s="53"/>
@@ -23348,7 +23666,7 @@
       <c r="J647" s="84"/>
       <c r="K647" s="84"/>
       <c r="L647" s="53"/>
-      <c r="M647" s="41"/>
+      <c r="M647" s="53"/>
       <c r="N647" s="53"/>
       <c r="O647" s="41"/>
       <c r="P647" s="41"/>
@@ -23389,7 +23707,7 @@
       <c r="G649" s="53"/>
       <c r="H649" s="53"/>
       <c r="I649" s="41"/>
-      <c r="J649" s="84"/>
+      <c r="J649" s="54"/>
       <c r="K649" s="84"/>
       <c r="L649" s="53"/>
       <c r="M649" s="53"/>
@@ -23412,7 +23730,7 @@
       <c r="H650" s="53"/>
       <c r="I650" s="41"/>
       <c r="J650" s="54"/>
-      <c r="K650" s="84"/>
+      <c r="K650" s="41"/>
       <c r="L650" s="53"/>
       <c r="M650" s="53"/>
       <c r="N650" s="53"/>
@@ -23433,16 +23751,16 @@
       <c r="G651" s="53"/>
       <c r="H651" s="53"/>
       <c r="I651" s="41"/>
-      <c r="J651" s="54"/>
+      <c r="J651" s="84"/>
       <c r="K651" s="41"/>
-      <c r="L651" s="53"/>
-      <c r="M651" s="53"/>
+      <c r="L651" s="41"/>
+      <c r="M651" s="41"/>
       <c r="N651" s="53"/>
       <c r="O651" s="41"/>
       <c r="P651" s="41"/>
       <c r="Q651" s="41"/>
       <c r="R651" s="41"/>
-      <c r="S651" s="35"/>
+      <c r="S651" s="42"/>
       <c r="T651" s="35"/>
     </row>
     <row r="652" spans="1:20" ht="16" customHeight="1">
@@ -23450,13 +23768,13 @@
       <c r="B652" s="53"/>
       <c r="C652" s="53"/>
       <c r="D652" s="53"/>
-      <c r="E652" s="53"/>
+      <c r="E652" s="41"/>
       <c r="F652" s="53"/>
       <c r="G652" s="53"/>
       <c r="H652" s="53"/>
       <c r="I652" s="41"/>
       <c r="J652" s="84"/>
-      <c r="K652" s="41"/>
+      <c r="K652" s="84"/>
       <c r="L652" s="41"/>
       <c r="M652" s="41"/>
       <c r="N652" s="53"/>
@@ -23479,8 +23797,8 @@
       <c r="I653" s="41"/>
       <c r="J653" s="84"/>
       <c r="K653" s="84"/>
-      <c r="L653" s="41"/>
-      <c r="M653" s="41"/>
+      <c r="L653" s="53"/>
+      <c r="M653" s="53"/>
       <c r="N653" s="53"/>
       <c r="O653" s="41"/>
       <c r="P653" s="41"/>
@@ -23494,7 +23812,7 @@
       <c r="B654" s="53"/>
       <c r="C654" s="53"/>
       <c r="D654" s="53"/>
-      <c r="E654" s="41"/>
+      <c r="E654" s="53"/>
       <c r="F654" s="53"/>
       <c r="G654" s="53"/>
       <c r="H654" s="53"/>
@@ -23521,7 +23839,7 @@
       <c r="G655" s="53"/>
       <c r="H655" s="53"/>
       <c r="I655" s="41"/>
-      <c r="J655" s="84"/>
+      <c r="J655" s="54"/>
       <c r="K655" s="84"/>
       <c r="L655" s="53"/>
       <c r="M655" s="53"/>
@@ -23538,13 +23856,13 @@
       <c r="B656" s="53"/>
       <c r="C656" s="53"/>
       <c r="D656" s="53"/>
-      <c r="E656" s="53"/>
+      <c r="E656" s="41"/>
       <c r="F656" s="53"/>
       <c r="G656" s="53"/>
       <c r="H656" s="53"/>
       <c r="I656" s="41"/>
       <c r="J656" s="54"/>
-      <c r="K656" s="84"/>
+      <c r="K656" s="41"/>
       <c r="L656" s="53"/>
       <c r="M656" s="53"/>
       <c r="N656" s="53"/>
@@ -23582,7 +23900,7 @@
       <c r="B658" s="53"/>
       <c r="C658" s="53"/>
       <c r="D658" s="53"/>
-      <c r="E658" s="41"/>
+      <c r="E658" s="53"/>
       <c r="F658" s="53"/>
       <c r="G658" s="53"/>
       <c r="H658" s="53"/>
@@ -23626,7 +23944,7 @@
       <c r="B660" s="53"/>
       <c r="C660" s="53"/>
       <c r="D660" s="53"/>
-      <c r="E660" s="53"/>
+      <c r="E660" s="41"/>
       <c r="F660" s="53"/>
       <c r="G660" s="53"/>
       <c r="H660" s="53"/>
@@ -23670,7 +23988,7 @@
       <c r="B662" s="53"/>
       <c r="C662" s="53"/>
       <c r="D662" s="53"/>
-      <c r="E662" s="41"/>
+      <c r="E662" s="53"/>
       <c r="F662" s="53"/>
       <c r="G662" s="53"/>
       <c r="H662" s="53"/>
@@ -23714,7 +24032,7 @@
       <c r="B664" s="53"/>
       <c r="C664" s="53"/>
       <c r="D664" s="53"/>
-      <c r="E664" s="53"/>
+      <c r="E664" s="41"/>
       <c r="F664" s="53"/>
       <c r="G664" s="53"/>
       <c r="H664" s="53"/>
@@ -23758,7 +24076,7 @@
       <c r="B666" s="53"/>
       <c r="C666" s="53"/>
       <c r="D666" s="53"/>
-      <c r="E666" s="41"/>
+      <c r="E666" s="53"/>
       <c r="F666" s="53"/>
       <c r="G666" s="53"/>
       <c r="H666" s="53"/>
@@ -23780,7 +24098,7 @@
       <c r="B667" s="53"/>
       <c r="C667" s="53"/>
       <c r="D667" s="53"/>
-      <c r="E667" s="53"/>
+      <c r="E667" s="41"/>
       <c r="F667" s="53"/>
       <c r="G667" s="53"/>
       <c r="H667" s="53"/>
@@ -23824,7 +24142,7 @@
       <c r="B669" s="53"/>
       <c r="C669" s="53"/>
       <c r="D669" s="53"/>
-      <c r="E669" s="41"/>
+      <c r="E669" s="53"/>
       <c r="F669" s="53"/>
       <c r="G669" s="53"/>
       <c r="H669" s="53"/>
@@ -23851,7 +24169,7 @@
       <c r="G670" s="53"/>
       <c r="H670" s="53"/>
       <c r="I670" s="41"/>
-      <c r="J670" s="54"/>
+      <c r="J670" s="84"/>
       <c r="K670" s="41"/>
       <c r="L670" s="53"/>
       <c r="M670" s="53"/>
@@ -23864,7 +24182,7 @@
       <c r="T670" s="35"/>
     </row>
     <row r="671" spans="1:20" ht="16" customHeight="1">
-      <c r="A671" s="53"/>
+      <c r="A671" s="41"/>
       <c r="B671" s="53"/>
       <c r="C671" s="53"/>
       <c r="D671" s="53"/>
@@ -23893,7 +24211,7 @@
       <c r="E672" s="53"/>
       <c r="F672" s="53"/>
       <c r="G672" s="53"/>
-      <c r="H672" s="53"/>
+      <c r="H672" s="41"/>
       <c r="I672" s="41"/>
       <c r="J672" s="84"/>
       <c r="K672" s="41"/>
@@ -23915,7 +24233,7 @@
       <c r="E673" s="53"/>
       <c r="F673" s="53"/>
       <c r="G673" s="53"/>
-      <c r="H673" s="41"/>
+      <c r="H673" s="53"/>
       <c r="I673" s="41"/>
       <c r="J673" s="84"/>
       <c r="K673" s="41"/>
@@ -23937,7 +24255,7 @@
       <c r="E674" s="53"/>
       <c r="F674" s="53"/>
       <c r="G674" s="53"/>
-      <c r="H674" s="53"/>
+      <c r="H674" s="41"/>
       <c r="I674" s="41"/>
       <c r="J674" s="84"/>
       <c r="K674" s="41"/>
@@ -23959,7 +24277,7 @@
       <c r="E675" s="53"/>
       <c r="F675" s="53"/>
       <c r="G675" s="53"/>
-      <c r="H675" s="41"/>
+      <c r="H675" s="53"/>
       <c r="I675" s="41"/>
       <c r="J675" s="84"/>
       <c r="K675" s="41"/>
@@ -23981,9 +24299,9 @@
       <c r="E676" s="53"/>
       <c r="F676" s="53"/>
       <c r="G676" s="53"/>
-      <c r="H676" s="53"/>
+      <c r="H676" s="41"/>
       <c r="I676" s="41"/>
-      <c r="J676" s="84"/>
+      <c r="J676" s="54"/>
       <c r="K676" s="41"/>
       <c r="L676" s="53"/>
       <c r="M676" s="53"/>
@@ -24000,7 +24318,7 @@
       <c r="B677" s="53"/>
       <c r="C677" s="53"/>
       <c r="D677" s="53"/>
-      <c r="E677" s="53"/>
+      <c r="E677" s="41"/>
       <c r="F677" s="53"/>
       <c r="G677" s="53"/>
       <c r="H677" s="41"/>
@@ -24027,10 +24345,10 @@
       <c r="G678" s="53"/>
       <c r="H678" s="41"/>
       <c r="I678" s="41"/>
-      <c r="J678" s="54"/>
+      <c r="J678" s="84"/>
       <c r="K678" s="41"/>
       <c r="L678" s="53"/>
-      <c r="M678" s="53"/>
+      <c r="M678" s="41"/>
       <c r="N678" s="53"/>
       <c r="O678" s="41"/>
       <c r="P678" s="41"/>
@@ -24041,16 +24359,16 @@
     </row>
     <row r="679" spans="1:20" ht="16" customHeight="1">
       <c r="A679" s="41"/>
-      <c r="B679" s="53"/>
+      <c r="B679" s="96"/>
       <c r="C679" s="53"/>
       <c r="D679" s="53"/>
-      <c r="E679" s="41"/>
+      <c r="E679" s="53"/>
       <c r="F679" s="53"/>
       <c r="G679" s="53"/>
       <c r="H679" s="41"/>
       <c r="I679" s="41"/>
       <c r="J679" s="84"/>
-      <c r="K679" s="41"/>
+      <c r="K679" s="84"/>
       <c r="L679" s="53"/>
       <c r="M679" s="41"/>
       <c r="N679" s="53"/>
@@ -24071,10 +24389,10 @@
       <c r="G680" s="53"/>
       <c r="H680" s="41"/>
       <c r="I680" s="41"/>
-      <c r="J680" s="84"/>
+      <c r="J680" s="54"/>
       <c r="K680" s="84"/>
       <c r="L680" s="53"/>
-      <c r="M680" s="41"/>
+      <c r="M680" s="53"/>
       <c r="N680" s="53"/>
       <c r="O680" s="41"/>
       <c r="P680" s="41"/>
@@ -24094,7 +24412,7 @@
       <c r="H681" s="41"/>
       <c r="I681" s="41"/>
       <c r="J681" s="54"/>
-      <c r="K681" s="84"/>
+      <c r="K681" s="54"/>
       <c r="L681" s="53"/>
       <c r="M681" s="53"/>
       <c r="N681" s="53"/>
@@ -24159,7 +24477,7 @@
       <c r="G684" s="53"/>
       <c r="H684" s="41"/>
       <c r="I684" s="41"/>
-      <c r="J684" s="54"/>
+      <c r="J684" s="41"/>
       <c r="K684" s="54"/>
       <c r="L684" s="53"/>
       <c r="M684" s="53"/>
@@ -24173,16 +24491,16 @@
     </row>
     <row r="685" spans="1:20" ht="16" customHeight="1">
       <c r="A685" s="41"/>
-      <c r="B685" s="96"/>
-      <c r="C685" s="53"/>
-      <c r="D685" s="53"/>
-      <c r="E685" s="53"/>
-      <c r="F685" s="53"/>
-      <c r="G685" s="53"/>
+      <c r="B685" s="41"/>
+      <c r="C685" s="41"/>
+      <c r="D685" s="41"/>
+      <c r="E685" s="41"/>
+      <c r="F685" s="41"/>
+      <c r="G685" s="41"/>
       <c r="H685" s="41"/>
       <c r="I685" s="41"/>
       <c r="J685" s="41"/>
-      <c r="K685" s="54"/>
+      <c r="K685" s="41"/>
       <c r="L685" s="53"/>
       <c r="M685" s="53"/>
       <c r="N685" s="53"/>
@@ -24205,9 +24523,9 @@
       <c r="I686" s="41"/>
       <c r="J686" s="41"/>
       <c r="K686" s="41"/>
-      <c r="L686" s="53"/>
-      <c r="M686" s="53"/>
-      <c r="N686" s="53"/>
+      <c r="L686" s="41"/>
+      <c r="M686" s="41"/>
+      <c r="N686" s="41"/>
       <c r="O686" s="41"/>
       <c r="P686" s="41"/>
       <c r="Q686" s="41"/>
@@ -25268,7 +25586,7 @@
       <c r="P734" s="41"/>
       <c r="Q734" s="41"/>
       <c r="R734" s="41"/>
-      <c r="S734" s="42"/>
+      <c r="S734" s="35"/>
       <c r="T734" s="35"/>
     </row>
     <row r="735" spans="1:20" ht="16" customHeight="1">
@@ -25312,7 +25630,7 @@
       <c r="P736" s="41"/>
       <c r="Q736" s="41"/>
       <c r="R736" s="41"/>
-      <c r="S736" s="35"/>
+      <c r="S736" s="42"/>
       <c r="T736" s="35"/>
     </row>
     <row r="737" spans="1:20" ht="16" customHeight="1">
@@ -25598,7 +25916,7 @@
       <c r="P749" s="41"/>
       <c r="Q749" s="41"/>
       <c r="R749" s="41"/>
-      <c r="S749" s="42"/>
+      <c r="S749" s="35"/>
       <c r="T749" s="35"/>
     </row>
     <row r="750" spans="1:20" ht="16" customHeight="1">
@@ -27867,7 +28185,7 @@
       <c r="S852" s="35"/>
       <c r="T852" s="35"/>
     </row>
-    <row r="853" spans="1:20" ht="16" customHeight="1">
+    <row r="853" spans="1:20" ht="15" customHeight="1">
       <c r="A853" s="41"/>
       <c r="B853" s="41"/>
       <c r="C853" s="41"/>
@@ -27886,8 +28204,8 @@
       <c r="P853" s="41"/>
       <c r="Q853" s="41"/>
       <c r="R853" s="41"/>
-      <c r="S853" s="35"/>
-      <c r="T853" s="35"/>
+      <c r="S853" s="41"/>
+      <c r="T853" s="41"/>
     </row>
     <row r="854" spans="1:20" ht="15" customHeight="1">
       <c r="A854" s="41"/>
@@ -29717,7 +30035,6 @@
     </row>
     <row r="937" spans="1:20" ht="15" customHeight="1">
       <c r="A937" s="41"/>
-      <c r="B937" s="41"/>
       <c r="C937" s="41"/>
       <c r="D937" s="41"/>
       <c r="E937" s="41"/>
@@ -29844,14 +30161,12 @@
     </row>
     <row r="943" spans="1:20" ht="15" customHeight="1">
       <c r="A943" s="41"/>
-      <c r="C943" s="41"/>
       <c r="D943" s="41"/>
       <c r="E943" s="41"/>
       <c r="F943" s="41"/>
       <c r="G943" s="41"/>
       <c r="H943" s="41"/>
       <c r="I943" s="41"/>
-      <c r="J943" s="41"/>
       <c r="K943" s="41"/>
       <c r="L943" s="41"/>
       <c r="M943" s="41"/>
@@ -29870,8 +30185,6 @@
       <c r="F944" s="41"/>
       <c r="G944" s="41"/>
       <c r="H944" s="41"/>
-      <c r="I944" s="41"/>
-      <c r="K944" s="41"/>
       <c r="L944" s="41"/>
       <c r="M944" s="41"/>
       <c r="N944" s="41"/>
@@ -29940,7 +30253,6 @@
       <c r="F948" s="41"/>
       <c r="G948" s="41"/>
       <c r="H948" s="41"/>
-      <c r="L948" s="41"/>
       <c r="M948" s="41"/>
       <c r="N948" s="41"/>
       <c r="O948" s="41"/>
@@ -29960,7 +30272,6 @@
       <c r="M949" s="41"/>
       <c r="N949" s="41"/>
       <c r="O949" s="41"/>
-      <c r="P949" s="41"/>
       <c r="Q949" s="41"/>
       <c r="R949" s="41"/>
       <c r="S949" s="41"/>
@@ -30006,7 +30317,6 @@
       <c r="M952" s="41"/>
       <c r="N952" s="41"/>
       <c r="O952" s="41"/>
-      <c r="Q952" s="41"/>
       <c r="R952" s="41"/>
       <c r="S952" s="41"/>
       <c r="T952" s="41"/>
@@ -30040,12 +30350,6 @@
       <c r="T954" s="41"/>
     </row>
     <row r="955" spans="1:20" ht="15" customHeight="1">
-      <c r="A955" s="41"/>
-      <c r="D955" s="41"/>
-      <c r="E955" s="41"/>
-      <c r="F955" s="41"/>
-      <c r="G955" s="41"/>
-      <c r="H955" s="41"/>
       <c r="M955" s="41"/>
       <c r="N955" s="41"/>
       <c r="O955" s="41"/>
@@ -30054,15 +30358,12 @@
       <c r="T955" s="41"/>
     </row>
     <row r="956" spans="1:20" ht="15" customHeight="1">
-      <c r="M956" s="41"/>
-      <c r="N956" s="41"/>
       <c r="O956" s="41"/>
       <c r="R956" s="41"/>
       <c r="S956" s="41"/>
       <c r="T956" s="41"/>
     </row>
     <row r="957" spans="1:20" ht="15" customHeight="1">
-      <c r="O957" s="41"/>
       <c r="R957" s="41"/>
       <c r="S957" s="41"/>
       <c r="T957" s="41"/>
@@ -30076,11 +30377,6 @@
       <c r="R959" s="41"/>
       <c r="S959" s="41"/>
       <c r="T959" s="41"/>
-    </row>
-    <row r="960" spans="1:20" ht="15" customHeight="1">
-      <c r="R960" s="41"/>
-      <c r="S960" s="41"/>
-      <c r="T960" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.intermet.2023.107947`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A021E5C2-0366-2742-BA67-1FA45D7DF366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A049DAE2-E9E3-7248-A293-5BB80E925390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2398" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2416" uniqueCount="286">
   <si>
     <r>
       <rPr>
@@ -964,6 +964,30 @@
   </si>
   <si>
     <t>10.1016/j.jallcom.2020.154101</t>
+  </si>
+  <si>
+    <t>10.1016/j.intermet.2023.107947</t>
+  </si>
+  <si>
+    <t>Ti35 Zr25 Ta15 Nb15 Sn10</t>
+  </si>
+  <si>
+    <t>VAM+HW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minor secondary disordered ZrSn-rich BCC </t>
+  </si>
+  <si>
+    <t>BCC+BCC+HCP+Zr5Sn3</t>
+  </si>
+  <si>
+    <t>as cast ingot was slowly pressed up to 4000MPa and held at 1800K for 10min and releived without any quench; majority disordered BCC with nanoscale Zr5Sn3 and BCC precipitation with nanoscale LRO</t>
+  </si>
+  <si>
+    <t>nanohardness</t>
+  </si>
+  <si>
+    <t>F3b</t>
   </si>
 </sst>
 </file>
@@ -14922,19 +14946,41 @@
     </row>
     <row r="250" spans="1:20" ht="18" customHeight="1">
       <c r="A250" s="106"/>
-      <c r="B250" s="99"/>
-      <c r="C250" s="86"/>
-      <c r="D250" s="86"/>
-      <c r="E250" s="99"/>
-      <c r="F250" s="49"/>
-      <c r="G250" s="31"/>
+      <c r="B250" s="99" t="s">
+        <v>279</v>
+      </c>
+      <c r="C250" s="86" t="s">
+        <v>110</v>
+      </c>
+      <c r="D250" s="86" t="s">
+        <v>108</v>
+      </c>
+      <c r="E250" s="99" t="s">
+        <v>281</v>
+      </c>
+      <c r="F250" s="49" t="s">
+        <v>284</v>
+      </c>
+      <c r="G250" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H250" s="52"/>
-      <c r="I250" s="50"/>
-      <c r="J250" s="38"/>
+      <c r="I250" s="50">
+        <v>298</v>
+      </c>
+      <c r="J250" s="107">
+        <v>5990000000</v>
+      </c>
       <c r="K250" s="36"/>
-      <c r="L250" s="38"/>
-      <c r="M250" s="38"/>
-      <c r="N250" s="29"/>
+      <c r="L250" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M250" s="38" t="s">
+        <v>285</v>
+      </c>
+      <c r="N250" s="29" t="s">
+        <v>278</v>
+      </c>
       <c r="O250" s="41"/>
       <c r="P250" s="41"/>
       <c r="Q250" s="41"/>
@@ -14944,19 +14990,41 @@
     </row>
     <row r="251" spans="1:20" ht="18" customHeight="1">
       <c r="A251" s="106"/>
-      <c r="B251" s="99"/>
-      <c r="C251" s="86"/>
-      <c r="D251" s="86"/>
-      <c r="E251" s="99"/>
-      <c r="F251" s="49"/>
-      <c r="G251" s="31"/>
+      <c r="B251" s="99" t="s">
+        <v>279</v>
+      </c>
+      <c r="C251" s="86" t="s">
+        <v>282</v>
+      </c>
+      <c r="D251" s="86" t="s">
+        <v>280</v>
+      </c>
+      <c r="E251" s="99" t="s">
+        <v>283</v>
+      </c>
+      <c r="F251" s="49" t="s">
+        <v>284</v>
+      </c>
+      <c r="G251" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H251" s="52"/>
-      <c r="I251" s="50"/>
-      <c r="J251" s="38"/>
+      <c r="I251" s="50">
+        <v>298</v>
+      </c>
+      <c r="J251" s="107">
+        <v>7470000000</v>
+      </c>
       <c r="K251" s="36"/>
-      <c r="L251" s="38"/>
-      <c r="M251" s="38"/>
-      <c r="N251" s="29"/>
+      <c r="L251" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M251" s="38" t="s">
+        <v>285</v>
+      </c>
+      <c r="N251" s="29" t="s">
+        <v>278</v>
+      </c>
       <c r="O251" s="41"/>
       <c r="P251" s="41"/>
       <c r="Q251" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.3390/coatings12040531 `
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A049DAE2-E9E3-7248-A293-5BB80E925390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09163D7C-2230-CC4E-ABA6-01099121CE79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2416" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="292">
   <si>
     <r>
       <rPr>
@@ -988,6 +988,24 @@
   </si>
   <si>
     <t>F3b</t>
+  </si>
+  <si>
+    <t>Mg30 Zn30 Sn30 Sr5 Bi5</t>
+  </si>
+  <si>
+    <t>AIM</t>
+  </si>
+  <si>
+    <t>Mg2Sn+MgSnSr+Mg38Sr9+alpha+MgZn</t>
+  </si>
+  <si>
+    <t>very complex as-solidified microstrcuture with 5-8 phases detected / discussed by authors but treat data with caution</t>
+  </si>
+  <si>
+    <t>melting point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.3390/coatings12040531 </t>
   </si>
 </sst>
 </file>
@@ -15034,41 +15052,91 @@
     </row>
     <row r="252" spans="1:20" ht="18" customHeight="1">
       <c r="A252" s="106"/>
-      <c r="B252" s="99"/>
-      <c r="C252" s="86"/>
-      <c r="D252" s="86"/>
-      <c r="E252" s="99"/>
-      <c r="F252" s="49"/>
-      <c r="G252" s="31"/>
+      <c r="B252" s="99" t="s">
+        <v>286</v>
+      </c>
+      <c r="C252" s="86" t="s">
+        <v>288</v>
+      </c>
+      <c r="D252" s="86" t="s">
+        <v>287</v>
+      </c>
+      <c r="E252" s="99" t="s">
+        <v>289</v>
+      </c>
+      <c r="F252" s="49" t="s">
+        <v>111</v>
+      </c>
+      <c r="G252" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H252" s="52"/>
-      <c r="I252" s="50"/>
-      <c r="J252" s="38"/>
-      <c r="K252" s="36"/>
-      <c r="L252" s="38"/>
+      <c r="I252" s="50">
+        <v>298</v>
+      </c>
+      <c r="J252" s="84">
+        <f t="shared" ref="J252:K252" si="6">P252*9807000</f>
+        <v>1716225000</v>
+      </c>
+      <c r="K252" s="84">
+        <f t="shared" si="6"/>
+        <v>735525000</v>
+      </c>
+      <c r="L252" s="38" t="s">
+        <v>32</v>
+      </c>
       <c r="M252" s="38"/>
-      <c r="N252" s="29"/>
+      <c r="N252" s="29" t="s">
+        <v>291</v>
+      </c>
       <c r="O252" s="41"/>
-      <c r="P252" s="41"/>
-      <c r="Q252" s="41"/>
+      <c r="P252" s="41">
+        <v>175</v>
+      </c>
+      <c r="Q252" s="41">
+        <v>75</v>
+      </c>
       <c r="R252" s="41"/>
       <c r="S252" s="35"/>
       <c r="T252" s="35"/>
     </row>
     <row r="253" spans="1:20" ht="18" customHeight="1">
       <c r="A253" s="106"/>
-      <c r="B253" s="99"/>
-      <c r="C253" s="86"/>
-      <c r="D253" s="86"/>
-      <c r="E253" s="99"/>
-      <c r="F253" s="49"/>
-      <c r="G253" s="31"/>
+      <c r="B253" s="99" t="s">
+        <v>286</v>
+      </c>
+      <c r="C253" s="86" t="s">
+        <v>288</v>
+      </c>
+      <c r="D253" s="86" t="s">
+        <v>287</v>
+      </c>
+      <c r="E253" s="99" t="s">
+        <v>289</v>
+      </c>
+      <c r="F253" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="G253" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H253" s="52"/>
-      <c r="I253" s="50"/>
-      <c r="J253" s="38"/>
+      <c r="I253" s="50">
+        <v>298</v>
+      </c>
+      <c r="J253" s="107">
+        <v>17980000000</v>
+      </c>
       <c r="K253" s="36"/>
-      <c r="L253" s="38"/>
-      <c r="M253" s="38"/>
-      <c r="N253" s="29"/>
+      <c r="L253" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M253" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N253" s="29" t="s">
+        <v>291</v>
+      </c>
       <c r="O253" s="41"/>
       <c r="P253" s="41"/>
       <c r="Q253" s="41"/>
@@ -15078,19 +15146,41 @@
     </row>
     <row r="254" spans="1:20" ht="18" customHeight="1">
       <c r="A254" s="106"/>
-      <c r="B254" s="99"/>
-      <c r="C254" s="86"/>
-      <c r="D254" s="86"/>
-      <c r="E254" s="99"/>
-      <c r="F254" s="49"/>
-      <c r="G254" s="31"/>
+      <c r="B254" s="99" t="s">
+        <v>286</v>
+      </c>
+      <c r="C254" s="86" t="s">
+        <v>288</v>
+      </c>
+      <c r="D254" s="86" t="s">
+        <v>287</v>
+      </c>
+      <c r="E254" s="99" t="s">
+        <v>289</v>
+      </c>
+      <c r="F254" s="49" t="s">
+        <v>112</v>
+      </c>
+      <c r="G254" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H254" s="52"/>
-      <c r="I254" s="50"/>
-      <c r="J254" s="38"/>
+      <c r="I254" s="50">
+        <v>298</v>
+      </c>
+      <c r="J254" s="38">
+        <v>192.84</v>
+      </c>
       <c r="K254" s="36"/>
-      <c r="L254" s="38"/>
-      <c r="M254" s="38"/>
-      <c r="N254" s="29"/>
+      <c r="L254" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M254" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="N254" s="29" t="s">
+        <v>291</v>
+      </c>
       <c r="O254" s="41"/>
       <c r="P254" s="41"/>
       <c r="Q254" s="41"/>
@@ -15100,19 +15190,38 @@
     </row>
     <row r="255" spans="1:20" ht="18" customHeight="1">
       <c r="A255" s="105"/>
-      <c r="B255" s="97"/>
-      <c r="C255" s="85"/>
-      <c r="D255" s="85"/>
-      <c r="E255" s="97"/>
-      <c r="F255" s="49"/>
-      <c r="G255" s="31"/>
+      <c r="B255" s="99" t="s">
+        <v>286</v>
+      </c>
+      <c r="C255" s="86" t="s">
+        <v>288</v>
+      </c>
+      <c r="D255" s="86" t="s">
+        <v>287</v>
+      </c>
+      <c r="E255" s="99" t="s">
+        <v>289</v>
+      </c>
+      <c r="F255" s="49" t="s">
+        <v>290</v>
+      </c>
+      <c r="G255" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H255" s="52"/>
       <c r="I255" s="50"/>
-      <c r="J255" s="38"/>
+      <c r="J255" s="38">
+        <f>420+273</f>
+        <v>693</v>
+      </c>
       <c r="K255" s="36"/>
-      <c r="L255" s="38"/>
+      <c r="L255" s="38" t="s">
+        <v>223</v>
+      </c>
       <c r="M255" s="38"/>
-      <c r="N255" s="29"/>
+      <c r="N255" s="29" t="s">
+        <v>291</v>
+      </c>
       <c r="O255" s="41"/>
       <c r="P255" s="41"/>
       <c r="Q255" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.3390/ma18235261 `
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09163D7C-2230-CC4E-ABA6-01099121CE79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603F80F0-9B84-ED43-9398-FC07AAE938AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="297">
   <si>
     <r>
       <rPr>
@@ -1006,6 +1006,21 @@
   </si>
   <si>
     <t xml:space="preserve">10.3390/coatings12040531 </t>
+  </si>
+  <si>
+    <t>Cr16 Mn16 Fe16 Co16 Ni16 P20</t>
+  </si>
+  <si>
+    <t>FCC+CrCoP+Ni3P+MnNiP</t>
+  </si>
+  <si>
+    <t>complex eutectic-like microstructure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melt spun onto copper at 20m/s resulting in 20um thick ribbons </t>
+  </si>
+  <si>
+    <t>10.3390/ma18235261</t>
   </si>
 </sst>
 </file>
@@ -15231,10 +15246,18 @@
     </row>
     <row r="256" spans="1:20" ht="18" customHeight="1">
       <c r="A256" s="106"/>
-      <c r="B256" s="99"/>
-      <c r="C256" s="86"/>
-      <c r="D256" s="86"/>
-      <c r="E256" s="99"/>
+      <c r="B256" s="99" t="s">
+        <v>292</v>
+      </c>
+      <c r="C256" s="86" t="s">
+        <v>293</v>
+      </c>
+      <c r="D256" s="86" t="s">
+        <v>164</v>
+      </c>
+      <c r="E256" s="99" t="s">
+        <v>294</v>
+      </c>
       <c r="F256" s="49"/>
       <c r="G256" s="31"/>
       <c r="H256" s="52"/>
@@ -15243,7 +15266,9 @@
       <c r="K256" s="36"/>
       <c r="L256" s="38"/>
       <c r="M256" s="38"/>
-      <c r="N256" s="29"/>
+      <c r="N256" s="29" t="s">
+        <v>296</v>
+      </c>
       <c r="O256" s="41"/>
       <c r="P256" s="41"/>
       <c r="Q256" s="41"/>
@@ -15253,10 +15278,18 @@
     </row>
     <row r="257" spans="1:20" ht="18" customHeight="1">
       <c r="A257" s="106"/>
-      <c r="B257" s="99"/>
-      <c r="C257" s="86"/>
-      <c r="D257" s="86"/>
-      <c r="E257" s="99"/>
+      <c r="B257" s="99" t="s">
+        <v>292</v>
+      </c>
+      <c r="C257" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D257" s="86" t="s">
+        <v>268</v>
+      </c>
+      <c r="E257" s="99" t="s">
+        <v>295</v>
+      </c>
       <c r="F257" s="49"/>
       <c r="G257" s="31"/>
       <c r="H257" s="52"/>
@@ -15265,7 +15298,9 @@
       <c r="K257" s="36"/>
       <c r="L257" s="38"/>
       <c r="M257" s="38"/>
-      <c r="N257" s="29"/>
+      <c r="N257" s="29" t="s">
+        <v>296</v>
+      </c>
       <c r="O257" s="41"/>
       <c r="P257" s="41"/>
       <c r="Q257" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1063/1.3575562 `
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603F80F0-9B84-ED43-9398-FC07AAE938AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B71DDC8-168B-0C4E-BDD4-506451E1E257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="11220" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="320" yWindow="11020" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2522" uniqueCount="306">
   <si>
     <r>
       <rPr>
@@ -1021,6 +1021,33 @@
   </si>
   <si>
     <t>10.3390/ma18235261</t>
+  </si>
+  <si>
+    <t>VIM+DC</t>
+  </si>
+  <si>
+    <t>Zn20 Ca20 Sr20 Yb20 (Li0.55 Mg0.45)20</t>
+  </si>
+  <si>
+    <t>remarkable homogenous deformation at room temperature with 4 times lower strength at 1e-5 strain rate compared to 1e-4</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">electrical resistivity </t>
+  </si>
+  <si>
+    <t>Ohm*m</t>
+  </si>
+  <si>
+    <t>viscosity</t>
+  </si>
+  <si>
+    <t>Pa*s</t>
+  </si>
+  <si>
+    <t>10.1063/1.3575562</t>
   </si>
 </sst>
 </file>
@@ -15310,19 +15337,43 @@
     </row>
     <row r="258" spans="1:20" ht="18" customHeight="1">
       <c r="A258" s="106"/>
-      <c r="B258" s="99"/>
-      <c r="C258" s="86"/>
-      <c r="D258" s="86"/>
-      <c r="E258" s="99"/>
-      <c r="F258" s="49"/>
-      <c r="G258" s="31"/>
-      <c r="H258" s="52"/>
-      <c r="I258" s="50"/>
-      <c r="J258" s="38"/>
+      <c r="B258" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C258" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D258" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E258" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F258" s="49" t="s">
+        <v>244</v>
+      </c>
+      <c r="G258" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H258" s="52" t="s">
+        <v>248</v>
+      </c>
+      <c r="I258" s="50">
+        <v>298</v>
+      </c>
+      <c r="J258" s="38">
+        <v>70</v>
+      </c>
       <c r="K258" s="36"/>
-      <c r="L258" s="38"/>
-      <c r="M258" s="38"/>
-      <c r="N258" s="29"/>
+      <c r="L258" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="M258" s="38" t="s">
+        <v>300</v>
+      </c>
+      <c r="N258" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O258" s="41"/>
       <c r="P258" s="41"/>
       <c r="Q258" s="41"/>
@@ -15332,19 +15383,43 @@
     </row>
     <row r="259" spans="1:20" ht="18" customHeight="1">
       <c r="A259" s="106"/>
-      <c r="B259" s="99"/>
-      <c r="C259" s="86"/>
-      <c r="D259" s="86"/>
-      <c r="E259" s="99"/>
-      <c r="F259" s="49"/>
-      <c r="G259" s="31"/>
-      <c r="H259" s="52"/>
-      <c r="I259" s="50"/>
-      <c r="J259" s="38"/>
+      <c r="B259" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C259" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D259" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E259" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F259" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="G259" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H259" s="52" t="s">
+        <v>248</v>
+      </c>
+      <c r="I259" s="50">
+        <v>298</v>
+      </c>
+      <c r="J259" s="107">
+        <v>363000000</v>
+      </c>
       <c r="K259" s="36"/>
-      <c r="L259" s="38"/>
-      <c r="M259" s="38"/>
-      <c r="N259" s="29"/>
+      <c r="L259" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M259" s="38" t="s">
+        <v>300</v>
+      </c>
+      <c r="N259" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O259" s="41"/>
       <c r="P259" s="41"/>
       <c r="Q259" s="41"/>
@@ -15354,19 +15429,41 @@
     </row>
     <row r="260" spans="1:20" ht="18" customHeight="1">
       <c r="A260" s="106"/>
-      <c r="B260" s="99"/>
-      <c r="C260" s="86"/>
-      <c r="D260" s="86"/>
-      <c r="E260" s="99"/>
-      <c r="F260" s="49"/>
-      <c r="G260" s="31"/>
-      <c r="H260" s="52"/>
+      <c r="B260" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C260" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D260" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E260" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F260" s="49" t="s">
+        <v>112</v>
+      </c>
+      <c r="G260" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H260" s="52" t="s">
+        <v>248</v>
+      </c>
       <c r="I260" s="50"/>
-      <c r="J260" s="38"/>
+      <c r="J260" s="107">
+        <v>320000000</v>
+      </c>
       <c r="K260" s="36"/>
-      <c r="L260" s="38"/>
-      <c r="M260" s="38"/>
-      <c r="N260" s="29"/>
+      <c r="L260" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="M260" s="38" t="s">
+        <v>300</v>
+      </c>
+      <c r="N260" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O260" s="41"/>
       <c r="P260" s="41"/>
       <c r="Q260" s="41"/>
@@ -15376,19 +15473,37 @@
     </row>
     <row r="261" spans="1:20" ht="18" customHeight="1">
       <c r="A261" s="106"/>
-      <c r="B261" s="99"/>
-      <c r="C261" s="86"/>
-      <c r="D261" s="86"/>
-      <c r="E261" s="99"/>
-      <c r="F261" s="49"/>
-      <c r="G261" s="31"/>
+      <c r="B261" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C261" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D261" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E261" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F261" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G261" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H261" s="52"/>
       <c r="I261" s="50"/>
-      <c r="J261" s="38"/>
+      <c r="J261" s="38">
+        <v>323</v>
+      </c>
       <c r="K261" s="36"/>
-      <c r="L261" s="38"/>
+      <c r="L261" s="38" t="s">
+        <v>223</v>
+      </c>
       <c r="M261" s="38"/>
-      <c r="N261" s="29"/>
+      <c r="N261" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O261" s="41"/>
       <c r="P261" s="41"/>
       <c r="Q261" s="41"/>
@@ -15398,19 +15513,39 @@
     </row>
     <row r="262" spans="1:20" ht="18" customHeight="1">
       <c r="A262" s="106"/>
-      <c r="B262" s="99"/>
-      <c r="C262" s="86"/>
-      <c r="D262" s="86"/>
-      <c r="E262" s="99"/>
-      <c r="F262" s="49"/>
-      <c r="G262" s="31"/>
+      <c r="B262" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C262" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D262" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E262" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F262" s="49" t="s">
+        <v>301</v>
+      </c>
+      <c r="G262" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H262" s="52"/>
-      <c r="I262" s="50"/>
-      <c r="J262" s="107"/>
+      <c r="I262" s="50">
+        <v>298</v>
+      </c>
+      <c r="J262" s="107">
+        <v>1.3999999999999999E-6</v>
+      </c>
       <c r="K262" s="36"/>
-      <c r="L262" s="38"/>
+      <c r="L262" s="38" t="s">
+        <v>302</v>
+      </c>
       <c r="M262" s="38"/>
-      <c r="N262" s="29"/>
+      <c r="N262" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O262" s="41"/>
       <c r="P262" s="41"/>
       <c r="Q262" s="41"/>
@@ -15420,19 +15555,39 @@
     </row>
     <row r="263" spans="1:20" ht="18" customHeight="1">
       <c r="A263" s="53"/>
-      <c r="B263" s="39"/>
-      <c r="C263" s="29"/>
-      <c r="D263" s="29"/>
-      <c r="E263" s="30"/>
-      <c r="F263" s="49"/>
-      <c r="G263" s="31"/>
+      <c r="B263" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C263" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D263" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E263" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F263" s="49" t="s">
+        <v>303</v>
+      </c>
+      <c r="G263" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H263" s="52"/>
-      <c r="I263" s="50"/>
-      <c r="J263" s="107"/>
+      <c r="I263" s="50">
+        <v>298</v>
+      </c>
+      <c r="J263" s="107">
+        <v>10000000000000</v>
+      </c>
       <c r="K263" s="36"/>
-      <c r="L263" s="38"/>
+      <c r="L263" s="38" t="s">
+        <v>304</v>
+      </c>
       <c r="M263" s="38"/>
-      <c r="N263" s="29"/>
+      <c r="N263" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O263" s="41"/>
       <c r="P263" s="41"/>
       <c r="Q263" s="41"/>
@@ -15442,19 +15597,39 @@
     </row>
     <row r="264" spans="1:20" ht="18" customHeight="1">
       <c r="A264" s="53"/>
-      <c r="B264" s="39"/>
-      <c r="C264" s="29"/>
-      <c r="D264" s="29"/>
-      <c r="E264" s="30"/>
-      <c r="F264" s="49"/>
-      <c r="G264" s="31"/>
+      <c r="B264" s="99" t="s">
+        <v>298</v>
+      </c>
+      <c r="C264" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D264" s="86" t="s">
+        <v>297</v>
+      </c>
+      <c r="E264" s="99" t="s">
+        <v>299</v>
+      </c>
+      <c r="F264" s="49" t="s">
+        <v>111</v>
+      </c>
+      <c r="G264" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H264" s="52"/>
-      <c r="I264" s="50"/>
-      <c r="J264" s="107"/>
+      <c r="I264" s="50">
+        <v>298</v>
+      </c>
+      <c r="J264" s="107">
+        <v>820000000</v>
+      </c>
       <c r="K264" s="36"/>
-      <c r="L264" s="38"/>
+      <c r="L264" s="38" t="s">
+        <v>32</v>
+      </c>
       <c r="M264" s="38"/>
-      <c r="N264" s="38"/>
+      <c r="N264" s="29" t="s">
+        <v>305</v>
+      </c>
       <c r="O264" s="41"/>
       <c r="P264" s="41"/>
       <c r="Q264" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jnoncrysol.2013.01.022`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B71DDC8-168B-0C4E-BDD4-506451E1E257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FF67FC-3A5F-7A49-B6CE-C1ADA51F935B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="11020" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2522" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="311">
   <si>
     <r>
       <rPr>
@@ -1048,6 +1048,21 @@
   </si>
   <si>
     <t>10.1063/1.3575562</t>
+  </si>
+  <si>
+    <t>AAM+A</t>
+  </si>
+  <si>
+    <t>annealed at 813K for 1h to crystallize</t>
+  </si>
+  <si>
+    <t>FCC+BCC+Ni7Zr2</t>
+  </si>
+  <si>
+    <t>Ti20 Zr20 Cu20 Ni20 Be20</t>
+  </si>
+  <si>
+    <t>10.1016/j.jnoncrysol.2013.01.022</t>
   </si>
 </sst>
 </file>
@@ -15639,19 +15654,41 @@
     </row>
     <row r="265" spans="1:20" ht="18" customHeight="1">
       <c r="A265" s="53"/>
-      <c r="B265" s="39"/>
-      <c r="C265" s="29"/>
-      <c r="D265" s="29"/>
+      <c r="B265" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C265" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D265" s="29" t="s">
+        <v>259</v>
+      </c>
       <c r="E265" s="30"/>
-      <c r="F265" s="49"/>
-      <c r="G265" s="31"/>
+      <c r="F265" s="49" t="s">
+        <v>111</v>
+      </c>
+      <c r="G265" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H265" s="52"/>
-      <c r="I265" s="50"/>
-      <c r="J265" s="107"/>
-      <c r="K265" s="36"/>
-      <c r="L265" s="38"/>
+      <c r="I265" s="50">
+        <v>298</v>
+      </c>
+      <c r="J265" s="107">
+        <f>9807000*680.3</f>
+        <v>6671702100</v>
+      </c>
+      <c r="K265" s="107">
+        <f>9807000*8.2</f>
+        <v>80417400</v>
+      </c>
+      <c r="L265" s="38" t="s">
+        <v>32</v>
+      </c>
       <c r="M265" s="38"/>
-      <c r="N265" s="38"/>
+      <c r="N265" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="O265" s="41"/>
       <c r="P265" s="41"/>
       <c r="Q265" s="41"/>
@@ -15661,10 +15698,18 @@
     </row>
     <row r="266" spans="1:20" ht="18" customHeight="1">
       <c r="A266" s="53"/>
-      <c r="B266" s="39"/>
-      <c r="C266" s="29"/>
-      <c r="D266" s="29"/>
-      <c r="E266" s="30"/>
+      <c r="B266" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C266" s="29" t="s">
+        <v>308</v>
+      </c>
+      <c r="D266" s="29" t="s">
+        <v>306</v>
+      </c>
+      <c r="E266" s="30" t="s">
+        <v>307</v>
+      </c>
       <c r="F266" s="49"/>
       <c r="G266" s="31"/>
       <c r="H266" s="52"/>
@@ -15673,7 +15718,9 @@
       <c r="K266" s="36"/>
       <c r="L266" s="38"/>
       <c r="M266" s="38"/>
-      <c r="N266" s="38"/>
+      <c r="N266" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="O266" s="41"/>
       <c r="P266" s="41"/>
       <c r="Q266" s="41"/>
@@ -15683,19 +15730,37 @@
     </row>
     <row r="267" spans="1:20" ht="18" customHeight="1">
       <c r="A267" s="53"/>
-      <c r="B267" s="39"/>
-      <c r="C267" s="29"/>
-      <c r="D267" s="29"/>
-      <c r="E267" s="51"/>
-      <c r="F267" s="49"/>
-      <c r="G267" s="31"/>
+      <c r="B267" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C267" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D267" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="E267" s="30"/>
+      <c r="F267" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="G267" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H267" s="52"/>
-      <c r="I267" s="50"/>
-      <c r="J267" s="33"/>
+      <c r="I267" s="50">
+        <v>298</v>
+      </c>
+      <c r="J267" s="33">
+        <v>2315000000</v>
+      </c>
       <c r="K267" s="36"/>
-      <c r="L267" s="38"/>
+      <c r="L267" s="38" t="s">
+        <v>32</v>
+      </c>
       <c r="M267" s="38"/>
-      <c r="N267" s="38"/>
+      <c r="N267" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="O267" s="41"/>
       <c r="P267" s="41"/>
       <c r="Q267" s="41"/>
@@ -15705,19 +15770,37 @@
     </row>
     <row r="268" spans="1:20" ht="18" customHeight="1">
       <c r="A268" s="53"/>
-      <c r="B268" s="39"/>
-      <c r="C268" s="29"/>
-      <c r="D268" s="29"/>
-      <c r="E268" s="51"/>
-      <c r="F268" s="49"/>
-      <c r="G268" s="31"/>
+      <c r="B268" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C268" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D268" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="E268" s="30"/>
+      <c r="F268" s="49" t="s">
+        <v>114</v>
+      </c>
+      <c r="G268" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H268" s="52"/>
-      <c r="I268" s="50"/>
-      <c r="J268" s="47"/>
+      <c r="I268" s="50">
+        <v>298</v>
+      </c>
+      <c r="J268" s="47">
+        <v>2</v>
+      </c>
       <c r="K268" s="36"/>
-      <c r="L268" s="38"/>
+      <c r="L268" s="38" t="s">
+        <v>66</v>
+      </c>
       <c r="M268" s="38"/>
-      <c r="N268" s="38"/>
+      <c r="N268" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="O268" s="41"/>
       <c r="P268" s="41"/>
       <c r="Q268" s="41"/>
@@ -15727,19 +15810,35 @@
     </row>
     <row r="269" spans="1:20" ht="18" customHeight="1">
       <c r="A269" s="53"/>
-      <c r="B269" s="39"/>
-      <c r="C269" s="29"/>
-      <c r="D269" s="29"/>
-      <c r="E269" s="51"/>
-      <c r="F269" s="53"/>
-      <c r="G269" s="31"/>
+      <c r="B269" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C269" s="86" t="s">
+        <v>219</v>
+      </c>
+      <c r="D269" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="E269" s="30"/>
+      <c r="F269" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="G269" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H269" s="52"/>
       <c r="I269" s="50"/>
-      <c r="J269" s="47"/>
+      <c r="J269" s="47">
+        <v>683</v>
+      </c>
       <c r="K269" s="36"/>
-      <c r="L269" s="38"/>
+      <c r="L269" s="38" t="s">
+        <v>223</v>
+      </c>
       <c r="M269" s="38"/>
-      <c r="N269" s="38"/>
+      <c r="N269" s="38" t="s">
+        <v>310</v>
+      </c>
       <c r="O269" s="41"/>
       <c r="P269" s="41"/>
       <c r="Q269" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1007/s40195-019-00977-1`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA52C82E-2FA8-FF47-91E3-E4F3D8B6DE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7FEED8-F5AD-174A-82EF-E1B3AEC1DCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2715" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2731" uniqueCount="330">
   <si>
     <r>
       <rPr>
@@ -1108,6 +1108,18 @@
   </si>
   <si>
     <t>10.1016/j.wear.2018.05.023</t>
+  </si>
+  <si>
+    <t>Fe3 Cr2 Al2 Cu Ni4 Si5</t>
+  </si>
+  <si>
+    <t>MA+CIP</t>
+  </si>
+  <si>
+    <t>amorphous with BCC nanocrystals; ball milled at 900rpm with 60:1 ratio for 40h with steel rods in argon and compacted under ultrahigh 6000MPa at low 573K into 10mmx10mm cylinders</t>
+  </si>
+  <si>
+    <t>10.1007/s40195-019-00977-1</t>
   </si>
 </sst>
 </file>
@@ -16687,21 +16699,44 @@
     </row>
     <row r="286" spans="1:20" ht="18" customHeight="1">
       <c r="A286" s="53"/>
-      <c r="B286" s="53"/>
-      <c r="C286" s="53"/>
-      <c r="D286" s="53"/>
-      <c r="E286" s="53"/>
-      <c r="F286" s="53"/>
-      <c r="G286" s="31"/>
-      <c r="H286" s="53"/>
-      <c r="I286" s="50"/>
-      <c r="J286" s="41"/>
+      <c r="B286" s="53" t="s">
+        <v>326</v>
+      </c>
+      <c r="C286" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="D286" s="53" t="s">
+        <v>327</v>
+      </c>
+      <c r="E286" s="53" t="s">
+        <v>328</v>
+      </c>
+      <c r="F286" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="G286" s="93" t="s">
+        <v>28</v>
+      </c>
+      <c r="H286" s="155"/>
+      <c r="I286" s="156">
+        <v>298</v>
+      </c>
+      <c r="J286" s="84">
+        <f t="shared" ref="J286" si="9">P286*9807000</f>
+        <v>11278050000</v>
+      </c>
       <c r="K286" s="41"/>
-      <c r="L286" s="53"/>
+      <c r="L286" s="53" t="s">
+        <v>32</v>
+      </c>
       <c r="M286" s="53"/>
-      <c r="N286" s="38"/>
+      <c r="N286" s="38" t="s">
+        <v>329</v>
+      </c>
       <c r="O286" s="41"/>
-      <c r="P286" s="41"/>
+      <c r="P286" s="41">
+        <v>1150</v>
+      </c>
       <c r="Q286" s="41"/>
       <c r="R286" s="41"/>
       <c r="S286" s="35"/>
@@ -16709,19 +16744,39 @@
     </row>
     <row r="287" spans="1:20" ht="18" customHeight="1">
       <c r="A287" s="53"/>
-      <c r="B287" s="53"/>
-      <c r="C287" s="53"/>
-      <c r="D287" s="53"/>
-      <c r="E287" s="53"/>
-      <c r="F287" s="53"/>
-      <c r="G287" s="31"/>
-      <c r="H287" s="53"/>
-      <c r="I287" s="50"/>
-      <c r="J287" s="41"/>
+      <c r="B287" s="53" t="s">
+        <v>326</v>
+      </c>
+      <c r="C287" s="53" t="s">
+        <v>219</v>
+      </c>
+      <c r="D287" s="53" t="s">
+        <v>327</v>
+      </c>
+      <c r="E287" s="53" t="s">
+        <v>328</v>
+      </c>
+      <c r="F287" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="G287" s="93" t="s">
+        <v>28</v>
+      </c>
+      <c r="H287" s="155"/>
+      <c r="I287" s="156">
+        <v>298</v>
+      </c>
+      <c r="J287" s="41">
+        <v>-0.19</v>
+      </c>
       <c r="K287" s="41"/>
-      <c r="L287" s="53"/>
+      <c r="L287" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="M287" s="53"/>
-      <c r="N287" s="38"/>
+      <c r="N287" s="38" t="s">
+        <v>329</v>
+      </c>
       <c r="O287" s="41"/>
       <c r="P287" s="41"/>
       <c r="Q287" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1080/09500839.2022.2120644`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7FEED8-F5AD-174A-82EF-E1B3AEC1DCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7456D7A-E664-5744-91B3-113E7A28F973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2731" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2822" uniqueCount="349">
   <si>
     <r>
       <rPr>
@@ -1120,6 +1120,63 @@
   </si>
   <si>
     <t>10.1007/s40195-019-00977-1</t>
+  </si>
+  <si>
+    <t>Ti Zr Hf</t>
+  </si>
+  <si>
+    <t>(Ti0.333 Zr0.333 Hf0.333)95 Re5</t>
+  </si>
+  <si>
+    <t>TZH</t>
+  </si>
+  <si>
+    <t>TZHR5</t>
+  </si>
+  <si>
+    <t>TZHR10</t>
+  </si>
+  <si>
+    <t>TZHR</t>
+  </si>
+  <si>
+    <t>(Ti0.333 Zr0.333 Hf0.333)90 Re10</t>
+  </si>
+  <si>
+    <t>Ti Zr Hf Re</t>
+  </si>
+  <si>
+    <t>(Ti0.333 Zr0.333 Hf0.333)90 Re5 Al5</t>
+  </si>
+  <si>
+    <t>(Ti0.333 Zr0.333 Hf0.333)88 Re5 Al7</t>
+  </si>
+  <si>
+    <t>TZHR5A5</t>
+  </si>
+  <si>
+    <t>TZHR5A7</t>
+  </si>
+  <si>
+    <t>HCP</t>
+  </si>
+  <si>
+    <t>HCP+HCP</t>
+  </si>
+  <si>
+    <t>HCP+L12</t>
+  </si>
+  <si>
+    <t>L12 is Zr3Al intermetallic</t>
+  </si>
+  <si>
+    <t>HCP+HCP+laves</t>
+  </si>
+  <si>
+    <t>annealed at 1273K for 24h; HfRe2 cubic laves phase</t>
+  </si>
+  <si>
+    <t>10.1080/09500839.2022.2120644</t>
   </si>
 </sst>
 </file>
@@ -16785,10 +16842,18 @@
       <c r="T287" s="35"/>
     </row>
     <row r="288" spans="1:20" ht="18" customHeight="1">
-      <c r="A288" s="53"/>
-      <c r="B288" s="53"/>
-      <c r="C288" s="53"/>
-      <c r="D288" s="53"/>
+      <c r="A288" s="53" t="s">
+        <v>332</v>
+      </c>
+      <c r="B288" s="53" t="s">
+        <v>330</v>
+      </c>
+      <c r="C288" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D288" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E288" s="53"/>
       <c r="F288" s="53"/>
       <c r="G288" s="31"/>
@@ -16798,7 +16863,9 @@
       <c r="K288" s="41"/>
       <c r="L288" s="53"/>
       <c r="M288" s="53"/>
-      <c r="N288" s="38"/>
+      <c r="N288" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O288" s="41"/>
       <c r="P288" s="41"/>
       <c r="Q288" s="41"/>
@@ -16807,10 +16874,18 @@
       <c r="T288" s="35"/>
     </row>
     <row r="289" spans="1:20" ht="18" customHeight="1">
-      <c r="A289" s="53"/>
-      <c r="B289" s="53"/>
-      <c r="C289" s="53"/>
-      <c r="D289" s="53"/>
+      <c r="A289" s="53" t="s">
+        <v>333</v>
+      </c>
+      <c r="B289" s="53" t="s">
+        <v>331</v>
+      </c>
+      <c r="C289" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D289" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E289" s="51"/>
       <c r="F289" s="53"/>
       <c r="G289" s="31"/>
@@ -16820,7 +16895,9 @@
       <c r="K289" s="41"/>
       <c r="L289" s="53"/>
       <c r="M289" s="53"/>
-      <c r="N289" s="38"/>
+      <c r="N289" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O289" s="41"/>
       <c r="P289" s="41"/>
       <c r="Q289" s="41"/>
@@ -16829,10 +16906,18 @@
       <c r="T289" s="35"/>
     </row>
     <row r="290" spans="1:20" ht="18" customHeight="1">
-      <c r="A290" s="53"/>
-      <c r="B290" s="53"/>
-      <c r="C290" s="53"/>
-      <c r="D290" s="53"/>
+      <c r="A290" s="53" t="s">
+        <v>334</v>
+      </c>
+      <c r="B290" s="53" t="s">
+        <v>336</v>
+      </c>
+      <c r="C290" s="53" t="s">
+        <v>343</v>
+      </c>
+      <c r="D290" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E290" s="51"/>
       <c r="F290" s="53"/>
       <c r="G290" s="31"/>
@@ -16842,7 +16927,9 @@
       <c r="K290" s="41"/>
       <c r="L290" s="53"/>
       <c r="M290" s="53"/>
-      <c r="N290" s="38"/>
+      <c r="N290" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O290" s="41"/>
       <c r="P290" s="41"/>
       <c r="Q290" s="41"/>
@@ -16851,10 +16938,18 @@
       <c r="T290" s="35"/>
     </row>
     <row r="291" spans="1:20" ht="18" customHeight="1">
-      <c r="A291" s="53"/>
-      <c r="B291" s="53"/>
-      <c r="C291" s="53"/>
-      <c r="D291" s="53"/>
+      <c r="A291" s="53" t="s">
+        <v>335</v>
+      </c>
+      <c r="B291" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="C291" s="53" t="s">
+        <v>343</v>
+      </c>
+      <c r="D291" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E291" s="51"/>
       <c r="F291" s="53"/>
       <c r="G291" s="31"/>
@@ -16864,7 +16959,9 @@
       <c r="K291" s="41"/>
       <c r="L291" s="53"/>
       <c r="M291" s="53"/>
-      <c r="N291" s="38"/>
+      <c r="N291" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O291" s="41"/>
       <c r="P291" s="41"/>
       <c r="Q291" s="41"/>
@@ -16873,10 +16970,18 @@
       <c r="T291" s="35"/>
     </row>
     <row r="292" spans="1:20" ht="18" customHeight="1">
-      <c r="A292" s="53"/>
-      <c r="B292" s="53"/>
-      <c r="C292" s="53"/>
-      <c r="D292" s="53"/>
+      <c r="A292" s="53" t="s">
+        <v>340</v>
+      </c>
+      <c r="B292" s="53" t="s">
+        <v>338</v>
+      </c>
+      <c r="C292" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D292" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E292" s="51"/>
       <c r="F292" s="53"/>
       <c r="G292" s="31"/>
@@ -16886,7 +16991,9 @@
       <c r="K292" s="41"/>
       <c r="L292" s="53"/>
       <c r="M292" s="53"/>
-      <c r="N292" s="38"/>
+      <c r="N292" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O292" s="41"/>
       <c r="P292" s="41"/>
       <c r="Q292" s="41"/>
@@ -16895,11 +17002,21 @@
       <c r="T292" s="35"/>
     </row>
     <row r="293" spans="1:20" ht="18" customHeight="1">
-      <c r="A293" s="53"/>
-      <c r="B293" s="53"/>
-      <c r="C293" s="53"/>
-      <c r="D293" s="53"/>
-      <c r="E293" s="51"/>
+      <c r="A293" s="53" t="s">
+        <v>341</v>
+      </c>
+      <c r="B293" s="53" t="s">
+        <v>339</v>
+      </c>
+      <c r="C293" s="53" t="s">
+        <v>344</v>
+      </c>
+      <c r="D293" s="53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E293" s="51" t="s">
+        <v>345</v>
+      </c>
       <c r="F293" s="53"/>
       <c r="G293" s="31"/>
       <c r="H293" s="53"/>
@@ -16908,7 +17025,9 @@
       <c r="K293" s="41"/>
       <c r="L293" s="53"/>
       <c r="M293" s="53"/>
-      <c r="N293" s="38"/>
+      <c r="N293" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O293" s="41"/>
       <c r="P293" s="41"/>
       <c r="Q293" s="41"/>
@@ -16917,11 +17036,21 @@
       <c r="T293" s="35"/>
     </row>
     <row r="294" spans="1:20" ht="18" customHeight="1">
-      <c r="A294" s="53"/>
-      <c r="B294" s="53"/>
-      <c r="C294" s="53"/>
-      <c r="D294" s="53"/>
-      <c r="E294" s="51"/>
+      <c r="A294" s="53" t="s">
+        <v>340</v>
+      </c>
+      <c r="B294" s="53" t="s">
+        <v>338</v>
+      </c>
+      <c r="C294" s="53" t="s">
+        <v>346</v>
+      </c>
+      <c r="D294" s="53" t="s">
+        <v>306</v>
+      </c>
+      <c r="E294" s="51" t="s">
+        <v>347</v>
+      </c>
       <c r="F294" s="53"/>
       <c r="G294" s="31"/>
       <c r="H294" s="53"/>
@@ -16930,7 +17059,9 @@
       <c r="K294" s="41"/>
       <c r="L294" s="53"/>
       <c r="M294" s="53"/>
-      <c r="N294" s="38"/>
+      <c r="N294" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O294" s="41"/>
       <c r="P294" s="41"/>
       <c r="Q294" s="41"/>
@@ -16939,20 +17070,44 @@
       <c r="T294" s="35"/>
     </row>
     <row r="295" spans="1:20" ht="18" customHeight="1">
-      <c r="A295" s="53"/>
-      <c r="B295" s="53"/>
-      <c r="C295" s="53"/>
-      <c r="D295" s="53"/>
+      <c r="A295" s="53" t="s">
+        <v>332</v>
+      </c>
+      <c r="B295" s="53" t="s">
+        <v>330</v>
+      </c>
+      <c r="C295" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D295" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E295" s="51"/>
-      <c r="F295" s="53"/>
-      <c r="G295" s="31"/>
+      <c r="F295" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="G295" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H295" s="53"/>
-      <c r="I295" s="36"/>
-      <c r="J295" s="54"/>
-      <c r="K295" s="41"/>
-      <c r="L295" s="53"/>
-      <c r="M295" s="53"/>
-      <c r="N295" s="38"/>
+      <c r="I295" s="36">
+        <v>298</v>
+      </c>
+      <c r="J295" s="54">
+        <v>7850000000</v>
+      </c>
+      <c r="K295" s="54">
+        <v>370000000</v>
+      </c>
+      <c r="L295" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M295" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N295" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O295" s="41"/>
       <c r="P295" s="41"/>
       <c r="Q295" s="41"/>
@@ -16961,20 +17116,44 @@
       <c r="T295" s="35"/>
     </row>
     <row r="296" spans="1:20" ht="18" customHeight="1">
-      <c r="A296" s="53"/>
-      <c r="B296" s="53"/>
-      <c r="C296" s="53"/>
-      <c r="D296" s="53"/>
+      <c r="A296" s="53" t="s">
+        <v>333</v>
+      </c>
+      <c r="B296" s="53" t="s">
+        <v>331</v>
+      </c>
+      <c r="C296" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D296" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E296" s="51"/>
-      <c r="F296" s="53"/>
-      <c r="G296" s="31"/>
+      <c r="F296" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="G296" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H296" s="53"/>
-      <c r="I296" s="36"/>
-      <c r="J296" s="54"/>
-      <c r="K296" s="41"/>
-      <c r="L296" s="53"/>
-      <c r="M296" s="53"/>
-      <c r="N296" s="38"/>
+      <c r="I296" s="36">
+        <v>298</v>
+      </c>
+      <c r="J296" s="54">
+        <v>7980000000</v>
+      </c>
+      <c r="K296" s="54">
+        <v>380000000</v>
+      </c>
+      <c r="L296" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M296" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N296" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O296" s="41"/>
       <c r="P296" s="41"/>
       <c r="Q296" s="41"/>
@@ -16983,20 +17162,44 @@
       <c r="T296" s="35"/>
     </row>
     <row r="297" spans="1:20" ht="18" customHeight="1">
-      <c r="A297" s="88"/>
-      <c r="B297" s="53"/>
-      <c r="C297" s="53"/>
-      <c r="D297" s="53"/>
+      <c r="A297" s="53" t="s">
+        <v>340</v>
+      </c>
+      <c r="B297" s="53" t="s">
+        <v>338</v>
+      </c>
+      <c r="C297" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D297" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E297" s="51"/>
-      <c r="F297" s="53"/>
-      <c r="G297" s="31"/>
+      <c r="F297" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="G297" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H297" s="53"/>
-      <c r="I297" s="36"/>
-      <c r="J297" s="54"/>
-      <c r="K297" s="41"/>
-      <c r="L297" s="53"/>
-      <c r="M297" s="53"/>
-      <c r="N297" s="38"/>
+      <c r="I297" s="36">
+        <v>298</v>
+      </c>
+      <c r="J297" s="54">
+        <v>8350000000</v>
+      </c>
+      <c r="K297" s="54">
+        <v>420000000</v>
+      </c>
+      <c r="L297" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M297" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N297" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O297" s="41"/>
       <c r="P297" s="41"/>
       <c r="Q297" s="41"/>
@@ -17005,20 +17208,44 @@
       <c r="T297" s="35"/>
     </row>
     <row r="298" spans="1:20" ht="18" customHeight="1">
-      <c r="A298" s="90"/>
-      <c r="B298" s="53"/>
-      <c r="C298" s="53"/>
-      <c r="D298" s="53"/>
+      <c r="A298" s="53" t="s">
+        <v>332</v>
+      </c>
+      <c r="B298" s="53" t="s">
+        <v>330</v>
+      </c>
+      <c r="C298" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D298" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E298" s="51"/>
-      <c r="F298" s="53"/>
-      <c r="G298" s="31"/>
+      <c r="F298" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="G298" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H298" s="53"/>
-      <c r="I298" s="36"/>
-      <c r="J298" s="54"/>
-      <c r="K298" s="41"/>
-      <c r="L298" s="53"/>
-      <c r="M298" s="53"/>
-      <c r="N298" s="38"/>
+      <c r="I298" s="36">
+        <v>298</v>
+      </c>
+      <c r="J298" s="54">
+        <v>116500000000</v>
+      </c>
+      <c r="K298" s="54">
+        <v>2800000000</v>
+      </c>
+      <c r="L298" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M298" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N298" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O298" s="41"/>
       <c r="P298" s="41"/>
       <c r="Q298" s="41"/>
@@ -17027,20 +17254,44 @@
       <c r="T298" s="35"/>
     </row>
     <row r="299" spans="1:20" ht="18" customHeight="1">
-      <c r="A299" s="90"/>
-      <c r="B299" s="53"/>
-      <c r="C299" s="53"/>
-      <c r="D299" s="53"/>
+      <c r="A299" s="53" t="s">
+        <v>333</v>
+      </c>
+      <c r="B299" s="53" t="s">
+        <v>331</v>
+      </c>
+      <c r="C299" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D299" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E299" s="51"/>
-      <c r="F299" s="89"/>
-      <c r="G299" s="31"/>
+      <c r="F299" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="G299" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H299" s="53"/>
-      <c r="I299" s="36"/>
-      <c r="J299" s="54"/>
-      <c r="K299" s="41"/>
-      <c r="L299" s="53"/>
-      <c r="M299" s="53"/>
-      <c r="N299" s="38"/>
+      <c r="I299" s="36">
+        <v>298</v>
+      </c>
+      <c r="J299" s="54">
+        <v>121200000000</v>
+      </c>
+      <c r="K299" s="54">
+        <v>1900000000</v>
+      </c>
+      <c r="L299" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M299" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N299" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O299" s="41"/>
       <c r="P299" s="41"/>
       <c r="Q299" s="41"/>
@@ -17049,20 +17300,44 @@
       <c r="T299" s="35"/>
     </row>
     <row r="300" spans="1:20" ht="18" customHeight="1">
-      <c r="A300" s="88"/>
-      <c r="B300" s="53"/>
-      <c r="C300" s="53"/>
-      <c r="D300" s="53"/>
+      <c r="A300" s="53" t="s">
+        <v>340</v>
+      </c>
+      <c r="B300" s="53" t="s">
+        <v>338</v>
+      </c>
+      <c r="C300" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D300" s="53" t="s">
+        <v>164</v>
+      </c>
       <c r="E300" s="51"/>
-      <c r="F300" s="89"/>
-      <c r="G300" s="31"/>
+      <c r="F300" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="G300" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H300" s="53"/>
-      <c r="I300" s="36"/>
-      <c r="J300" s="54"/>
-      <c r="K300" s="41"/>
-      <c r="L300" s="53"/>
-      <c r="M300" s="53"/>
-      <c r="N300" s="38"/>
+      <c r="I300" s="36">
+        <v>298</v>
+      </c>
+      <c r="J300" s="54">
+        <v>129800000000</v>
+      </c>
+      <c r="K300" s="54">
+        <v>2000000000</v>
+      </c>
+      <c r="L300" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M300" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N300" s="38" t="s">
+        <v>348</v>
+      </c>
       <c r="O300" s="41"/>
       <c r="P300" s="41"/>
       <c r="Q300" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.msea.2026.150740`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7456D7A-E664-5744-91B3-113E7A28F973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6298A2F7-91AC-1D41-9F5C-C4B9CF0737B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2822" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2861" uniqueCount="353">
   <si>
     <r>
       <rPr>
@@ -1177,6 +1177,18 @@
   </si>
   <si>
     <t>10.1080/09500839.2022.2120644</t>
+  </si>
+  <si>
+    <t>Al15 Ti40 Nb20 Hf10 V15</t>
+  </si>
+  <si>
+    <t>drop cast into a copper mold for rectangular shape instead of button</t>
+  </si>
+  <si>
+    <t>10.1016/j.msea.2026.150740</t>
+  </si>
+  <si>
+    <t>drop cast into a copper mold for rectangular shape instead of button; average and SD from 3 tests</t>
   </si>
 </sst>
 </file>
@@ -2406,6 +2418,68 @@
     <xf numFmtId="49" fontId="13" fillId="10" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2466,68 +2540,6 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="9" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="9" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="10" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3744,19 +3756,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="12"/>
-      <c r="D2" s="115" t="s">
+      <c r="D2" s="137" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="116"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="121"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="120"/>
-      <c r="M2" s="120"/>
-      <c r="N2" s="123"/>
+      <c r="E2" s="138"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="145"/>
       <c r="O2" s="13"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -3772,17 +3784,17 @@
         <v>72</v>
       </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="118"/>
-      <c r="F3" s="124"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="125"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="124"/>
-      <c r="M3" s="124"/>
-      <c r="N3" s="127"/>
+      <c r="D3" s="139"/>
+      <c r="E3" s="140"/>
+      <c r="F3" s="146"/>
+      <c r="G3" s="146"/>
+      <c r="H3" s="146"/>
+      <c r="I3" s="147"/>
+      <c r="J3" s="148"/>
+      <c r="K3" s="148"/>
+      <c r="L3" s="146"/>
+      <c r="M3" s="146"/>
+      <c r="N3" s="149"/>
       <c r="O3" s="13"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -3823,43 +3835,43 @@
       <c r="B5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="128" t="s">
+      <c r="C5" s="150" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="130" t="s">
+      <c r="D5" s="152" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="130" t="s">
+      <c r="E5" s="152" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="130" t="s">
+      <c r="F5" s="152" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="130" t="s">
+      <c r="G5" s="152" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="131" t="s">
+      <c r="H5" s="153" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="130" t="s">
+      <c r="I5" s="152" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="130" t="s">
+      <c r="J5" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="130" t="s">
+      <c r="K5" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="130" t="s">
+      <c r="L5" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="130" t="s">
+      <c r="M5" s="152" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="130" t="s">
+      <c r="N5" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="135" t="s">
+      <c r="O5" s="120" t="s">
         <v>19</v>
       </c>
       <c r="P5" s="24"/>
@@ -3875,19 +3887,19 @@
       <c r="B6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="129"/>
-      <c r="D6" s="129"/>
-      <c r="E6" s="129"/>
-      <c r="F6" s="129"/>
-      <c r="G6" s="129"/>
-      <c r="H6" s="132"/>
-      <c r="I6" s="133"/>
-      <c r="J6" s="134"/>
-      <c r="K6" s="134"/>
-      <c r="L6" s="129"/>
-      <c r="M6" s="129"/>
-      <c r="N6" s="129"/>
-      <c r="O6" s="136"/>
+      <c r="C6" s="151"/>
+      <c r="D6" s="151"/>
+      <c r="E6" s="151"/>
+      <c r="F6" s="151"/>
+      <c r="G6" s="151"/>
+      <c r="H6" s="154"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="156"/>
+      <c r="K6" s="156"/>
+      <c r="L6" s="151"/>
+      <c r="M6" s="151"/>
+      <c r="N6" s="151"/>
+      <c r="O6" s="121"/>
       <c r="P6" s="24"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="9"/>
@@ -3937,7 +3949,7 @@
       <c r="N7" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="O7" s="137"/>
+      <c r="O7" s="122"/>
       <c r="P7" s="60" t="s">
         <v>61</v>
       </c>
@@ -3952,35 +3964,35 @@
     </row>
     <row r="8" spans="1:20" ht="20.25" customHeight="1" thickBot="1">
       <c r="A8" s="55"/>
-      <c r="B8" s="138" t="s">
+      <c r="B8" s="123" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="139"/>
-      <c r="D8" s="139"/>
-      <c r="E8" s="140"/>
-      <c r="F8" s="141" t="s">
+      <c r="C8" s="124"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="125"/>
+      <c r="F8" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="142"/>
-      <c r="H8" s="142"/>
-      <c r="I8" s="143"/>
-      <c r="J8" s="144"/>
-      <c r="K8" s="144"/>
-      <c r="L8" s="145"/>
-      <c r="M8" s="146" t="s">
+      <c r="G8" s="127"/>
+      <c r="H8" s="127"/>
+      <c r="I8" s="128"/>
+      <c r="J8" s="129"/>
+      <c r="K8" s="129"/>
+      <c r="L8" s="130"/>
+      <c r="M8" s="131" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="147"/>
+      <c r="N8" s="132"/>
       <c r="O8" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="P8" s="148" t="s">
+      <c r="P8" s="133" t="s">
         <v>41</v>
       </c>
-      <c r="Q8" s="149"/>
-      <c r="R8" s="150"/>
-      <c r="S8" s="150"/>
-      <c r="T8" s="151"/>
+      <c r="Q8" s="134"/>
+      <c r="R8" s="135"/>
+      <c r="S8" s="135"/>
+      <c r="T8" s="136"/>
     </row>
     <row r="9" spans="1:20" ht="21" customHeight="1" thickBot="1">
       <c r="A9" s="56" t="s">
@@ -14979,7 +14991,7 @@
       <c r="E246" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="F246" s="152" t="s">
+      <c r="F246" s="115" t="s">
         <v>224</v>
       </c>
       <c r="G246" s="31" t="s">
@@ -15023,7 +15035,7 @@
       <c r="E247" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="F247" s="152" t="s">
+      <c r="F247" s="115" t="s">
         <v>224</v>
       </c>
       <c r="G247" s="31" t="s">
@@ -15067,7 +15079,7 @@
       <c r="E248" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="F248" s="152" t="s">
+      <c r="F248" s="115" t="s">
         <v>224</v>
       </c>
       <c r="G248" s="31" t="s">
@@ -15111,7 +15123,7 @@
       <c r="E249" s="99" t="s">
         <v>275</v>
       </c>
-      <c r="F249" s="152" t="s">
+      <c r="F249" s="115" t="s">
         <v>224</v>
       </c>
       <c r="G249" s="31" t="s">
@@ -16350,8 +16362,8 @@
       <c r="G277" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="H277" s="153"/>
-      <c r="I277" s="154">
+      <c r="H277" s="116"/>
+      <c r="I277" s="117">
         <v>298</v>
       </c>
       <c r="J277" s="54">
@@ -16396,8 +16408,8 @@
       <c r="G278" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H278" s="155"/>
-      <c r="I278" s="156">
+      <c r="H278" s="118"/>
+      <c r="I278" s="119">
         <v>298</v>
       </c>
       <c r="J278" s="54">
@@ -16442,8 +16454,8 @@
       <c r="G279" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H279" s="155"/>
-      <c r="I279" s="156">
+      <c r="H279" s="118"/>
+      <c r="I279" s="119">
         <v>298</v>
       </c>
       <c r="J279" s="54">
@@ -16488,8 +16500,8 @@
       <c r="G280" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="H280" s="153"/>
-      <c r="I280" s="154">
+      <c r="H280" s="116"/>
+      <c r="I280" s="117">
         <v>298</v>
       </c>
       <c r="J280" s="54">
@@ -16536,8 +16548,8 @@
       <c r="G281" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H281" s="155"/>
-      <c r="I281" s="156">
+      <c r="H281" s="118"/>
+      <c r="I281" s="119">
         <v>298</v>
       </c>
       <c r="J281" s="54">
@@ -16584,8 +16596,8 @@
       <c r="G282" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H282" s="155"/>
-      <c r="I282" s="156">
+      <c r="H282" s="118"/>
+      <c r="I282" s="119">
         <v>298</v>
       </c>
       <c r="J282" s="54">
@@ -16632,8 +16644,8 @@
       <c r="G283" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="H283" s="153"/>
-      <c r="I283" s="154">
+      <c r="H283" s="116"/>
+      <c r="I283" s="117">
         <v>298</v>
       </c>
       <c r="J283" s="54">
@@ -16680,8 +16692,8 @@
       <c r="G284" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H284" s="155"/>
-      <c r="I284" s="156">
+      <c r="H284" s="118"/>
+      <c r="I284" s="119">
         <v>298</v>
       </c>
       <c r="J284" s="47">
@@ -16728,8 +16740,8 @@
       <c r="G285" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H285" s="155"/>
-      <c r="I285" s="156">
+      <c r="H285" s="118"/>
+      <c r="I285" s="119">
         <v>298</v>
       </c>
       <c r="J285" s="41">
@@ -16774,8 +16786,8 @@
       <c r="G286" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H286" s="155"/>
-      <c r="I286" s="156">
+      <c r="H286" s="118"/>
+      <c r="I286" s="119">
         <v>298</v>
       </c>
       <c r="J286" s="84">
@@ -16819,8 +16831,8 @@
       <c r="G287" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H287" s="155"/>
-      <c r="I287" s="156">
+      <c r="H287" s="118"/>
+      <c r="I287" s="119">
         <v>298</v>
       </c>
       <c r="J287" s="41">
@@ -17347,19 +17359,45 @@
     </row>
     <row r="301" spans="1:20" ht="18" customHeight="1">
       <c r="A301" s="90"/>
-      <c r="B301" s="53"/>
-      <c r="C301" s="53"/>
-      <c r="D301" s="53"/>
-      <c r="E301" s="51"/>
-      <c r="F301" s="89"/>
-      <c r="G301" s="31"/>
-      <c r="H301" s="53"/>
-      <c r="I301" s="36"/>
-      <c r="J301" s="54"/>
-      <c r="K301" s="41"/>
-      <c r="L301" s="53"/>
-      <c r="M301" s="53"/>
-      <c r="N301" s="38"/>
+      <c r="B301" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="C301" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="D301" s="53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E301" s="51" t="s">
+        <v>352</v>
+      </c>
+      <c r="F301" s="89" t="s">
+        <v>67</v>
+      </c>
+      <c r="G301" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H301" s="53" t="s">
+        <v>248</v>
+      </c>
+      <c r="I301" s="36">
+        <v>298</v>
+      </c>
+      <c r="J301" s="54">
+        <v>1222200000</v>
+      </c>
+      <c r="K301" s="54">
+        <v>4100000</v>
+      </c>
+      <c r="L301" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M301" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="N301" s="38" t="s">
+        <v>351</v>
+      </c>
       <c r="O301" s="41"/>
       <c r="P301" s="41"/>
       <c r="Q301" s="41"/>
@@ -17369,19 +17407,45 @@
     </row>
     <row r="302" spans="1:20" ht="18" customHeight="1">
       <c r="A302" s="90"/>
-      <c r="B302" s="53"/>
-      <c r="C302" s="53"/>
-      <c r="D302" s="53"/>
-      <c r="E302" s="51"/>
-      <c r="F302" s="89"/>
-      <c r="G302" s="31"/>
-      <c r="H302" s="53"/>
-      <c r="I302" s="36"/>
-      <c r="J302" s="54"/>
-      <c r="K302" s="41"/>
-      <c r="L302" s="53"/>
-      <c r="M302" s="53"/>
-      <c r="N302" s="38"/>
+      <c r="B302" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="C302" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="D302" s="53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E302" s="51" t="s">
+        <v>352</v>
+      </c>
+      <c r="F302" s="89" t="s">
+        <v>70</v>
+      </c>
+      <c r="G302" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H302" s="53" t="s">
+        <v>248</v>
+      </c>
+      <c r="I302" s="36">
+        <v>298</v>
+      </c>
+      <c r="J302" s="54">
+        <v>1264400000</v>
+      </c>
+      <c r="K302" s="54">
+        <v>12600000</v>
+      </c>
+      <c r="L302" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M302" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="N302" s="38" t="s">
+        <v>351</v>
+      </c>
       <c r="O302" s="41"/>
       <c r="P302" s="41"/>
       <c r="Q302" s="41"/>
@@ -17391,19 +17455,45 @@
     </row>
     <row r="303" spans="1:20" ht="18" customHeight="1">
       <c r="A303" s="53"/>
-      <c r="B303" s="53"/>
-      <c r="C303" s="53"/>
-      <c r="D303" s="53"/>
-      <c r="E303" s="51"/>
-      <c r="F303" s="89"/>
-      <c r="G303" s="31"/>
-      <c r="H303" s="53"/>
-      <c r="I303" s="36"/>
-      <c r="J303" s="41"/>
-      <c r="K303" s="41"/>
-      <c r="L303" s="53"/>
-      <c r="M303" s="53"/>
-      <c r="N303" s="38"/>
+      <c r="B303" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="C303" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="D303" s="53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E303" s="51" t="s">
+        <v>352</v>
+      </c>
+      <c r="F303" s="89" t="s">
+        <v>69</v>
+      </c>
+      <c r="G303" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H303" s="53" t="s">
+        <v>248</v>
+      </c>
+      <c r="I303" s="36">
+        <v>298</v>
+      </c>
+      <c r="J303" s="41">
+        <v>19.7</v>
+      </c>
+      <c r="K303" s="41">
+        <v>0.9</v>
+      </c>
+      <c r="L303" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="M303" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="N303" s="38" t="s">
+        <v>351</v>
+      </c>
       <c r="O303" s="41"/>
       <c r="P303" s="41"/>
       <c r="Q303" s="41"/>
@@ -17413,19 +17503,41 @@
     </row>
     <row r="304" spans="1:20" ht="18" customHeight="1">
       <c r="A304" s="53"/>
-      <c r="B304" s="88"/>
-      <c r="C304" s="89"/>
-      <c r="D304" s="89"/>
-      <c r="E304" s="100"/>
-      <c r="F304" s="53"/>
-      <c r="G304" s="31"/>
-      <c r="H304" s="53"/>
-      <c r="I304" s="36"/>
-      <c r="J304" s="41"/>
+      <c r="B304" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="C304" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="D304" s="53" t="s">
+        <v>164</v>
+      </c>
+      <c r="E304" s="51" t="s">
+        <v>350</v>
+      </c>
+      <c r="F304" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="G304" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H304" s="53" t="s">
+        <v>248</v>
+      </c>
+      <c r="I304" s="36">
+        <v>298</v>
+      </c>
+      <c r="J304" s="41">
+        <v>16</v>
+      </c>
       <c r="K304" s="41"/>
-      <c r="L304" s="53"/>
+      <c r="L304" s="53" t="s">
+        <v>66</v>
+      </c>
       <c r="M304" s="53"/>
-      <c r="N304" s="38"/>
+      <c r="N304" s="38" t="s">
+        <v>351</v>
+      </c>
       <c r="O304" s="41"/>
       <c r="P304" s="41"/>
       <c r="Q304" s="41"/>
@@ -31595,11 +31707,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:L8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="P8:T8"/>
     <mergeCell ref="D2:E3"/>
     <mergeCell ref="F2:N3"/>
     <mergeCell ref="C5:C6"/>
@@ -31614,6 +31721,11 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
+    <mergeCell ref="O5:O7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="P8:T8"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.msea.2019.138192`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6298A2F7-91AC-1D41-9F5C-C4B9CF0737B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99AFA67-1EAC-644E-B7F1-31DF4D772849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2861" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2977" uniqueCount="367">
   <si>
     <r>
       <rPr>
@@ -1189,6 +1189,48 @@
   </si>
   <si>
     <t>drop cast into a copper mold for rectangular shape instead of button; average and SD from 3 tests</t>
+  </si>
+  <si>
+    <t>CoCrFeMnNi</t>
+  </si>
+  <si>
+    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99.9 Nd0.1</t>
+  </si>
+  <si>
+    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99.5 Nd0.5</t>
+  </si>
+  <si>
+    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99 Nd1</t>
+  </si>
+  <si>
+    <t>Nd0</t>
+  </si>
+  <si>
+    <t>Nd0.1</t>
+  </si>
+  <si>
+    <t>Nd0.5</t>
+  </si>
+  <si>
+    <t>Nd1.0</t>
+  </si>
+  <si>
+    <t>AAM+A+WQ+CR+A+WQ</t>
+  </si>
+  <si>
+    <t>FCC</t>
+  </si>
+  <si>
+    <t>FCC+HCP</t>
+  </si>
+  <si>
+    <t>cast samples annealed in argon at 1273K for 100h and water quenched then cold rolled to 80% reduction in 10 passes then annealed again in argon at 1173K for 1h and again water quenched; ductile fracture</t>
+  </si>
+  <si>
+    <t>cast samples annealed in argon at 1273K for 100h and water quenched then cold rolled to 80% reduction in 10 passes then annealed again in argon at 1173K for 1h and again water quenched; minor NdNiMn-rich HCP nanoprecipitates with 150% hardness of matrix; ductile fracture</t>
+  </si>
+  <si>
+    <t>10.1016/j.msea.2019.138192</t>
   </si>
 </sst>
 </file>
@@ -17546,20 +17588,42 @@
       <c r="T304" s="35"/>
     </row>
     <row r="305" spans="1:20" ht="18" customHeight="1">
-      <c r="A305" s="53"/>
-      <c r="B305" s="90"/>
-      <c r="C305" s="91"/>
-      <c r="D305" s="91"/>
-      <c r="E305" s="101"/>
-      <c r="F305" s="53"/>
-      <c r="G305" s="31"/>
+      <c r="A305" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B305" s="90" t="s">
+        <v>353</v>
+      </c>
+      <c r="C305" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D305" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E305" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F305" s="53" t="s">
+        <v>67</v>
+      </c>
+      <c r="G305" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H305" s="53"/>
-      <c r="I305" s="36"/>
-      <c r="J305" s="41"/>
+      <c r="I305" s="36">
+        <v>298</v>
+      </c>
+      <c r="J305" s="54">
+        <v>226000000</v>
+      </c>
       <c r="K305" s="41"/>
-      <c r="L305" s="53"/>
+      <c r="L305" s="53" t="s">
+        <v>32</v>
+      </c>
       <c r="M305" s="53"/>
-      <c r="N305" s="38"/>
+      <c r="N305" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O305" s="41"/>
       <c r="P305" s="41"/>
       <c r="Q305" s="41"/>
@@ -17568,20 +17632,42 @@
       <c r="T305" s="35"/>
     </row>
     <row r="306" spans="1:20" ht="18" customHeight="1">
-      <c r="A306" s="53"/>
-      <c r="B306" s="90"/>
-      <c r="C306" s="91"/>
-      <c r="D306" s="91"/>
-      <c r="E306" s="101"/>
-      <c r="F306" s="53"/>
-      <c r="G306" s="31"/>
+      <c r="A306" s="53" t="s">
+        <v>358</v>
+      </c>
+      <c r="B306" s="90" t="s">
+        <v>354</v>
+      </c>
+      <c r="C306" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D306" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E306" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F306" s="53" t="s">
+        <v>67</v>
+      </c>
+      <c r="G306" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H306" s="53"/>
-      <c r="I306" s="36"/>
-      <c r="J306" s="41"/>
+      <c r="I306" s="36">
+        <v>298</v>
+      </c>
+      <c r="J306" s="54">
+        <v>219000000</v>
+      </c>
       <c r="K306" s="41"/>
-      <c r="L306" s="53"/>
+      <c r="L306" s="53" t="s">
+        <v>32</v>
+      </c>
       <c r="M306" s="53"/>
-      <c r="N306" s="38"/>
+      <c r="N306" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O306" s="41"/>
       <c r="P306" s="41"/>
       <c r="Q306" s="41"/>
@@ -17590,20 +17676,42 @@
       <c r="T306" s="35"/>
     </row>
     <row r="307" spans="1:20" ht="18" customHeight="1">
-      <c r="A307" s="53"/>
-      <c r="B307" s="90"/>
-      <c r="C307" s="91"/>
-      <c r="D307" s="91"/>
-      <c r="E307" s="101"/>
-      <c r="F307" s="53"/>
-      <c r="G307" s="31"/>
+      <c r="A307" s="53" t="s">
+        <v>359</v>
+      </c>
+      <c r="B307" s="90" t="s">
+        <v>355</v>
+      </c>
+      <c r="C307" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D307" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E307" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F307" s="53" t="s">
+        <v>67</v>
+      </c>
+      <c r="G307" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H307" s="53"/>
-      <c r="I307" s="36"/>
-      <c r="J307" s="41"/>
+      <c r="I307" s="36">
+        <v>298</v>
+      </c>
+      <c r="J307" s="54">
+        <v>270000000</v>
+      </c>
       <c r="K307" s="41"/>
-      <c r="L307" s="53"/>
+      <c r="L307" s="53" t="s">
+        <v>32</v>
+      </c>
       <c r="M307" s="53"/>
-      <c r="N307" s="38"/>
+      <c r="N307" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O307" s="41"/>
       <c r="P307" s="41"/>
       <c r="Q307" s="41"/>
@@ -17612,20 +17720,42 @@
       <c r="T307" s="35"/>
     </row>
     <row r="308" spans="1:20" ht="18" customHeight="1">
-      <c r="A308" s="53"/>
-      <c r="B308" s="90"/>
-      <c r="C308" s="91"/>
-      <c r="D308" s="91"/>
-      <c r="E308" s="101"/>
-      <c r="F308" s="53"/>
-      <c r="G308" s="31"/>
+      <c r="A308" s="53" t="s">
+        <v>360</v>
+      </c>
+      <c r="B308" s="90" t="s">
+        <v>356</v>
+      </c>
+      <c r="C308" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D308" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E308" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F308" s="53" t="s">
+        <v>67</v>
+      </c>
+      <c r="G308" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H308" s="53"/>
-      <c r="I308" s="36"/>
-      <c r="J308" s="33"/>
+      <c r="I308" s="36">
+        <v>298</v>
+      </c>
+      <c r="J308" s="33">
+        <v>322000000</v>
+      </c>
       <c r="K308" s="41"/>
-      <c r="L308" s="53"/>
+      <c r="L308" s="53" t="s">
+        <v>32</v>
+      </c>
       <c r="M308" s="53"/>
-      <c r="N308" s="38"/>
+      <c r="N308" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O308" s="41"/>
       <c r="P308" s="41"/>
       <c r="Q308" s="41"/>
@@ -17634,20 +17764,44 @@
       <c r="T308" s="35"/>
     </row>
     <row r="309" spans="1:20" ht="18" customHeight="1">
-      <c r="A309" s="53"/>
-      <c r="B309" s="88"/>
-      <c r="C309" s="89"/>
-      <c r="D309" s="89"/>
-      <c r="E309" s="100"/>
-      <c r="F309" s="53"/>
-      <c r="G309" s="31"/>
+      <c r="A309" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B309" s="90" t="s">
+        <v>353</v>
+      </c>
+      <c r="C309" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D309" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E309" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F309" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="G309" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H309" s="53"/>
-      <c r="I309" s="36"/>
-      <c r="J309" s="33"/>
+      <c r="I309" s="36">
+        <v>298</v>
+      </c>
+      <c r="J309" s="33">
+        <v>587000000</v>
+      </c>
       <c r="K309" s="33"/>
-      <c r="L309" s="53"/>
-      <c r="M309" s="53"/>
-      <c r="N309" s="38"/>
+      <c r="L309" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M309" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N309" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O309" s="41"/>
       <c r="P309" s="41"/>
       <c r="Q309" s="41"/>
@@ -17656,20 +17810,44 @@
       <c r="T309" s="35"/>
     </row>
     <row r="310" spans="1:20" ht="18" customHeight="1">
-      <c r="A310" s="53"/>
-      <c r="B310" s="90"/>
-      <c r="C310" s="91"/>
-      <c r="D310" s="91"/>
-      <c r="E310" s="101"/>
-      <c r="F310" s="53"/>
-      <c r="G310" s="31"/>
+      <c r="A310" s="53" t="s">
+        <v>358</v>
+      </c>
+      <c r="B310" s="90" t="s">
+        <v>354</v>
+      </c>
+      <c r="C310" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D310" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E310" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F310" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="G310" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H310" s="53"/>
-      <c r="I310" s="36"/>
-      <c r="J310" s="33"/>
+      <c r="I310" s="36">
+        <v>298</v>
+      </c>
+      <c r="J310" s="33">
+        <v>581000000</v>
+      </c>
       <c r="K310" s="33"/>
-      <c r="L310" s="53"/>
-      <c r="M310" s="53"/>
-      <c r="N310" s="38"/>
+      <c r="L310" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M310" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N310" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O310" s="41"/>
       <c r="P310" s="41"/>
       <c r="Q310" s="41"/>
@@ -17678,20 +17856,44 @@
       <c r="T310" s="35"/>
     </row>
     <row r="311" spans="1:20" ht="18" customHeight="1">
-      <c r="A311" s="53"/>
-      <c r="B311" s="90"/>
-      <c r="C311" s="91"/>
-      <c r="D311" s="91"/>
-      <c r="E311" s="101"/>
-      <c r="F311" s="53"/>
-      <c r="G311" s="31"/>
+      <c r="A311" s="53" t="s">
+        <v>359</v>
+      </c>
+      <c r="B311" s="90" t="s">
+        <v>355</v>
+      </c>
+      <c r="C311" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D311" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E311" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F311" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="G311" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H311" s="53"/>
-      <c r="I311" s="36"/>
-      <c r="J311" s="33"/>
+      <c r="I311" s="36">
+        <v>298</v>
+      </c>
+      <c r="J311" s="33">
+        <v>707000000</v>
+      </c>
       <c r="K311" s="33"/>
-      <c r="L311" s="53"/>
-      <c r="M311" s="53"/>
-      <c r="N311" s="38"/>
+      <c r="L311" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M311" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N311" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O311" s="41"/>
       <c r="P311" s="41"/>
       <c r="Q311" s="41"/>
@@ -17700,20 +17902,44 @@
       <c r="T311" s="35"/>
     </row>
     <row r="312" spans="1:20" ht="18" customHeight="1">
-      <c r="A312" s="53"/>
-      <c r="B312" s="90"/>
-      <c r="C312" s="91"/>
-      <c r="D312" s="91"/>
-      <c r="E312" s="101"/>
-      <c r="F312" s="53"/>
-      <c r="G312" s="31"/>
+      <c r="A312" s="53" t="s">
+        <v>360</v>
+      </c>
+      <c r="B312" s="90" t="s">
+        <v>356</v>
+      </c>
+      <c r="C312" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D312" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E312" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F312" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="G312" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H312" s="53"/>
-      <c r="I312" s="36"/>
-      <c r="J312" s="33"/>
+      <c r="I312" s="36">
+        <v>298</v>
+      </c>
+      <c r="J312" s="33">
+        <v>819000000</v>
+      </c>
       <c r="K312" s="33"/>
-      <c r="L312" s="53"/>
-      <c r="M312" s="53"/>
-      <c r="N312" s="38"/>
+      <c r="L312" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="M312" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N312" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O312" s="41"/>
       <c r="P312" s="41"/>
       <c r="Q312" s="41"/>
@@ -17722,20 +17948,44 @@
       <c r="T312" s="35"/>
     </row>
     <row r="313" spans="1:20" ht="18" customHeight="1">
-      <c r="A313" s="53"/>
-      <c r="B313" s="90"/>
-      <c r="C313" s="91"/>
-      <c r="D313" s="91"/>
-      <c r="E313" s="101"/>
-      <c r="F313" s="53"/>
-      <c r="G313" s="31"/>
-      <c r="H313" s="53"/>
-      <c r="I313" s="36"/>
-      <c r="J313" s="41"/>
+      <c r="A313" s="88" t="s">
+        <v>357</v>
+      </c>
+      <c r="B313" s="91" t="s">
+        <v>353</v>
+      </c>
+      <c r="C313" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D313" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E313" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F313" s="89" t="s">
+        <v>69</v>
+      </c>
+      <c r="G313" s="92" t="s">
+        <v>28</v>
+      </c>
+      <c r="H313" s="89"/>
+      <c r="I313" s="117">
+        <v>298</v>
+      </c>
+      <c r="J313" s="41">
+        <v>65.7</v>
+      </c>
       <c r="K313" s="33"/>
-      <c r="L313" s="53"/>
-      <c r="M313" s="53"/>
-      <c r="N313" s="38"/>
+      <c r="L313" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="M313" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N313" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O313" s="41"/>
       <c r="P313" s="41"/>
       <c r="Q313" s="41"/>
@@ -17744,20 +17994,44 @@
       <c r="T313" s="35"/>
     </row>
     <row r="314" spans="1:20" ht="18" customHeight="1">
-      <c r="A314" s="53"/>
-      <c r="B314" s="88"/>
-      <c r="C314" s="89"/>
-      <c r="D314" s="53"/>
-      <c r="E314" s="53"/>
-      <c r="F314" s="53"/>
-      <c r="G314" s="31"/>
-      <c r="H314" s="53"/>
-      <c r="I314" s="41"/>
-      <c r="J314" s="41"/>
+      <c r="A314" s="90" t="s">
+        <v>358</v>
+      </c>
+      <c r="B314" s="91" t="s">
+        <v>354</v>
+      </c>
+      <c r="C314" s="91" t="s">
+        <v>362</v>
+      </c>
+      <c r="D314" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E314" s="101" t="s">
+        <v>364</v>
+      </c>
+      <c r="F314" s="89" t="s">
+        <v>69</v>
+      </c>
+      <c r="G314" s="93" t="s">
+        <v>28</v>
+      </c>
+      <c r="H314" s="91"/>
+      <c r="I314" s="119">
+        <v>298</v>
+      </c>
+      <c r="J314" s="41">
+        <v>56.4</v>
+      </c>
       <c r="K314" s="41"/>
-      <c r="L314" s="53"/>
-      <c r="M314" s="53"/>
-      <c r="N314" s="38"/>
+      <c r="L314" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="M314" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N314" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O314" s="41"/>
       <c r="P314" s="41"/>
       <c r="Q314" s="41"/>
@@ -17766,20 +18040,44 @@
       <c r="T314" s="35"/>
     </row>
     <row r="315" spans="1:20" ht="18" customHeight="1">
-      <c r="A315" s="53"/>
-      <c r="B315" s="90"/>
-      <c r="C315" s="91"/>
-      <c r="D315" s="53"/>
-      <c r="E315" s="53"/>
-      <c r="F315" s="53"/>
-      <c r="G315" s="31"/>
-      <c r="H315" s="53"/>
-      <c r="I315" s="41"/>
-      <c r="J315" s="41"/>
+      <c r="A315" s="90" t="s">
+        <v>359</v>
+      </c>
+      <c r="B315" s="91" t="s">
+        <v>355</v>
+      </c>
+      <c r="C315" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D315" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E315" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F315" s="89" t="s">
+        <v>69</v>
+      </c>
+      <c r="G315" s="93" t="s">
+        <v>28</v>
+      </c>
+      <c r="H315" s="91"/>
+      <c r="I315" s="119">
+        <v>298</v>
+      </c>
+      <c r="J315" s="41">
+        <v>46.1</v>
+      </c>
       <c r="K315" s="44"/>
-      <c r="L315" s="53"/>
-      <c r="M315" s="53"/>
-      <c r="N315" s="38"/>
+      <c r="L315" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="M315" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N315" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O315" s="41"/>
       <c r="P315" s="41"/>
       <c r="Q315" s="41"/>
@@ -17788,20 +18086,44 @@
       <c r="T315" s="35"/>
     </row>
     <row r="316" spans="1:20" ht="18" customHeight="1">
-      <c r="A316" s="53"/>
-      <c r="B316" s="90"/>
-      <c r="C316" s="91"/>
-      <c r="D316" s="53"/>
-      <c r="E316" s="53"/>
-      <c r="F316" s="53"/>
-      <c r="G316" s="31"/>
-      <c r="H316" s="53"/>
-      <c r="I316" s="41"/>
-      <c r="J316" s="41"/>
+      <c r="A316" s="90" t="s">
+        <v>360</v>
+      </c>
+      <c r="B316" s="91" t="s">
+        <v>356</v>
+      </c>
+      <c r="C316" s="91" t="s">
+        <v>363</v>
+      </c>
+      <c r="D316" s="91" t="s">
+        <v>361</v>
+      </c>
+      <c r="E316" s="101" t="s">
+        <v>365</v>
+      </c>
+      <c r="F316" s="89" t="s">
+        <v>69</v>
+      </c>
+      <c r="G316" s="93" t="s">
+        <v>28</v>
+      </c>
+      <c r="H316" s="91"/>
+      <c r="I316" s="119">
+        <v>298</v>
+      </c>
+      <c r="J316" s="41">
+        <v>34.200000000000003</v>
+      </c>
       <c r="K316" s="44"/>
-      <c r="L316" s="53"/>
-      <c r="M316" s="53"/>
-      <c r="N316" s="38"/>
+      <c r="L316" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="M316" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="N316" s="38" t="s">
+        <v>366</v>
+      </c>
       <c r="O316" s="41"/>
       <c r="P316" s="41"/>
       <c r="Q316" s="41"/>

</xml_diff>

<commit_message>
- composition bugfix in `10.1016/j.msea.2019.138192`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99AFA67-1EAC-644E-B7F1-31DF4D772849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443F67C5-EBEF-0A46-97E8-7A93DD7FBEEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1194,15 +1194,6 @@
     <t>CoCrFeMnNi</t>
   </si>
   <si>
-    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99.9 Nd0.1</t>
-  </si>
-  <si>
-    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99.5 Nd0.5</t>
-  </si>
-  <si>
-    <t>(Co20 Cr20 Fe20 Mn20 Ni20)99 Nd1</t>
-  </si>
-  <si>
     <t>Nd0</t>
   </si>
   <si>
@@ -1231,6 +1222,15 @@
   </si>
   <si>
     <t>10.1016/j.msea.2019.138192</t>
+  </si>
+  <si>
+    <t>(Co0.2 Cr0.2 Fe0.2 Mn0.2 Ni0.2)99.9 Nd0.1</t>
+  </si>
+  <si>
+    <t>(Co0.2 Cr0.2 Fe0.2 Mn0.2 Ni0.2)99.5 Nd0.5</t>
+  </si>
+  <si>
+    <t>(Co0.2 Cr0.2 Fe0.2 Mn0.2 Ni0.2)99 Nd1</t>
   </si>
 </sst>
 </file>
@@ -17589,19 +17589,19 @@
     </row>
     <row r="305" spans="1:20" ht="18" customHeight="1">
       <c r="A305" s="53" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B305" s="90" t="s">
         <v>353</v>
       </c>
       <c r="C305" s="91" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D305" s="91" t="s">
+        <v>358</v>
+      </c>
+      <c r="E305" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E305" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F305" s="53" t="s">
         <v>67</v>
@@ -17622,7 +17622,7 @@
       </c>
       <c r="M305" s="53"/>
       <c r="N305" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O305" s="41"/>
       <c r="P305" s="41"/>
@@ -17633,19 +17633,19 @@
     </row>
     <row r="306" spans="1:20" ht="18" customHeight="1">
       <c r="A306" s="53" t="s">
+        <v>355</v>
+      </c>
+      <c r="B306" s="90" t="s">
+        <v>364</v>
+      </c>
+      <c r="C306" s="91" t="s">
+        <v>359</v>
+      </c>
+      <c r="D306" s="91" t="s">
         <v>358</v>
       </c>
-      <c r="B306" s="90" t="s">
-        <v>354</v>
-      </c>
-      <c r="C306" s="91" t="s">
-        <v>362</v>
-      </c>
-      <c r="D306" s="91" t="s">
+      <c r="E306" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E306" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F306" s="53" t="s">
         <v>67</v>
@@ -17666,7 +17666,7 @@
       </c>
       <c r="M306" s="53"/>
       <c r="N306" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O306" s="41"/>
       <c r="P306" s="41"/>
@@ -17677,19 +17677,19 @@
     </row>
     <row r="307" spans="1:20" ht="18" customHeight="1">
       <c r="A307" s="53" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B307" s="90" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C307" s="91" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D307" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E307" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F307" s="53" t="s">
         <v>67</v>
@@ -17710,7 +17710,7 @@
       </c>
       <c r="M307" s="53"/>
       <c r="N307" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O307" s="41"/>
       <c r="P307" s="41"/>
@@ -17721,19 +17721,19 @@
     </row>
     <row r="308" spans="1:20" ht="18" customHeight="1">
       <c r="A308" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B308" s="90" t="s">
+        <v>366</v>
+      </c>
+      <c r="C308" s="91" t="s">
         <v>360</v>
       </c>
-      <c r="B308" s="90" t="s">
-        <v>356</v>
-      </c>
-      <c r="C308" s="91" t="s">
-        <v>363</v>
-      </c>
       <c r="D308" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E308" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F308" s="53" t="s">
         <v>67</v>
@@ -17754,7 +17754,7 @@
       </c>
       <c r="M308" s="53"/>
       <c r="N308" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O308" s="41"/>
       <c r="P308" s="41"/>
@@ -17765,19 +17765,19 @@
     </row>
     <row r="309" spans="1:20" ht="18" customHeight="1">
       <c r="A309" s="53" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B309" s="90" t="s">
         <v>353</v>
       </c>
       <c r="C309" s="91" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D309" s="91" t="s">
+        <v>358</v>
+      </c>
+      <c r="E309" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E309" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F309" s="53" t="s">
         <v>70</v>
@@ -17800,7 +17800,7 @@
         <v>115</v>
       </c>
       <c r="N309" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O309" s="41"/>
       <c r="P309" s="41"/>
@@ -17811,19 +17811,19 @@
     </row>
     <row r="310" spans="1:20" ht="18" customHeight="1">
       <c r="A310" s="53" t="s">
+        <v>355</v>
+      </c>
+      <c r="B310" s="90" t="s">
+        <v>364</v>
+      </c>
+      <c r="C310" s="91" t="s">
+        <v>359</v>
+      </c>
+      <c r="D310" s="91" t="s">
         <v>358</v>
       </c>
-      <c r="B310" s="90" t="s">
-        <v>354</v>
-      </c>
-      <c r="C310" s="91" t="s">
-        <v>362</v>
-      </c>
-      <c r="D310" s="91" t="s">
+      <c r="E310" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E310" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F310" s="53" t="s">
         <v>70</v>
@@ -17846,7 +17846,7 @@
         <v>115</v>
       </c>
       <c r="N310" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O310" s="41"/>
       <c r="P310" s="41"/>
@@ -17857,19 +17857,19 @@
     </row>
     <row r="311" spans="1:20" ht="18" customHeight="1">
       <c r="A311" s="53" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B311" s="90" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="C311" s="91" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D311" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E311" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F311" s="53" t="s">
         <v>70</v>
@@ -17892,7 +17892,7 @@
         <v>115</v>
       </c>
       <c r="N311" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O311" s="41"/>
       <c r="P311" s="41"/>
@@ -17903,19 +17903,19 @@
     </row>
     <row r="312" spans="1:20" ht="18" customHeight="1">
       <c r="A312" s="53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B312" s="90" t="s">
+        <v>366</v>
+      </c>
+      <c r="C312" s="91" t="s">
         <v>360</v>
       </c>
-      <c r="B312" s="90" t="s">
-        <v>356</v>
-      </c>
-      <c r="C312" s="91" t="s">
-        <v>363</v>
-      </c>
       <c r="D312" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E312" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F312" s="53" t="s">
         <v>70</v>
@@ -17938,7 +17938,7 @@
         <v>115</v>
       </c>
       <c r="N312" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O312" s="41"/>
       <c r="P312" s="41"/>
@@ -17949,19 +17949,19 @@
     </row>
     <row r="313" spans="1:20" ht="18" customHeight="1">
       <c r="A313" s="88" t="s">
-        <v>357</v>
-      </c>
-      <c r="B313" s="91" t="s">
+        <v>354</v>
+      </c>
+      <c r="B313" s="90" t="s">
         <v>353</v>
       </c>
       <c r="C313" s="91" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D313" s="91" t="s">
+        <v>358</v>
+      </c>
+      <c r="E313" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E313" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F313" s="89" t="s">
         <v>69</v>
@@ -17984,7 +17984,7 @@
         <v>115</v>
       </c>
       <c r="N313" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O313" s="41"/>
       <c r="P313" s="41"/>
@@ -17995,19 +17995,19 @@
     </row>
     <row r="314" spans="1:20" ht="18" customHeight="1">
       <c r="A314" s="90" t="s">
+        <v>355</v>
+      </c>
+      <c r="B314" s="90" t="s">
+        <v>364</v>
+      </c>
+      <c r="C314" s="91" t="s">
+        <v>359</v>
+      </c>
+      <c r="D314" s="91" t="s">
         <v>358</v>
       </c>
-      <c r="B314" s="91" t="s">
-        <v>354</v>
-      </c>
-      <c r="C314" s="91" t="s">
-        <v>362</v>
-      </c>
-      <c r="D314" s="91" t="s">
+      <c r="E314" s="101" t="s">
         <v>361</v>
-      </c>
-      <c r="E314" s="101" t="s">
-        <v>364</v>
       </c>
       <c r="F314" s="89" t="s">
         <v>69</v>
@@ -18030,7 +18030,7 @@
         <v>115</v>
       </c>
       <c r="N314" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O314" s="41"/>
       <c r="P314" s="41"/>
@@ -18041,19 +18041,19 @@
     </row>
     <row r="315" spans="1:20" ht="18" customHeight="1">
       <c r="A315" s="90" t="s">
-        <v>359</v>
-      </c>
-      <c r="B315" s="91" t="s">
-        <v>355</v>
+        <v>356</v>
+      </c>
+      <c r="B315" s="90" t="s">
+        <v>365</v>
       </c>
       <c r="C315" s="91" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D315" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E315" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F315" s="89" t="s">
         <v>69</v>
@@ -18076,7 +18076,7 @@
         <v>115</v>
       </c>
       <c r="N315" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O315" s="41"/>
       <c r="P315" s="41"/>
@@ -18087,19 +18087,19 @@
     </row>
     <row r="316" spans="1:20" ht="18" customHeight="1">
       <c r="A316" s="90" t="s">
+        <v>357</v>
+      </c>
+      <c r="B316" s="90" t="s">
+        <v>366</v>
+      </c>
+      <c r="C316" s="91" t="s">
         <v>360</v>
       </c>
-      <c r="B316" s="91" t="s">
-        <v>356</v>
-      </c>
-      <c r="C316" s="91" t="s">
-        <v>363</v>
-      </c>
       <c r="D316" s="91" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E316" s="101" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F316" s="89" t="s">
         <v>69</v>
@@ -18122,7 +18122,7 @@
         <v>115</v>
       </c>
       <c r="N316" s="38" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="O316" s="41"/>
       <c r="P316" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.corsci.2023.110979`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443F67C5-EBEF-0A46-97E8-7A93DD7FBEEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F6E330-7B9B-FD46-83FE-1C5DDE89E7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2977" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3018" uniqueCount="373">
   <si>
     <r>
       <rPr>
@@ -1231,6 +1231,24 @@
   </si>
   <si>
     <t>(Co0.2 Cr0.2 Fe0.2 Mn0.2 Ni0.2)99 Nd1</t>
+  </si>
+  <si>
+    <t>Fe Co Ni Cr Mo0.25 B0.237 Si0.137</t>
+  </si>
+  <si>
+    <t>Zr22.5 Ti22.5 Hf22.5 Ni22.5 Ta10</t>
+  </si>
+  <si>
+    <t>3.5 wt.% NaCl solution</t>
+  </si>
+  <si>
+    <t>passive current density</t>
+  </si>
+  <si>
+    <t>pitting potential</t>
+  </si>
+  <si>
+    <t>10.1016/j.corsci.2023.110979</t>
   </si>
 </sst>
 </file>
@@ -1410,7 +1428,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="58">
+  <borders count="63">
     <border>
       <left/>
       <right/>
@@ -2249,12 +2267,83 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA7A7A7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA7A7A7"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA7A7A7"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA7A7A7"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA7A7A7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA7A7A7"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2582,6 +2671,12 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -16873,7 +16968,9 @@
       <c r="G287" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H287" s="118"/>
+      <c r="H287" s="118" t="s">
+        <v>369</v>
+      </c>
       <c r="I287" s="119">
         <v>298</v>
       </c>
@@ -18133,19 +18230,39 @@
     </row>
     <row r="317" spans="1:20" ht="18" customHeight="1">
       <c r="A317" s="53"/>
-      <c r="B317" s="90"/>
-      <c r="C317" s="91"/>
-      <c r="D317" s="53"/>
-      <c r="E317" s="53"/>
-      <c r="F317" s="53"/>
-      <c r="G317" s="31"/>
+      <c r="B317" s="159" t="s">
+        <v>368</v>
+      </c>
+      <c r="C317" s="91" t="s">
+        <v>219</v>
+      </c>
+      <c r="D317" s="53" t="s">
+        <v>268</v>
+      </c>
+      <c r="E317" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="F317" s="53" t="s">
+        <v>265</v>
+      </c>
+      <c r="G317" s="31" t="s">
+        <v>28</v>
+      </c>
       <c r="H317" s="41"/>
       <c r="I317" s="41"/>
-      <c r="J317" s="41"/>
+      <c r="J317" s="41">
+        <v>745</v>
+      </c>
       <c r="K317" s="44"/>
-      <c r="L317" s="53"/>
-      <c r="M317" s="53"/>
-      <c r="N317" s="38"/>
+      <c r="L317" s="53" t="s">
+        <v>223</v>
+      </c>
+      <c r="M317" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="N317" s="38" t="s">
+        <v>372</v>
+      </c>
       <c r="O317" s="41"/>
       <c r="P317" s="41"/>
       <c r="Q317" s="41"/>
@@ -18155,19 +18272,43 @@
     </row>
     <row r="318" spans="1:20" ht="18" customHeight="1">
       <c r="A318" s="53"/>
-      <c r="B318" s="90"/>
-      <c r="C318" s="91"/>
-      <c r="D318" s="53"/>
-      <c r="E318" s="53"/>
-      <c r="F318" s="53"/>
-      <c r="G318" s="31"/>
-      <c r="H318" s="41"/>
-      <c r="I318" s="41"/>
-      <c r="J318" s="54"/>
+      <c r="B318" s="160" t="s">
+        <v>368</v>
+      </c>
+      <c r="C318" s="91" t="s">
+        <v>219</v>
+      </c>
+      <c r="D318" s="53" t="s">
+        <v>268</v>
+      </c>
+      <c r="E318" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="F318" s="53" t="s">
+        <v>370</v>
+      </c>
+      <c r="G318" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H318" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I318" s="41">
+        <v>298</v>
+      </c>
+      <c r="J318" s="54">
+        <v>3.6610000000000002E-3</v>
+      </c>
       <c r="K318" s="44"/>
-      <c r="L318" s="53"/>
-      <c r="M318" s="53"/>
-      <c r="N318" s="38"/>
+      <c r="L318" s="53" t="s">
+        <v>157</v>
+      </c>
+      <c r="M318" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N318" s="38" t="s">
+        <v>372</v>
+      </c>
       <c r="O318" s="41"/>
       <c r="P318" s="41"/>
       <c r="Q318" s="41"/>
@@ -18177,19 +18318,43 @@
     </row>
     <row r="319" spans="1:20" ht="18" customHeight="1">
       <c r="A319" s="53"/>
-      <c r="B319" s="88"/>
-      <c r="C319" s="89"/>
-      <c r="D319" s="53"/>
-      <c r="E319" s="53"/>
-      <c r="F319" s="53"/>
-      <c r="G319" s="31"/>
-      <c r="H319" s="41"/>
-      <c r="I319" s="41"/>
-      <c r="J319" s="54"/>
+      <c r="B319" s="160" t="s">
+        <v>368</v>
+      </c>
+      <c r="C319" s="91" t="s">
+        <v>219</v>
+      </c>
+      <c r="D319" s="53" t="s">
+        <v>268</v>
+      </c>
+      <c r="E319" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="F319" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="G319" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H319" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I319" s="41">
+        <v>298</v>
+      </c>
+      <c r="J319" s="54">
+        <v>-0.21</v>
+      </c>
       <c r="K319" s="44"/>
-      <c r="L319" s="53"/>
-      <c r="M319" s="53"/>
-      <c r="N319" s="38"/>
+      <c r="L319" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="M319" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N319" s="38" t="s">
+        <v>372</v>
+      </c>
       <c r="O319" s="41"/>
       <c r="P319" s="41"/>
       <c r="Q319" s="41"/>
@@ -18199,19 +18364,43 @@
     </row>
     <row r="320" spans="1:20" ht="18" customHeight="1">
       <c r="A320" s="53"/>
-      <c r="B320" s="90"/>
-      <c r="C320" s="91"/>
-      <c r="D320" s="53"/>
-      <c r="E320" s="53"/>
-      <c r="F320" s="53"/>
-      <c r="G320" s="31"/>
-      <c r="H320" s="41"/>
-      <c r="I320" s="41"/>
-      <c r="J320" s="54"/>
+      <c r="B320" s="158" t="s">
+        <v>368</v>
+      </c>
+      <c r="C320" s="161" t="s">
+        <v>219</v>
+      </c>
+      <c r="D320" s="162" t="s">
+        <v>268</v>
+      </c>
+      <c r="E320" s="162" t="s">
+        <v>275</v>
+      </c>
+      <c r="F320" s="53" t="s">
+        <v>371</v>
+      </c>
+      <c r="G320" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H320" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I320" s="41">
+        <v>298</v>
+      </c>
+      <c r="J320" s="54">
+        <v>0.28999999999999998</v>
+      </c>
       <c r="K320" s="44"/>
-      <c r="L320" s="53"/>
-      <c r="M320" s="53"/>
-      <c r="N320" s="38"/>
+      <c r="L320" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="M320" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="N320" s="38" t="s">
+        <v>372</v>
+      </c>
       <c r="O320" s="41"/>
       <c r="P320" s="41"/>
       <c r="Q320" s="41"/>
@@ -18221,10 +18410,12 @@
     </row>
     <row r="321" spans="1:20" ht="18" customHeight="1">
       <c r="A321" s="53"/>
-      <c r="B321" s="90"/>
+      <c r="B321" s="90" t="s">
+        <v>367</v>
+      </c>
       <c r="C321" s="91"/>
-      <c r="D321" s="53"/>
-      <c r="E321" s="53"/>
+      <c r="D321" s="157"/>
+      <c r="E321" s="157"/>
       <c r="F321" s="53"/>
       <c r="G321" s="31"/>
       <c r="H321" s="41"/>
@@ -18287,7 +18478,7 @@
     </row>
     <row r="324" spans="1:20" ht="18" customHeight="1">
       <c r="A324" s="53"/>
-      <c r="B324" s="88"/>
+      <c r="B324" s="90"/>
       <c r="C324" s="89"/>
       <c r="D324" s="89"/>
       <c r="E324" s="89"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.ijheatmasstransfer.2024.125628`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F6E330-7B9B-FD46-83FE-1C5DDE89E7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC59352-2812-F740-8827-8437E6D23C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3018" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3022" uniqueCount="377">
   <si>
     <r>
       <rPr>
@@ -1249,6 +1249,18 @@
   </si>
   <si>
     <t>10.1016/j.corsci.2023.110979</t>
+  </si>
+  <si>
+    <t>GA</t>
+  </si>
+  <si>
+    <t>gas atomized in bulk at 1650K in argon; VIGA-150-type atomization apparatus; estimated cooling rate of 10^5 K/s</t>
+  </si>
+  <si>
+    <t>FCC+FCC</t>
+  </si>
+  <si>
+    <t>10.1016/j.ijheatmasstransfer.2024.125628</t>
   </si>
 </sst>
 </file>
@@ -18413,9 +18425,15 @@
       <c r="B321" s="90" t="s">
         <v>367</v>
       </c>
-      <c r="C321" s="91"/>
-      <c r="D321" s="157"/>
-      <c r="E321" s="157"/>
+      <c r="C321" s="91" t="s">
+        <v>375</v>
+      </c>
+      <c r="D321" s="157" t="s">
+        <v>373</v>
+      </c>
+      <c r="E321" s="157" t="s">
+        <v>374</v>
+      </c>
       <c r="F321" s="53"/>
       <c r="G321" s="31"/>
       <c r="H321" s="41"/>
@@ -18424,7 +18442,9 @@
       <c r="K321" s="44"/>
       <c r="L321" s="53"/>
       <c r="M321" s="53"/>
-      <c r="N321" s="38"/>
+      <c r="N321" s="38" t="s">
+        <v>376</v>
+      </c>
       <c r="O321" s="41"/>
       <c r="P321" s="41"/>
       <c r="Q321" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1016/j.jmrt.2023.11.247`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC59352-2812-F740-8827-8437E6D23C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF4629C-3AF2-C840-AB97-1E92AF552C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3022" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3090" uniqueCount="381">
   <si>
     <r>
       <rPr>
@@ -1261,6 +1261,18 @@
   </si>
   <si>
     <t>10.1016/j.ijheatmasstransfer.2024.125628</t>
+  </si>
+  <si>
+    <t>Cr Nb Ta Ti V</t>
+  </si>
+  <si>
+    <t>Nb Ta Ti V</t>
+  </si>
+  <si>
+    <t>minor hexagonal laves phase detected between dendrites</t>
+  </si>
+  <si>
+    <t>10.1016/j.jmrt.2023.11.247</t>
   </si>
 </sst>
 </file>
@@ -1440,7 +1452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="63">
+  <borders count="65">
     <border>
       <left/>
       <right/>
@@ -2280,6 +2292,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFA7A7A7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color theme="3"/>
       </left>
@@ -2350,12 +2371,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2683,12 +2715,14 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -18242,7 +18276,7 @@
     </row>
     <row r="317" spans="1:20" ht="18" customHeight="1">
       <c r="A317" s="53"/>
-      <c r="B317" s="159" t="s">
+      <c r="B317" s="160" t="s">
         <v>368</v>
       </c>
       <c r="C317" s="91" t="s">
@@ -18284,7 +18318,7 @@
     </row>
     <row r="318" spans="1:20" ht="18" customHeight="1">
       <c r="A318" s="53"/>
-      <c r="B318" s="160" t="s">
+      <c r="B318" s="161" t="s">
         <v>368</v>
       </c>
       <c r="C318" s="91" t="s">
@@ -18330,7 +18364,7 @@
     </row>
     <row r="319" spans="1:20" ht="18" customHeight="1">
       <c r="A319" s="53"/>
-      <c r="B319" s="160" t="s">
+      <c r="B319" s="161" t="s">
         <v>368</v>
       </c>
       <c r="C319" s="91" t="s">
@@ -18376,16 +18410,16 @@
     </row>
     <row r="320" spans="1:20" ht="18" customHeight="1">
       <c r="A320" s="53"/>
-      <c r="B320" s="158" t="s">
+      <c r="B320" s="159" t="s">
         <v>368</v>
       </c>
-      <c r="C320" s="161" t="s">
+      <c r="C320" s="162" t="s">
         <v>219</v>
       </c>
-      <c r="D320" s="162" t="s">
+      <c r="D320" s="163" t="s">
         <v>268</v>
       </c>
-      <c r="E320" s="162" t="s">
+      <c r="E320" s="163" t="s">
         <v>275</v>
       </c>
       <c r="F320" s="53" t="s">
@@ -18428,10 +18462,10 @@
       <c r="C321" s="91" t="s">
         <v>375</v>
       </c>
-      <c r="D321" s="157" t="s">
+      <c r="D321" s="158" t="s">
         <v>373</v>
       </c>
-      <c r="E321" s="157" t="s">
+      <c r="E321" s="158" t="s">
         <v>374</v>
       </c>
       <c r="F321" s="53"/>
@@ -18454,19 +18488,39 @@
     </row>
     <row r="322" spans="1:20" ht="18" customHeight="1">
       <c r="A322" s="53"/>
-      <c r="B322" s="90"/>
-      <c r="C322" s="91"/>
-      <c r="D322" s="53"/>
+      <c r="B322" s="90" t="s">
+        <v>378</v>
+      </c>
+      <c r="C322" s="157" t="s">
+        <v>63</v>
+      </c>
+      <c r="D322" s="91" t="s">
+        <v>108</v>
+      </c>
       <c r="E322" s="53"/>
-      <c r="F322" s="53"/>
-      <c r="G322" s="31"/>
-      <c r="H322" s="41"/>
-      <c r="I322" s="41"/>
-      <c r="J322" s="54"/>
+      <c r="F322" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="G322" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H322" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I322" s="41">
+        <v>298</v>
+      </c>
+      <c r="J322" s="54">
+        <v>-0.35</v>
+      </c>
       <c r="K322" s="44"/>
-      <c r="L322" s="53"/>
+      <c r="L322" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="M322" s="53"/>
-      <c r="N322" s="38"/>
+      <c r="N322" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O322" s="41"/>
       <c r="P322" s="41"/>
       <c r="Q322" s="41"/>
@@ -18476,19 +18530,41 @@
     </row>
     <row r="323" spans="1:20" ht="18" customHeight="1">
       <c r="A323" s="53"/>
-      <c r="B323" s="90"/>
-      <c r="C323" s="91"/>
-      <c r="D323" s="53"/>
-      <c r="E323" s="53"/>
-      <c r="F323" s="53"/>
-      <c r="G323" s="31"/>
-      <c r="H323" s="41"/>
-      <c r="I323" s="41"/>
-      <c r="J323" s="41"/>
+      <c r="B323" s="90" t="s">
+        <v>377</v>
+      </c>
+      <c r="C323" s="91" t="s">
+        <v>173</v>
+      </c>
+      <c r="D323" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E323" s="53" t="s">
+        <v>379</v>
+      </c>
+      <c r="F323" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="G323" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H323" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I323" s="41">
+        <v>298</v>
+      </c>
+      <c r="J323" s="41">
+        <v>-0.44</v>
+      </c>
       <c r="K323" s="44"/>
-      <c r="L323" s="53"/>
+      <c r="L323" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="M323" s="53"/>
-      <c r="N323" s="38"/>
+      <c r="N323" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O323" s="41"/>
       <c r="P323" s="41"/>
       <c r="Q323" s="41"/>
@@ -18498,19 +18574,39 @@
     </row>
     <row r="324" spans="1:20" ht="18" customHeight="1">
       <c r="A324" s="53"/>
-      <c r="B324" s="90"/>
-      <c r="C324" s="89"/>
-      <c r="D324" s="89"/>
-      <c r="E324" s="89"/>
-      <c r="F324" s="89"/>
-      <c r="G324" s="92"/>
-      <c r="H324" s="41"/>
-      <c r="I324" s="41"/>
-      <c r="J324" s="41"/>
+      <c r="B324" s="90" t="s">
+        <v>378</v>
+      </c>
+      <c r="C324" s="157" t="s">
+        <v>63</v>
+      </c>
+      <c r="D324" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E324" s="53"/>
+      <c r="F324" s="89" t="s">
+        <v>155</v>
+      </c>
+      <c r="G324" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H324" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I324" s="41">
+        <v>298</v>
+      </c>
+      <c r="J324" s="41">
+        <v>4.3600000000000002E-3</v>
+      </c>
       <c r="K324" s="44"/>
-      <c r="L324" s="53"/>
+      <c r="L324" s="53" t="s">
+        <v>157</v>
+      </c>
       <c r="M324" s="53"/>
-      <c r="N324" s="38"/>
+      <c r="N324" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O324" s="41"/>
       <c r="P324" s="41"/>
       <c r="Q324" s="41"/>
@@ -18520,19 +18616,41 @@
     </row>
     <row r="325" spans="1:20" ht="18" customHeight="1">
       <c r="A325" s="53"/>
-      <c r="B325" s="90"/>
-      <c r="C325" s="91"/>
-      <c r="D325" s="91"/>
-      <c r="E325" s="91"/>
-      <c r="F325" s="89"/>
-      <c r="G325" s="93"/>
-      <c r="H325" s="41"/>
-      <c r="I325" s="41"/>
-      <c r="J325" s="41"/>
+      <c r="B325" s="90" t="s">
+        <v>377</v>
+      </c>
+      <c r="C325" s="91" t="s">
+        <v>173</v>
+      </c>
+      <c r="D325" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E325" s="53" t="s">
+        <v>379</v>
+      </c>
+      <c r="F325" s="89" t="s">
+        <v>155</v>
+      </c>
+      <c r="G325" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H325" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I325" s="41">
+        <v>298</v>
+      </c>
+      <c r="J325" s="41">
+        <v>7.8799999999999999E-3</v>
+      </c>
       <c r="K325" s="44"/>
-      <c r="L325" s="53"/>
+      <c r="L325" s="53" t="s">
+        <v>157</v>
+      </c>
       <c r="M325" s="53"/>
-      <c r="N325" s="38"/>
+      <c r="N325" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O325" s="41"/>
       <c r="P325" s="41"/>
       <c r="Q325" s="41"/>
@@ -18542,19 +18660,39 @@
     </row>
     <row r="326" spans="1:20" ht="18" customHeight="1">
       <c r="A326" s="53"/>
-      <c r="B326" s="90"/>
-      <c r="C326" s="91"/>
-      <c r="D326" s="91"/>
-      <c r="E326" s="91"/>
-      <c r="F326" s="89"/>
-      <c r="G326" s="93"/>
-      <c r="H326" s="41"/>
-      <c r="I326" s="41"/>
-      <c r="J326" s="41"/>
+      <c r="B326" s="90" t="s">
+        <v>378</v>
+      </c>
+      <c r="C326" s="157" t="s">
+        <v>63</v>
+      </c>
+      <c r="D326" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E326" s="53"/>
+      <c r="F326" s="89" t="s">
+        <v>370</v>
+      </c>
+      <c r="G326" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H326" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I326" s="41">
+        <v>298</v>
+      </c>
+      <c r="J326" s="41">
+        <v>5.4800000000000001E-2</v>
+      </c>
       <c r="K326" s="44"/>
-      <c r="L326" s="53"/>
+      <c r="L326" s="53" t="s">
+        <v>157</v>
+      </c>
       <c r="M326" s="53"/>
-      <c r="N326" s="38"/>
+      <c r="N326" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O326" s="41"/>
       <c r="P326" s="41"/>
       <c r="Q326" s="41"/>
@@ -18564,19 +18702,41 @@
     </row>
     <row r="327" spans="1:20" ht="18" customHeight="1">
       <c r="A327" s="53"/>
-      <c r="B327" s="90"/>
-      <c r="C327" s="91"/>
-      <c r="D327" s="91"/>
-      <c r="E327" s="91"/>
-      <c r="F327" s="89"/>
-      <c r="G327" s="93"/>
-      <c r="H327" s="41"/>
-      <c r="I327" s="41"/>
-      <c r="J327" s="41"/>
+      <c r="B327" s="90" t="s">
+        <v>377</v>
+      </c>
+      <c r="C327" s="91" t="s">
+        <v>173</v>
+      </c>
+      <c r="D327" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E327" s="53" t="s">
+        <v>379</v>
+      </c>
+      <c r="F327" s="89" t="s">
+        <v>370</v>
+      </c>
+      <c r="G327" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H327" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I327" s="41">
+        <v>298</v>
+      </c>
+      <c r="J327" s="41">
+        <v>0.1321</v>
+      </c>
       <c r="K327" s="44"/>
-      <c r="L327" s="53"/>
+      <c r="L327" s="53" t="s">
+        <v>157</v>
+      </c>
       <c r="M327" s="53"/>
-      <c r="N327" s="38"/>
+      <c r="N327" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O327" s="41"/>
       <c r="P327" s="41"/>
       <c r="Q327" s="41"/>
@@ -18586,19 +18746,39 @@
     </row>
     <row r="328" spans="1:20" ht="18" customHeight="1">
       <c r="A328" s="53"/>
-      <c r="B328" s="90"/>
-      <c r="C328" s="91"/>
-      <c r="D328" s="91"/>
-      <c r="E328" s="91"/>
-      <c r="F328" s="89"/>
-      <c r="G328" s="93"/>
-      <c r="H328" s="41"/>
-      <c r="I328" s="41"/>
-      <c r="J328" s="41"/>
+      <c r="B328" s="90" t="s">
+        <v>378</v>
+      </c>
+      <c r="C328" s="157" t="s">
+        <v>63</v>
+      </c>
+      <c r="D328" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E328" s="53"/>
+      <c r="F328" s="89" t="s">
+        <v>371</v>
+      </c>
+      <c r="G328" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H328" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I328" s="41">
+        <v>298</v>
+      </c>
+      <c r="J328" s="41">
+        <v>1.94</v>
+      </c>
       <c r="K328" s="44"/>
-      <c r="L328" s="53"/>
+      <c r="L328" s="164" t="s">
+        <v>156</v>
+      </c>
       <c r="M328" s="53"/>
-      <c r="N328" s="38"/>
+      <c r="N328" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O328" s="41"/>
       <c r="P328" s="41"/>
       <c r="Q328" s="41"/>
@@ -18608,19 +18788,41 @@
     </row>
     <row r="329" spans="1:20" ht="18" customHeight="1">
       <c r="A329" s="41"/>
-      <c r="B329" s="53"/>
-      <c r="C329" s="53"/>
-      <c r="D329" s="53"/>
-      <c r="E329" s="53"/>
-      <c r="F329" s="53"/>
-      <c r="G329" s="31"/>
-      <c r="H329" s="41"/>
-      <c r="I329" s="41"/>
-      <c r="J329" s="41"/>
+      <c r="B329" s="90" t="s">
+        <v>377</v>
+      </c>
+      <c r="C329" s="91" t="s">
+        <v>173</v>
+      </c>
+      <c r="D329" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E329" s="53" t="s">
+        <v>379</v>
+      </c>
+      <c r="F329" s="53" t="s">
+        <v>371</v>
+      </c>
+      <c r="G329" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H329" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="I329" s="41">
+        <v>298</v>
+      </c>
+      <c r="J329" s="41">
+        <v>1.52</v>
+      </c>
       <c r="K329" s="44"/>
-      <c r="L329" s="53"/>
+      <c r="L329" s="53" t="s">
+        <v>156</v>
+      </c>
       <c r="M329" s="53"/>
-      <c r="N329" s="38"/>
+      <c r="N329" s="38" t="s">
+        <v>380</v>
+      </c>
       <c r="O329" s="41"/>
       <c r="P329" s="41"/>
       <c r="Q329" s="41"/>

</xml_diff>

<commit_message>
- parsed data from `10.1007/s12613-024-2933-5`
</commit_message>
<xml_diff>
--- a/MiscSmallUploads_Spring2026.xlsx
+++ b/MiscSmallUploads_Spring2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/VSCode Projects/ULTERA-contribute-amkrajewski/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF4629C-3AF2-C840-AB97-1E92AF552C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E787184-83B4-D34B-A26A-EDA2B071896A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="9940" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="4000" windowWidth="34560" windowHeight="9780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3090" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3095" uniqueCount="384">
   <si>
     <r>
       <rPr>
@@ -1273,6 +1273,15 @@
   </si>
   <si>
     <t>10.1016/j.jmrt.2023.11.247</t>
+  </si>
+  <si>
+    <t>Y Gd Tb Dy Ho</t>
+  </si>
+  <si>
+    <t>excellent hydrogen storage of 2.33wt% resulting in FCC hydride (Y Gd Tb Dy Ho)4.48 H77.62</t>
+  </si>
+  <si>
+    <t>10.1007/s12613-024-2933-5</t>
   </si>
 </sst>
 </file>
@@ -18832,10 +18841,18 @@
     </row>
     <row r="330" spans="1:20" ht="18" customHeight="1">
       <c r="A330" s="41"/>
-      <c r="B330" s="53"/>
-      <c r="C330" s="53"/>
-      <c r="D330" s="53"/>
-      <c r="E330" s="53"/>
+      <c r="B330" s="53" t="s">
+        <v>381</v>
+      </c>
+      <c r="C330" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="D330" s="53" t="s">
+        <v>108</v>
+      </c>
+      <c r="E330" s="53" t="s">
+        <v>382</v>
+      </c>
       <c r="F330" s="53"/>
       <c r="G330" s="31"/>
       <c r="H330" s="41"/>
@@ -18844,7 +18861,9 @@
       <c r="K330" s="44"/>
       <c r="L330" s="53"/>
       <c r="M330" s="53"/>
-      <c r="N330" s="53"/>
+      <c r="N330" s="53" t="s">
+        <v>383</v>
+      </c>
       <c r="O330" s="41"/>
       <c r="P330" s="41"/>
       <c r="Q330" s="41"/>

</xml_diff>